<commit_message>
Add explicit date picker validation to all four semester date cells
Sem 1 and Sem 2 start/end date cells now have DataValidation(type='date')
applied, which is what tells Excel to show the calendar picker popup.
Previously only MM/DD/YYYY number format was set (which handles display
but not the picker in older Excel versions).

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -1310,6 +1310,16 @@
     <mergeCell ref="A2:J2"/>
     <mergeCell ref="G15:J15"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="C10:F10 C11:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="date" operator="between">
+      <formula1>DATE(2000,1,1)</formula1>
+      <formula2>DATE(2099,12,31)</formula2>
+    </dataValidation>
+    <dataValidation sqref="C15:F15 C16:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="date" operator="between">
+      <formula1>DATE(2000,1,1)</formula1>
+      <formula2>DATE(2099,12,31)</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix grade formula: handle empty S2 end date
When C19 (S2 End Date) is blank, Excel treated it as year 1900, producing
nonsense grades. Formula now falls back to: (1) last 4 chars of the School
Year text field, then (2) YEAR(TODAY()) as a last resort.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -1184,7 +1184,7 @@
       <c r="D29" s="7" t="n"/>
       <c r="E29" s="16" t="n"/>
       <c r="F29" s="17">
-        <f>IF(OR(B29="",E29=""),"",LET(g,12-(E29-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B29="",E29=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E29-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G29" s="5" t="n"/>
@@ -1197,7 +1197,7 @@
       <c r="D30" s="19" t="n"/>
       <c r="E30" s="20" t="n"/>
       <c r="F30" s="17">
-        <f>IF(OR(B30="",E30=""),"",LET(g,12-(E30-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B30="",E30=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E30-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G30" s="18" t="n"/>
@@ -1210,7 +1210,7 @@
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="16" t="n"/>
       <c r="F31" s="17">
-        <f>IF(OR(B31="",E31=""),"",LET(g,12-(E31-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B31="",E31=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E31-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G31" s="5" t="n"/>
@@ -1223,7 +1223,7 @@
       <c r="D32" s="19" t="n"/>
       <c r="E32" s="20" t="n"/>
       <c r="F32" s="17">
-        <f>IF(OR(B32="",E32=""),"",LET(g,12-(E32-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B32="",E32=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E32-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G32" s="18" t="n"/>
@@ -1236,7 +1236,7 @@
       <c r="D33" s="7" t="n"/>
       <c r="E33" s="16" t="n"/>
       <c r="F33" s="17">
-        <f>IF(OR(B33="",E33=""),"",LET(g,12-(E33-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B33="",E33=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E33-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G33" s="5" t="n"/>
@@ -1249,7 +1249,7 @@
       <c r="D34" s="19" t="n"/>
       <c r="E34" s="20" t="n"/>
       <c r="F34" s="17">
-        <f>IF(OR(B34="",E34=""),"",LET(g,12-(E34-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B34="",E34=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E34-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G34" s="18" t="n"/>
@@ -1262,7 +1262,7 @@
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="16" t="n"/>
       <c r="F35" s="17">
-        <f>IF(OR(B35="",E35=""),"",LET(g,12-(E35-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B35="",E35=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E35-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G35" s="5" t="n"/>
@@ -1275,7 +1275,7 @@
       <c r="D36" s="19" t="n"/>
       <c r="E36" s="20" t="n"/>
       <c r="F36" s="17">
-        <f>IF(OR(B36="",E36=""),"",LET(g,12-(E36-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B36="",E36=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E36-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G36" s="18" t="n"/>
@@ -1288,7 +1288,7 @@
       <c r="D37" s="7" t="n"/>
       <c r="E37" s="16" t="n"/>
       <c r="F37" s="17">
-        <f>IF(OR(B37="",E37=""),"",LET(g,12-(E37-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B37="",E37=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E37-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G37" s="5" t="n"/>
@@ -1301,7 +1301,7 @@
       <c r="D38" s="19" t="n"/>
       <c r="E38" s="20" t="n"/>
       <c r="F38" s="17">
-        <f>IF(OR(B38="",E38=""),"",LET(g,12-(E38-YEAR($C$19)),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
+        <f>IF(OR(B38="",E38=""),"",LET(yr,IF($C$19&lt;&gt;"",YEAR($C$19),IF($C$6&lt;&gt;"",VALUE(RIGHT($C$6,4)),YEAR(TODAY()))),g,12-(E38-yr),IF(g=11,"11th",IF(g=12,"12th",IF(g=1,"1st",IF(g=2,"2nd",IF(g=3,"3rd",g&amp;"th")))))))</f>
         <v/>
       </c>
       <c r="G38" s="18" t="n"/>

</xml_diff>

<commit_message>
Add unit type dropdown: pages, lessons, chapters, units, assignments, projects
Both curriculum slots on every subject row (Group Studies + all 10
student sections) now have a dropdown instead of the hardcoded 'pages'.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -5163,6 +5163,11 @@
     <mergeCell ref="A151:J151"/>
     <mergeCell ref="A71:J71"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C56 C57 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67 C68 C69 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C83 C84 C85 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C104 C105 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C120 C121 C122 C123 C124 C125 C126 C127 C128 C129 C130 C131 C132 C133 C136 C137 C138 C139 C140 C141 C142 C143 C144 C145 C146 C147 C148 C149 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C162 C163 C164 C165 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H120 H121 H122 H123 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H146 H147 H148 H149 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"pages,lessons,chapters,units,assignments,projects"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 10 distinct student colors + restore Student 1 tab
- Each student gets a unique, print-friendly color (dusty rose, sage,
  sky blue, amber, lavender, teal, terracotta, periwinkle, olive, plum)
- Course Content student header rows use the matching color per student
- Student 1 tab banner and sheet tab use the same color
- CC->student sheet references updated to new column layout (Slot 1)
- When remaining student tabs are added they'll pull from STUDENT_COLORS

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Getting Started" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Course Content" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Student 1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="MM/DD/YYYY"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,8 +117,64 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005C7A52"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FAF8F6"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008A6A30"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="006B5C55"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005C7A52"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="005C7A52"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="008A6A30"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="008A6A30"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="006B5C55"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -184,8 +241,74 @@
         <bgColor rgb="00F5EDE3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007A9E7E"/>
+        <bgColor rgb="007A9E7E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007AA0C4"/>
+        <bgColor rgb="007AA0C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C4A462"/>
+        <bgColor rgb="00C4A462"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009B8EC4"/>
+        <bgColor rgb="009B8EC4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006AADA6"/>
+        <bgColor rgb="006AADA6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C47A6A"/>
+        <bgColor rgb="00C47A6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007A8EC4"/>
+        <bgColor rgb="007A8EC4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008FA87A"/>
+        <bgColor rgb="008FA87A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A87A9E"/>
+        <bgColor rgb="00A87A9E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005C7A52"/>
+        <bgColor rgb="005C7A52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008A6A30"/>
+        <bgColor rgb="008A6A30"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -221,11 +344,16 @@
         <color rgb="00D4C4BB"/>
       </bottom>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D4C4BB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -330,7 +458,88 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1261,7 +1470,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00A08878"/>
+    <tabColor rgb="006B5C55"/>
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2400,7 +2609,7 @@
     </row>
     <row r="54" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="36">
+      <c r="A55" s="37">
         <f>IF('Getting Started'!B31&lt;&gt;"","  "&amp;UPPER('Getting Started'!B31)&amp;"   ·   "&amp;'Getting Started'!F31,"  STUDENT 3")</f>
         <v/>
       </c>
@@ -2743,7 +2952,7 @@
     </row>
     <row r="70" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="71" ht="26" customHeight="1">
-      <c r="A71" s="36">
+      <c r="A71" s="38">
         <f>IF('Getting Started'!B32&lt;&gt;"","  "&amp;UPPER('Getting Started'!B32)&amp;"   ·   "&amp;'Getting Started'!F32,"  STUDENT 4")</f>
         <v/>
       </c>
@@ -3086,7 +3295,7 @@
     </row>
     <row r="86" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="87" ht="26" customHeight="1">
-      <c r="A87" s="36">
+      <c r="A87" s="39">
         <f>IF('Getting Started'!B33&lt;&gt;"","  "&amp;UPPER('Getting Started'!B33)&amp;"   ·   "&amp;'Getting Started'!F33,"  STUDENT 5")</f>
         <v/>
       </c>
@@ -3429,7 +3638,7 @@
     </row>
     <row r="102" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="103" ht="26" customHeight="1">
-      <c r="A103" s="36">
+      <c r="A103" s="40">
         <f>IF('Getting Started'!B34&lt;&gt;"","  "&amp;UPPER('Getting Started'!B34)&amp;"   ·   "&amp;'Getting Started'!F34,"  STUDENT 6")</f>
         <v/>
       </c>
@@ -3772,7 +3981,7 @@
     </row>
     <row r="118" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="119" ht="26" customHeight="1">
-      <c r="A119" s="36">
+      <c r="A119" s="41">
         <f>IF('Getting Started'!B35&lt;&gt;"","  "&amp;UPPER('Getting Started'!B35)&amp;"   ·   "&amp;'Getting Started'!F35,"  STUDENT 7")</f>
         <v/>
       </c>
@@ -4115,7 +4324,7 @@
     </row>
     <row r="134" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="135" ht="26" customHeight="1">
-      <c r="A135" s="36">
+      <c r="A135" s="42">
         <f>IF('Getting Started'!B36&lt;&gt;"","  "&amp;UPPER('Getting Started'!B36)&amp;"   ·   "&amp;'Getting Started'!F36,"  STUDENT 8")</f>
         <v/>
       </c>
@@ -4458,7 +4667,7 @@
     </row>
     <row r="150" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="151" ht="26" customHeight="1">
-      <c r="A151" s="36">
+      <c r="A151" s="43">
         <f>IF('Getting Started'!B37&lt;&gt;"","  "&amp;UPPER('Getting Started'!B37)&amp;"   ·   "&amp;'Getting Started'!F37,"  STUDENT 9")</f>
         <v/>
       </c>
@@ -4801,7 +5010,7 @@
     </row>
     <row r="166" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
     <row r="167" ht="26" customHeight="1">
-      <c r="A167" s="36">
+      <c r="A167" s="44">
         <f>IF('Getting Started'!B38&lt;&gt;"","  "&amp;UPPER('Getting Started'!B38)&amp;"   ·   "&amp;'Getting Started'!F38,"  STUDENT 10")</f>
         <v/>
       </c>
@@ -5170,4 +5379,3538 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00CE8282"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J173"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1">
+        <f>IF('Getting Started'!B29="","Student 1",'Getting Started'!B29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="45">
+        <f>IFERROR("Grade: "&amp;'Getting Started'!F29&amp;"   ·   School Year: "&amp;'Getting Started'!C6,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="46">
+        <f>IFERROR("SEMESTER 1   "&amp;TEXT('Getting Started'!C10,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C11,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C15&amp;" wks)","SEMESTER 1")</f>
+        <v/>
+      </c>
+      <c r="F4" s="26" t="n"/>
+      <c r="G4" s="47">
+        <f>IFERROR("SEMESTER 2   "&amp;TEXT('Getting Started'!C18,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C19,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C23&amp;" wks)","SEMESTER 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>Subject  /  Curriculum</t>
+        </is>
+      </c>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Sem 1
+Units</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>/ Week</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
+        <is>
+          <t>/ Day</t>
+        </is>
+      </c>
+      <c r="E5" s="49" t="inlineStr">
+        <is>
+          <t>Est. End</t>
+        </is>
+      </c>
+      <c r="F5" s="50" t="inlineStr"/>
+      <c r="G5" s="51" t="inlineStr">
+        <is>
+          <t>Sem 2
+Units</t>
+        </is>
+      </c>
+      <c r="H5" s="51" t="inlineStr">
+        <is>
+          <t>/ Week</t>
+        </is>
+      </c>
+      <c r="I5" s="51" t="inlineStr">
+        <is>
+          <t>/ Day</t>
+        </is>
+      </c>
+      <c r="J5" s="51" t="inlineStr">
+        <is>
+          <t>Est. End</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  BIBLE</t>
+        </is>
+      </c>
+      <c r="E7" s="53">
+        <f>IFERROR(IF('Course Content'!B24="","← enter on Course Content tab",'Course Content'!B24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="54">
+        <f>'Course Content'!D24</f>
+        <v/>
+      </c>
+      <c r="C8" s="55">
+        <f>IFERROR(IF(B8="","",ROUND(B8/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D8" s="55">
+        <f>IFERROR(IF(C8="","",ROUND(C8/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E8" s="56">
+        <f>IFERROR(IF(B8="","",TEXT('Getting Started'!C10+(B8/D8),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="26" t="n"/>
+      <c r="G8" s="57">
+        <f>'Course Content'!E24</f>
+        <v/>
+      </c>
+      <c r="H8" s="58">
+        <f>IFERROR(IF(G8="","",ROUND(G8/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="58">
+        <f>IFERROR(IF(H8="","",ROUND(H8/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="59">
+        <f>IFERROR(IF(G8="","",TEXT('Getting Started'!C18+(G8/I8),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F10" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G10" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H10" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I10" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J10" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="F11" s="33" t="n"/>
+      <c r="G11" s="17">
+        <f>IFERROR(SUM(F11:F11),"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="17">
+        <f>IF(F11="","",1)</f>
+        <v/>
+      </c>
+      <c r="I11" s="17">
+        <f>IFERROR(IF(F11="","",CEILING(G11/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="62">
+        <f>IFERROR(IF(F11="","",TEXT('Getting Started'!C10+(H11-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I11*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="18" t="n"/>
+      <c r="F12" s="32" t="n"/>
+      <c r="G12" s="17">
+        <f>IFERROR(SUM(F11:F12),"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="17">
+        <f>IFERROR(IF(F12="","",FLOOR(G11/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="17">
+        <f>IFERROR(IF(F12="","",CEILING(G12/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="62">
+        <f>IFERROR(IF(F12="","",TEXT('Getting Started'!C10+(H12-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I12*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="F13" s="33" t="n"/>
+      <c r="G13" s="17">
+        <f>IFERROR(SUM(F11:F13),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="17">
+        <f>IFERROR(IF(F13="","",FLOOR(G12/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="17">
+        <f>IFERROR(IF(F13="","",CEILING(G13/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="62">
+        <f>IFERROR(IF(F13="","",TEXT('Getting Started'!C10+(H13-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I13*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="18" t="n"/>
+      <c r="F14" s="32" t="n"/>
+      <c r="G14" s="17">
+        <f>IFERROR(SUM(F11:F14),"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="17">
+        <f>IFERROR(IF(F14="","",FLOOR(G13/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="17">
+        <f>IFERROR(IF(F14="","",CEILING(G14/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="62">
+        <f>IFERROR(IF(F14="","",TEXT('Getting Started'!C10+(H14-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I14*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="F15" s="33" t="n"/>
+      <c r="G15" s="17">
+        <f>IFERROR(SUM(F11:F15),"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="17">
+        <f>IFERROR(IF(F15="","",FLOOR(G14/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="17">
+        <f>IFERROR(IF(F15="","",CEILING(G15/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="62">
+        <f>IFERROR(IF(F15="","",TEXT('Getting Started'!C10+(H15-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I15*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="18" t="n"/>
+      <c r="F16" s="32" t="n"/>
+      <c r="G16" s="17">
+        <f>IFERROR(SUM(F11:F16),"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="17">
+        <f>IFERROR(IF(F16="","",FLOOR(G15/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="17">
+        <f>IFERROR(IF(F16="","",CEILING(G16/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="62">
+        <f>IFERROR(IF(F16="","",TEXT('Getting Started'!C10+(H16-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I16*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="63" t="n"/>
+    </row>
+    <row r="18" ht="8" customHeight="1"/>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MATH</t>
+        </is>
+      </c>
+      <c r="E19" s="53">
+        <f>IFERROR(IF('Course Content'!B25="","← enter on Course Content tab",'Course Content'!B25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="54">
+        <f>'Course Content'!D25</f>
+        <v/>
+      </c>
+      <c r="C20" s="55">
+        <f>IFERROR(IF(B20="","",ROUND(B20/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D20" s="55">
+        <f>IFERROR(IF(C20="","",ROUND(C20/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="56">
+        <f>IFERROR(IF(B20="","",TEXT('Getting Started'!C10+(B20/D20),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="26" t="n"/>
+      <c r="G20" s="57">
+        <f>'Course Content'!E25</f>
+        <v/>
+      </c>
+      <c r="H20" s="58">
+        <f>IFERROR(IF(G20="","",ROUND(G20/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="58">
+        <f>IFERROR(IF(H20="","",ROUND(H20/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="59">
+        <f>IFERROR(IF(G20="","",TEXT('Getting Started'!C18+(G20/I20),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F22" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G22" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H22" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I22" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J22" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="F23" s="33" t="n"/>
+      <c r="G23" s="17">
+        <f>IFERROR(SUM(F23:F23),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="17">
+        <f>IF(F23="","",1)</f>
+        <v/>
+      </c>
+      <c r="I23" s="17">
+        <f>IFERROR(IF(F23="","",CEILING(G23/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="62">
+        <f>IFERROR(IF(F23="","",TEXT('Getting Started'!C10+(H23-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I23*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="18" t="n"/>
+      <c r="F24" s="32" t="n"/>
+      <c r="G24" s="17">
+        <f>IFERROR(SUM(F23:F24),"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="17">
+        <f>IFERROR(IF(F24="","",FLOOR(G23/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="17">
+        <f>IFERROR(IF(F24="","",CEILING(G24/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="62">
+        <f>IFERROR(IF(F24="","",TEXT('Getting Started'!C10+(H24-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I24*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" s="5" t="n"/>
+      <c r="F25" s="33" t="n"/>
+      <c r="G25" s="17">
+        <f>IFERROR(SUM(F23:F25),"")</f>
+        <v/>
+      </c>
+      <c r="H25" s="17">
+        <f>IFERROR(IF(F25="","",FLOOR(G24/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I25" s="17">
+        <f>IFERROR(IF(F25="","",CEILING(G25/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J25" s="62">
+        <f>IFERROR(IF(F25="","",TEXT('Getting Started'!C10+(H25-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I25*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="18" t="n"/>
+      <c r="F26" s="32" t="n"/>
+      <c r="G26" s="17">
+        <f>IFERROR(SUM(F23:F26),"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="17">
+        <f>IFERROR(IF(F26="","",FLOOR(G25/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="17">
+        <f>IFERROR(IF(F26="","",CEILING(G26/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="62">
+        <f>IFERROR(IF(F26="","",TEXT('Getting Started'!C10+(H26-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I26*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" s="5" t="n"/>
+      <c r="F27" s="33" t="n"/>
+      <c r="G27" s="17">
+        <f>IFERROR(SUM(F23:F27),"")</f>
+        <v/>
+      </c>
+      <c r="H27" s="17">
+        <f>IFERROR(IF(F27="","",FLOOR(G26/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I27" s="17">
+        <f>IFERROR(IF(F27="","",CEILING(G27/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J27" s="62">
+        <f>IFERROR(IF(F27="","",TEXT('Getting Started'!C10+(H27-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I27*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" s="18" t="n"/>
+      <c r="F28" s="32" t="n"/>
+      <c r="G28" s="17">
+        <f>IFERROR(SUM(F23:F28),"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="17">
+        <f>IFERROR(IF(F28="","",FLOOR(G27/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="17">
+        <f>IFERROR(IF(F28="","",CEILING(G28/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="62">
+        <f>IFERROR(IF(F28="","",TEXT('Getting Started'!C10+(H28-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I28*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="63" t="n"/>
+    </row>
+    <row r="30" ht="8" customHeight="1"/>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ENGLISH / LANGUAGE ARTS</t>
+        </is>
+      </c>
+      <c r="E31" s="53">
+        <f>IFERROR(IF('Course Content'!B26="","← enter on Course Content tab",'Course Content'!B26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="54">
+        <f>'Course Content'!D26</f>
+        <v/>
+      </c>
+      <c r="C32" s="55">
+        <f>IFERROR(IF(B32="","",ROUND(B32/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D32" s="55">
+        <f>IFERROR(IF(C32="","",ROUND(C32/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E32" s="56">
+        <f>IFERROR(IF(B32="","",TEXT('Getting Started'!C10+(B32/D32),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F32" s="26" t="n"/>
+      <c r="G32" s="57">
+        <f>'Course Content'!E26</f>
+        <v/>
+      </c>
+      <c r="H32" s="58">
+        <f>IFERROR(IF(G32="","",ROUND(G32/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="58">
+        <f>IFERROR(IF(H32="","",ROUND(H32/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J32" s="59">
+        <f>IFERROR(IF(G32="","",TEXT('Getting Started'!C18+(G32/I32),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B34" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F34" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G34" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H34" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I34" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J34" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="5" t="n"/>
+      <c r="F35" s="33" t="n"/>
+      <c r="G35" s="17">
+        <f>IFERROR(SUM(F35:F35),"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="17">
+        <f>IF(F35="","",1)</f>
+        <v/>
+      </c>
+      <c r="I35" s="17">
+        <f>IFERROR(IF(F35="","",CEILING(G35/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J35" s="62">
+        <f>IFERROR(IF(F35="","",TEXT('Getting Started'!C10+(H35-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I35*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="18" t="n"/>
+      <c r="F36" s="32" t="n"/>
+      <c r="G36" s="17">
+        <f>IFERROR(SUM(F35:F36),"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="17">
+        <f>IFERROR(IF(F36="","",FLOOR(G35/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I36" s="17">
+        <f>IFERROR(IF(F36="","",CEILING(G36/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J36" s="62">
+        <f>IFERROR(IF(F36="","",TEXT('Getting Started'!C10+(H36-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I36*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="F37" s="33" t="n"/>
+      <c r="G37" s="17">
+        <f>IFERROR(SUM(F35:F37),"")</f>
+        <v/>
+      </c>
+      <c r="H37" s="17">
+        <f>IFERROR(IF(F37="","",FLOOR(G36/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I37" s="17">
+        <f>IFERROR(IF(F37="","",CEILING(G37/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J37" s="62">
+        <f>IFERROR(IF(F37="","",TEXT('Getting Started'!C10+(H37-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I37*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B38" s="18" t="n"/>
+      <c r="F38" s="32" t="n"/>
+      <c r="G38" s="17">
+        <f>IFERROR(SUM(F35:F38),"")</f>
+        <v/>
+      </c>
+      <c r="H38" s="17">
+        <f>IFERROR(IF(F38="","",FLOOR(G37/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I38" s="17">
+        <f>IFERROR(IF(F38="","",CEILING(G38/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J38" s="62">
+        <f>IFERROR(IF(F38="","",TEXT('Getting Started'!C10+(H38-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I38*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B39" s="5" t="n"/>
+      <c r="F39" s="33" t="n"/>
+      <c r="G39" s="17">
+        <f>IFERROR(SUM(F35:F39),"")</f>
+        <v/>
+      </c>
+      <c r="H39" s="17">
+        <f>IFERROR(IF(F39="","",FLOOR(G38/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I39" s="17">
+        <f>IFERROR(IF(F39="","",CEILING(G39/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J39" s="62">
+        <f>IFERROR(IF(F39="","",TEXT('Getting Started'!C10+(H39-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I39*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B40" s="18" t="n"/>
+      <c r="F40" s="32" t="n"/>
+      <c r="G40" s="17">
+        <f>IFERROR(SUM(F35:F40),"")</f>
+        <v/>
+      </c>
+      <c r="H40" s="17">
+        <f>IFERROR(IF(F40="","",FLOOR(G39/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I40" s="17">
+        <f>IFERROR(IF(F40="","",CEILING(G40/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J40" s="62">
+        <f>IFERROR(IF(F40="","",TEXT('Getting Started'!C10+(H40-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I40*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="63" t="n"/>
+    </row>
+    <row r="42" ht="8" customHeight="1"/>
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  READING</t>
+        </is>
+      </c>
+      <c r="E43" s="53">
+        <f>IFERROR(IF('Course Content'!B27="","← enter on Course Content tab",'Course Content'!B27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="B44" s="54">
+        <f>'Course Content'!D27</f>
+        <v/>
+      </c>
+      <c r="C44" s="55">
+        <f>IFERROR(IF(B44="","",ROUND(B44/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D44" s="55">
+        <f>IFERROR(IF(C44="","",ROUND(C44/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="56">
+        <f>IFERROR(IF(B44="","",TEXT('Getting Started'!C10+(B44/D44),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="26" t="n"/>
+      <c r="G44" s="57">
+        <f>'Course Content'!E27</f>
+        <v/>
+      </c>
+      <c r="H44" s="58">
+        <f>IFERROR(IF(G44="","",ROUND(G44/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I44" s="58">
+        <f>IFERROR(IF(H44="","",ROUND(H44/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J44" s="59">
+        <f>IFERROR(IF(G44="","",TEXT('Getting Started'!C18+(G44/I44),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B46" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F46" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G46" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H46" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I46" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J46" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="F47" s="33" t="n"/>
+      <c r="G47" s="17">
+        <f>IFERROR(SUM(F47:F47),"")</f>
+        <v/>
+      </c>
+      <c r="H47" s="17">
+        <f>IF(F47="","",1)</f>
+        <v/>
+      </c>
+      <c r="I47" s="17">
+        <f>IFERROR(IF(F47="","",CEILING(G47/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J47" s="62">
+        <f>IFERROR(IF(F47="","",TEXT('Getting Started'!C10+(H47-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I47*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="18" t="n"/>
+      <c r="F48" s="32" t="n"/>
+      <c r="G48" s="17">
+        <f>IFERROR(SUM(F47:F48),"")</f>
+        <v/>
+      </c>
+      <c r="H48" s="17">
+        <f>IFERROR(IF(F48="","",FLOOR(G47/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I48" s="17">
+        <f>IFERROR(IF(F48="","",CEILING(G48/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J48" s="62">
+        <f>IFERROR(IF(F48="","",TEXT('Getting Started'!C10+(H48-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I48*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" s="5" t="n"/>
+      <c r="F49" s="33" t="n"/>
+      <c r="G49" s="17">
+        <f>IFERROR(SUM(F47:F49),"")</f>
+        <v/>
+      </c>
+      <c r="H49" s="17">
+        <f>IFERROR(IF(F49="","",FLOOR(G48/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I49" s="17">
+        <f>IFERROR(IF(F49="","",CEILING(G49/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J49" s="62">
+        <f>IFERROR(IF(F49="","",TEXT('Getting Started'!C10+(H49-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I49*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B50" s="18" t="n"/>
+      <c r="F50" s="32" t="n"/>
+      <c r="G50" s="17">
+        <f>IFERROR(SUM(F47:F50),"")</f>
+        <v/>
+      </c>
+      <c r="H50" s="17">
+        <f>IFERROR(IF(F50="","",FLOOR(G49/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I50" s="17">
+        <f>IFERROR(IF(F50="","",CEILING(G50/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J50" s="62">
+        <f>IFERROR(IF(F50="","",TEXT('Getting Started'!C10+(H50-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I50*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" s="5" t="n"/>
+      <c r="F51" s="33" t="n"/>
+      <c r="G51" s="17">
+        <f>IFERROR(SUM(F47:F51),"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="17">
+        <f>IFERROR(IF(F51="","",FLOOR(G50/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I51" s="17">
+        <f>IFERROR(IF(F51="","",CEILING(G51/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="62">
+        <f>IFERROR(IF(F51="","",TEXT('Getting Started'!C10+(H51-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I51*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B52" s="18" t="n"/>
+      <c r="F52" s="32" t="n"/>
+      <c r="G52" s="17">
+        <f>IFERROR(SUM(F47:F52),"")</f>
+        <v/>
+      </c>
+      <c r="H52" s="17">
+        <f>IFERROR(IF(F52="","",FLOOR(G51/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I52" s="17">
+        <f>IFERROR(IF(F52="","",CEILING(G52/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J52" s="62">
+        <f>IFERROR(IF(F52="","",TEXT('Getting Started'!C10+(H52-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I52*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="63" t="n"/>
+    </row>
+    <row r="54" ht="8" customHeight="1"/>
+    <row r="55" ht="24" customHeight="1">
+      <c r="A55" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WRITING / COMPOSITION</t>
+        </is>
+      </c>
+      <c r="E55" s="53">
+        <f>IFERROR(IF('Course Content'!B28="","← enter on Course Content tab",'Course Content'!B28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="B56" s="54">
+        <f>'Course Content'!D28</f>
+        <v/>
+      </c>
+      <c r="C56" s="55">
+        <f>IFERROR(IF(B56="","",ROUND(B56/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D56" s="55">
+        <f>IFERROR(IF(C56="","",ROUND(C56/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E56" s="56">
+        <f>IFERROR(IF(B56="","",TEXT('Getting Started'!C10+(B56/D56),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F56" s="26" t="n"/>
+      <c r="G56" s="57">
+        <f>'Course Content'!E28</f>
+        <v/>
+      </c>
+      <c r="H56" s="58">
+        <f>IFERROR(IF(G56="","",ROUND(G56/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I56" s="58">
+        <f>IFERROR(IF(H56="","",ROUND(H56/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J56" s="59">
+        <f>IFERROR(IF(G56="","",TEXT('Getting Started'!C18+(G56/I56),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B58" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F58" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G58" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H58" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I58" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J58" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B59" s="5" t="n"/>
+      <c r="F59" s="33" t="n"/>
+      <c r="G59" s="17">
+        <f>IFERROR(SUM(F59:F59),"")</f>
+        <v/>
+      </c>
+      <c r="H59" s="17">
+        <f>IF(F59="","",1)</f>
+        <v/>
+      </c>
+      <c r="I59" s="17">
+        <f>IFERROR(IF(F59="","",CEILING(G59/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J59" s="62">
+        <f>IFERROR(IF(F59="","",TEXT('Getting Started'!C10+(H59-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I59*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" s="18" t="n"/>
+      <c r="F60" s="32" t="n"/>
+      <c r="G60" s="17">
+        <f>IFERROR(SUM(F59:F60),"")</f>
+        <v/>
+      </c>
+      <c r="H60" s="17">
+        <f>IFERROR(IF(F60="","",FLOOR(G59/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I60" s="17">
+        <f>IFERROR(IF(F60="","",CEILING(G60/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J60" s="62">
+        <f>IFERROR(IF(F60="","",TEXT('Getting Started'!C10+(H60-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I60*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B61" s="5" t="n"/>
+      <c r="F61" s="33" t="n"/>
+      <c r="G61" s="17">
+        <f>IFERROR(SUM(F59:F61),"")</f>
+        <v/>
+      </c>
+      <c r="H61" s="17">
+        <f>IFERROR(IF(F61="","",FLOOR(G60/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I61" s="17">
+        <f>IFERROR(IF(F61="","",CEILING(G61/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J61" s="62">
+        <f>IFERROR(IF(F61="","",TEXT('Getting Started'!C10+(H61-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I61*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B62" s="18" t="n"/>
+      <c r="F62" s="32" t="n"/>
+      <c r="G62" s="17">
+        <f>IFERROR(SUM(F59:F62),"")</f>
+        <v/>
+      </c>
+      <c r="H62" s="17">
+        <f>IFERROR(IF(F62="","",FLOOR(G61/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I62" s="17">
+        <f>IFERROR(IF(F62="","",CEILING(G62/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J62" s="62">
+        <f>IFERROR(IF(F62="","",TEXT('Getting Started'!C10+(H62-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I62*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B63" s="5" t="n"/>
+      <c r="F63" s="33" t="n"/>
+      <c r="G63" s="17">
+        <f>IFERROR(SUM(F59:F63),"")</f>
+        <v/>
+      </c>
+      <c r="H63" s="17">
+        <f>IFERROR(IF(F63="","",FLOOR(G62/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I63" s="17">
+        <f>IFERROR(IF(F63="","",CEILING(G63/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J63" s="62">
+        <f>IFERROR(IF(F63="","",TEXT('Getting Started'!C10+(H63-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I63*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B64" s="18" t="n"/>
+      <c r="F64" s="32" t="n"/>
+      <c r="G64" s="17">
+        <f>IFERROR(SUM(F59:F64),"")</f>
+        <v/>
+      </c>
+      <c r="H64" s="17">
+        <f>IFERROR(IF(F64="","",FLOOR(G63/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I64" s="17">
+        <f>IFERROR(IF(F64="","",CEILING(G64/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J64" s="62">
+        <f>IFERROR(IF(F64="","",TEXT('Getting Started'!C10+(H64-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I64*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="63" t="n"/>
+    </row>
+    <row r="66" ht="8" customHeight="1"/>
+    <row r="67" ht="24" customHeight="1">
+      <c r="A67" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SCIENCE</t>
+        </is>
+      </c>
+      <c r="E67" s="53">
+        <f>IFERROR(IF('Course Content'!B29="","← enter on Course Content tab",'Course Content'!B29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="B68" s="54">
+        <f>'Course Content'!D29</f>
+        <v/>
+      </c>
+      <c r="C68" s="55">
+        <f>IFERROR(IF(B68="","",ROUND(B68/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D68" s="55">
+        <f>IFERROR(IF(C68="","",ROUND(C68/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E68" s="56">
+        <f>IFERROR(IF(B68="","",TEXT('Getting Started'!C10+(B68/D68),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F68" s="26" t="n"/>
+      <c r="G68" s="57">
+        <f>'Course Content'!E29</f>
+        <v/>
+      </c>
+      <c r="H68" s="58">
+        <f>IFERROR(IF(G68="","",ROUND(G68/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I68" s="58">
+        <f>IFERROR(IF(H68="","",ROUND(H68/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J68" s="59">
+        <f>IFERROR(IF(G68="","",TEXT('Getting Started'!C18+(G68/I68),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="16" customHeight="1">
+      <c r="A69" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B70" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F70" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G70" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H70" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I70" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J70" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B71" s="5" t="n"/>
+      <c r="F71" s="33" t="n"/>
+      <c r="G71" s="17">
+        <f>IFERROR(SUM(F71:F71),"")</f>
+        <v/>
+      </c>
+      <c r="H71" s="17">
+        <f>IF(F71="","",1)</f>
+        <v/>
+      </c>
+      <c r="I71" s="17">
+        <f>IFERROR(IF(F71="","",CEILING(G71/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J71" s="62">
+        <f>IFERROR(IF(F71="","",TEXT('Getting Started'!C10+(H71-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I71*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B72" s="18" t="n"/>
+      <c r="F72" s="32" t="n"/>
+      <c r="G72" s="17">
+        <f>IFERROR(SUM(F71:F72),"")</f>
+        <v/>
+      </c>
+      <c r="H72" s="17">
+        <f>IFERROR(IF(F72="","",FLOOR(G71/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I72" s="17">
+        <f>IFERROR(IF(F72="","",CEILING(G72/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J72" s="62">
+        <f>IFERROR(IF(F72="","",TEXT('Getting Started'!C10+(H72-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I72*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B73" s="5" t="n"/>
+      <c r="F73" s="33" t="n"/>
+      <c r="G73" s="17">
+        <f>IFERROR(SUM(F71:F73),"")</f>
+        <v/>
+      </c>
+      <c r="H73" s="17">
+        <f>IFERROR(IF(F73="","",FLOOR(G72/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I73" s="17">
+        <f>IFERROR(IF(F73="","",CEILING(G73/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J73" s="62">
+        <f>IFERROR(IF(F73="","",TEXT('Getting Started'!C10+(H73-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I73*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B74" s="18" t="n"/>
+      <c r="F74" s="32" t="n"/>
+      <c r="G74" s="17">
+        <f>IFERROR(SUM(F71:F74),"")</f>
+        <v/>
+      </c>
+      <c r="H74" s="17">
+        <f>IFERROR(IF(F74="","",FLOOR(G73/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I74" s="17">
+        <f>IFERROR(IF(F74="","",CEILING(G74/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J74" s="62">
+        <f>IFERROR(IF(F74="","",TEXT('Getting Started'!C10+(H74-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I74*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B75" s="5" t="n"/>
+      <c r="F75" s="33" t="n"/>
+      <c r="G75" s="17">
+        <f>IFERROR(SUM(F71:F75),"")</f>
+        <v/>
+      </c>
+      <c r="H75" s="17">
+        <f>IFERROR(IF(F75="","",FLOOR(G74/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I75" s="17">
+        <f>IFERROR(IF(F75="","",CEILING(G75/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J75" s="62">
+        <f>IFERROR(IF(F75="","",TEXT('Getting Started'!C10+(H75-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I75*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B76" s="18" t="n"/>
+      <c r="F76" s="32" t="n"/>
+      <c r="G76" s="17">
+        <f>IFERROR(SUM(F71:F76),"")</f>
+        <v/>
+      </c>
+      <c r="H76" s="17">
+        <f>IFERROR(IF(F76="","",FLOOR(G75/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I76" s="17">
+        <f>IFERROR(IF(F76="","",CEILING(G76/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J76" s="62">
+        <f>IFERROR(IF(F76="","",TEXT('Getting Started'!C10+(H76-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I76*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="63" t="n"/>
+    </row>
+    <row r="78" ht="8" customHeight="1"/>
+    <row r="79" ht="24" customHeight="1">
+      <c r="A79" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SOCIAL STUDIES / HISTORY</t>
+        </is>
+      </c>
+      <c r="E79" s="53">
+        <f>IFERROR(IF('Course Content'!B30="","← enter on Course Content tab",'Course Content'!B30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="B80" s="54">
+        <f>'Course Content'!D30</f>
+        <v/>
+      </c>
+      <c r="C80" s="55">
+        <f>IFERROR(IF(B80="","",ROUND(B80/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D80" s="55">
+        <f>IFERROR(IF(C80="","",ROUND(C80/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E80" s="56">
+        <f>IFERROR(IF(B80="","",TEXT('Getting Started'!C10+(B80/D80),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F80" s="26" t="n"/>
+      <c r="G80" s="57">
+        <f>'Course Content'!E30</f>
+        <v/>
+      </c>
+      <c r="H80" s="58">
+        <f>IFERROR(IF(G80="","",ROUND(G80/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I80" s="58">
+        <f>IFERROR(IF(H80="","",ROUND(H80/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J80" s="59">
+        <f>IFERROR(IF(G80="","",TEXT('Getting Started'!C18+(G80/I80),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" ht="16" customHeight="1">
+      <c r="A81" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B82" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F82" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G82" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H82" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I82" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J82" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B83" s="5" t="n"/>
+      <c r="F83" s="33" t="n"/>
+      <c r="G83" s="17">
+        <f>IFERROR(SUM(F83:F83),"")</f>
+        <v/>
+      </c>
+      <c r="H83" s="17">
+        <f>IF(F83="","",1)</f>
+        <v/>
+      </c>
+      <c r="I83" s="17">
+        <f>IFERROR(IF(F83="","",CEILING(G83/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J83" s="62">
+        <f>IFERROR(IF(F83="","",TEXT('Getting Started'!C10+(H83-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I83*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B84" s="18" t="n"/>
+      <c r="F84" s="32" t="n"/>
+      <c r="G84" s="17">
+        <f>IFERROR(SUM(F83:F84),"")</f>
+        <v/>
+      </c>
+      <c r="H84" s="17">
+        <f>IFERROR(IF(F84="","",FLOOR(G83/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I84" s="17">
+        <f>IFERROR(IF(F84="","",CEILING(G84/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J84" s="62">
+        <f>IFERROR(IF(F84="","",TEXT('Getting Started'!C10+(H84-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I84*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B85" s="5" t="n"/>
+      <c r="F85" s="33" t="n"/>
+      <c r="G85" s="17">
+        <f>IFERROR(SUM(F83:F85),"")</f>
+        <v/>
+      </c>
+      <c r="H85" s="17">
+        <f>IFERROR(IF(F85="","",FLOOR(G84/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I85" s="17">
+        <f>IFERROR(IF(F85="","",CEILING(G85/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J85" s="62">
+        <f>IFERROR(IF(F85="","",TEXT('Getting Started'!C10+(H85-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I85*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B86" s="18" t="n"/>
+      <c r="F86" s="32" t="n"/>
+      <c r="G86" s="17">
+        <f>IFERROR(SUM(F83:F86),"")</f>
+        <v/>
+      </c>
+      <c r="H86" s="17">
+        <f>IFERROR(IF(F86="","",FLOOR(G85/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I86" s="17">
+        <f>IFERROR(IF(F86="","",CEILING(G86/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J86" s="62">
+        <f>IFERROR(IF(F86="","",TEXT('Getting Started'!C10+(H86-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I86*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B87" s="5" t="n"/>
+      <c r="F87" s="33" t="n"/>
+      <c r="G87" s="17">
+        <f>IFERROR(SUM(F83:F87),"")</f>
+        <v/>
+      </c>
+      <c r="H87" s="17">
+        <f>IFERROR(IF(F87="","",FLOOR(G86/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I87" s="17">
+        <f>IFERROR(IF(F87="","",CEILING(G87/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J87" s="62">
+        <f>IFERROR(IF(F87="","",TEXT('Getting Started'!C10+(H87-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I87*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B88" s="18" t="n"/>
+      <c r="F88" s="32" t="n"/>
+      <c r="G88" s="17">
+        <f>IFERROR(SUM(F83:F88),"")</f>
+        <v/>
+      </c>
+      <c r="H88" s="17">
+        <f>IFERROR(IF(F88="","",FLOOR(G87/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I88" s="17">
+        <f>IFERROR(IF(F88="","",CEILING(G88/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J88" s="62">
+        <f>IFERROR(IF(F88="","",TEXT('Getting Started'!C10+(H88-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I88*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="63" t="n"/>
+    </row>
+    <row r="90" ht="8" customHeight="1"/>
+    <row r="91" ht="24" customHeight="1">
+      <c r="A91" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HEALTH</t>
+        </is>
+      </c>
+      <c r="E91" s="53">
+        <f>IFERROR(IF('Course Content'!B31="","← enter on Course Content tab",'Course Content'!B31),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="B92" s="54">
+        <f>'Course Content'!D31</f>
+        <v/>
+      </c>
+      <c r="C92" s="55">
+        <f>IFERROR(IF(B92="","",ROUND(B92/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D92" s="55">
+        <f>IFERROR(IF(C92="","",ROUND(C92/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E92" s="56">
+        <f>IFERROR(IF(B92="","",TEXT('Getting Started'!C10+(B92/D92),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F92" s="26" t="n"/>
+      <c r="G92" s="57">
+        <f>'Course Content'!E31</f>
+        <v/>
+      </c>
+      <c r="H92" s="58">
+        <f>IFERROR(IF(G92="","",ROUND(G92/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I92" s="58">
+        <f>IFERROR(IF(H92="","",ROUND(H92/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J92" s="59">
+        <f>IFERROR(IF(G92="","",TEXT('Getting Started'!C18+(G92/I92),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" ht="16" customHeight="1">
+      <c r="A93" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B94" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F94" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G94" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H94" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I94" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J94" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B95" s="5" t="n"/>
+      <c r="F95" s="33" t="n"/>
+      <c r="G95" s="17">
+        <f>IFERROR(SUM(F95:F95),"")</f>
+        <v/>
+      </c>
+      <c r="H95" s="17">
+        <f>IF(F95="","",1)</f>
+        <v/>
+      </c>
+      <c r="I95" s="17">
+        <f>IFERROR(IF(F95="","",CEILING(G95/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J95" s="62">
+        <f>IFERROR(IF(F95="","",TEXT('Getting Started'!C10+(H95-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I95*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B96" s="18" t="n"/>
+      <c r="F96" s="32" t="n"/>
+      <c r="G96" s="17">
+        <f>IFERROR(SUM(F95:F96),"")</f>
+        <v/>
+      </c>
+      <c r="H96" s="17">
+        <f>IFERROR(IF(F96="","",FLOOR(G95/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I96" s="17">
+        <f>IFERROR(IF(F96="","",CEILING(G96/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J96" s="62">
+        <f>IFERROR(IF(F96="","",TEXT('Getting Started'!C10+(H96-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I96*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B97" s="5" t="n"/>
+      <c r="F97" s="33" t="n"/>
+      <c r="G97" s="17">
+        <f>IFERROR(SUM(F95:F97),"")</f>
+        <v/>
+      </c>
+      <c r="H97" s="17">
+        <f>IFERROR(IF(F97="","",FLOOR(G96/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I97" s="17">
+        <f>IFERROR(IF(F97="","",CEILING(G97/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J97" s="62">
+        <f>IFERROR(IF(F97="","",TEXT('Getting Started'!C10+(H97-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I97*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B98" s="18" t="n"/>
+      <c r="F98" s="32" t="n"/>
+      <c r="G98" s="17">
+        <f>IFERROR(SUM(F95:F98),"")</f>
+        <v/>
+      </c>
+      <c r="H98" s="17">
+        <f>IFERROR(IF(F98="","",FLOOR(G97/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I98" s="17">
+        <f>IFERROR(IF(F98="","",CEILING(G98/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J98" s="62">
+        <f>IFERROR(IF(F98="","",TEXT('Getting Started'!C10+(H98-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I98*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B99" s="5" t="n"/>
+      <c r="F99" s="33" t="n"/>
+      <c r="G99" s="17">
+        <f>IFERROR(SUM(F95:F99),"")</f>
+        <v/>
+      </c>
+      <c r="H99" s="17">
+        <f>IFERROR(IF(F99="","",FLOOR(G98/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I99" s="17">
+        <f>IFERROR(IF(F99="","",CEILING(G99/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J99" s="62">
+        <f>IFERROR(IF(F99="","",TEXT('Getting Started'!C10+(H99-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I99*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B100" s="18" t="n"/>
+      <c r="F100" s="32" t="n"/>
+      <c r="G100" s="17">
+        <f>IFERROR(SUM(F95:F100),"")</f>
+        <v/>
+      </c>
+      <c r="H100" s="17">
+        <f>IFERROR(IF(F100="","",FLOOR(G99/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I100" s="17">
+        <f>IFERROR(IF(F100="","",CEILING(G100/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J100" s="62">
+        <f>IFERROR(IF(F100="","",TEXT('Getting Started'!C10+(H100-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I100*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="63" t="n"/>
+    </row>
+    <row r="102" ht="8" customHeight="1"/>
+    <row r="103" ht="24" customHeight="1">
+      <c r="A103" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  PHYSICAL EDUCATION</t>
+        </is>
+      </c>
+      <c r="E103" s="53">
+        <f>IFERROR(IF('Course Content'!B32="","← enter on Course Content tab",'Course Content'!B32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="B104" s="54">
+        <f>'Course Content'!D32</f>
+        <v/>
+      </c>
+      <c r="C104" s="55">
+        <f>IFERROR(IF(B104="","",ROUND(B104/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D104" s="55">
+        <f>IFERROR(IF(C104="","",ROUND(C104/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E104" s="56">
+        <f>IFERROR(IF(B104="","",TEXT('Getting Started'!C10+(B104/D104),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F104" s="26" t="n"/>
+      <c r="G104" s="57">
+        <f>'Course Content'!E32</f>
+        <v/>
+      </c>
+      <c r="H104" s="58">
+        <f>IFERROR(IF(G104="","",ROUND(G104/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I104" s="58">
+        <f>IFERROR(IF(H104="","",ROUND(H104/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J104" s="59">
+        <f>IFERROR(IF(G104="","",TEXT('Getting Started'!C18+(G104/I104),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105" ht="16" customHeight="1">
+      <c r="A105" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B106" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F106" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G106" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H106" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I106" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J106" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B107" s="5" t="n"/>
+      <c r="F107" s="33" t="n"/>
+      <c r="G107" s="17">
+        <f>IFERROR(SUM(F107:F107),"")</f>
+        <v/>
+      </c>
+      <c r="H107" s="17">
+        <f>IF(F107="","",1)</f>
+        <v/>
+      </c>
+      <c r="I107" s="17">
+        <f>IFERROR(IF(F107="","",CEILING(G107/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J107" s="62">
+        <f>IFERROR(IF(F107="","",TEXT('Getting Started'!C10+(H107-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I107*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B108" s="18" t="n"/>
+      <c r="F108" s="32" t="n"/>
+      <c r="G108" s="17">
+        <f>IFERROR(SUM(F107:F108),"")</f>
+        <v/>
+      </c>
+      <c r="H108" s="17">
+        <f>IFERROR(IF(F108="","",FLOOR(G107/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I108" s="17">
+        <f>IFERROR(IF(F108="","",CEILING(G108/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J108" s="62">
+        <f>IFERROR(IF(F108="","",TEXT('Getting Started'!C10+(H108-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I108*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B109" s="5" t="n"/>
+      <c r="F109" s="33" t="n"/>
+      <c r="G109" s="17">
+        <f>IFERROR(SUM(F107:F109),"")</f>
+        <v/>
+      </c>
+      <c r="H109" s="17">
+        <f>IFERROR(IF(F109="","",FLOOR(G108/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I109" s="17">
+        <f>IFERROR(IF(F109="","",CEILING(G109/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J109" s="62">
+        <f>IFERROR(IF(F109="","",TEXT('Getting Started'!C10+(H109-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I109*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B110" s="18" t="n"/>
+      <c r="F110" s="32" t="n"/>
+      <c r="G110" s="17">
+        <f>IFERROR(SUM(F107:F110),"")</f>
+        <v/>
+      </c>
+      <c r="H110" s="17">
+        <f>IFERROR(IF(F110="","",FLOOR(G109/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I110" s="17">
+        <f>IFERROR(IF(F110="","",CEILING(G110/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J110" s="62">
+        <f>IFERROR(IF(F110="","",TEXT('Getting Started'!C10+(H110-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I110*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B111" s="5" t="n"/>
+      <c r="F111" s="33" t="n"/>
+      <c r="G111" s="17">
+        <f>IFERROR(SUM(F107:F111),"")</f>
+        <v/>
+      </c>
+      <c r="H111" s="17">
+        <f>IFERROR(IF(F111="","",FLOOR(G110/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I111" s="17">
+        <f>IFERROR(IF(F111="","",CEILING(G111/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J111" s="62">
+        <f>IFERROR(IF(F111="","",TEXT('Getting Started'!C10+(H111-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I111*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B112" s="18" t="n"/>
+      <c r="F112" s="32" t="n"/>
+      <c r="G112" s="17">
+        <f>IFERROR(SUM(F107:F112),"")</f>
+        <v/>
+      </c>
+      <c r="H112" s="17">
+        <f>IFERROR(IF(F112="","",FLOOR(G111/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I112" s="17">
+        <f>IFERROR(IF(F112="","",CEILING(G112/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J112" s="62">
+        <f>IFERROR(IF(F112="","",TEXT('Getting Started'!C10+(H112-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I112*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="63" t="n"/>
+    </row>
+    <row r="114" ht="8" customHeight="1"/>
+    <row r="115" ht="24" customHeight="1">
+      <c r="A115" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ART / MUSIC</t>
+        </is>
+      </c>
+      <c r="E115" s="53">
+        <f>IFERROR(IF('Course Content'!B33="","← enter on Course Content tab",'Course Content'!B33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="B116" s="54">
+        <f>'Course Content'!D33</f>
+        <v/>
+      </c>
+      <c r="C116" s="55">
+        <f>IFERROR(IF(B116="","",ROUND(B116/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D116" s="55">
+        <f>IFERROR(IF(C116="","",ROUND(C116/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E116" s="56">
+        <f>IFERROR(IF(B116="","",TEXT('Getting Started'!C10+(B116/D116),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F116" s="26" t="n"/>
+      <c r="G116" s="57">
+        <f>'Course Content'!E33</f>
+        <v/>
+      </c>
+      <c r="H116" s="58">
+        <f>IFERROR(IF(G116="","",ROUND(G116/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I116" s="58">
+        <f>IFERROR(IF(H116="","",ROUND(H116/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J116" s="59">
+        <f>IFERROR(IF(G116="","",TEXT('Getting Started'!C18+(G116/I116),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117" ht="16" customHeight="1">
+      <c r="A117" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B118" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F118" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G118" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H118" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I118" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J118" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B119" s="5" t="n"/>
+      <c r="F119" s="33" t="n"/>
+      <c r="G119" s="17">
+        <f>IFERROR(SUM(F119:F119),"")</f>
+        <v/>
+      </c>
+      <c r="H119" s="17">
+        <f>IF(F119="","",1)</f>
+        <v/>
+      </c>
+      <c r="I119" s="17">
+        <f>IFERROR(IF(F119="","",CEILING(G119/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J119" s="62">
+        <f>IFERROR(IF(F119="","",TEXT('Getting Started'!C10+(H119-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I119*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B120" s="18" t="n"/>
+      <c r="F120" s="32" t="n"/>
+      <c r="G120" s="17">
+        <f>IFERROR(SUM(F119:F120),"")</f>
+        <v/>
+      </c>
+      <c r="H120" s="17">
+        <f>IFERROR(IF(F120="","",FLOOR(G119/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I120" s="17">
+        <f>IFERROR(IF(F120="","",CEILING(G120/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J120" s="62">
+        <f>IFERROR(IF(F120="","",TEXT('Getting Started'!C10+(H120-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I120*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" ht="18" customHeight="1">
+      <c r="A121" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B121" s="5" t="n"/>
+      <c r="F121" s="33" t="n"/>
+      <c r="G121" s="17">
+        <f>IFERROR(SUM(F119:F121),"")</f>
+        <v/>
+      </c>
+      <c r="H121" s="17">
+        <f>IFERROR(IF(F121="","",FLOOR(G120/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I121" s="17">
+        <f>IFERROR(IF(F121="","",CEILING(G121/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J121" s="62">
+        <f>IFERROR(IF(F121="","",TEXT('Getting Started'!C10+(H121-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I121*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122" ht="18" customHeight="1">
+      <c r="A122" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B122" s="18" t="n"/>
+      <c r="F122" s="32" t="n"/>
+      <c r="G122" s="17">
+        <f>IFERROR(SUM(F119:F122),"")</f>
+        <v/>
+      </c>
+      <c r="H122" s="17">
+        <f>IFERROR(IF(F122="","",FLOOR(G121/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I122" s="17">
+        <f>IFERROR(IF(F122="","",CEILING(G122/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J122" s="62">
+        <f>IFERROR(IF(F122="","",TEXT('Getting Started'!C10+(H122-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I122*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" ht="18" customHeight="1">
+      <c r="A123" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B123" s="5" t="n"/>
+      <c r="F123" s="33" t="n"/>
+      <c r="G123" s="17">
+        <f>IFERROR(SUM(F119:F123),"")</f>
+        <v/>
+      </c>
+      <c r="H123" s="17">
+        <f>IFERROR(IF(F123="","",FLOOR(G122/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I123" s="17">
+        <f>IFERROR(IF(F123="","",CEILING(G123/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J123" s="62">
+        <f>IFERROR(IF(F123="","",TEXT('Getting Started'!C10+(H123-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I123*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124" ht="18" customHeight="1">
+      <c r="A124" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B124" s="18" t="n"/>
+      <c r="F124" s="32" t="n"/>
+      <c r="G124" s="17">
+        <f>IFERROR(SUM(F119:F124),"")</f>
+        <v/>
+      </c>
+      <c r="H124" s="17">
+        <f>IFERROR(IF(F124="","",FLOOR(G123/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I124" s="17">
+        <f>IFERROR(IF(F124="","",CEILING(G124/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J124" s="62">
+        <f>IFERROR(IF(F124="","",TEXT('Getting Started'!C10+(H124-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I124*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="63" t="n"/>
+    </row>
+    <row r="126" ht="8" customHeight="1"/>
+    <row r="127" ht="24" customHeight="1">
+      <c r="A127" s="52">
+        <f>IF('Course Content'!A34="","  ELECTIVE / OTHER 1","  "&amp;UPPER('Course Content'!A34))</f>
+        <v/>
+      </c>
+      <c r="E127" s="53">
+        <f>IFERROR(IF('Course Content'!B34="","← enter on Course Content tab",'Course Content'!B34),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128" ht="22" customHeight="1">
+      <c r="B128" s="54">
+        <f>'Course Content'!D34</f>
+        <v/>
+      </c>
+      <c r="C128" s="55">
+        <f>IFERROR(IF(B128="","",ROUND(B128/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D128" s="55">
+        <f>IFERROR(IF(C128="","",ROUND(C128/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E128" s="56">
+        <f>IFERROR(IF(B128="","",TEXT('Getting Started'!C10+(B128/D128),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F128" s="26" t="n"/>
+      <c r="G128" s="57">
+        <f>'Course Content'!E34</f>
+        <v/>
+      </c>
+      <c r="H128" s="58">
+        <f>IFERROR(IF(G128="","",ROUND(G128/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I128" s="58">
+        <f>IFERROR(IF(H128="","",ROUND(H128/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J128" s="59">
+        <f>IFERROR(IF(G128="","",TEXT('Getting Started'!C18+(G128/I128),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129" ht="16" customHeight="1">
+      <c r="A129" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="22" customHeight="1">
+      <c r="A130" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B130" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F130" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G130" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H130" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I130" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J130" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="18" customHeight="1">
+      <c r="A131" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B131" s="5" t="n"/>
+      <c r="F131" s="33" t="n"/>
+      <c r="G131" s="17">
+        <f>IFERROR(SUM(F131:F131),"")</f>
+        <v/>
+      </c>
+      <c r="H131" s="17">
+        <f>IF(F131="","",1)</f>
+        <v/>
+      </c>
+      <c r="I131" s="17">
+        <f>IFERROR(IF(F131="","",CEILING(G131/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J131" s="62">
+        <f>IFERROR(IF(F131="","",TEXT('Getting Started'!C10+(H131-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I131*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132" ht="18" customHeight="1">
+      <c r="A132" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B132" s="18" t="n"/>
+      <c r="F132" s="32" t="n"/>
+      <c r="G132" s="17">
+        <f>IFERROR(SUM(F131:F132),"")</f>
+        <v/>
+      </c>
+      <c r="H132" s="17">
+        <f>IFERROR(IF(F132="","",FLOOR(G131/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I132" s="17">
+        <f>IFERROR(IF(F132="","",CEILING(G132/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J132" s="62">
+        <f>IFERROR(IF(F132="","",TEXT('Getting Started'!C10+(H132-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I132*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133" ht="18" customHeight="1">
+      <c r="A133" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B133" s="5" t="n"/>
+      <c r="F133" s="33" t="n"/>
+      <c r="G133" s="17">
+        <f>IFERROR(SUM(F131:F133),"")</f>
+        <v/>
+      </c>
+      <c r="H133" s="17">
+        <f>IFERROR(IF(F133="","",FLOOR(G132/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I133" s="17">
+        <f>IFERROR(IF(F133="","",CEILING(G133/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J133" s="62">
+        <f>IFERROR(IF(F133="","",TEXT('Getting Started'!C10+(H133-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I133*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134" ht="18" customHeight="1">
+      <c r="A134" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B134" s="18" t="n"/>
+      <c r="F134" s="32" t="n"/>
+      <c r="G134" s="17">
+        <f>IFERROR(SUM(F131:F134),"")</f>
+        <v/>
+      </c>
+      <c r="H134" s="17">
+        <f>IFERROR(IF(F134="","",FLOOR(G133/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I134" s="17">
+        <f>IFERROR(IF(F134="","",CEILING(G134/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J134" s="62">
+        <f>IFERROR(IF(F134="","",TEXT('Getting Started'!C10+(H134-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I134*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B135" s="5" t="n"/>
+      <c r="F135" s="33" t="n"/>
+      <c r="G135" s="17">
+        <f>IFERROR(SUM(F131:F135),"")</f>
+        <v/>
+      </c>
+      <c r="H135" s="17">
+        <f>IFERROR(IF(F135="","",FLOOR(G134/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I135" s="17">
+        <f>IFERROR(IF(F135="","",CEILING(G135/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J135" s="62">
+        <f>IFERROR(IF(F135="","",TEXT('Getting Started'!C10+(H135-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I135*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136" ht="18" customHeight="1">
+      <c r="A136" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B136" s="18" t="n"/>
+      <c r="F136" s="32" t="n"/>
+      <c r="G136" s="17">
+        <f>IFERROR(SUM(F131:F136),"")</f>
+        <v/>
+      </c>
+      <c r="H136" s="17">
+        <f>IFERROR(IF(F136="","",FLOOR(G135/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I136" s="17">
+        <f>IFERROR(IF(F136="","",CEILING(G136/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J136" s="62">
+        <f>IFERROR(IF(F136="","",TEXT('Getting Started'!C10+(H136-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I136*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="63" t="n"/>
+    </row>
+    <row r="138" ht="8" customHeight="1"/>
+    <row r="139" ht="24" customHeight="1">
+      <c r="A139" s="52">
+        <f>IF('Course Content'!A35="","  ELECTIVE / OTHER 2","  "&amp;UPPER('Course Content'!A35))</f>
+        <v/>
+      </c>
+      <c r="E139" s="53">
+        <f>IFERROR(IF('Course Content'!B35="","← enter on Course Content tab",'Course Content'!B35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140" ht="22" customHeight="1">
+      <c r="B140" s="54">
+        <f>'Course Content'!D35</f>
+        <v/>
+      </c>
+      <c r="C140" s="55">
+        <f>IFERROR(IF(B140="","",ROUND(B140/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D140" s="55">
+        <f>IFERROR(IF(C140="","",ROUND(C140/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E140" s="56">
+        <f>IFERROR(IF(B140="","",TEXT('Getting Started'!C10+(B140/D140),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F140" s="26" t="n"/>
+      <c r="G140" s="57">
+        <f>'Course Content'!E35</f>
+        <v/>
+      </c>
+      <c r="H140" s="58">
+        <f>IFERROR(IF(G140="","",ROUND(G140/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I140" s="58">
+        <f>IFERROR(IF(H140="","",ROUND(H140/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J140" s="59">
+        <f>IFERROR(IF(G140="","",TEXT('Getting Started'!C18+(G140/I140),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141" ht="16" customHeight="1">
+      <c r="A141" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="22" customHeight="1">
+      <c r="A142" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B142" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F142" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G142" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H142" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I142" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J142" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="18" customHeight="1">
+      <c r="A143" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B143" s="5" t="n"/>
+      <c r="F143" s="33" t="n"/>
+      <c r="G143" s="17">
+        <f>IFERROR(SUM(F143:F143),"")</f>
+        <v/>
+      </c>
+      <c r="H143" s="17">
+        <f>IF(F143="","",1)</f>
+        <v/>
+      </c>
+      <c r="I143" s="17">
+        <f>IFERROR(IF(F143="","",CEILING(G143/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J143" s="62">
+        <f>IFERROR(IF(F143="","",TEXT('Getting Started'!C10+(H143-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I143*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="A144" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B144" s="18" t="n"/>
+      <c r="F144" s="32" t="n"/>
+      <c r="G144" s="17">
+        <f>IFERROR(SUM(F143:F144),"")</f>
+        <v/>
+      </c>
+      <c r="H144" s="17">
+        <f>IFERROR(IF(F144="","",FLOOR(G143/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I144" s="17">
+        <f>IFERROR(IF(F144="","",CEILING(G144/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J144" s="62">
+        <f>IFERROR(IF(F144="","",TEXT('Getting Started'!C10+(H144-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I144*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145" ht="18" customHeight="1">
+      <c r="A145" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B145" s="5" t="n"/>
+      <c r="F145" s="33" t="n"/>
+      <c r="G145" s="17">
+        <f>IFERROR(SUM(F143:F145),"")</f>
+        <v/>
+      </c>
+      <c r="H145" s="17">
+        <f>IFERROR(IF(F145="","",FLOOR(G144/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I145" s="17">
+        <f>IFERROR(IF(F145="","",CEILING(G145/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J145" s="62">
+        <f>IFERROR(IF(F145="","",TEXT('Getting Started'!C10+(H145-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I145*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146" ht="18" customHeight="1">
+      <c r="A146" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B146" s="18" t="n"/>
+      <c r="F146" s="32" t="n"/>
+      <c r="G146" s="17">
+        <f>IFERROR(SUM(F143:F146),"")</f>
+        <v/>
+      </c>
+      <c r="H146" s="17">
+        <f>IFERROR(IF(F146="","",FLOOR(G145/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I146" s="17">
+        <f>IFERROR(IF(F146="","",CEILING(G146/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J146" s="62">
+        <f>IFERROR(IF(F146="","",TEXT('Getting Started'!C10+(H146-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I146*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147" ht="18" customHeight="1">
+      <c r="A147" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B147" s="5" t="n"/>
+      <c r="F147" s="33" t="n"/>
+      <c r="G147" s="17">
+        <f>IFERROR(SUM(F143:F147),"")</f>
+        <v/>
+      </c>
+      <c r="H147" s="17">
+        <f>IFERROR(IF(F147="","",FLOOR(G146/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I147" s="17">
+        <f>IFERROR(IF(F147="","",CEILING(G147/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J147" s="62">
+        <f>IFERROR(IF(F147="","",TEXT('Getting Started'!C10+(H147-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I147*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148" ht="18" customHeight="1">
+      <c r="A148" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B148" s="18" t="n"/>
+      <c r="F148" s="32" t="n"/>
+      <c r="G148" s="17">
+        <f>IFERROR(SUM(F143:F148),"")</f>
+        <v/>
+      </c>
+      <c r="H148" s="17">
+        <f>IFERROR(IF(F148="","",FLOOR(G147/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I148" s="17">
+        <f>IFERROR(IF(F148="","",CEILING(G148/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J148" s="62">
+        <f>IFERROR(IF(F148="","",TEXT('Getting Started'!C10+(H148-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I148*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149" ht="20" customHeight="1">
+      <c r="A149" s="63" t="n"/>
+    </row>
+    <row r="150" ht="8" customHeight="1"/>
+    <row r="151" ht="24" customHeight="1">
+      <c r="A151" s="52">
+        <f>IF('Course Content'!A36="","  ELECTIVE / OTHER 3","  "&amp;UPPER('Course Content'!A36))</f>
+        <v/>
+      </c>
+      <c r="E151" s="53">
+        <f>IFERROR(IF('Course Content'!B36="","← enter on Course Content tab",'Course Content'!B36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152" ht="22" customHeight="1">
+      <c r="B152" s="54">
+        <f>'Course Content'!D36</f>
+        <v/>
+      </c>
+      <c r="C152" s="55">
+        <f>IFERROR(IF(B152="","",ROUND(B152/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D152" s="55">
+        <f>IFERROR(IF(C152="","",ROUND(C152/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E152" s="56">
+        <f>IFERROR(IF(B152="","",TEXT('Getting Started'!C10+(B152/D152),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F152" s="26" t="n"/>
+      <c r="G152" s="57">
+        <f>'Course Content'!E36</f>
+        <v/>
+      </c>
+      <c r="H152" s="58">
+        <f>IFERROR(IF(G152="","",ROUND(G152/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I152" s="58">
+        <f>IFERROR(IF(H152="","",ROUND(H152/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J152" s="59">
+        <f>IFERROR(IF(G152="","",TEXT('Getting Started'!C18+(G152/I152),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153" ht="16" customHeight="1">
+      <c r="A153" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="22" customHeight="1">
+      <c r="A154" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B154" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F154" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G154" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H154" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I154" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J154" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="18" customHeight="1">
+      <c r="A155" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B155" s="5" t="n"/>
+      <c r="F155" s="33" t="n"/>
+      <c r="G155" s="17">
+        <f>IFERROR(SUM(F155:F155),"")</f>
+        <v/>
+      </c>
+      <c r="H155" s="17">
+        <f>IF(F155="","",1)</f>
+        <v/>
+      </c>
+      <c r="I155" s="17">
+        <f>IFERROR(IF(F155="","",CEILING(G155/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J155" s="62">
+        <f>IFERROR(IF(F155="","",TEXT('Getting Started'!C10+(H155-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I155*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="156" ht="18" customHeight="1">
+      <c r="A156" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B156" s="18" t="n"/>
+      <c r="F156" s="32" t="n"/>
+      <c r="G156" s="17">
+        <f>IFERROR(SUM(F155:F156),"")</f>
+        <v/>
+      </c>
+      <c r="H156" s="17">
+        <f>IFERROR(IF(F156="","",FLOOR(G155/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I156" s="17">
+        <f>IFERROR(IF(F156="","",CEILING(G156/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J156" s="62">
+        <f>IFERROR(IF(F156="","",TEXT('Getting Started'!C10+(H156-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I156*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157" ht="18" customHeight="1">
+      <c r="A157" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B157" s="5" t="n"/>
+      <c r="F157" s="33" t="n"/>
+      <c r="G157" s="17">
+        <f>IFERROR(SUM(F155:F157),"")</f>
+        <v/>
+      </c>
+      <c r="H157" s="17">
+        <f>IFERROR(IF(F157="","",FLOOR(G156/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I157" s="17">
+        <f>IFERROR(IF(F157="","",CEILING(G157/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J157" s="62">
+        <f>IFERROR(IF(F157="","",TEXT('Getting Started'!C10+(H157-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I157*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B158" s="18" t="n"/>
+      <c r="F158" s="32" t="n"/>
+      <c r="G158" s="17">
+        <f>IFERROR(SUM(F155:F158),"")</f>
+        <v/>
+      </c>
+      <c r="H158" s="17">
+        <f>IFERROR(IF(F158="","",FLOOR(G157/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I158" s="17">
+        <f>IFERROR(IF(F158="","",CEILING(G158/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J158" s="62">
+        <f>IFERROR(IF(F158="","",TEXT('Getting Started'!C10+(H158-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I158*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159" ht="18" customHeight="1">
+      <c r="A159" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B159" s="5" t="n"/>
+      <c r="F159" s="33" t="n"/>
+      <c r="G159" s="17">
+        <f>IFERROR(SUM(F155:F159),"")</f>
+        <v/>
+      </c>
+      <c r="H159" s="17">
+        <f>IFERROR(IF(F159="","",FLOOR(G158/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I159" s="17">
+        <f>IFERROR(IF(F159="","",CEILING(G159/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J159" s="62">
+        <f>IFERROR(IF(F159="","",TEXT('Getting Started'!C10+(H159-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I159*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B160" s="18" t="n"/>
+      <c r="F160" s="32" t="n"/>
+      <c r="G160" s="17">
+        <f>IFERROR(SUM(F155:F160),"")</f>
+        <v/>
+      </c>
+      <c r="H160" s="17">
+        <f>IFERROR(IF(F160="","",FLOOR(G159/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I160" s="17">
+        <f>IFERROR(IF(F160="","",CEILING(G160/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J160" s="62">
+        <f>IFERROR(IF(F160="","",TEXT('Getting Started'!C10+(H160-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I160*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="161" ht="20" customHeight="1">
+      <c r="A161" s="63" t="n"/>
+    </row>
+    <row r="162" ht="8" customHeight="1"/>
+    <row r="163" ht="24" customHeight="1">
+      <c r="A163" s="52">
+        <f>IF('Course Content'!A37="","  ELECTIVE / OTHER 4","  "&amp;UPPER('Course Content'!A37))</f>
+        <v/>
+      </c>
+      <c r="E163" s="53">
+        <f>IFERROR(IF('Course Content'!B37="","← enter on Course Content tab",'Course Content'!B37),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164" ht="22" customHeight="1">
+      <c r="B164" s="54">
+        <f>'Course Content'!D37</f>
+        <v/>
+      </c>
+      <c r="C164" s="55">
+        <f>IFERROR(IF(B164="","",ROUND(B164/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="D164" s="55">
+        <f>IFERROR(IF(C164="","",ROUND(C164/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E164" s="56">
+        <f>IFERROR(IF(B164="","",TEXT('Getting Started'!C10+(B164/D164),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+      <c r="F164" s="26" t="n"/>
+      <c r="G164" s="57">
+        <f>'Course Content'!E37</f>
+        <v/>
+      </c>
+      <c r="H164" s="58">
+        <f>IFERROR(IF(G164="","",ROUND(G164/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I164" s="58">
+        <f>IFERROR(IF(H164="","",ROUND(H164/'Getting Started'!C7,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J164" s="59">
+        <f>IFERROR(IF(G164="","",TEXT('Getting Started'!C18+(G164/I164),"MMM D, YYYY")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="165" ht="16" customHeight="1">
+      <c r="A165" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="22" customHeight="1">
+      <c r="A166" s="48" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B166" s="48" t="inlineStr">
+        <is>
+          <t>Book / Component Title</t>
+        </is>
+      </c>
+      <c r="F166" s="48" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="G166" s="48" t="inlineStr">
+        <is>
+          <t>Cumul.</t>
+        </is>
+      </c>
+      <c r="H166" s="48" t="inlineStr">
+        <is>
+          <t>Start
+Week</t>
+        </is>
+      </c>
+      <c r="I166" s="48" t="inlineStr">
+        <is>
+          <t>End
+Week</t>
+        </is>
+      </c>
+      <c r="J166" s="48" t="inlineStr">
+        <is>
+          <t>Est. Dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="18" customHeight="1">
+      <c r="A167" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="B167" s="5" t="n"/>
+      <c r="F167" s="33" t="n"/>
+      <c r="G167" s="17">
+        <f>IFERROR(SUM(F167:F167),"")</f>
+        <v/>
+      </c>
+      <c r="H167" s="17">
+        <f>IF(F167="","",1)</f>
+        <v/>
+      </c>
+      <c r="I167" s="17">
+        <f>IFERROR(IF(F167="","",CEILING(G167/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J167" s="62">
+        <f>IFERROR(IF(F167="","",TEXT('Getting Started'!C10+(H167-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I167*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="168" ht="18" customHeight="1">
+      <c r="A168" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B168" s="18" t="n"/>
+      <c r="F168" s="32" t="n"/>
+      <c r="G168" s="17">
+        <f>IFERROR(SUM(F167:F168),"")</f>
+        <v/>
+      </c>
+      <c r="H168" s="17">
+        <f>IFERROR(IF(F168="","",FLOOR(G167/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I168" s="17">
+        <f>IFERROR(IF(F168="","",CEILING(G168/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J168" s="62">
+        <f>IFERROR(IF(F168="","",TEXT('Getting Started'!C10+(H168-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I168*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169" ht="18" customHeight="1">
+      <c r="A169" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B169" s="5" t="n"/>
+      <c r="F169" s="33" t="n"/>
+      <c r="G169" s="17">
+        <f>IFERROR(SUM(F167:F169),"")</f>
+        <v/>
+      </c>
+      <c r="H169" s="17">
+        <f>IFERROR(IF(F169="","",FLOOR(G168/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I169" s="17">
+        <f>IFERROR(IF(F169="","",CEILING(G169/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J169" s="62">
+        <f>IFERROR(IF(F169="","",TEXT('Getting Started'!C10+(H169-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I169*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="170" ht="18" customHeight="1">
+      <c r="A170" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B170" s="18" t="n"/>
+      <c r="F170" s="32" t="n"/>
+      <c r="G170" s="17">
+        <f>IFERROR(SUM(F167:F170),"")</f>
+        <v/>
+      </c>
+      <c r="H170" s="17">
+        <f>IFERROR(IF(F170="","",FLOOR(G169/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I170" s="17">
+        <f>IFERROR(IF(F170="","",CEILING(G170/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J170" s="62">
+        <f>IFERROR(IF(F170="","",TEXT('Getting Started'!C10+(H170-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I170*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171" ht="18" customHeight="1">
+      <c r="A171" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B171" s="5" t="n"/>
+      <c r="F171" s="33" t="n"/>
+      <c r="G171" s="17">
+        <f>IFERROR(SUM(F167:F171),"")</f>
+        <v/>
+      </c>
+      <c r="H171" s="17">
+        <f>IFERROR(IF(F171="","",FLOOR(G170/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I171" s="17">
+        <f>IFERROR(IF(F171="","",CEILING(G171/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J171" s="62">
+        <f>IFERROR(IF(F171="","",TEXT('Getting Started'!C10+(H171-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I171*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="A172" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B172" s="18" t="n"/>
+      <c r="F172" s="32" t="n"/>
+      <c r="G172" s="17">
+        <f>IFERROR(SUM(F167:F172),"")</f>
+        <v/>
+      </c>
+      <c r="H172" s="17">
+        <f>IFERROR(IF(F172="","",FLOOR(G171/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
+        <v/>
+      </c>
+      <c r="I172" s="17">
+        <f>IFERROR(IF(F172="","",CEILING(G172/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
+        <v/>
+      </c>
+      <c r="J172" s="62">
+        <f>IFERROR(IF(F172="","",TEXT('Getting Started'!C10+(H172-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I172*7,"MMM D")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="173" ht="20" customHeight="1">
+      <c r="A173" s="63" t="n"/>
+    </row>
+    <row r="174" ht="8" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="158">
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="E19:J19"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="A165:J165"/>
+    <mergeCell ref="B123:E123"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B110:E110"/>
+    <mergeCell ref="A93:J93"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A173:J173"/>
+    <mergeCell ref="B100:E100"/>
+    <mergeCell ref="A77:J77"/>
+    <mergeCell ref="B109:E109"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B155:E155"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="A69:J69"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="E139:J139"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B136:E136"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="A163:D163"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B112:E112"/>
+    <mergeCell ref="E79:J79"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A81:J81"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="A161:J161"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B154:E154"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B106:E106"/>
+    <mergeCell ref="A127:D127"/>
+    <mergeCell ref="E163:J163"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B156:E156"/>
+    <mergeCell ref="E91:J91"/>
+    <mergeCell ref="B131:E131"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="A79:D79"/>
+    <mergeCell ref="E115:J115"/>
+    <mergeCell ref="B130:E130"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B132:E132"/>
+    <mergeCell ref="B166:E166"/>
+    <mergeCell ref="A149:J149"/>
+    <mergeCell ref="B119:E119"/>
+    <mergeCell ref="E127:J127"/>
+    <mergeCell ref="A139:D139"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="B168:E168"/>
+    <mergeCell ref="B84:E84"/>
+    <mergeCell ref="B118:E118"/>
+    <mergeCell ref="A141:J141"/>
+    <mergeCell ref="A91:D91"/>
+    <mergeCell ref="B158:E158"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="B142:E142"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="A125:J125"/>
+    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="B160:E160"/>
+    <mergeCell ref="B169:E169"/>
+    <mergeCell ref="B144:E144"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B134:E134"/>
+    <mergeCell ref="B121:E121"/>
+    <mergeCell ref="A103:D103"/>
+    <mergeCell ref="B122:E122"/>
+    <mergeCell ref="B71:E71"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="A153:J153"/>
+    <mergeCell ref="B120:E120"/>
+    <mergeCell ref="A137:J137"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="A41:J41"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="E151:J151"/>
+    <mergeCell ref="B170:E170"/>
+    <mergeCell ref="E55:J55"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B157:E157"/>
+    <mergeCell ref="E67:J67"/>
+    <mergeCell ref="B171:E171"/>
+    <mergeCell ref="A101:J101"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B172:E172"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="E103:J103"/>
+    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="B143:E143"/>
+    <mergeCell ref="A53:J53"/>
+    <mergeCell ref="E31:J31"/>
+    <mergeCell ref="B124:E124"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="B133:E133"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="A117:J117"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="B135:E135"/>
+    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B159:E159"/>
+    <mergeCell ref="E7:J7"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A45:J45"/>
+    <mergeCell ref="B96:E96"/>
+    <mergeCell ref="B167:E167"/>
+    <mergeCell ref="B70:E70"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="A65:J65"/>
+    <mergeCell ref="E43:J43"/>
+    <mergeCell ref="B111:E111"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="A89:J89"/>
+    <mergeCell ref="B73:E73"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B82:E82"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A55:D55"/>
+    <mergeCell ref="A105:J105"/>
+    <mergeCell ref="B147:E147"/>
+    <mergeCell ref="A57:J57"/>
+    <mergeCell ref="A113:J113"/>
+    <mergeCell ref="A151:D151"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="A129:J129"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Redesign student tab: school days selector + clean schedule table
- School days selector (Mon–Sat): mark any day with X, Days/Week
  auto-counts via COUNTA and feeds all pace calculations
- Simple one-row-per-subject schedule table:
  Subject | Curriculum | S1 Total | S1/Week | S1/Day | S2 Total | S2/Week | S2/Day | Unit Type
- All curriculum data pulled from Course Content (Slot 1)
- Semester date strips reference Getting Started dates
- Removed complex component breakdown and old add_subject_section

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="MM/DD/YYYY"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -119,19 +119,31 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="005C7A52"/>
-      <sz val="9"/>
+      <color rgb="00CE8282"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FAF8F6"/>
+      <color rgb="006B5C55"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="005C7A52"/>
       <sz val="9"/>
     </font>
     <font>
@@ -143,35 +155,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="006B5C55"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="005C7A52"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="005C7A52"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="008A6A30"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="008A6A30"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="006B5C55"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="23">
@@ -345,15 +336,24 @@
       </bottom>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="00CE8282"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CE8282"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CE8282"/>
+      </top>
       <bottom style="thin">
-        <color rgb="00D4C4BB"/>
+        <color rgb="00CE8282"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -485,7 +485,10 @@
     <xf numFmtId="0" fontId="15" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -494,26 +497,26 @@
     <xf numFmtId="0" fontId="10" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -521,26 +524,17 @@
     <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5388,3528 +5382,729 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J173"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="4" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="1">
+    <row r="1" ht="44" customHeight="1">
+      <c r="A1" s="45">
         <f>IF('Getting Started'!B29="","Student 1",'Getting Started'!B29)</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="45">
+      <c r="A2" s="46">
         <f>IFERROR("Grade: "&amp;'Getting Started'!F29&amp;"   ·   School Year: "&amp;'Getting Started'!C6,"")</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="46">
-        <f>IFERROR("SEMESTER 1   "&amp;TEXT('Getting Started'!C10,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C11,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C15&amp;" wks)","SEMESTER 1")</f>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="47">
+        <f>IFERROR("SEM 1   "&amp;TEXT('Getting Started'!C10,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C11,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C15&amp;" school wks)","SEMESTER 1")</f>
         <v/>
       </c>
       <c r="F4" s="26" t="n"/>
-      <c r="G4" s="47">
-        <f>IFERROR("SEMESTER 2   "&amp;TEXT('Getting Started'!C18,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C19,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C23&amp;" wks)","SEMESTER 2")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="48" t="inlineStr">
-        <is>
-          <t>Subject  /  Curriculum</t>
-        </is>
-      </c>
-      <c r="B5" s="49" t="inlineStr">
+      <c r="G4" s="48">
+        <f>IFERROR("SEM 2   "&amp;TEXT('Getting Started'!C18,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C19,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C23&amp;" school wks)","SEMESTER 2")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="8" customHeight="1"/>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SCHOOL DAYS  ·  Mark each day this student attends</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="50" t="inlineStr">
+        <is>
+          <t>Mark with  X  →</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>Days / Week:</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="26" t="n"/>
+      <c r="B8" s="51" t="n"/>
+      <c r="C8" s="51" t="n"/>
+      <c r="D8" s="51" t="n"/>
+      <c r="E8" s="51" t="n"/>
+      <c r="F8" s="51" t="n"/>
+      <c r="G8" s="51" t="n"/>
+      <c r="H8" s="52">
+        <f>MAX(1,COUNTA(B8:G8))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="8" customHeight="1"/>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="53" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="B10" s="53" t="inlineStr">
+        <is>
+          <t>Curriculum  /  Book</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
         <is>
           <t>Sem 1
-Units</t>
-        </is>
-      </c>
-      <c r="C5" s="49" t="inlineStr">
-        <is>
-          <t>/ Week</t>
-        </is>
-      </c>
-      <c r="D5" s="49" t="inlineStr">
-        <is>
-          <t>/ Day</t>
-        </is>
-      </c>
-      <c r="E5" s="49" t="inlineStr">
-        <is>
-          <t>Est. End</t>
-        </is>
-      </c>
-      <c r="F5" s="50" t="inlineStr"/>
-      <c r="G5" s="51" t="inlineStr">
+Total</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>Sem 1
+/ Week</t>
+        </is>
+      </c>
+      <c r="E10" s="54" t="inlineStr">
+        <is>
+          <t>Sem 1
+/ Day</t>
+        </is>
+      </c>
+      <c r="F10" s="26" t="n"/>
+      <c r="G10" s="55" t="inlineStr">
         <is>
           <t>Sem 2
-Units</t>
-        </is>
-      </c>
-      <c r="H5" s="51" t="inlineStr">
-        <is>
-          <t>/ Week</t>
-        </is>
-      </c>
-      <c r="I5" s="51" t="inlineStr">
-        <is>
-          <t>/ Day</t>
-        </is>
-      </c>
-      <c r="J5" s="51" t="inlineStr">
-        <is>
-          <t>Est. End</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="8" customHeight="1"/>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  BIBLE</t>
-        </is>
-      </c>
-      <c r="E7" s="53">
-        <f>IFERROR(IF('Course Content'!B24="","← enter on Course Content tab",'Course Content'!B24),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="54">
-        <f>'Course Content'!D24</f>
-        <v/>
-      </c>
-      <c r="C8" s="55">
-        <f>IFERROR(IF(B8="","",ROUND(B8/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D8" s="55">
-        <f>IFERROR(IF(C8="","",ROUND(C8/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E8" s="56">
-        <f>IFERROR(IF(B8="","",TEXT('Getting Started'!C10+(B8/D8),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="26" t="n"/>
-      <c r="G8" s="57">
-        <f>'Course Content'!E24</f>
-        <v/>
-      </c>
-      <c r="H8" s="58">
-        <f>IFERROR(IF(G8="","",ROUND(G8/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="58">
-        <f>IFERROR(IF(H8="","",ROUND(H8/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="59">
-        <f>IFERROR(IF(G8="","",TEXT('Getting Started'!C18+(G8/I8),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B10" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F10" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G10" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H10" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I10" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J10" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="F11" s="33" t="n"/>
-      <c r="G11" s="17">
-        <f>IFERROR(SUM(F11:F11),"")</f>
-        <v/>
-      </c>
-      <c r="H11" s="17">
-        <f>IF(F11="","",1)</f>
-        <v/>
-      </c>
-      <c r="I11" s="17">
-        <f>IFERROR(IF(F11="","",CEILING(G11/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="62">
-        <f>IFERROR(IF(F11="","",TEXT('Getting Started'!C10+(H11-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I11*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" s="18" t="n"/>
-      <c r="F12" s="32" t="n"/>
-      <c r="G12" s="17">
-        <f>IFERROR(SUM(F11:F12),"")</f>
-        <v/>
-      </c>
-      <c r="H12" s="17">
-        <f>IFERROR(IF(F12="","",FLOOR(G11/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="17">
-        <f>IFERROR(IF(F12="","",CEILING(G12/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="62">
-        <f>IFERROR(IF(F12="","",TEXT('Getting Started'!C10+(H12-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I12*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="F13" s="33" t="n"/>
-      <c r="G13" s="17">
-        <f>IFERROR(SUM(F11:F13),"")</f>
-        <v/>
-      </c>
-      <c r="H13" s="17">
-        <f>IFERROR(IF(F13="","",FLOOR(G12/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I13" s="17">
-        <f>IFERROR(IF(F13="","",CEILING(G13/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="62">
-        <f>IFERROR(IF(F13="","",TEXT('Getting Started'!C10+(H13-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I13*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B14" s="18" t="n"/>
-      <c r="F14" s="32" t="n"/>
-      <c r="G14" s="17">
-        <f>IFERROR(SUM(F11:F14),"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="17">
-        <f>IFERROR(IF(F14="","",FLOOR(G13/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="17">
-        <f>IFERROR(IF(F14="","",CEILING(G14/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="62">
-        <f>IFERROR(IF(F14="","",TEXT('Getting Started'!C10+(H14-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I14*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="F15" s="33" t="n"/>
-      <c r="G15" s="17">
-        <f>IFERROR(SUM(F11:F15),"")</f>
-        <v/>
-      </c>
-      <c r="H15" s="17">
-        <f>IFERROR(IF(F15="","",FLOOR(G14/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="17">
-        <f>IFERROR(IF(F15="","",CEILING(G15/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="62">
-        <f>IFERROR(IF(F15="","",TEXT('Getting Started'!C10+(H15-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I15*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B16" s="18" t="n"/>
-      <c r="F16" s="32" t="n"/>
-      <c r="G16" s="17">
-        <f>IFERROR(SUM(F11:F16),"")</f>
-        <v/>
-      </c>
-      <c r="H16" s="17">
-        <f>IFERROR(IF(F16="","",FLOOR(G15/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="17">
-        <f>IFERROR(IF(F16="","",CEILING(G16/((IFERROR(B8,0)+IFERROR(G8,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="62">
-        <f>IFERROR(IF(F16="","",TEXT('Getting Started'!C10+(H16-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I16*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="63" t="n"/>
-    </row>
-    <row r="18" ht="8" customHeight="1"/>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MATH</t>
-        </is>
-      </c>
-      <c r="E19" s="53">
-        <f>IFERROR(IF('Course Content'!B25="","← enter on Course Content tab",'Course Content'!B25),"")</f>
+Total</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>Sem 2
+/ Week</t>
+        </is>
+      </c>
+      <c r="I10" s="55" t="inlineStr">
+        <is>
+          <t>Sem 2
+/ Day</t>
+        </is>
+      </c>
+      <c r="J10" s="53" t="inlineStr">
+        <is>
+          <t>Unit
+Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Bible</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>IFERROR(IF('Course Content'!B24="","—",'Course Content'!B24),"")</f>
+        <v/>
+      </c>
+      <c r="C11" s="56">
+        <f>IFERROR(IF('Course Content'!D24="","—",'Course Content'!D24),"")</f>
+        <v/>
+      </c>
+      <c r="D11" s="56">
+        <f>IFERROR(IF('Course Content'!D24="","",ROUND('Course Content'!D24/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E11" s="57">
+        <f>IFERROR(IF(D11="","",ROUND(D11/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="26" t="n"/>
+      <c r="G11" s="58">
+        <f>IFERROR(IF('Course Content'!E24="","—",'Course Content'!E24),"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="58">
+        <f>IFERROR(IF('Course Content'!E24="","",ROUND('Course Content'!E24/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="59">
+        <f>IFERROR(IF(H11="","",ROUND(H11/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="60">
+        <f>IFERROR(IF('Course Content'!C24="","",'Course Content'!C24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>Math</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <f>IFERROR(IF('Course Content'!B25="","—",'Course Content'!B25),"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="56">
+        <f>IFERROR(IF('Course Content'!D25="","—",'Course Content'!D25),"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="56">
+        <f>IFERROR(IF('Course Content'!D25="","",ROUND('Course Content'!D25/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="57">
+        <f>IFERROR(IF(D12="","",ROUND(D12/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="58">
+        <f>IFERROR(IF('Course Content'!E25="","—",'Course Content'!E25),"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="58">
+        <f>IFERROR(IF('Course Content'!E25="","",ROUND('Course Content'!E25/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="59">
+        <f>IFERROR(IF(H12="","",ROUND(H12/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="61">
+        <f>IFERROR(IF('Course Content'!C25="","",'Course Content'!C25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>IFERROR(IF('Course Content'!B26="","—",'Course Content'!B26),"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="56">
+        <f>IFERROR(IF('Course Content'!D26="","—",'Course Content'!D26),"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="56">
+        <f>IFERROR(IF('Course Content'!D26="","",ROUND('Course Content'!D26/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="57">
+        <f>IFERROR(IF(D13="","",ROUND(D13/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="58">
+        <f>IFERROR(IF('Course Content'!E26="","—",'Course Content'!E26),"")</f>
+        <v/>
+      </c>
+      <c r="H13" s="58">
+        <f>IFERROR(IF('Course Content'!E26="","",ROUND('Course Content'!E26/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="59">
+        <f>IFERROR(IF(H13="","",ROUND(H13/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="60">
+        <f>IFERROR(IF('Course Content'!C26="","",'Course Content'!C26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B14" s="18">
+        <f>IFERROR(IF('Course Content'!B27="","—",'Course Content'!B27),"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="56">
+        <f>IFERROR(IF('Course Content'!D27="","—",'Course Content'!D27),"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="56">
+        <f>IFERROR(IF('Course Content'!D27="","",ROUND('Course Content'!D27/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="57">
+        <f>IFERROR(IF(D14="","",ROUND(D14/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="26" t="n"/>
+      <c r="G14" s="58">
+        <f>IFERROR(IF('Course Content'!E27="","—",'Course Content'!E27),"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="58">
+        <f>IFERROR(IF('Course Content'!E27="","",ROUND('Course Content'!E27/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="59">
+        <f>IFERROR(IF(H14="","",ROUND(H14/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="61">
+        <f>IFERROR(IF('Course Content'!C27="","",'Course Content'!C27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>Writing / Composition</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>IFERROR(IF('Course Content'!B28="","—",'Course Content'!B28),"")</f>
+        <v/>
+      </c>
+      <c r="C15" s="56">
+        <f>IFERROR(IF('Course Content'!D28="","—",'Course Content'!D28),"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="56">
+        <f>IFERROR(IF('Course Content'!D28="","",ROUND('Course Content'!D28/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="57">
+        <f>IFERROR(IF(D15="","",ROUND(D15/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="26" t="n"/>
+      <c r="G15" s="58">
+        <f>IFERROR(IF('Course Content'!E28="","—",'Course Content'!E28),"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="58">
+        <f>IFERROR(IF('Course Content'!E28="","",ROUND('Course Content'!E28/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="59">
+        <f>IFERROR(IF(H15="","",ROUND(H15/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="60">
+        <f>IFERROR(IF('Course Content'!C28="","",'Course Content'!C28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="B16" s="18">
+        <f>IFERROR(IF('Course Content'!B29="","—",'Course Content'!B29),"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="56">
+        <f>IFERROR(IF('Course Content'!D29="","—",'Course Content'!D29),"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="56">
+        <f>IFERROR(IF('Course Content'!D29="","",ROUND('Course Content'!D29/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="57">
+        <f>IFERROR(IF(D16="","",ROUND(D16/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="26" t="n"/>
+      <c r="G16" s="58">
+        <f>IFERROR(IF('Course Content'!E29="","—",'Course Content'!E29),"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="58">
+        <f>IFERROR(IF('Course Content'!E29="","",ROUND('Course Content'!E29/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="59">
+        <f>IFERROR(IF(H16="","",ROUND(H16/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="61">
+        <f>IFERROR(IF('Course Content'!C29="","",'Course Content'!C29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>IFERROR(IF('Course Content'!B30="","—",'Course Content'!B30),"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="56">
+        <f>IFERROR(IF('Course Content'!D30="","—",'Course Content'!D30),"")</f>
+        <v/>
+      </c>
+      <c r="D17" s="56">
+        <f>IFERROR(IF('Course Content'!D30="","",ROUND('Course Content'!D30/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E17" s="57">
+        <f>IFERROR(IF(D17="","",ROUND(D17/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="26" t="n"/>
+      <c r="G17" s="58">
+        <f>IFERROR(IF('Course Content'!E30="","—",'Course Content'!E30),"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="58">
+        <f>IFERROR(IF('Course Content'!E30="","",ROUND('Course Content'!E30/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="59">
+        <f>IFERROR(IF(H17="","",ROUND(H17/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="60">
+        <f>IFERROR(IF('Course Content'!C30="","",'Course Content'!C30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B18" s="18">
+        <f>IFERROR(IF('Course Content'!B31="","—",'Course Content'!B31),"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="56">
+        <f>IFERROR(IF('Course Content'!D31="","—",'Course Content'!D31),"")</f>
+        <v/>
+      </c>
+      <c r="D18" s="56">
+        <f>IFERROR(IF('Course Content'!D31="","",ROUND('Course Content'!D31/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E18" s="57">
+        <f>IFERROR(IF(D18="","",ROUND(D18/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="26" t="n"/>
+      <c r="G18" s="58">
+        <f>IFERROR(IF('Course Content'!E31="","—",'Course Content'!E31),"")</f>
+        <v/>
+      </c>
+      <c r="H18" s="58">
+        <f>IFERROR(IF('Course Content'!E31="","",ROUND('Course Content'!E31/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="59">
+        <f>IFERROR(IF(H18="","",ROUND(H18/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="61">
+        <f>IFERROR(IF('Course Content'!C31="","",'Course Content'!C31),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>IFERROR(IF('Course Content'!B32="","—",'Course Content'!B32),"")</f>
+        <v/>
+      </c>
+      <c r="C19" s="56">
+        <f>IFERROR(IF('Course Content'!D32="","—",'Course Content'!D32),"")</f>
+        <v/>
+      </c>
+      <c r="D19" s="56">
+        <f>IFERROR(IF('Course Content'!D32="","",ROUND('Course Content'!D32/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="57">
+        <f>IFERROR(IF(D19="","",ROUND(D19/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="58">
+        <f>IFERROR(IF('Course Content'!E32="","—",'Course Content'!E32),"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="58">
+        <f>IFERROR(IF('Course Content'!E32="","",ROUND('Course Content'!E32/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="59">
+        <f>IFERROR(IF(H19="","",ROUND(H19/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="60">
+        <f>IFERROR(IF('Course Content'!C32="","",'Course Content'!C32),"")</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
-      <c r="B20" s="54">
-        <f>'Course Content'!D25</f>
-        <v/>
-      </c>
-      <c r="C20" s="55">
-        <f>IFERROR(IF(B20="","",ROUND(B20/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D20" s="55">
-        <f>IFERROR(IF(C20="","",ROUND(C20/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E20" s="56">
-        <f>IFERROR(IF(B20="","",TEXT('Getting Started'!C10+(B20/D20),"MMM D, YYYY")),"")</f>
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>IFERROR(IF('Course Content'!B33="","—",'Course Content'!B33),"")</f>
+        <v/>
+      </c>
+      <c r="C20" s="56">
+        <f>IFERROR(IF('Course Content'!D33="","—",'Course Content'!D33),"")</f>
+        <v/>
+      </c>
+      <c r="D20" s="56">
+        <f>IFERROR(IF('Course Content'!D33="","",ROUND('Course Content'!D33/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="57">
+        <f>IFERROR(IF(D20="","",ROUND(D20/I9,1)),"")</f>
         <v/>
       </c>
       <c r="F20" s="26" t="n"/>
-      <c r="G20" s="57">
-        <f>'Course Content'!E25</f>
+      <c r="G20" s="58">
+        <f>IFERROR(IF('Course Content'!E33="","—",'Course Content'!E33),"")</f>
         <v/>
       </c>
       <c r="H20" s="58">
-        <f>IFERROR(IF(G20="","",ROUND(G20/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="58">
-        <f>IFERROR(IF(H20="","",ROUND(H20/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="59">
-        <f>IFERROR(IF(G20="","",TEXT('Getting Started'!C18+(G20/I20),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
+        <f>IFERROR(IF('Course Content'!E33="","",ROUND('Course Content'!E33/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="59">
+        <f>IFERROR(IF(H20="","",ROUND(H20/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="61">
+        <f>IFERROR(IF('Course Content'!C33="","",'Course Content'!C33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="31">
+        <f>IF('Course Content'!A34="Elective / Other 1","Elective / Other 1",'Course Content'!A34)</f>
+        <v/>
+      </c>
+      <c r="B21" s="5">
+        <f>IFERROR(IF('Course Content'!B34="","—",'Course Content'!B34),"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="56">
+        <f>IFERROR(IF('Course Content'!D34="","—",'Course Content'!D34),"")</f>
+        <v/>
+      </c>
+      <c r="D21" s="56">
+        <f>IFERROR(IF('Course Content'!D34="","",ROUND('Course Content'!D34/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E21" s="57">
+        <f>IFERROR(IF(D21="","",ROUND(D21/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F21" s="26" t="n"/>
+      <c r="G21" s="58">
+        <f>IFERROR(IF('Course Content'!E34="","—",'Course Content'!E34),"")</f>
+        <v/>
+      </c>
+      <c r="H21" s="58">
+        <f>IFERROR(IF('Course Content'!E34="","",ROUND('Course Content'!E34/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I21" s="59">
+        <f>IFERROR(IF(H21="","",ROUND(H21/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J21" s="60">
+        <f>IFERROR(IF('Course Content'!C34="","",'Course Content'!C34),"")</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B22" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F22" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G22" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H22" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I22" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J22" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" s="5" t="n"/>
-      <c r="F23" s="33" t="n"/>
-      <c r="G23" s="17">
-        <f>IFERROR(SUM(F23:F23),"")</f>
-        <v/>
-      </c>
-      <c r="H23" s="17">
-        <f>IF(F23="","",1)</f>
-        <v/>
-      </c>
-      <c r="I23" s="17">
-        <f>IFERROR(IF(F23="","",CEILING(G23/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J23" s="62">
-        <f>IFERROR(IF(F23="","",TEXT('Getting Started'!C10+(H23-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I23*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B24" s="18" t="n"/>
-      <c r="F24" s="32" t="n"/>
-      <c r="G24" s="17">
-        <f>IFERROR(SUM(F23:F24),"")</f>
-        <v/>
-      </c>
-      <c r="H24" s="17">
-        <f>IFERROR(IF(F24="","",FLOOR(G23/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I24" s="17">
-        <f>IFERROR(IF(F24="","",CEILING(G24/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J24" s="62">
-        <f>IFERROR(IF(F24="","",TEXT('Getting Started'!C10+(H24-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I24*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B25" s="5" t="n"/>
-      <c r="F25" s="33" t="n"/>
-      <c r="G25" s="17">
-        <f>IFERROR(SUM(F23:F25),"")</f>
-        <v/>
-      </c>
-      <c r="H25" s="17">
-        <f>IFERROR(IF(F25="","",FLOOR(G24/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I25" s="17">
-        <f>IFERROR(IF(F25="","",CEILING(G25/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="62">
-        <f>IFERROR(IF(F25="","",TEXT('Getting Started'!C10+(H25-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I25*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B26" s="18" t="n"/>
-      <c r="F26" s="32" t="n"/>
-      <c r="G26" s="17">
-        <f>IFERROR(SUM(F23:F26),"")</f>
-        <v/>
-      </c>
-      <c r="H26" s="17">
-        <f>IFERROR(IF(F26="","",FLOOR(G25/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I26" s="17">
-        <f>IFERROR(IF(F26="","",CEILING(G26/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J26" s="62">
-        <f>IFERROR(IF(F26="","",TEXT('Getting Started'!C10+(H26-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I26*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B27" s="5" t="n"/>
-      <c r="F27" s="33" t="n"/>
-      <c r="G27" s="17">
-        <f>IFERROR(SUM(F23:F27),"")</f>
-        <v/>
-      </c>
-      <c r="H27" s="17">
-        <f>IFERROR(IF(F27="","",FLOOR(G26/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I27" s="17">
-        <f>IFERROR(IF(F27="","",CEILING(G27/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J27" s="62">
-        <f>IFERROR(IF(F27="","",TEXT('Getting Started'!C10+(H27-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I27*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B28" s="18" t="n"/>
-      <c r="F28" s="32" t="n"/>
-      <c r="G28" s="17">
-        <f>IFERROR(SUM(F23:F28),"")</f>
-        <v/>
-      </c>
-      <c r="H28" s="17">
-        <f>IFERROR(IF(F28="","",FLOOR(G27/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I28" s="17">
-        <f>IFERROR(IF(F28="","",CEILING(G28/((IFERROR(B20,0)+IFERROR(G20,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J28" s="62">
-        <f>IFERROR(IF(F28="","",TEXT('Getting Started'!C10+(H28-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I28*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="63" t="n"/>
-    </row>
-    <row r="30" ht="8" customHeight="1"/>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ENGLISH / LANGUAGE ARTS</t>
-        </is>
-      </c>
-      <c r="E31" s="53">
-        <f>IFERROR(IF('Course Content'!B26="","← enter on Course Content tab",'Course Content'!B26),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="54">
-        <f>'Course Content'!D26</f>
-        <v/>
-      </c>
-      <c r="C32" s="55">
-        <f>IFERROR(IF(B32="","",ROUND(B32/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D32" s="55">
-        <f>IFERROR(IF(C32="","",ROUND(C32/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E32" s="56">
-        <f>IFERROR(IF(B32="","",TEXT('Getting Started'!C10+(B32/D32),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F32" s="26" t="n"/>
-      <c r="G32" s="57">
-        <f>'Course Content'!E26</f>
-        <v/>
-      </c>
-      <c r="H32" s="58">
-        <f>IFERROR(IF(G32="","",ROUND(G32/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I32" s="58">
-        <f>IFERROR(IF(H32="","",ROUND(H32/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="59">
-        <f>IFERROR(IF(G32="","",TEXT('Getting Started'!C18+(G32/I32),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B34" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F34" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G34" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H34" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I34" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J34" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B35" s="5" t="n"/>
-      <c r="F35" s="33" t="n"/>
-      <c r="G35" s="17">
-        <f>IFERROR(SUM(F35:F35),"")</f>
-        <v/>
-      </c>
-      <c r="H35" s="17">
-        <f>IF(F35="","",1)</f>
-        <v/>
-      </c>
-      <c r="I35" s="17">
-        <f>IFERROR(IF(F35="","",CEILING(G35/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J35" s="62">
-        <f>IFERROR(IF(F35="","",TEXT('Getting Started'!C10+(H35-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I35*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B36" s="18" t="n"/>
-      <c r="F36" s="32" t="n"/>
-      <c r="G36" s="17">
-        <f>IFERROR(SUM(F35:F36),"")</f>
-        <v/>
-      </c>
-      <c r="H36" s="17">
-        <f>IFERROR(IF(F36="","",FLOOR(G35/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I36" s="17">
-        <f>IFERROR(IF(F36="","",CEILING(G36/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J36" s="62">
-        <f>IFERROR(IF(F36="","",TEXT('Getting Started'!C10+(H36-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I36*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B37" s="5" t="n"/>
-      <c r="F37" s="33" t="n"/>
-      <c r="G37" s="17">
-        <f>IFERROR(SUM(F35:F37),"")</f>
-        <v/>
-      </c>
-      <c r="H37" s="17">
-        <f>IFERROR(IF(F37="","",FLOOR(G36/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I37" s="17">
-        <f>IFERROR(IF(F37="","",CEILING(G37/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J37" s="62">
-        <f>IFERROR(IF(F37="","",TEXT('Getting Started'!C10+(H37-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I37*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B38" s="18" t="n"/>
-      <c r="F38" s="32" t="n"/>
-      <c r="G38" s="17">
-        <f>IFERROR(SUM(F35:F38),"")</f>
-        <v/>
-      </c>
-      <c r="H38" s="17">
-        <f>IFERROR(IF(F38="","",FLOOR(G37/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I38" s="17">
-        <f>IFERROR(IF(F38="","",CEILING(G38/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J38" s="62">
-        <f>IFERROR(IF(F38="","",TEXT('Getting Started'!C10+(H38-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I38*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B39" s="5" t="n"/>
-      <c r="F39" s="33" t="n"/>
-      <c r="G39" s="17">
-        <f>IFERROR(SUM(F35:F39),"")</f>
-        <v/>
-      </c>
-      <c r="H39" s="17">
-        <f>IFERROR(IF(F39="","",FLOOR(G38/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I39" s="17">
-        <f>IFERROR(IF(F39="","",CEILING(G39/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J39" s="62">
-        <f>IFERROR(IF(F39="","",TEXT('Getting Started'!C10+(H39-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I39*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B40" s="18" t="n"/>
-      <c r="F40" s="32" t="n"/>
-      <c r="G40" s="17">
-        <f>IFERROR(SUM(F35:F40),"")</f>
-        <v/>
-      </c>
-      <c r="H40" s="17">
-        <f>IFERROR(IF(F40="","",FLOOR(G39/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I40" s="17">
-        <f>IFERROR(IF(F40="","",CEILING(G40/((IFERROR(B32,0)+IFERROR(G32,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J40" s="62">
-        <f>IFERROR(IF(F40="","",TEXT('Getting Started'!C10+(H40-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I40*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="63" t="n"/>
-    </row>
-    <row r="42" ht="8" customHeight="1"/>
-    <row r="43" ht="24" customHeight="1">
-      <c r="A43" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  READING</t>
-        </is>
-      </c>
-      <c r="E43" s="53">
-        <f>IFERROR(IF('Course Content'!B27="","← enter on Course Content tab",'Course Content'!B27),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="B44" s="54">
-        <f>'Course Content'!D27</f>
-        <v/>
-      </c>
-      <c r="C44" s="55">
-        <f>IFERROR(IF(B44="","",ROUND(B44/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D44" s="55">
-        <f>IFERROR(IF(C44="","",ROUND(C44/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E44" s="56">
-        <f>IFERROR(IF(B44="","",TEXT('Getting Started'!C10+(B44/D44),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F44" s="26" t="n"/>
-      <c r="G44" s="57">
-        <f>'Course Content'!E27</f>
-        <v/>
-      </c>
-      <c r="H44" s="58">
-        <f>IFERROR(IF(G44="","",ROUND(G44/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I44" s="58">
-        <f>IFERROR(IF(H44="","",ROUND(H44/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J44" s="59">
-        <f>IFERROR(IF(G44="","",TEXT('Getting Started'!C18+(G44/I44),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B46" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F46" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G46" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H46" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I46" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J46" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B47" s="5" t="n"/>
-      <c r="F47" s="33" t="n"/>
-      <c r="G47" s="17">
-        <f>IFERROR(SUM(F47:F47),"")</f>
-        <v/>
-      </c>
-      <c r="H47" s="17">
-        <f>IF(F47="","",1)</f>
-        <v/>
-      </c>
-      <c r="I47" s="17">
-        <f>IFERROR(IF(F47="","",CEILING(G47/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J47" s="62">
-        <f>IFERROR(IF(F47="","",TEXT('Getting Started'!C10+(H47-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I47*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B48" s="18" t="n"/>
-      <c r="F48" s="32" t="n"/>
-      <c r="G48" s="17">
-        <f>IFERROR(SUM(F47:F48),"")</f>
-        <v/>
-      </c>
-      <c r="H48" s="17">
-        <f>IFERROR(IF(F48="","",FLOOR(G47/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I48" s="17">
-        <f>IFERROR(IF(F48="","",CEILING(G48/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J48" s="62">
-        <f>IFERROR(IF(F48="","",TEXT('Getting Started'!C10+(H48-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I48*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B49" s="5" t="n"/>
-      <c r="F49" s="33" t="n"/>
-      <c r="G49" s="17">
-        <f>IFERROR(SUM(F47:F49),"")</f>
-        <v/>
-      </c>
-      <c r="H49" s="17">
-        <f>IFERROR(IF(F49="","",FLOOR(G48/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I49" s="17">
-        <f>IFERROR(IF(F49="","",CEILING(G49/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J49" s="62">
-        <f>IFERROR(IF(F49="","",TEXT('Getting Started'!C10+(H49-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I49*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B50" s="18" t="n"/>
-      <c r="F50" s="32" t="n"/>
-      <c r="G50" s="17">
-        <f>IFERROR(SUM(F47:F50),"")</f>
-        <v/>
-      </c>
-      <c r="H50" s="17">
-        <f>IFERROR(IF(F50="","",FLOOR(G49/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I50" s="17">
-        <f>IFERROR(IF(F50="","",CEILING(G50/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J50" s="62">
-        <f>IFERROR(IF(F50="","",TEXT('Getting Started'!C10+(H50-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I50*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B51" s="5" t="n"/>
-      <c r="F51" s="33" t="n"/>
-      <c r="G51" s="17">
-        <f>IFERROR(SUM(F47:F51),"")</f>
-        <v/>
-      </c>
-      <c r="H51" s="17">
-        <f>IFERROR(IF(F51="","",FLOOR(G50/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I51" s="17">
-        <f>IFERROR(IF(F51="","",CEILING(G51/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J51" s="62">
-        <f>IFERROR(IF(F51="","",TEXT('Getting Started'!C10+(H51-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I51*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B52" s="18" t="n"/>
-      <c r="F52" s="32" t="n"/>
-      <c r="G52" s="17">
-        <f>IFERROR(SUM(F47:F52),"")</f>
-        <v/>
-      </c>
-      <c r="H52" s="17">
-        <f>IFERROR(IF(F52="","",FLOOR(G51/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I52" s="17">
-        <f>IFERROR(IF(F52="","",CEILING(G52/((IFERROR(B44,0)+IFERROR(G44,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J52" s="62">
-        <f>IFERROR(IF(F52="","",TEXT('Getting Started'!C10+(H52-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I52*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="63" t="n"/>
-    </row>
-    <row r="54" ht="8" customHeight="1"/>
-    <row r="55" ht="24" customHeight="1">
-      <c r="A55" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  WRITING / COMPOSITION</t>
-        </is>
-      </c>
-      <c r="E55" s="53">
-        <f>IFERROR(IF('Course Content'!B28="","← enter on Course Content tab",'Course Content'!B28),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="B56" s="54">
-        <f>'Course Content'!D28</f>
-        <v/>
-      </c>
-      <c r="C56" s="55">
-        <f>IFERROR(IF(B56="","",ROUND(B56/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D56" s="55">
-        <f>IFERROR(IF(C56="","",ROUND(C56/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E56" s="56">
-        <f>IFERROR(IF(B56="","",TEXT('Getting Started'!C10+(B56/D56),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F56" s="26" t="n"/>
-      <c r="G56" s="57">
-        <f>'Course Content'!E28</f>
-        <v/>
-      </c>
-      <c r="H56" s="58">
-        <f>IFERROR(IF(G56="","",ROUND(G56/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I56" s="58">
-        <f>IFERROR(IF(H56="","",ROUND(H56/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J56" s="59">
-        <f>IFERROR(IF(G56="","",TEXT('Getting Started'!C18+(G56/I56),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="22" customHeight="1">
-      <c r="A58" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B58" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F58" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G58" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H58" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I58" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J58" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B59" s="5" t="n"/>
-      <c r="F59" s="33" t="n"/>
-      <c r="G59" s="17">
-        <f>IFERROR(SUM(F59:F59),"")</f>
-        <v/>
-      </c>
-      <c r="H59" s="17">
-        <f>IF(F59="","",1)</f>
-        <v/>
-      </c>
-      <c r="I59" s="17">
-        <f>IFERROR(IF(F59="","",CEILING(G59/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J59" s="62">
-        <f>IFERROR(IF(F59="","",TEXT('Getting Started'!C10+(H59-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I59*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B60" s="18" t="n"/>
-      <c r="F60" s="32" t="n"/>
-      <c r="G60" s="17">
-        <f>IFERROR(SUM(F59:F60),"")</f>
-        <v/>
-      </c>
-      <c r="H60" s="17">
-        <f>IFERROR(IF(F60="","",FLOOR(G59/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I60" s="17">
-        <f>IFERROR(IF(F60="","",CEILING(G60/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J60" s="62">
-        <f>IFERROR(IF(F60="","",TEXT('Getting Started'!C10+(H60-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I60*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B61" s="5" t="n"/>
-      <c r="F61" s="33" t="n"/>
-      <c r="G61" s="17">
-        <f>IFERROR(SUM(F59:F61),"")</f>
-        <v/>
-      </c>
-      <c r="H61" s="17">
-        <f>IFERROR(IF(F61="","",FLOOR(G60/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I61" s="17">
-        <f>IFERROR(IF(F61="","",CEILING(G61/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J61" s="62">
-        <f>IFERROR(IF(F61="","",TEXT('Getting Started'!C10+(H61-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I61*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B62" s="18" t="n"/>
-      <c r="F62" s="32" t="n"/>
-      <c r="G62" s="17">
-        <f>IFERROR(SUM(F59:F62),"")</f>
-        <v/>
-      </c>
-      <c r="H62" s="17">
-        <f>IFERROR(IF(F62="","",FLOOR(G61/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I62" s="17">
-        <f>IFERROR(IF(F62="","",CEILING(G62/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J62" s="62">
-        <f>IFERROR(IF(F62="","",TEXT('Getting Started'!C10+(H62-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I62*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B63" s="5" t="n"/>
-      <c r="F63" s="33" t="n"/>
-      <c r="G63" s="17">
-        <f>IFERROR(SUM(F59:F63),"")</f>
-        <v/>
-      </c>
-      <c r="H63" s="17">
-        <f>IFERROR(IF(F63="","",FLOOR(G62/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I63" s="17">
-        <f>IFERROR(IF(F63="","",CEILING(G63/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J63" s="62">
-        <f>IFERROR(IF(F63="","",TEXT('Getting Started'!C10+(H63-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I63*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B64" s="18" t="n"/>
-      <c r="F64" s="32" t="n"/>
-      <c r="G64" s="17">
-        <f>IFERROR(SUM(F59:F64),"")</f>
-        <v/>
-      </c>
-      <c r="H64" s="17">
-        <f>IFERROR(IF(F64="","",FLOOR(G63/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I64" s="17">
-        <f>IFERROR(IF(F64="","",CEILING(G64/((IFERROR(B56,0)+IFERROR(G56,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J64" s="62">
-        <f>IFERROR(IF(F64="","",TEXT('Getting Started'!C10+(H64-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I64*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="A65" s="63" t="n"/>
-    </row>
-    <row r="66" ht="8" customHeight="1"/>
-    <row r="67" ht="24" customHeight="1">
-      <c r="A67" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SCIENCE</t>
-        </is>
-      </c>
-      <c r="E67" s="53">
-        <f>IFERROR(IF('Course Content'!B29="","← enter on Course Content tab",'Course Content'!B29),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" ht="22" customHeight="1">
-      <c r="B68" s="54">
-        <f>'Course Content'!D29</f>
-        <v/>
-      </c>
-      <c r="C68" s="55">
-        <f>IFERROR(IF(B68="","",ROUND(B68/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D68" s="55">
-        <f>IFERROR(IF(C68="","",ROUND(C68/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E68" s="56">
-        <f>IFERROR(IF(B68="","",TEXT('Getting Started'!C10+(B68/D68),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F68" s="26" t="n"/>
-      <c r="G68" s="57">
-        <f>'Course Content'!E29</f>
-        <v/>
-      </c>
-      <c r="H68" s="58">
-        <f>IFERROR(IF(G68="","",ROUND(G68/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I68" s="58">
-        <f>IFERROR(IF(H68="","",ROUND(H68/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J68" s="59">
-        <f>IFERROR(IF(G68="","",TEXT('Getting Started'!C18+(G68/I68),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" ht="16" customHeight="1">
-      <c r="A69" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B70" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F70" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G70" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H70" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I70" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J70" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B71" s="5" t="n"/>
-      <c r="F71" s="33" t="n"/>
-      <c r="G71" s="17">
-        <f>IFERROR(SUM(F71:F71),"")</f>
-        <v/>
-      </c>
-      <c r="H71" s="17">
-        <f>IF(F71="","",1)</f>
-        <v/>
-      </c>
-      <c r="I71" s="17">
-        <f>IFERROR(IF(F71="","",CEILING(G71/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J71" s="62">
-        <f>IFERROR(IF(F71="","",TEXT('Getting Started'!C10+(H71-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I71*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" ht="18" customHeight="1">
-      <c r="A72" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B72" s="18" t="n"/>
-      <c r="F72" s="32" t="n"/>
-      <c r="G72" s="17">
-        <f>IFERROR(SUM(F71:F72),"")</f>
-        <v/>
-      </c>
-      <c r="H72" s="17">
-        <f>IFERROR(IF(F72="","",FLOOR(G71/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I72" s="17">
-        <f>IFERROR(IF(F72="","",CEILING(G72/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J72" s="62">
-        <f>IFERROR(IF(F72="","",TEXT('Getting Started'!C10+(H72-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I72*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B73" s="5" t="n"/>
-      <c r="F73" s="33" t="n"/>
-      <c r="G73" s="17">
-        <f>IFERROR(SUM(F71:F73),"")</f>
-        <v/>
-      </c>
-      <c r="H73" s="17">
-        <f>IFERROR(IF(F73="","",FLOOR(G72/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I73" s="17">
-        <f>IFERROR(IF(F73="","",CEILING(G73/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J73" s="62">
-        <f>IFERROR(IF(F73="","",TEXT('Getting Started'!C10+(H73-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I73*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" ht="18" customHeight="1">
-      <c r="A74" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B74" s="18" t="n"/>
-      <c r="F74" s="32" t="n"/>
-      <c r="G74" s="17">
-        <f>IFERROR(SUM(F71:F74),"")</f>
-        <v/>
-      </c>
-      <c r="H74" s="17">
-        <f>IFERROR(IF(F74="","",FLOOR(G73/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I74" s="17">
-        <f>IFERROR(IF(F74="","",CEILING(G74/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J74" s="62">
-        <f>IFERROR(IF(F74="","",TEXT('Getting Started'!C10+(H74-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I74*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B75" s="5" t="n"/>
-      <c r="F75" s="33" t="n"/>
-      <c r="G75" s="17">
-        <f>IFERROR(SUM(F71:F75),"")</f>
-        <v/>
-      </c>
-      <c r="H75" s="17">
-        <f>IFERROR(IF(F75="","",FLOOR(G74/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I75" s="17">
-        <f>IFERROR(IF(F75="","",CEILING(G75/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J75" s="62">
-        <f>IFERROR(IF(F75="","",TEXT('Getting Started'!C10+(H75-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I75*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B76" s="18" t="n"/>
-      <c r="F76" s="32" t="n"/>
-      <c r="G76" s="17">
-        <f>IFERROR(SUM(F71:F76),"")</f>
-        <v/>
-      </c>
-      <c r="H76" s="17">
-        <f>IFERROR(IF(F76="","",FLOOR(G75/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I76" s="17">
-        <f>IFERROR(IF(F76="","",CEILING(G76/((IFERROR(B68,0)+IFERROR(G68,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J76" s="62">
-        <f>IFERROR(IF(F76="","",TEXT('Getting Started'!C10+(H76-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I76*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" ht="20" customHeight="1">
-      <c r="A77" s="63" t="n"/>
-    </row>
-    <row r="78" ht="8" customHeight="1"/>
-    <row r="79" ht="24" customHeight="1">
-      <c r="A79" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SOCIAL STUDIES / HISTORY</t>
-        </is>
-      </c>
-      <c r="E79" s="53">
-        <f>IFERROR(IF('Course Content'!B30="","← enter on Course Content tab",'Course Content'!B30),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80" ht="22" customHeight="1">
-      <c r="B80" s="54">
-        <f>'Course Content'!D30</f>
-        <v/>
-      </c>
-      <c r="C80" s="55">
-        <f>IFERROR(IF(B80="","",ROUND(B80/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D80" s="55">
-        <f>IFERROR(IF(C80="","",ROUND(C80/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E80" s="56">
-        <f>IFERROR(IF(B80="","",TEXT('Getting Started'!C10+(B80/D80),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F80" s="26" t="n"/>
-      <c r="G80" s="57">
-        <f>'Course Content'!E30</f>
-        <v/>
-      </c>
-      <c r="H80" s="58">
-        <f>IFERROR(IF(G80="","",ROUND(G80/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I80" s="58">
-        <f>IFERROR(IF(H80="","",ROUND(H80/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J80" s="59">
-        <f>IFERROR(IF(G80="","",TEXT('Getting Started'!C18+(G80/I80),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" ht="16" customHeight="1">
-      <c r="A81" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="22" customHeight="1">
-      <c r="A82" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B82" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F82" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G82" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H82" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I82" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J82" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B83" s="5" t="n"/>
-      <c r="F83" s="33" t="n"/>
-      <c r="G83" s="17">
-        <f>IFERROR(SUM(F83:F83),"")</f>
-        <v/>
-      </c>
-      <c r="H83" s="17">
-        <f>IF(F83="","",1)</f>
-        <v/>
-      </c>
-      <c r="I83" s="17">
-        <f>IFERROR(IF(F83="","",CEILING(G83/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J83" s="62">
-        <f>IFERROR(IF(F83="","",TEXT('Getting Started'!C10+(H83-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I83*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" ht="18" customHeight="1">
-      <c r="A84" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B84" s="18" t="n"/>
-      <c r="F84" s="32" t="n"/>
-      <c r="G84" s="17">
-        <f>IFERROR(SUM(F83:F84),"")</f>
-        <v/>
-      </c>
-      <c r="H84" s="17">
-        <f>IFERROR(IF(F84="","",FLOOR(G83/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I84" s="17">
-        <f>IFERROR(IF(F84="","",CEILING(G84/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J84" s="62">
-        <f>IFERROR(IF(F84="","",TEXT('Getting Started'!C10+(H84-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I84*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B85" s="5" t="n"/>
-      <c r="F85" s="33" t="n"/>
-      <c r="G85" s="17">
-        <f>IFERROR(SUM(F83:F85),"")</f>
-        <v/>
-      </c>
-      <c r="H85" s="17">
-        <f>IFERROR(IF(F85="","",FLOOR(G84/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I85" s="17">
-        <f>IFERROR(IF(F85="","",CEILING(G85/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J85" s="62">
-        <f>IFERROR(IF(F85="","",TEXT('Getting Started'!C10+(H85-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I85*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B86" s="18" t="n"/>
-      <c r="F86" s="32" t="n"/>
-      <c r="G86" s="17">
-        <f>IFERROR(SUM(F83:F86),"")</f>
-        <v/>
-      </c>
-      <c r="H86" s="17">
-        <f>IFERROR(IF(F86="","",FLOOR(G85/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I86" s="17">
-        <f>IFERROR(IF(F86="","",CEILING(G86/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J86" s="62">
-        <f>IFERROR(IF(F86="","",TEXT('Getting Started'!C10+(H86-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I86*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B87" s="5" t="n"/>
-      <c r="F87" s="33" t="n"/>
-      <c r="G87" s="17">
-        <f>IFERROR(SUM(F83:F87),"")</f>
-        <v/>
-      </c>
-      <c r="H87" s="17">
-        <f>IFERROR(IF(F87="","",FLOOR(G86/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I87" s="17">
-        <f>IFERROR(IF(F87="","",CEILING(G87/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J87" s="62">
-        <f>IFERROR(IF(F87="","",TEXT('Getting Started'!C10+(H87-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I87*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" ht="18" customHeight="1">
-      <c r="A88" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B88" s="18" t="n"/>
-      <c r="F88" s="32" t="n"/>
-      <c r="G88" s="17">
-        <f>IFERROR(SUM(F83:F88),"")</f>
-        <v/>
-      </c>
-      <c r="H88" s="17">
-        <f>IFERROR(IF(F88="","",FLOOR(G87/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I88" s="17">
-        <f>IFERROR(IF(F88="","",CEILING(G88/((IFERROR(B80,0)+IFERROR(G80,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J88" s="62">
-        <f>IFERROR(IF(F88="","",TEXT('Getting Started'!C10+(H88-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I88*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" ht="20" customHeight="1">
-      <c r="A89" s="63" t="n"/>
-    </row>
-    <row r="90" ht="8" customHeight="1"/>
-    <row r="91" ht="24" customHeight="1">
-      <c r="A91" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  HEALTH</t>
-        </is>
-      </c>
-      <c r="E91" s="53">
-        <f>IFERROR(IF('Course Content'!B31="","← enter on Course Content tab",'Course Content'!B31),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" ht="22" customHeight="1">
-      <c r="B92" s="54">
-        <f>'Course Content'!D31</f>
-        <v/>
-      </c>
-      <c r="C92" s="55">
-        <f>IFERROR(IF(B92="","",ROUND(B92/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D92" s="55">
-        <f>IFERROR(IF(C92="","",ROUND(C92/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E92" s="56">
-        <f>IFERROR(IF(B92="","",TEXT('Getting Started'!C10+(B92/D92),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F92" s="26" t="n"/>
-      <c r="G92" s="57">
-        <f>'Course Content'!E31</f>
-        <v/>
-      </c>
-      <c r="H92" s="58">
-        <f>IFERROR(IF(G92="","",ROUND(G92/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I92" s="58">
-        <f>IFERROR(IF(H92="","",ROUND(H92/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J92" s="59">
-        <f>IFERROR(IF(G92="","",TEXT('Getting Started'!C18+(G92/I92),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" ht="16" customHeight="1">
-      <c r="A93" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="22" customHeight="1">
-      <c r="A94" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B94" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F94" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G94" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H94" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I94" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J94" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B95" s="5" t="n"/>
-      <c r="F95" s="33" t="n"/>
-      <c r="G95" s="17">
-        <f>IFERROR(SUM(F95:F95),"")</f>
-        <v/>
-      </c>
-      <c r="H95" s="17">
-        <f>IF(F95="","",1)</f>
-        <v/>
-      </c>
-      <c r="I95" s="17">
-        <f>IFERROR(IF(F95="","",CEILING(G95/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J95" s="62">
-        <f>IFERROR(IF(F95="","",TEXT('Getting Started'!C10+(H95-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I95*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96" ht="18" customHeight="1">
-      <c r="A96" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B96" s="18" t="n"/>
-      <c r="F96" s="32" t="n"/>
-      <c r="G96" s="17">
-        <f>IFERROR(SUM(F95:F96),"")</f>
-        <v/>
-      </c>
-      <c r="H96" s="17">
-        <f>IFERROR(IF(F96="","",FLOOR(G95/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I96" s="17">
-        <f>IFERROR(IF(F96="","",CEILING(G96/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J96" s="62">
-        <f>IFERROR(IF(F96="","",TEXT('Getting Started'!C10+(H96-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I96*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B97" s="5" t="n"/>
-      <c r="F97" s="33" t="n"/>
-      <c r="G97" s="17">
-        <f>IFERROR(SUM(F95:F97),"")</f>
-        <v/>
-      </c>
-      <c r="H97" s="17">
-        <f>IFERROR(IF(F97="","",FLOOR(G96/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I97" s="17">
-        <f>IFERROR(IF(F97="","",CEILING(G97/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J97" s="62">
-        <f>IFERROR(IF(F97="","",TEXT('Getting Started'!C10+(H97-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I97*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98" ht="18" customHeight="1">
-      <c r="A98" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B98" s="18" t="n"/>
-      <c r="F98" s="32" t="n"/>
-      <c r="G98" s="17">
-        <f>IFERROR(SUM(F95:F98),"")</f>
-        <v/>
-      </c>
-      <c r="H98" s="17">
-        <f>IFERROR(IF(F98="","",FLOOR(G97/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I98" s="17">
-        <f>IFERROR(IF(F98="","",CEILING(G98/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J98" s="62">
-        <f>IFERROR(IF(F98="","",TEXT('Getting Started'!C10+(H98-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I98*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99" ht="18" customHeight="1">
-      <c r="A99" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B99" s="5" t="n"/>
-      <c r="F99" s="33" t="n"/>
-      <c r="G99" s="17">
-        <f>IFERROR(SUM(F95:F99),"")</f>
-        <v/>
-      </c>
-      <c r="H99" s="17">
-        <f>IFERROR(IF(F99="","",FLOOR(G98/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I99" s="17">
-        <f>IFERROR(IF(F99="","",CEILING(G99/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J99" s="62">
-        <f>IFERROR(IF(F99="","",TEXT('Getting Started'!C10+(H99-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I99*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="100" ht="18" customHeight="1">
-      <c r="A100" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B100" s="18" t="n"/>
-      <c r="F100" s="32" t="n"/>
-      <c r="G100" s="17">
-        <f>IFERROR(SUM(F95:F100),"")</f>
-        <v/>
-      </c>
-      <c r="H100" s="17">
-        <f>IFERROR(IF(F100="","",FLOOR(G99/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I100" s="17">
-        <f>IFERROR(IF(F100="","",CEILING(G100/((IFERROR(B92,0)+IFERROR(G92,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J100" s="62">
-        <f>IFERROR(IF(F100="","",TEXT('Getting Started'!C10+(H100-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I100*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101" ht="20" customHeight="1">
-      <c r="A101" s="63" t="n"/>
-    </row>
-    <row r="102" ht="8" customHeight="1"/>
-    <row r="103" ht="24" customHeight="1">
-      <c r="A103" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  PHYSICAL EDUCATION</t>
-        </is>
-      </c>
-      <c r="E103" s="53">
-        <f>IFERROR(IF('Course Content'!B32="","← enter on Course Content tab",'Course Content'!B32),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="104" ht="22" customHeight="1">
-      <c r="B104" s="54">
-        <f>'Course Content'!D32</f>
-        <v/>
-      </c>
-      <c r="C104" s="55">
-        <f>IFERROR(IF(B104="","",ROUND(B104/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D104" s="55">
-        <f>IFERROR(IF(C104="","",ROUND(C104/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E104" s="56">
-        <f>IFERROR(IF(B104="","",TEXT('Getting Started'!C10+(B104/D104),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F104" s="26" t="n"/>
-      <c r="G104" s="57">
-        <f>'Course Content'!E32</f>
-        <v/>
-      </c>
-      <c r="H104" s="58">
-        <f>IFERROR(IF(G104="","",ROUND(G104/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I104" s="58">
-        <f>IFERROR(IF(H104="","",ROUND(H104/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J104" s="59">
-        <f>IFERROR(IF(G104="","",TEXT('Getting Started'!C18+(G104/I104),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="105" ht="16" customHeight="1">
-      <c r="A105" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="22" customHeight="1">
-      <c r="A106" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B106" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F106" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G106" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H106" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I106" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J106" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B107" s="5" t="n"/>
-      <c r="F107" s="33" t="n"/>
-      <c r="G107" s="17">
-        <f>IFERROR(SUM(F107:F107),"")</f>
-        <v/>
-      </c>
-      <c r="H107" s="17">
-        <f>IF(F107="","",1)</f>
-        <v/>
-      </c>
-      <c r="I107" s="17">
-        <f>IFERROR(IF(F107="","",CEILING(G107/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J107" s="62">
-        <f>IFERROR(IF(F107="","",TEXT('Getting Started'!C10+(H107-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I107*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="108" ht="18" customHeight="1">
-      <c r="A108" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B108" s="18" t="n"/>
-      <c r="F108" s="32" t="n"/>
-      <c r="G108" s="17">
-        <f>IFERROR(SUM(F107:F108),"")</f>
-        <v/>
-      </c>
-      <c r="H108" s="17">
-        <f>IFERROR(IF(F108="","",FLOOR(G107/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I108" s="17">
-        <f>IFERROR(IF(F108="","",CEILING(G108/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J108" s="62">
-        <f>IFERROR(IF(F108="","",TEXT('Getting Started'!C10+(H108-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I108*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="109" ht="18" customHeight="1">
-      <c r="A109" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B109" s="5" t="n"/>
-      <c r="F109" s="33" t="n"/>
-      <c r="G109" s="17">
-        <f>IFERROR(SUM(F107:F109),"")</f>
-        <v/>
-      </c>
-      <c r="H109" s="17">
-        <f>IFERROR(IF(F109="","",FLOOR(G108/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I109" s="17">
-        <f>IFERROR(IF(F109="","",CEILING(G109/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J109" s="62">
-        <f>IFERROR(IF(F109="","",TEXT('Getting Started'!C10+(H109-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I109*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="110" ht="18" customHeight="1">
-      <c r="A110" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B110" s="18" t="n"/>
-      <c r="F110" s="32" t="n"/>
-      <c r="G110" s="17">
-        <f>IFERROR(SUM(F107:F110),"")</f>
-        <v/>
-      </c>
-      <c r="H110" s="17">
-        <f>IFERROR(IF(F110="","",FLOOR(G109/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I110" s="17">
-        <f>IFERROR(IF(F110="","",CEILING(G110/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J110" s="62">
-        <f>IFERROR(IF(F110="","",TEXT('Getting Started'!C10+(H110-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I110*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="111" ht="18" customHeight="1">
-      <c r="A111" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B111" s="5" t="n"/>
-      <c r="F111" s="33" t="n"/>
-      <c r="G111" s="17">
-        <f>IFERROR(SUM(F107:F111),"")</f>
-        <v/>
-      </c>
-      <c r="H111" s="17">
-        <f>IFERROR(IF(F111="","",FLOOR(G110/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I111" s="17">
-        <f>IFERROR(IF(F111="","",CEILING(G111/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J111" s="62">
-        <f>IFERROR(IF(F111="","",TEXT('Getting Started'!C10+(H111-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I111*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B112" s="18" t="n"/>
-      <c r="F112" s="32" t="n"/>
-      <c r="G112" s="17">
-        <f>IFERROR(SUM(F107:F112),"")</f>
-        <v/>
-      </c>
-      <c r="H112" s="17">
-        <f>IFERROR(IF(F112="","",FLOOR(G111/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I112" s="17">
-        <f>IFERROR(IF(F112="","",CEILING(G112/((IFERROR(B104,0)+IFERROR(G104,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J112" s="62">
-        <f>IFERROR(IF(F112="","",TEXT('Getting Started'!C10+(H112-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I112*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="63" t="n"/>
-    </row>
-    <row r="114" ht="8" customHeight="1"/>
-    <row r="115" ht="24" customHeight="1">
-      <c r="A115" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ART / MUSIC</t>
-        </is>
-      </c>
-      <c r="E115" s="53">
-        <f>IFERROR(IF('Course Content'!B33="","← enter on Course Content tab",'Course Content'!B33),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="116" ht="22" customHeight="1">
-      <c r="B116" s="54">
-        <f>'Course Content'!D33</f>
-        <v/>
-      </c>
-      <c r="C116" s="55">
-        <f>IFERROR(IF(B116="","",ROUND(B116/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D116" s="55">
-        <f>IFERROR(IF(C116="","",ROUND(C116/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E116" s="56">
-        <f>IFERROR(IF(B116="","",TEXT('Getting Started'!C10+(B116/D116),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F116" s="26" t="n"/>
-      <c r="G116" s="57">
-        <f>'Course Content'!E33</f>
-        <v/>
-      </c>
-      <c r="H116" s="58">
-        <f>IFERROR(IF(G116="","",ROUND(G116/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I116" s="58">
-        <f>IFERROR(IF(H116="","",ROUND(H116/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J116" s="59">
-        <f>IFERROR(IF(G116="","",TEXT('Getting Started'!C18+(G116/I116),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="117" ht="16" customHeight="1">
-      <c r="A117" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="22" customHeight="1">
-      <c r="A118" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B118" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F118" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G118" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H118" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I118" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J118" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B119" s="5" t="n"/>
-      <c r="F119" s="33" t="n"/>
-      <c r="G119" s="17">
-        <f>IFERROR(SUM(F119:F119),"")</f>
-        <v/>
-      </c>
-      <c r="H119" s="17">
-        <f>IF(F119="","",1)</f>
-        <v/>
-      </c>
-      <c r="I119" s="17">
-        <f>IFERROR(IF(F119="","",CEILING(G119/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J119" s="62">
-        <f>IFERROR(IF(F119="","",TEXT('Getting Started'!C10+(H119-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I119*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="120" ht="18" customHeight="1">
-      <c r="A120" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B120" s="18" t="n"/>
-      <c r="F120" s="32" t="n"/>
-      <c r="G120" s="17">
-        <f>IFERROR(SUM(F119:F120),"")</f>
-        <v/>
-      </c>
-      <c r="H120" s="17">
-        <f>IFERROR(IF(F120="","",FLOOR(G119/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I120" s="17">
-        <f>IFERROR(IF(F120="","",CEILING(G120/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J120" s="62">
-        <f>IFERROR(IF(F120="","",TEXT('Getting Started'!C10+(H120-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I120*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="121" ht="18" customHeight="1">
-      <c r="A121" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B121" s="5" t="n"/>
-      <c r="F121" s="33" t="n"/>
-      <c r="G121" s="17">
-        <f>IFERROR(SUM(F119:F121),"")</f>
-        <v/>
-      </c>
-      <c r="H121" s="17">
-        <f>IFERROR(IF(F121="","",FLOOR(G120/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I121" s="17">
-        <f>IFERROR(IF(F121="","",CEILING(G121/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J121" s="62">
-        <f>IFERROR(IF(F121="","",TEXT('Getting Started'!C10+(H121-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I121*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="122" ht="18" customHeight="1">
-      <c r="A122" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B122" s="18" t="n"/>
-      <c r="F122" s="32" t="n"/>
-      <c r="G122" s="17">
-        <f>IFERROR(SUM(F119:F122),"")</f>
-        <v/>
-      </c>
-      <c r="H122" s="17">
-        <f>IFERROR(IF(F122="","",FLOOR(G121/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I122" s="17">
-        <f>IFERROR(IF(F122="","",CEILING(G122/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J122" s="62">
-        <f>IFERROR(IF(F122="","",TEXT('Getting Started'!C10+(H122-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I122*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="123" ht="18" customHeight="1">
-      <c r="A123" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B123" s="5" t="n"/>
-      <c r="F123" s="33" t="n"/>
-      <c r="G123" s="17">
-        <f>IFERROR(SUM(F119:F123),"")</f>
-        <v/>
-      </c>
-      <c r="H123" s="17">
-        <f>IFERROR(IF(F123="","",FLOOR(G122/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I123" s="17">
-        <f>IFERROR(IF(F123="","",CEILING(G123/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J123" s="62">
-        <f>IFERROR(IF(F123="","",TEXT('Getting Started'!C10+(H123-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I123*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="124" ht="18" customHeight="1">
-      <c r="A124" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B124" s="18" t="n"/>
-      <c r="F124" s="32" t="n"/>
-      <c r="G124" s="17">
-        <f>IFERROR(SUM(F119:F124),"")</f>
-        <v/>
-      </c>
-      <c r="H124" s="17">
-        <f>IFERROR(IF(F124="","",FLOOR(G123/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I124" s="17">
-        <f>IFERROR(IF(F124="","",CEILING(G124/((IFERROR(B116,0)+IFERROR(G116,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J124" s="62">
-        <f>IFERROR(IF(F124="","",TEXT('Getting Started'!C10+(H124-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I124*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="125" ht="20" customHeight="1">
-      <c r="A125" s="63" t="n"/>
-    </row>
-    <row r="126" ht="8" customHeight="1"/>
-    <row r="127" ht="24" customHeight="1">
-      <c r="A127" s="52">
-        <f>IF('Course Content'!A34="","  ELECTIVE / OTHER 1","  "&amp;UPPER('Course Content'!A34))</f>
-        <v/>
-      </c>
-      <c r="E127" s="53">
-        <f>IFERROR(IF('Course Content'!B34="","← enter on Course Content tab",'Course Content'!B34),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="128" ht="22" customHeight="1">
-      <c r="B128" s="54">
-        <f>'Course Content'!D34</f>
-        <v/>
-      </c>
-      <c r="C128" s="55">
-        <f>IFERROR(IF(B128="","",ROUND(B128/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D128" s="55">
-        <f>IFERROR(IF(C128="","",ROUND(C128/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E128" s="56">
-        <f>IFERROR(IF(B128="","",TEXT('Getting Started'!C10+(B128/D128),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F128" s="26" t="n"/>
-      <c r="G128" s="57">
-        <f>'Course Content'!E34</f>
-        <v/>
-      </c>
-      <c r="H128" s="58">
-        <f>IFERROR(IF(G128="","",ROUND(G128/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I128" s="58">
-        <f>IFERROR(IF(H128="","",ROUND(H128/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J128" s="59">
-        <f>IFERROR(IF(G128="","",TEXT('Getting Started'!C18+(G128/I128),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="129" ht="16" customHeight="1">
-      <c r="A129" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="22" customHeight="1">
-      <c r="A130" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B130" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F130" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G130" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H130" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I130" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J130" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" ht="18" customHeight="1">
-      <c r="A131" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B131" s="5" t="n"/>
-      <c r="F131" s="33" t="n"/>
-      <c r="G131" s="17">
-        <f>IFERROR(SUM(F131:F131),"")</f>
-        <v/>
-      </c>
-      <c r="H131" s="17">
-        <f>IF(F131="","",1)</f>
-        <v/>
-      </c>
-      <c r="I131" s="17">
-        <f>IFERROR(IF(F131="","",CEILING(G131/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J131" s="62">
-        <f>IFERROR(IF(F131="","",TEXT('Getting Started'!C10+(H131-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I131*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="132" ht="18" customHeight="1">
-      <c r="A132" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B132" s="18" t="n"/>
-      <c r="F132" s="32" t="n"/>
-      <c r="G132" s="17">
-        <f>IFERROR(SUM(F131:F132),"")</f>
-        <v/>
-      </c>
-      <c r="H132" s="17">
-        <f>IFERROR(IF(F132="","",FLOOR(G131/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I132" s="17">
-        <f>IFERROR(IF(F132="","",CEILING(G132/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J132" s="62">
-        <f>IFERROR(IF(F132="","",TEXT('Getting Started'!C10+(H132-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I132*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="133" ht="18" customHeight="1">
-      <c r="A133" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B133" s="5" t="n"/>
-      <c r="F133" s="33" t="n"/>
-      <c r="G133" s="17">
-        <f>IFERROR(SUM(F131:F133),"")</f>
-        <v/>
-      </c>
-      <c r="H133" s="17">
-        <f>IFERROR(IF(F133="","",FLOOR(G132/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I133" s="17">
-        <f>IFERROR(IF(F133="","",CEILING(G133/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J133" s="62">
-        <f>IFERROR(IF(F133="","",TEXT('Getting Started'!C10+(H133-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I133*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="134" ht="18" customHeight="1">
-      <c r="A134" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B134" s="18" t="n"/>
-      <c r="F134" s="32" t="n"/>
-      <c r="G134" s="17">
-        <f>IFERROR(SUM(F131:F134),"")</f>
-        <v/>
-      </c>
-      <c r="H134" s="17">
-        <f>IFERROR(IF(F134="","",FLOOR(G133/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I134" s="17">
-        <f>IFERROR(IF(F134="","",CEILING(G134/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J134" s="62">
-        <f>IFERROR(IF(F134="","",TEXT('Getting Started'!C10+(H134-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I134*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="135" ht="18" customHeight="1">
-      <c r="A135" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B135" s="5" t="n"/>
-      <c r="F135" s="33" t="n"/>
-      <c r="G135" s="17">
-        <f>IFERROR(SUM(F131:F135),"")</f>
-        <v/>
-      </c>
-      <c r="H135" s="17">
-        <f>IFERROR(IF(F135="","",FLOOR(G134/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I135" s="17">
-        <f>IFERROR(IF(F135="","",CEILING(G135/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J135" s="62">
-        <f>IFERROR(IF(F135="","",TEXT('Getting Started'!C10+(H135-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I135*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="136" ht="18" customHeight="1">
-      <c r="A136" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B136" s="18" t="n"/>
-      <c r="F136" s="32" t="n"/>
-      <c r="G136" s="17">
-        <f>IFERROR(SUM(F131:F136),"")</f>
-        <v/>
-      </c>
-      <c r="H136" s="17">
-        <f>IFERROR(IF(F136="","",FLOOR(G135/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I136" s="17">
-        <f>IFERROR(IF(F136="","",CEILING(G136/((IFERROR(B128,0)+IFERROR(G128,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J136" s="62">
-        <f>IFERROR(IF(F136="","",TEXT('Getting Started'!C10+(H136-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I136*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="137" ht="20" customHeight="1">
-      <c r="A137" s="63" t="n"/>
-    </row>
-    <row r="138" ht="8" customHeight="1"/>
-    <row r="139" ht="24" customHeight="1">
-      <c r="A139" s="52">
-        <f>IF('Course Content'!A35="","  ELECTIVE / OTHER 2","  "&amp;UPPER('Course Content'!A35))</f>
-        <v/>
-      </c>
-      <c r="E139" s="53">
-        <f>IFERROR(IF('Course Content'!B35="","← enter on Course Content tab",'Course Content'!B35),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="140" ht="22" customHeight="1">
-      <c r="B140" s="54">
-        <f>'Course Content'!D35</f>
-        <v/>
-      </c>
-      <c r="C140" s="55">
-        <f>IFERROR(IF(B140="","",ROUND(B140/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D140" s="55">
-        <f>IFERROR(IF(C140="","",ROUND(C140/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E140" s="56">
-        <f>IFERROR(IF(B140="","",TEXT('Getting Started'!C10+(B140/D140),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F140" s="26" t="n"/>
-      <c r="G140" s="57">
-        <f>'Course Content'!E35</f>
-        <v/>
-      </c>
-      <c r="H140" s="58">
-        <f>IFERROR(IF(G140="","",ROUND(G140/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I140" s="58">
-        <f>IFERROR(IF(H140="","",ROUND(H140/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J140" s="59">
-        <f>IFERROR(IF(G140="","",TEXT('Getting Started'!C18+(G140/I140),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="141" ht="16" customHeight="1">
-      <c r="A141" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="22" customHeight="1">
-      <c r="A142" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B142" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F142" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G142" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H142" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I142" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J142" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="143" ht="18" customHeight="1">
-      <c r="A143" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B143" s="5" t="n"/>
-      <c r="F143" s="33" t="n"/>
-      <c r="G143" s="17">
-        <f>IFERROR(SUM(F143:F143),"")</f>
-        <v/>
-      </c>
-      <c r="H143" s="17">
-        <f>IF(F143="","",1)</f>
-        <v/>
-      </c>
-      <c r="I143" s="17">
-        <f>IFERROR(IF(F143="","",CEILING(G143/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J143" s="62">
-        <f>IFERROR(IF(F143="","",TEXT('Getting Started'!C10+(H143-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I143*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="144" ht="18" customHeight="1">
-      <c r="A144" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B144" s="18" t="n"/>
-      <c r="F144" s="32" t="n"/>
-      <c r="G144" s="17">
-        <f>IFERROR(SUM(F143:F144),"")</f>
-        <v/>
-      </c>
-      <c r="H144" s="17">
-        <f>IFERROR(IF(F144="","",FLOOR(G143/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I144" s="17">
-        <f>IFERROR(IF(F144="","",CEILING(G144/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J144" s="62">
-        <f>IFERROR(IF(F144="","",TEXT('Getting Started'!C10+(H144-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I144*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="145" ht="18" customHeight="1">
-      <c r="A145" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B145" s="5" t="n"/>
-      <c r="F145" s="33" t="n"/>
-      <c r="G145" s="17">
-        <f>IFERROR(SUM(F143:F145),"")</f>
-        <v/>
-      </c>
-      <c r="H145" s="17">
-        <f>IFERROR(IF(F145="","",FLOOR(G144/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I145" s="17">
-        <f>IFERROR(IF(F145="","",CEILING(G145/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J145" s="62">
-        <f>IFERROR(IF(F145="","",TEXT('Getting Started'!C10+(H145-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I145*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="146" ht="18" customHeight="1">
-      <c r="A146" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B146" s="18" t="n"/>
-      <c r="F146" s="32" t="n"/>
-      <c r="G146" s="17">
-        <f>IFERROR(SUM(F143:F146),"")</f>
-        <v/>
-      </c>
-      <c r="H146" s="17">
-        <f>IFERROR(IF(F146="","",FLOOR(G145/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I146" s="17">
-        <f>IFERROR(IF(F146="","",CEILING(G146/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J146" s="62">
-        <f>IFERROR(IF(F146="","",TEXT('Getting Started'!C10+(H146-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I146*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="147" ht="18" customHeight="1">
-      <c r="A147" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B147" s="5" t="n"/>
-      <c r="F147" s="33" t="n"/>
-      <c r="G147" s="17">
-        <f>IFERROR(SUM(F143:F147),"")</f>
-        <v/>
-      </c>
-      <c r="H147" s="17">
-        <f>IFERROR(IF(F147="","",FLOOR(G146/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I147" s="17">
-        <f>IFERROR(IF(F147="","",CEILING(G147/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J147" s="62">
-        <f>IFERROR(IF(F147="","",TEXT('Getting Started'!C10+(H147-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I147*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="148" ht="18" customHeight="1">
-      <c r="A148" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B148" s="18" t="n"/>
-      <c r="F148" s="32" t="n"/>
-      <c r="G148" s="17">
-        <f>IFERROR(SUM(F143:F148),"")</f>
-        <v/>
-      </c>
-      <c r="H148" s="17">
-        <f>IFERROR(IF(F148="","",FLOOR(G147/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I148" s="17">
-        <f>IFERROR(IF(F148="","",CEILING(G148/((IFERROR(B140,0)+IFERROR(G140,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J148" s="62">
-        <f>IFERROR(IF(F148="","",TEXT('Getting Started'!C10+(H148-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I148*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="149" ht="20" customHeight="1">
-      <c r="A149" s="63" t="n"/>
-    </row>
-    <row r="150" ht="8" customHeight="1"/>
-    <row r="151" ht="24" customHeight="1">
-      <c r="A151" s="52">
-        <f>IF('Course Content'!A36="","  ELECTIVE / OTHER 3","  "&amp;UPPER('Course Content'!A36))</f>
-        <v/>
-      </c>
-      <c r="E151" s="53">
-        <f>IFERROR(IF('Course Content'!B36="","← enter on Course Content tab",'Course Content'!B36),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="152" ht="22" customHeight="1">
-      <c r="B152" s="54">
-        <f>'Course Content'!D36</f>
-        <v/>
-      </c>
-      <c r="C152" s="55">
-        <f>IFERROR(IF(B152="","",ROUND(B152/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D152" s="55">
-        <f>IFERROR(IF(C152="","",ROUND(C152/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E152" s="56">
-        <f>IFERROR(IF(B152="","",TEXT('Getting Started'!C10+(B152/D152),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F152" s="26" t="n"/>
-      <c r="G152" s="57">
-        <f>'Course Content'!E36</f>
-        <v/>
-      </c>
-      <c r="H152" s="58">
-        <f>IFERROR(IF(G152="","",ROUND(G152/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I152" s="58">
-        <f>IFERROR(IF(H152="","",ROUND(H152/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J152" s="59">
-        <f>IFERROR(IF(G152="","",TEXT('Getting Started'!C18+(G152/I152),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="153" ht="16" customHeight="1">
-      <c r="A153" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="22" customHeight="1">
-      <c r="A154" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B154" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F154" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G154" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H154" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I154" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J154" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="18" customHeight="1">
-      <c r="A155" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B155" s="5" t="n"/>
-      <c r="F155" s="33" t="n"/>
-      <c r="G155" s="17">
-        <f>IFERROR(SUM(F155:F155),"")</f>
-        <v/>
-      </c>
-      <c r="H155" s="17">
-        <f>IF(F155="","",1)</f>
-        <v/>
-      </c>
-      <c r="I155" s="17">
-        <f>IFERROR(IF(F155="","",CEILING(G155/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J155" s="62">
-        <f>IFERROR(IF(F155="","",TEXT('Getting Started'!C10+(H155-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I155*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156" ht="18" customHeight="1">
-      <c r="A156" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B156" s="18" t="n"/>
-      <c r="F156" s="32" t="n"/>
-      <c r="G156" s="17">
-        <f>IFERROR(SUM(F155:F156),"")</f>
-        <v/>
-      </c>
-      <c r="H156" s="17">
-        <f>IFERROR(IF(F156="","",FLOOR(G155/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I156" s="17">
-        <f>IFERROR(IF(F156="","",CEILING(G156/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J156" s="62">
-        <f>IFERROR(IF(F156="","",TEXT('Getting Started'!C10+(H156-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I156*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157" ht="18" customHeight="1">
-      <c r="A157" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B157" s="5" t="n"/>
-      <c r="F157" s="33" t="n"/>
-      <c r="G157" s="17">
-        <f>IFERROR(SUM(F155:F157),"")</f>
-        <v/>
-      </c>
-      <c r="H157" s="17">
-        <f>IFERROR(IF(F157="","",FLOOR(G156/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I157" s="17">
-        <f>IFERROR(IF(F157="","",CEILING(G157/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J157" s="62">
-        <f>IFERROR(IF(F157="","",TEXT('Getting Started'!C10+(H157-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I157*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="158" ht="18" customHeight="1">
-      <c r="A158" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B158" s="18" t="n"/>
-      <c r="F158" s="32" t="n"/>
-      <c r="G158" s="17">
-        <f>IFERROR(SUM(F155:F158),"")</f>
-        <v/>
-      </c>
-      <c r="H158" s="17">
-        <f>IFERROR(IF(F158="","",FLOOR(G157/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I158" s="17">
-        <f>IFERROR(IF(F158="","",CEILING(G158/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J158" s="62">
-        <f>IFERROR(IF(F158="","",TEXT('Getting Started'!C10+(H158-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I158*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="159" ht="18" customHeight="1">
-      <c r="A159" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B159" s="5" t="n"/>
-      <c r="F159" s="33" t="n"/>
-      <c r="G159" s="17">
-        <f>IFERROR(SUM(F155:F159),"")</f>
-        <v/>
-      </c>
-      <c r="H159" s="17">
-        <f>IFERROR(IF(F159="","",FLOOR(G158/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I159" s="17">
-        <f>IFERROR(IF(F159="","",CEILING(G159/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J159" s="62">
-        <f>IFERROR(IF(F159="","",TEXT('Getting Started'!C10+(H159-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I159*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="160" ht="18" customHeight="1">
-      <c r="A160" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B160" s="18" t="n"/>
-      <c r="F160" s="32" t="n"/>
-      <c r="G160" s="17">
-        <f>IFERROR(SUM(F155:F160),"")</f>
-        <v/>
-      </c>
-      <c r="H160" s="17">
-        <f>IFERROR(IF(F160="","",FLOOR(G159/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I160" s="17">
-        <f>IFERROR(IF(F160="","",CEILING(G160/((IFERROR(B152,0)+IFERROR(G152,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J160" s="62">
-        <f>IFERROR(IF(F160="","",TEXT('Getting Started'!C10+(H160-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I160*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="161" ht="20" customHeight="1">
-      <c r="A161" s="63" t="n"/>
-    </row>
-    <row r="162" ht="8" customHeight="1"/>
-    <row r="163" ht="24" customHeight="1">
-      <c r="A163" s="52">
-        <f>IF('Course Content'!A37="","  ELECTIVE / OTHER 4","  "&amp;UPPER('Course Content'!A37))</f>
-        <v/>
-      </c>
-      <c r="E163" s="53">
-        <f>IFERROR(IF('Course Content'!B37="","← enter on Course Content tab",'Course Content'!B37),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="164" ht="22" customHeight="1">
-      <c r="B164" s="54">
-        <f>'Course Content'!D37</f>
-        <v/>
-      </c>
-      <c r="C164" s="55">
-        <f>IFERROR(IF(B164="","",ROUND(B164/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="D164" s="55">
-        <f>IFERROR(IF(C164="","",ROUND(C164/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E164" s="56">
-        <f>IFERROR(IF(B164="","",TEXT('Getting Started'!C10+(B164/D164),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-      <c r="F164" s="26" t="n"/>
-      <c r="G164" s="57">
-        <f>'Course Content'!E37</f>
-        <v/>
-      </c>
-      <c r="H164" s="58">
-        <f>IFERROR(IF(G164="","",ROUND(G164/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I164" s="58">
-        <f>IFERROR(IF(H164="","",ROUND(H164/'Getting Started'!C7,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J164" s="59">
-        <f>IFERROR(IF(G164="","",TEXT('Getting Started'!C18+(G164/I164),"MMM D, YYYY")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="165" ht="16" customHeight="1">
-      <c r="A165" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Component Breakdown  (optional — use for multi-volume curricula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="166" ht="22" customHeight="1">
-      <c r="A166" s="48" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B166" s="48" t="inlineStr">
-        <is>
-          <t>Book / Component Title</t>
-        </is>
-      </c>
-      <c r="F166" s="48" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="G166" s="48" t="inlineStr">
-        <is>
-          <t>Cumul.</t>
-        </is>
-      </c>
-      <c r="H166" s="48" t="inlineStr">
-        <is>
-          <t>Start
-Week</t>
-        </is>
-      </c>
-      <c r="I166" s="48" t="inlineStr">
-        <is>
-          <t>End
-Week</t>
-        </is>
-      </c>
-      <c r="J166" s="48" t="inlineStr">
-        <is>
-          <t>Est. Dates</t>
-        </is>
-      </c>
-    </row>
-    <row r="167" ht="18" customHeight="1">
-      <c r="A167" s="61" t="n">
-        <v>1</v>
-      </c>
-      <c r="B167" s="5" t="n"/>
-      <c r="F167" s="33" t="n"/>
-      <c r="G167" s="17">
-        <f>IFERROR(SUM(F167:F167),"")</f>
-        <v/>
-      </c>
-      <c r="H167" s="17">
-        <f>IF(F167="","",1)</f>
-        <v/>
-      </c>
-      <c r="I167" s="17">
-        <f>IFERROR(IF(F167="","",CEILING(G167/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J167" s="62">
-        <f>IFERROR(IF(F167="","",TEXT('Getting Started'!C10+(H167-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I167*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="168" ht="18" customHeight="1">
-      <c r="A168" s="61" t="n">
-        <v>2</v>
-      </c>
-      <c r="B168" s="18" t="n"/>
-      <c r="F168" s="32" t="n"/>
-      <c r="G168" s="17">
-        <f>IFERROR(SUM(F167:F168),"")</f>
-        <v/>
-      </c>
-      <c r="H168" s="17">
-        <f>IFERROR(IF(F168="","",FLOOR(G167/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I168" s="17">
-        <f>IFERROR(IF(F168="","",CEILING(G168/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J168" s="62">
-        <f>IFERROR(IF(F168="","",TEXT('Getting Started'!C10+(H168-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I168*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="169" ht="18" customHeight="1">
-      <c r="A169" s="61" t="n">
-        <v>3</v>
-      </c>
-      <c r="B169" s="5" t="n"/>
-      <c r="F169" s="33" t="n"/>
-      <c r="G169" s="17">
-        <f>IFERROR(SUM(F167:F169),"")</f>
-        <v/>
-      </c>
-      <c r="H169" s="17">
-        <f>IFERROR(IF(F169="","",FLOOR(G168/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I169" s="17">
-        <f>IFERROR(IF(F169="","",CEILING(G169/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J169" s="62">
-        <f>IFERROR(IF(F169="","",TEXT('Getting Started'!C10+(H169-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I169*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="170" ht="18" customHeight="1">
-      <c r="A170" s="61" t="n">
-        <v>4</v>
-      </c>
-      <c r="B170" s="18" t="n"/>
-      <c r="F170" s="32" t="n"/>
-      <c r="G170" s="17">
-        <f>IFERROR(SUM(F167:F170),"")</f>
-        <v/>
-      </c>
-      <c r="H170" s="17">
-        <f>IFERROR(IF(F170="","",FLOOR(G169/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I170" s="17">
-        <f>IFERROR(IF(F170="","",CEILING(G170/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J170" s="62">
-        <f>IFERROR(IF(F170="","",TEXT('Getting Started'!C10+(H170-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I170*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="171" ht="18" customHeight="1">
-      <c r="A171" s="61" t="n">
-        <v>5</v>
-      </c>
-      <c r="B171" s="5" t="n"/>
-      <c r="F171" s="33" t="n"/>
-      <c r="G171" s="17">
-        <f>IFERROR(SUM(F167:F171),"")</f>
-        <v/>
-      </c>
-      <c r="H171" s="17">
-        <f>IFERROR(IF(F171="","",FLOOR(G170/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I171" s="17">
-        <f>IFERROR(IF(F171="","",CEILING(G171/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J171" s="62">
-        <f>IFERROR(IF(F171="","",TEXT('Getting Started'!C10+(H171-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I171*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="172" ht="18" customHeight="1">
-      <c r="A172" s="61" t="n">
-        <v>6</v>
-      </c>
-      <c r="B172" s="18" t="n"/>
-      <c r="F172" s="32" t="n"/>
-      <c r="G172" s="17">
-        <f>IFERROR(SUM(F167:F172),"")</f>
-        <v/>
-      </c>
-      <c r="H172" s="17">
-        <f>IFERROR(IF(F172="","",FLOOR(G171/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)+1),"")</f>
-        <v/>
-      </c>
-      <c r="I172" s="17">
-        <f>IFERROR(IF(F172="","",CEILING(G172/((IFERROR(B164,0)+IFERROR(G164,0))/(IFERROR('Getting Started'!C15,0)+IFERROR('Getting Started'!C23,0))),1)),"")</f>
-        <v/>
-      </c>
-      <c r="J172" s="62">
-        <f>IFERROR(IF(F172="","",TEXT('Getting Started'!C10+(H172-1)*7,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C10+I172*7,"MMM D")),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="173" ht="20" customHeight="1">
-      <c r="A173" s="63" t="n"/>
-    </row>
-    <row r="174" ht="8" customHeight="1"/>
+      <c r="A22" s="31">
+        <f>IF('Course Content'!A35="Elective / Other 2","Elective / Other 2",'Course Content'!A35)</f>
+        <v/>
+      </c>
+      <c r="B22" s="18">
+        <f>IFERROR(IF('Course Content'!B35="","—",'Course Content'!B35),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="56">
+        <f>IFERROR(IF('Course Content'!D35="","—",'Course Content'!D35),"")</f>
+        <v/>
+      </c>
+      <c r="D22" s="56">
+        <f>IFERROR(IF('Course Content'!D35="","",ROUND('Course Content'!D35/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E22" s="57">
+        <f>IFERROR(IF(D22="","",ROUND(D22/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="58">
+        <f>IFERROR(IF('Course Content'!E35="","—",'Course Content'!E35),"")</f>
+        <v/>
+      </c>
+      <c r="H22" s="58">
+        <f>IFERROR(IF('Course Content'!E35="","",ROUND('Course Content'!E35/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I22" s="59">
+        <f>IFERROR(IF(H22="","",ROUND(H22/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J22" s="61">
+        <f>IFERROR(IF('Course Content'!C35="","",'Course Content'!C35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="31">
+        <f>IF('Course Content'!A36="Elective / Other 3","Elective / Other 3",'Course Content'!A36)</f>
+        <v/>
+      </c>
+      <c r="B23" s="5">
+        <f>IFERROR(IF('Course Content'!B36="","—",'Course Content'!B36),"")</f>
+        <v/>
+      </c>
+      <c r="C23" s="56">
+        <f>IFERROR(IF('Course Content'!D36="","—",'Course Content'!D36),"")</f>
+        <v/>
+      </c>
+      <c r="D23" s="56">
+        <f>IFERROR(IF('Course Content'!D36="","",ROUND('Course Content'!D36/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E23" s="57">
+        <f>IFERROR(IF(D23="","",ROUND(D23/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="58">
+        <f>IFERROR(IF('Course Content'!E36="","—",'Course Content'!E36),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="58">
+        <f>IFERROR(IF('Course Content'!E36="","",ROUND('Course Content'!E36/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I23" s="59">
+        <f>IFERROR(IF(H23="","",ROUND(H23/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J23" s="60">
+        <f>IFERROR(IF('Course Content'!C36="","",'Course Content'!C36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="31">
+        <f>IF('Course Content'!A37="Elective / Other 4","Elective / Other 4",'Course Content'!A37)</f>
+        <v/>
+      </c>
+      <c r="B24" s="18">
+        <f>IFERROR(IF('Course Content'!B37="","—",'Course Content'!B37),"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="56">
+        <f>IFERROR(IF('Course Content'!D37="","—",'Course Content'!D37),"")</f>
+        <v/>
+      </c>
+      <c r="D24" s="56">
+        <f>IFERROR(IF('Course Content'!D37="","",ROUND('Course Content'!D37/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="E24" s="57">
+        <f>IFERROR(IF(D24="","",ROUND(D24/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="58">
+        <f>IFERROR(IF('Course Content'!E37="","—",'Course Content'!E37),"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="58">
+        <f>IFERROR(IF('Course Content'!E37="","",ROUND('Course Content'!E37/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="I24" s="59">
+        <f>IFERROR(IF(H24="","",ROUND(H24/I9,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J24" s="61">
+        <f>IFERROR(IF('Course Content'!C37="","",'Course Content'!C37),"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="158">
-    <mergeCell ref="B146:E146"/>
-    <mergeCell ref="E19:J19"/>
-    <mergeCell ref="B74:E74"/>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A6:J6"/>
     <mergeCell ref="G4:J4"/>
-    <mergeCell ref="A165:J165"/>
-    <mergeCell ref="B123:E123"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="B76:E76"/>
-    <mergeCell ref="B110:E110"/>
-    <mergeCell ref="A93:J93"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A173:J173"/>
-    <mergeCell ref="B100:E100"/>
-    <mergeCell ref="A77:J77"/>
-    <mergeCell ref="B109:E109"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B155:E155"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="B86:E86"/>
-    <mergeCell ref="A69:J69"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="E139:J139"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="B136:E136"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B13:E13"/>
-    <mergeCell ref="A163:D163"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="B112:E112"/>
-    <mergeCell ref="E79:J79"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B49:E49"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="A29:J29"/>
-    <mergeCell ref="A81:J81"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="A161:J161"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B154:E154"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B106:E106"/>
-    <mergeCell ref="A127:D127"/>
-    <mergeCell ref="E163:J163"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="B156:E156"/>
-    <mergeCell ref="E91:J91"/>
-    <mergeCell ref="B131:E131"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="A79:D79"/>
-    <mergeCell ref="E115:J115"/>
-    <mergeCell ref="B130:E130"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B61:E61"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="B132:E132"/>
-    <mergeCell ref="B166:E166"/>
-    <mergeCell ref="A149:J149"/>
-    <mergeCell ref="B119:E119"/>
-    <mergeCell ref="E127:J127"/>
-    <mergeCell ref="A139:D139"/>
-    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="H8:J8"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="B168:E168"/>
-    <mergeCell ref="B84:E84"/>
-    <mergeCell ref="B118:E118"/>
-    <mergeCell ref="A141:J141"/>
-    <mergeCell ref="A91:D91"/>
-    <mergeCell ref="B158:E158"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B142:E142"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="A125:J125"/>
-    <mergeCell ref="B95:E95"/>
-    <mergeCell ref="A115:D115"/>
-    <mergeCell ref="B160:E160"/>
-    <mergeCell ref="B169:E169"/>
-    <mergeCell ref="B144:E144"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B134:E134"/>
-    <mergeCell ref="B121:E121"/>
-    <mergeCell ref="A103:D103"/>
-    <mergeCell ref="B122:E122"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B52:E52"/>
-    <mergeCell ref="A153:J153"/>
-    <mergeCell ref="B120:E120"/>
-    <mergeCell ref="A137:J137"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="A41:J41"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="E151:J151"/>
-    <mergeCell ref="B170:E170"/>
-    <mergeCell ref="E55:J55"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B157:E157"/>
-    <mergeCell ref="E67:J67"/>
-    <mergeCell ref="B171:E171"/>
-    <mergeCell ref="A101:J101"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="B172:E172"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="A33:J33"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="E103:J103"/>
-    <mergeCell ref="B83:E83"/>
-    <mergeCell ref="A17:J17"/>
-    <mergeCell ref="B143:E143"/>
-    <mergeCell ref="A53:J53"/>
-    <mergeCell ref="E31:J31"/>
-    <mergeCell ref="B124:E124"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="B133:E133"/>
-    <mergeCell ref="B85:E85"/>
-    <mergeCell ref="B94:E94"/>
-    <mergeCell ref="A117:J117"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="B75:E75"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="B135:E135"/>
-    <mergeCell ref="B62:E62"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B159:E159"/>
-    <mergeCell ref="E7:J7"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A45:J45"/>
-    <mergeCell ref="B96:E96"/>
-    <mergeCell ref="B167:E167"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="A65:J65"/>
-    <mergeCell ref="E43:J43"/>
-    <mergeCell ref="B111:E111"/>
-    <mergeCell ref="B145:E145"/>
-    <mergeCell ref="B98:E98"/>
-    <mergeCell ref="A89:J89"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B88:E88"/>
-    <mergeCell ref="B82:E82"/>
-    <mergeCell ref="A21:J21"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="A105:J105"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="A57:J57"/>
-    <mergeCell ref="A113:J113"/>
-    <mergeCell ref="A151:D151"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="A129:J129"/>
+    <mergeCell ref="H7:J7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update generated workbook with per-subject day scheduling
https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="MM/DD/YYYY"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,6 +130,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="006B5C55"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00CE8282"/>
       <sz val="14"/>
@@ -151,6 +157,12 @@
       <b val="1"/>
       <color rgb="008A6A30"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00CE8282"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -353,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -500,34 +512,41 @@
     <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5382,19 +5401,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
     <col width="4" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="2" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
@@ -5415,8 +5442,8 @@
         <f>IFERROR("SEM 1   "&amp;TEXT('Getting Started'!C10,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C11,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C15&amp;" school wks)","SEMESTER 1")</f>
         <v/>
       </c>
-      <c r="F4" s="26" t="n"/>
-      <c r="G4" s="48">
+      <c r="J4" s="26" t="n"/>
+      <c r="K4" s="48">
         <f>IFERROR("SEM 2   "&amp;TEXT('Getting Started'!C18,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C19,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C23&amp;" school wks)","SEMESTER 2")</f>
         <v/>
       </c>
@@ -5430,110 +5457,167 @@
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="50" t="inlineStr">
-        <is>
-          <t>Mark with  X  →</t>
-        </is>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr"/>
+      <c r="B7" s="51" t="inlineStr">
+        <is>
+          <t>Typical school week  →</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Mon</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>Tue</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Wed</t>
         </is>
       </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>Thu</t>
         </is>
       </c>
-      <c r="F7" s="24" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="G7" s="24" t="inlineStr">
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="H7" s="24" t="inlineStr">
-        <is>
-          <t>Days / Week:</t>
-        </is>
-      </c>
+      <c r="I7" s="24" t="inlineStr">
+        <is>
+          <t>Days /Wk</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="n"/>
+      <c r="K7" s="52" t="n"/>
+      <c r="L7" s="52" t="n"/>
+      <c r="M7" s="52" t="n"/>
+      <c r="N7" s="52" t="n"/>
+      <c r="O7" s="52" t="n"/>
+      <c r="P7" s="52" t="n"/>
+      <c r="Q7" s="52" t="n"/>
+      <c r="R7" s="52" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="26" t="n"/>
-      <c r="B8" s="51" t="n"/>
-      <c r="C8" s="51" t="n"/>
-      <c r="D8" s="51" t="n"/>
-      <c r="E8" s="51" t="n"/>
-      <c r="F8" s="51" t="n"/>
-      <c r="G8" s="51" t="n"/>
-      <c r="H8" s="52">
-        <f>MAX(1,COUNTA(B8:G8))</f>
-        <v/>
-      </c>
+      <c r="B8" s="26" t="n"/>
+      <c r="C8" s="53" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="53" t="n"/>
+      <c r="F8" s="53" t="n"/>
+      <c r="G8" s="53" t="n"/>
+      <c r="H8" s="53" t="n"/>
+      <c r="I8" s="54">
+        <f>MAX(1,COUNTA(C8:H8))</f>
+        <v/>
+      </c>
+      <c r="J8" s="26" t="n"/>
+      <c r="K8" s="26" t="n"/>
+      <c r="L8" s="26" t="n"/>
+      <c r="M8" s="26" t="n"/>
+      <c r="N8" s="26" t="n"/>
+      <c r="O8" s="26" t="n"/>
+      <c r="P8" s="26" t="n"/>
+      <c r="Q8" s="26" t="n"/>
+      <c r="R8" s="26" t="n"/>
     </row>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="53" t="inlineStr">
+      <c r="A10" s="55" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="B10" s="53" t="inlineStr">
-        <is>
-          <t>Curriculum  /  Book</t>
-        </is>
-      </c>
-      <c r="C10" s="54" t="inlineStr">
-        <is>
-          <t>Sem 1
+      <c r="B10" s="55" t="inlineStr">
+        <is>
+          <t>Curriculum / Book</t>
+        </is>
+      </c>
+      <c r="C10" s="55" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D10" s="55" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="E10" s="55" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="F10" s="55" t="inlineStr">
+        <is>
+          <t>Th</t>
+        </is>
+      </c>
+      <c r="G10" s="55" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H10" s="55" t="inlineStr">
+        <is>
+          <t>Sa</t>
+        </is>
+      </c>
+      <c r="I10" s="55" t="inlineStr">
+        <is>
+          <t>Days
+/Wk</t>
+        </is>
+      </c>
+      <c r="J10" s="26" t="n"/>
+      <c r="K10" s="56" t="inlineStr">
+        <is>
+          <t>S1
 Total</t>
         </is>
       </c>
-      <c r="D10" s="54" t="inlineStr">
-        <is>
-          <t>Sem 1
-/ Week</t>
-        </is>
-      </c>
-      <c r="E10" s="54" t="inlineStr">
-        <is>
-          <t>Sem 1
-/ Day</t>
-        </is>
-      </c>
-      <c r="F10" s="26" t="n"/>
-      <c r="G10" s="55" t="inlineStr">
-        <is>
-          <t>Sem 2
+      <c r="L10" s="56" t="inlineStr">
+        <is>
+          <t>S1
+/Wk</t>
+        </is>
+      </c>
+      <c r="M10" s="56" t="inlineStr">
+        <is>
+          <t>S1
+/Day</t>
+        </is>
+      </c>
+      <c r="N10" s="26" t="n"/>
+      <c r="O10" s="57" t="inlineStr">
+        <is>
+          <t>S2
 Total</t>
         </is>
       </c>
-      <c r="H10" s="55" t="inlineStr">
-        <is>
-          <t>Sem 2
-/ Week</t>
-        </is>
-      </c>
-      <c r="I10" s="55" t="inlineStr">
-        <is>
-          <t>Sem 2
-/ Day</t>
-        </is>
-      </c>
-      <c r="J10" s="53" t="inlineStr">
+      <c r="P10" s="57" t="inlineStr">
+        <is>
+          <t>S2
+/Wk</t>
+        </is>
+      </c>
+      <c r="Q10" s="57" t="inlineStr">
+        <is>
+          <t>S2
+/Day</t>
+        </is>
+      </c>
+      <c r="R10" s="55" t="inlineStr">
         <is>
           <t>Unit
 Type</t>
@@ -5550,32 +5634,43 @@
         <f>IFERROR(IF('Course Content'!B24="","—",'Course Content'!B24),"")</f>
         <v/>
       </c>
-      <c r="C11" s="56">
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="58" t="n"/>
+      <c r="E11" s="58" t="n"/>
+      <c r="F11" s="58" t="n"/>
+      <c r="G11" s="58" t="n"/>
+      <c r="H11" s="58" t="n"/>
+      <c r="I11" s="17">
+        <f>IF(COUNTA(C11:H11)=0,$I$8,COUNTA(C11:H11))</f>
+        <v/>
+      </c>
+      <c r="J11" s="26" t="n"/>
+      <c r="K11" s="59">
         <f>IFERROR(IF('Course Content'!D24="","—",'Course Content'!D24),"")</f>
         <v/>
       </c>
-      <c r="D11" s="56">
-        <f>IFERROR(IF('Course Content'!D24="","",ROUND('Course Content'!D24/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E11" s="57">
-        <f>IFERROR(IF(D11="","",ROUND(D11/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F11" s="26" t="n"/>
-      <c r="G11" s="58">
+      <c r="L11" s="59">
+        <f>IFERROR(IF('Course Content'!D24="","",FLOOR('Course Content'!D24/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="60">
+        <f>IFERROR(IF(L11="","",FLOOR(L11/I11,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="26" t="n"/>
+      <c r="O11" s="61">
         <f>IFERROR(IF('Course Content'!E24="","—",'Course Content'!E24),"")</f>
         <v/>
       </c>
-      <c r="H11" s="58">
-        <f>IFERROR(IF('Course Content'!E24="","",ROUND('Course Content'!E24/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I11" s="59">
-        <f>IFERROR(IF(H11="","",ROUND(H11/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="60">
+      <c r="P11" s="61">
+        <f>IFERROR(IF('Course Content'!E24="","",FLOOR('Course Content'!E24/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q11" s="62">
+        <f>IFERROR(IF(P11="","",FLOOR(P11/I11,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R11" s="63">
         <f>IFERROR(IF('Course Content'!C24="","",'Course Content'!C24),"")</f>
         <v/>
       </c>
@@ -5590,32 +5685,43 @@
         <f>IFERROR(IF('Course Content'!B25="","—",'Course Content'!B25),"")</f>
         <v/>
       </c>
-      <c r="C12" s="56">
+      <c r="C12" s="58" t="n"/>
+      <c r="D12" s="58" t="n"/>
+      <c r="E12" s="58" t="n"/>
+      <c r="F12" s="58" t="n"/>
+      <c r="G12" s="58" t="n"/>
+      <c r="H12" s="58" t="n"/>
+      <c r="I12" s="17">
+        <f>IF(COUNTA(C12:H12)=0,$I$8,COUNTA(C12:H12))</f>
+        <v/>
+      </c>
+      <c r="J12" s="26" t="n"/>
+      <c r="K12" s="59">
         <f>IFERROR(IF('Course Content'!D25="","—",'Course Content'!D25),"")</f>
         <v/>
       </c>
-      <c r="D12" s="56">
-        <f>IFERROR(IF('Course Content'!D25="","",ROUND('Course Content'!D25/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E12" s="57">
-        <f>IFERROR(IF(D12="","",ROUND(D12/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F12" s="26" t="n"/>
-      <c r="G12" s="58">
+      <c r="L12" s="59">
+        <f>IFERROR(IF('Course Content'!D25="","",FLOOR('Course Content'!D25/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="60">
+        <f>IFERROR(IF(L12="","",FLOOR(L12/I12,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="26" t="n"/>
+      <c r="O12" s="61">
         <f>IFERROR(IF('Course Content'!E25="","—",'Course Content'!E25),"")</f>
         <v/>
       </c>
-      <c r="H12" s="58">
-        <f>IFERROR(IF('Course Content'!E25="","",ROUND('Course Content'!E25/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="59">
-        <f>IFERROR(IF(H12="","",ROUND(H12/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="61">
+      <c r="P12" s="61">
+        <f>IFERROR(IF('Course Content'!E25="","",FLOOR('Course Content'!E25/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q12" s="62">
+        <f>IFERROR(IF(P12="","",FLOOR(P12/I12,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R12" s="64">
         <f>IFERROR(IF('Course Content'!C25="","",'Course Content'!C25),"")</f>
         <v/>
       </c>
@@ -5630,32 +5736,43 @@
         <f>IFERROR(IF('Course Content'!B26="","—",'Course Content'!B26),"")</f>
         <v/>
       </c>
-      <c r="C13" s="56">
+      <c r="C13" s="58" t="n"/>
+      <c r="D13" s="58" t="n"/>
+      <c r="E13" s="58" t="n"/>
+      <c r="F13" s="58" t="n"/>
+      <c r="G13" s="58" t="n"/>
+      <c r="H13" s="58" t="n"/>
+      <c r="I13" s="17">
+        <f>IF(COUNTA(C13:H13)=0,$I$8,COUNTA(C13:H13))</f>
+        <v/>
+      </c>
+      <c r="J13" s="26" t="n"/>
+      <c r="K13" s="59">
         <f>IFERROR(IF('Course Content'!D26="","—",'Course Content'!D26),"")</f>
         <v/>
       </c>
-      <c r="D13" s="56">
-        <f>IFERROR(IF('Course Content'!D26="","",ROUND('Course Content'!D26/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E13" s="57">
-        <f>IFERROR(IF(D13="","",ROUND(D13/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="58">
+      <c r="L13" s="59">
+        <f>IFERROR(IF('Course Content'!D26="","",FLOOR('Course Content'!D26/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="60">
+        <f>IFERROR(IF(L13="","",FLOOR(L13/I13,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="26" t="n"/>
+      <c r="O13" s="61">
         <f>IFERROR(IF('Course Content'!E26="","—",'Course Content'!E26),"")</f>
         <v/>
       </c>
-      <c r="H13" s="58">
-        <f>IFERROR(IF('Course Content'!E26="","",ROUND('Course Content'!E26/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I13" s="59">
-        <f>IFERROR(IF(H13="","",ROUND(H13/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="60">
+      <c r="P13" s="61">
+        <f>IFERROR(IF('Course Content'!E26="","",FLOOR('Course Content'!E26/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q13" s="62">
+        <f>IFERROR(IF(P13="","",FLOOR(P13/I13,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R13" s="63">
         <f>IFERROR(IF('Course Content'!C26="","",'Course Content'!C26),"")</f>
         <v/>
       </c>
@@ -5670,32 +5787,43 @@
         <f>IFERROR(IF('Course Content'!B27="","—",'Course Content'!B27),"")</f>
         <v/>
       </c>
-      <c r="C14" s="56">
+      <c r="C14" s="58" t="n"/>
+      <c r="D14" s="58" t="n"/>
+      <c r="E14" s="58" t="n"/>
+      <c r="F14" s="58" t="n"/>
+      <c r="G14" s="58" t="n"/>
+      <c r="H14" s="58" t="n"/>
+      <c r="I14" s="17">
+        <f>IF(COUNTA(C14:H14)=0,$I$8,COUNTA(C14:H14))</f>
+        <v/>
+      </c>
+      <c r="J14" s="26" t="n"/>
+      <c r="K14" s="59">
         <f>IFERROR(IF('Course Content'!D27="","—",'Course Content'!D27),"")</f>
         <v/>
       </c>
-      <c r="D14" s="56">
-        <f>IFERROR(IF('Course Content'!D27="","",ROUND('Course Content'!D27/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E14" s="57">
-        <f>IFERROR(IF(D14="","",ROUND(D14/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F14" s="26" t="n"/>
-      <c r="G14" s="58">
+      <c r="L14" s="59">
+        <f>IFERROR(IF('Course Content'!D27="","",FLOOR('Course Content'!D27/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="60">
+        <f>IFERROR(IF(L14="","",FLOOR(L14/I14,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="26" t="n"/>
+      <c r="O14" s="61">
         <f>IFERROR(IF('Course Content'!E27="","—",'Course Content'!E27),"")</f>
         <v/>
       </c>
-      <c r="H14" s="58">
-        <f>IFERROR(IF('Course Content'!E27="","",ROUND('Course Content'!E27/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="59">
-        <f>IFERROR(IF(H14="","",ROUND(H14/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="61">
+      <c r="P14" s="61">
+        <f>IFERROR(IF('Course Content'!E27="","",FLOOR('Course Content'!E27/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="62">
+        <f>IFERROR(IF(P14="","",FLOOR(P14/I14,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R14" s="64">
         <f>IFERROR(IF('Course Content'!C27="","",'Course Content'!C27),"")</f>
         <v/>
       </c>
@@ -5710,32 +5838,43 @@
         <f>IFERROR(IF('Course Content'!B28="","—",'Course Content'!B28),"")</f>
         <v/>
       </c>
-      <c r="C15" s="56">
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="n"/>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="58" t="n"/>
+      <c r="H15" s="58" t="n"/>
+      <c r="I15" s="17">
+        <f>IF(COUNTA(C15:H15)=0,$I$8,COUNTA(C15:H15))</f>
+        <v/>
+      </c>
+      <c r="J15" s="26" t="n"/>
+      <c r="K15" s="59">
         <f>IFERROR(IF('Course Content'!D28="","—",'Course Content'!D28),"")</f>
         <v/>
       </c>
-      <c r="D15" s="56">
-        <f>IFERROR(IF('Course Content'!D28="","",ROUND('Course Content'!D28/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E15" s="57">
-        <f>IFERROR(IF(D15="","",ROUND(D15/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="26" t="n"/>
-      <c r="G15" s="58">
+      <c r="L15" s="59">
+        <f>IFERROR(IF('Course Content'!D28="","",FLOOR('Course Content'!D28/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="60">
+        <f>IFERROR(IF(L15="","",FLOOR(L15/I15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="26" t="n"/>
+      <c r="O15" s="61">
         <f>IFERROR(IF('Course Content'!E28="","—",'Course Content'!E28),"")</f>
         <v/>
       </c>
-      <c r="H15" s="58">
-        <f>IFERROR(IF('Course Content'!E28="","",ROUND('Course Content'!E28/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="59">
-        <f>IFERROR(IF(H15="","",ROUND(H15/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="60">
+      <c r="P15" s="61">
+        <f>IFERROR(IF('Course Content'!E28="","",FLOOR('Course Content'!E28/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="62">
+        <f>IFERROR(IF(P15="","",FLOOR(P15/I15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="63">
         <f>IFERROR(IF('Course Content'!C28="","",'Course Content'!C28),"")</f>
         <v/>
       </c>
@@ -5750,32 +5889,43 @@
         <f>IFERROR(IF('Course Content'!B29="","—",'Course Content'!B29),"")</f>
         <v/>
       </c>
-      <c r="C16" s="56">
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="n"/>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="58" t="n"/>
+      <c r="I16" s="17">
+        <f>IF(COUNTA(C16:H16)=0,$I$8,COUNTA(C16:H16))</f>
+        <v/>
+      </c>
+      <c r="J16" s="26" t="n"/>
+      <c r="K16" s="59">
         <f>IFERROR(IF('Course Content'!D29="","—",'Course Content'!D29),"")</f>
         <v/>
       </c>
-      <c r="D16" s="56">
-        <f>IFERROR(IF('Course Content'!D29="","",ROUND('Course Content'!D29/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E16" s="57">
-        <f>IFERROR(IF(D16="","",ROUND(D16/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F16" s="26" t="n"/>
-      <c r="G16" s="58">
+      <c r="L16" s="59">
+        <f>IFERROR(IF('Course Content'!D29="","",FLOOR('Course Content'!D29/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="60">
+        <f>IFERROR(IF(L16="","",FLOOR(L16/I16,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="26" t="n"/>
+      <c r="O16" s="61">
         <f>IFERROR(IF('Course Content'!E29="","—",'Course Content'!E29),"")</f>
         <v/>
       </c>
-      <c r="H16" s="58">
-        <f>IFERROR(IF('Course Content'!E29="","",ROUND('Course Content'!E29/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="59">
-        <f>IFERROR(IF(H16="","",ROUND(H16/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="61">
+      <c r="P16" s="61">
+        <f>IFERROR(IF('Course Content'!E29="","",FLOOR('Course Content'!E29/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q16" s="62">
+        <f>IFERROR(IF(P16="","",FLOOR(P16/I16,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R16" s="64">
         <f>IFERROR(IF('Course Content'!C29="","",'Course Content'!C29),"")</f>
         <v/>
       </c>
@@ -5790,32 +5940,43 @@
         <f>IFERROR(IF('Course Content'!B30="","—",'Course Content'!B30),"")</f>
         <v/>
       </c>
-      <c r="C17" s="56">
+      <c r="C17" s="58" t="n"/>
+      <c r="D17" s="58" t="n"/>
+      <c r="E17" s="58" t="n"/>
+      <c r="F17" s="58" t="n"/>
+      <c r="G17" s="58" t="n"/>
+      <c r="H17" s="58" t="n"/>
+      <c r="I17" s="17">
+        <f>IF(COUNTA(C17:H17)=0,$I$8,COUNTA(C17:H17))</f>
+        <v/>
+      </c>
+      <c r="J17" s="26" t="n"/>
+      <c r="K17" s="59">
         <f>IFERROR(IF('Course Content'!D30="","—",'Course Content'!D30),"")</f>
         <v/>
       </c>
-      <c r="D17" s="56">
-        <f>IFERROR(IF('Course Content'!D30="","",ROUND('Course Content'!D30/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E17" s="57">
-        <f>IFERROR(IF(D17="","",ROUND(D17/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="26" t="n"/>
-      <c r="G17" s="58">
+      <c r="L17" s="59">
+        <f>IFERROR(IF('Course Content'!D30="","",FLOOR('Course Content'!D30/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="60">
+        <f>IFERROR(IF(L17="","",FLOOR(L17/I17,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="26" t="n"/>
+      <c r="O17" s="61">
         <f>IFERROR(IF('Course Content'!E30="","—",'Course Content'!E30),"")</f>
         <v/>
       </c>
-      <c r="H17" s="58">
-        <f>IFERROR(IF('Course Content'!E30="","",ROUND('Course Content'!E30/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I17" s="59">
-        <f>IFERROR(IF(H17="","",ROUND(H17/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="60">
+      <c r="P17" s="61">
+        <f>IFERROR(IF('Course Content'!E30="","",FLOOR('Course Content'!E30/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="62">
+        <f>IFERROR(IF(P17="","",FLOOR(P17/I17,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R17" s="63">
         <f>IFERROR(IF('Course Content'!C30="","",'Course Content'!C30),"")</f>
         <v/>
       </c>
@@ -5830,32 +5991,43 @@
         <f>IFERROR(IF('Course Content'!B31="","—",'Course Content'!B31),"")</f>
         <v/>
       </c>
-      <c r="C18" s="56">
+      <c r="C18" s="58" t="n"/>
+      <c r="D18" s="58" t="n"/>
+      <c r="E18" s="58" t="n"/>
+      <c r="F18" s="58" t="n"/>
+      <c r="G18" s="58" t="n"/>
+      <c r="H18" s="58" t="n"/>
+      <c r="I18" s="17">
+        <f>IF(COUNTA(C18:H18)=0,$I$8,COUNTA(C18:H18))</f>
+        <v/>
+      </c>
+      <c r="J18" s="26" t="n"/>
+      <c r="K18" s="59">
         <f>IFERROR(IF('Course Content'!D31="","—",'Course Content'!D31),"")</f>
         <v/>
       </c>
-      <c r="D18" s="56">
-        <f>IFERROR(IF('Course Content'!D31="","",ROUND('Course Content'!D31/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E18" s="57">
-        <f>IFERROR(IF(D18="","",ROUND(D18/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F18" s="26" t="n"/>
-      <c r="G18" s="58">
+      <c r="L18" s="59">
+        <f>IFERROR(IF('Course Content'!D31="","",FLOOR('Course Content'!D31/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="60">
+        <f>IFERROR(IF(L18="","",FLOOR(L18/I18,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="26" t="n"/>
+      <c r="O18" s="61">
         <f>IFERROR(IF('Course Content'!E31="","—",'Course Content'!E31),"")</f>
         <v/>
       </c>
-      <c r="H18" s="58">
-        <f>IFERROR(IF('Course Content'!E31="","",ROUND('Course Content'!E31/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I18" s="59">
-        <f>IFERROR(IF(H18="","",ROUND(H18/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="61">
+      <c r="P18" s="61">
+        <f>IFERROR(IF('Course Content'!E31="","",FLOOR('Course Content'!E31/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q18" s="62">
+        <f>IFERROR(IF(P18="","",FLOOR(P18/I18,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R18" s="64">
         <f>IFERROR(IF('Course Content'!C31="","",'Course Content'!C31),"")</f>
         <v/>
       </c>
@@ -5870,32 +6042,43 @@
         <f>IFERROR(IF('Course Content'!B32="","—",'Course Content'!B32),"")</f>
         <v/>
       </c>
-      <c r="C19" s="56">
+      <c r="C19" s="58" t="n"/>
+      <c r="D19" s="58" t="n"/>
+      <c r="E19" s="58" t="n"/>
+      <c r="F19" s="58" t="n"/>
+      <c r="G19" s="58" t="n"/>
+      <c r="H19" s="58" t="n"/>
+      <c r="I19" s="17">
+        <f>IF(COUNTA(C19:H19)=0,$I$8,COUNTA(C19:H19))</f>
+        <v/>
+      </c>
+      <c r="J19" s="26" t="n"/>
+      <c r="K19" s="59">
         <f>IFERROR(IF('Course Content'!D32="","—",'Course Content'!D32),"")</f>
         <v/>
       </c>
-      <c r="D19" s="56">
-        <f>IFERROR(IF('Course Content'!D32="","",ROUND('Course Content'!D32/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E19" s="57">
-        <f>IFERROR(IF(D19="","",ROUND(D19/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F19" s="26" t="n"/>
-      <c r="G19" s="58">
+      <c r="L19" s="59">
+        <f>IFERROR(IF('Course Content'!D32="","",FLOOR('Course Content'!D32/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="60">
+        <f>IFERROR(IF(L19="","",FLOOR(L19/I19,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="26" t="n"/>
+      <c r="O19" s="61">
         <f>IFERROR(IF('Course Content'!E32="","—",'Course Content'!E32),"")</f>
         <v/>
       </c>
-      <c r="H19" s="58">
-        <f>IFERROR(IF('Course Content'!E32="","",ROUND('Course Content'!E32/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I19" s="59">
-        <f>IFERROR(IF(H19="","",ROUND(H19/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="60">
+      <c r="P19" s="61">
+        <f>IFERROR(IF('Course Content'!E32="","",FLOOR('Course Content'!E32/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q19" s="62">
+        <f>IFERROR(IF(P19="","",FLOOR(P19/I19,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R19" s="63">
         <f>IFERROR(IF('Course Content'!C32="","",'Course Content'!C32),"")</f>
         <v/>
       </c>
@@ -5910,32 +6093,43 @@
         <f>IFERROR(IF('Course Content'!B33="","—",'Course Content'!B33),"")</f>
         <v/>
       </c>
-      <c r="C20" s="56">
+      <c r="C20" s="58" t="n"/>
+      <c r="D20" s="58" t="n"/>
+      <c r="E20" s="58" t="n"/>
+      <c r="F20" s="58" t="n"/>
+      <c r="G20" s="58" t="n"/>
+      <c r="H20" s="58" t="n"/>
+      <c r="I20" s="17">
+        <f>IF(COUNTA(C20:H20)=0,$I$8,COUNTA(C20:H20))</f>
+        <v/>
+      </c>
+      <c r="J20" s="26" t="n"/>
+      <c r="K20" s="59">
         <f>IFERROR(IF('Course Content'!D33="","—",'Course Content'!D33),"")</f>
         <v/>
       </c>
-      <c r="D20" s="56">
-        <f>IFERROR(IF('Course Content'!D33="","",ROUND('Course Content'!D33/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E20" s="57">
-        <f>IFERROR(IF(D20="","",ROUND(D20/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F20" s="26" t="n"/>
-      <c r="G20" s="58">
+      <c r="L20" s="59">
+        <f>IFERROR(IF('Course Content'!D33="","",FLOOR('Course Content'!D33/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M20" s="60">
+        <f>IFERROR(IF(L20="","",FLOOR(L20/I20,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="26" t="n"/>
+      <c r="O20" s="61">
         <f>IFERROR(IF('Course Content'!E33="","—",'Course Content'!E33),"")</f>
         <v/>
       </c>
-      <c r="H20" s="58">
-        <f>IFERROR(IF('Course Content'!E33="","",ROUND('Course Content'!E33/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="59">
-        <f>IFERROR(IF(H20="","",ROUND(H20/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="61">
+      <c r="P20" s="61">
+        <f>IFERROR(IF('Course Content'!E33="","",FLOOR('Course Content'!E33/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q20" s="62">
+        <f>IFERROR(IF(P20="","",FLOOR(P20/I20,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R20" s="64">
         <f>IFERROR(IF('Course Content'!C33="","",'Course Content'!C33),"")</f>
         <v/>
       </c>
@@ -5949,32 +6143,43 @@
         <f>IFERROR(IF('Course Content'!B34="","—",'Course Content'!B34),"")</f>
         <v/>
       </c>
-      <c r="C21" s="56">
+      <c r="C21" s="58" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="58" t="n"/>
+      <c r="F21" s="58" t="n"/>
+      <c r="G21" s="58" t="n"/>
+      <c r="H21" s="58" t="n"/>
+      <c r="I21" s="17">
+        <f>IF(COUNTA(C21:H21)=0,$I$8,COUNTA(C21:H21))</f>
+        <v/>
+      </c>
+      <c r="J21" s="26" t="n"/>
+      <c r="K21" s="59">
         <f>IFERROR(IF('Course Content'!D34="","—",'Course Content'!D34),"")</f>
         <v/>
       </c>
-      <c r="D21" s="56">
-        <f>IFERROR(IF('Course Content'!D34="","",ROUND('Course Content'!D34/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E21" s="57">
-        <f>IFERROR(IF(D21="","",ROUND(D21/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F21" s="26" t="n"/>
-      <c r="G21" s="58">
+      <c r="L21" s="59">
+        <f>IFERROR(IF('Course Content'!D34="","",FLOOR('Course Content'!D34/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M21" s="60">
+        <f>IFERROR(IF(L21="","",FLOOR(L21/I21,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N21" s="26" t="n"/>
+      <c r="O21" s="61">
         <f>IFERROR(IF('Course Content'!E34="","—",'Course Content'!E34),"")</f>
         <v/>
       </c>
-      <c r="H21" s="58">
-        <f>IFERROR(IF('Course Content'!E34="","",ROUND('Course Content'!E34/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I21" s="59">
-        <f>IFERROR(IF(H21="","",ROUND(H21/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J21" s="60">
+      <c r="P21" s="61">
+        <f>IFERROR(IF('Course Content'!E34="","",FLOOR('Course Content'!E34/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q21" s="62">
+        <f>IFERROR(IF(P21="","",FLOOR(P21/I21,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R21" s="63">
         <f>IFERROR(IF('Course Content'!C34="","",'Course Content'!C34),"")</f>
         <v/>
       </c>
@@ -5988,32 +6193,43 @@
         <f>IFERROR(IF('Course Content'!B35="","—",'Course Content'!B35),"")</f>
         <v/>
       </c>
-      <c r="C22" s="56">
+      <c r="C22" s="58" t="n"/>
+      <c r="D22" s="58" t="n"/>
+      <c r="E22" s="58" t="n"/>
+      <c r="F22" s="58" t="n"/>
+      <c r="G22" s="58" t="n"/>
+      <c r="H22" s="58" t="n"/>
+      <c r="I22" s="17">
+        <f>IF(COUNTA(C22:H22)=0,$I$8,COUNTA(C22:H22))</f>
+        <v/>
+      </c>
+      <c r="J22" s="26" t="n"/>
+      <c r="K22" s="59">
         <f>IFERROR(IF('Course Content'!D35="","—",'Course Content'!D35),"")</f>
         <v/>
       </c>
-      <c r="D22" s="56">
-        <f>IFERROR(IF('Course Content'!D35="","",ROUND('Course Content'!D35/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E22" s="57">
-        <f>IFERROR(IF(D22="","",ROUND(D22/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F22" s="26" t="n"/>
-      <c r="G22" s="58">
+      <c r="L22" s="59">
+        <f>IFERROR(IF('Course Content'!D35="","",FLOOR('Course Content'!D35/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="60">
+        <f>IFERROR(IF(L22="","",FLOOR(L22/I22,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N22" s="26" t="n"/>
+      <c r="O22" s="61">
         <f>IFERROR(IF('Course Content'!E35="","—",'Course Content'!E35),"")</f>
         <v/>
       </c>
-      <c r="H22" s="58">
-        <f>IFERROR(IF('Course Content'!E35="","",ROUND('Course Content'!E35/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I22" s="59">
-        <f>IFERROR(IF(H22="","",ROUND(H22/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="61">
+      <c r="P22" s="61">
+        <f>IFERROR(IF('Course Content'!E35="","",FLOOR('Course Content'!E35/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q22" s="62">
+        <f>IFERROR(IF(P22="","",FLOOR(P22/I22,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R22" s="64">
         <f>IFERROR(IF('Course Content'!C35="","",'Course Content'!C35),"")</f>
         <v/>
       </c>
@@ -6027,32 +6243,43 @@
         <f>IFERROR(IF('Course Content'!B36="","—",'Course Content'!B36),"")</f>
         <v/>
       </c>
-      <c r="C23" s="56">
+      <c r="C23" s="58" t="n"/>
+      <c r="D23" s="58" t="n"/>
+      <c r="E23" s="58" t="n"/>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="58" t="n"/>
+      <c r="H23" s="58" t="n"/>
+      <c r="I23" s="17">
+        <f>IF(COUNTA(C23:H23)=0,$I$8,COUNTA(C23:H23))</f>
+        <v/>
+      </c>
+      <c r="J23" s="26" t="n"/>
+      <c r="K23" s="59">
         <f>IFERROR(IF('Course Content'!D36="","—",'Course Content'!D36),"")</f>
         <v/>
       </c>
-      <c r="D23" s="56">
-        <f>IFERROR(IF('Course Content'!D36="","",ROUND('Course Content'!D36/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E23" s="57">
-        <f>IFERROR(IF(D23="","",ROUND(D23/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F23" s="26" t="n"/>
-      <c r="G23" s="58">
+      <c r="L23" s="59">
+        <f>IFERROR(IF('Course Content'!D36="","",FLOOR('Course Content'!D36/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="60">
+        <f>IFERROR(IF(L23="","",FLOOR(L23/I23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="26" t="n"/>
+      <c r="O23" s="61">
         <f>IFERROR(IF('Course Content'!E36="","—",'Course Content'!E36),"")</f>
         <v/>
       </c>
-      <c r="H23" s="58">
-        <f>IFERROR(IF('Course Content'!E36="","",ROUND('Course Content'!E36/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I23" s="59">
-        <f>IFERROR(IF(H23="","",ROUND(H23/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J23" s="60">
+      <c r="P23" s="61">
+        <f>IFERROR(IF('Course Content'!E36="","",FLOOR('Course Content'!E36/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q23" s="62">
+        <f>IFERROR(IF(P23="","",FLOOR(P23/I23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R23" s="63">
         <f>IFERROR(IF('Course Content'!C36="","",'Course Content'!C36),"")</f>
         <v/>
       </c>
@@ -6066,45 +6293,54 @@
         <f>IFERROR(IF('Course Content'!B37="","—",'Course Content'!B37),"")</f>
         <v/>
       </c>
-      <c r="C24" s="56">
+      <c r="C24" s="58" t="n"/>
+      <c r="D24" s="58" t="n"/>
+      <c r="E24" s="58" t="n"/>
+      <c r="F24" s="58" t="n"/>
+      <c r="G24" s="58" t="n"/>
+      <c r="H24" s="58" t="n"/>
+      <c r="I24" s="17">
+        <f>IF(COUNTA(C24:H24)=0,$I$8,COUNTA(C24:H24))</f>
+        <v/>
+      </c>
+      <c r="J24" s="26" t="n"/>
+      <c r="K24" s="59">
         <f>IFERROR(IF('Course Content'!D37="","—",'Course Content'!D37),"")</f>
         <v/>
       </c>
-      <c r="D24" s="56">
-        <f>IFERROR(IF('Course Content'!D37="","",ROUND('Course Content'!D37/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="E24" s="57">
-        <f>IFERROR(IF(D24="","",ROUND(D24/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="F24" s="26" t="n"/>
-      <c r="G24" s="58">
+      <c r="L24" s="59">
+        <f>IFERROR(IF('Course Content'!D37="","",FLOOR('Course Content'!D37/'Getting Started'!C15,1)),"")</f>
+        <v/>
+      </c>
+      <c r="M24" s="60">
+        <f>IFERROR(IF(L24="","",FLOOR(L24/I24,1)),"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="26" t="n"/>
+      <c r="O24" s="61">
         <f>IFERROR(IF('Course Content'!E37="","—",'Course Content'!E37),"")</f>
         <v/>
       </c>
-      <c r="H24" s="58">
-        <f>IFERROR(IF('Course Content'!E37="","",ROUND('Course Content'!E37/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="I24" s="59">
-        <f>IFERROR(IF(H24="","",ROUND(H24/I9,1)),"")</f>
-        <v/>
-      </c>
-      <c r="J24" s="61">
+      <c r="P24" s="61">
+        <f>IFERROR(IF('Course Content'!E37="","",FLOOR('Course Content'!E37/'Getting Started'!C23,1)),"")</f>
+        <v/>
+      </c>
+      <c r="Q24" s="62">
+        <f>IFERROR(IF(P24="","",FLOOR(P24/I24,1)),"")</f>
+        <v/>
+      </c>
+      <c r="R24" s="64">
         <f>IFERROR(IF('Course Content'!C37="","",'Course Content'!C37),"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="H7:J7"/>
+  <mergeCells count="5">
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="K4:R4"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A6:R6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Pull Group Studies and Slot 2 through to student tab
Student tab now aggregates all four curriculum sources per subject:
Group Studies Slot 1 & 2 plus per-student Slot 1 & 2. Curriculum column
shows all non-blank titles joined with " · " (group entries prefixed
[Grp]). S1/S2 totals sum all four slots; unit type uses first non-blank.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -365,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -534,6 +534,9 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -551,6 +554,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -5630,48 +5636,48 @@
           <t>Bible</t>
         </is>
       </c>
-      <c r="B11" s="5">
-        <f>IFERROR(IF('Course Content'!B24="","—",'Course Content'!B24),"")</f>
-        <v/>
-      </c>
-      <c r="C11" s="58" t="n"/>
-      <c r="D11" s="58" t="n"/>
-      <c r="E11" s="58" t="n"/>
-      <c r="F11" s="58" t="n"/>
-      <c r="G11" s="58" t="n"/>
-      <c r="H11" s="58" t="n"/>
+      <c r="B11" s="58">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,""),IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,""),IF('Course Content'!B24&lt;&gt;"",'Course Content'!B24,""),IF('Course Content'!G24&lt;&gt;"",'Course Content'!G24,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C11" s="59" t="n"/>
+      <c r="D11" s="59" t="n"/>
+      <c r="E11" s="59" t="n"/>
+      <c r="F11" s="59" t="n"/>
+      <c r="G11" s="59" t="n"/>
+      <c r="H11" s="59" t="n"/>
       <c r="I11" s="17">
         <f>IF(COUNTA(C11:H11)=0,$I$8,COUNTA(C11:H11))</f>
         <v/>
       </c>
       <c r="J11" s="26" t="n"/>
-      <c r="K11" s="59">
-        <f>IFERROR(IF('Course Content'!D24="","—",'Course Content'!D24),"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="59">
-        <f>IFERROR(IF('Course Content'!D24="","",FLOOR('Course Content'!D24/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="60">
-        <f>IFERROR(IF(L11="","",FLOOR(L11/I11,1)),"")</f>
+      <c r="K11" s="60">
+        <f>IFERROR(IF(('Course Content'!D8="")*('Course Content'!I8="")*('Course Content'!D24="")*('Course Content'!I24=""),"—",IFERROR('Course Content'!D8*1,0)+IFERROR('Course Content'!I8*1,0)+IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="60">
+        <f>IFERROR(IF(K11="","",IF(K11="—","",FLOOR(K11/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="61">
+        <f>IFERROR(IF(L11="","",IF(L11="—","",FLOOR(L11/I11,1))),"")</f>
         <v/>
       </c>
       <c r="N11" s="26" t="n"/>
-      <c r="O11" s="61">
-        <f>IFERROR(IF('Course Content'!E24="","—",'Course Content'!E24),"")</f>
-        <v/>
-      </c>
-      <c r="P11" s="61">
-        <f>IFERROR(IF('Course Content'!E24="","",FLOOR('Course Content'!E24/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q11" s="62">
-        <f>IFERROR(IF(P11="","",FLOOR(P11/I11,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R11" s="63">
-        <f>IFERROR(IF('Course Content'!C24="","",'Course Content'!C24),"")</f>
+      <c r="O11" s="62">
+        <f>IFERROR(IF(('Course Content'!E8="")*('Course Content'!J8="")*('Course Content'!E24="")*('Course Content'!J24=""),"—",IFERROR('Course Content'!E8*1,0)+IFERROR('Course Content'!J8*1,0)+IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="62">
+        <f>IFERROR(IF(O11="","",IF(O11="—","",FLOOR(O11/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q11" s="63">
+        <f>IFERROR(IF(P11="","",IF(P11="—","",FLOOR(P11/I11,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R11" s="64">
+        <f>IFERROR(IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,IF('Course Content'!H24&lt;&gt;"",'Course Content'!H24,IF('Course Content'!C8&lt;&gt;"",'Course Content'!C8,'Course Content'!H8))),"")</f>
         <v/>
       </c>
     </row>
@@ -5681,48 +5687,48 @@
           <t>Math</t>
         </is>
       </c>
-      <c r="B12" s="18">
-        <f>IFERROR(IF('Course Content'!B25="","—",'Course Content'!B25),"")</f>
-        <v/>
-      </c>
-      <c r="C12" s="58" t="n"/>
-      <c r="D12" s="58" t="n"/>
-      <c r="E12" s="58" t="n"/>
-      <c r="F12" s="58" t="n"/>
-      <c r="G12" s="58" t="n"/>
-      <c r="H12" s="58" t="n"/>
+      <c r="B12" s="65">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,""),IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,""),IF('Course Content'!B25&lt;&gt;"",'Course Content'!B25,""),IF('Course Content'!G25&lt;&gt;"",'Course Content'!G25,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C12" s="59" t="n"/>
+      <c r="D12" s="59" t="n"/>
+      <c r="E12" s="59" t="n"/>
+      <c r="F12" s="59" t="n"/>
+      <c r="G12" s="59" t="n"/>
+      <c r="H12" s="59" t="n"/>
       <c r="I12" s="17">
         <f>IF(COUNTA(C12:H12)=0,$I$8,COUNTA(C12:H12))</f>
         <v/>
       </c>
       <c r="J12" s="26" t="n"/>
-      <c r="K12" s="59">
-        <f>IFERROR(IF('Course Content'!D25="","—",'Course Content'!D25),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="59">
-        <f>IFERROR(IF('Course Content'!D25="","",FLOOR('Course Content'!D25/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="60">
-        <f>IFERROR(IF(L12="","",FLOOR(L12/I12,1)),"")</f>
+      <c r="K12" s="60">
+        <f>IFERROR(IF(('Course Content'!D9="")*('Course Content'!I9="")*('Course Content'!D25="")*('Course Content'!I25=""),"—",IFERROR('Course Content'!D9*1,0)+IFERROR('Course Content'!I9*1,0)+IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="60">
+        <f>IFERROR(IF(K12="","",IF(K12="—","",FLOOR(K12/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="61">
+        <f>IFERROR(IF(L12="","",IF(L12="—","",FLOOR(L12/I12,1))),"")</f>
         <v/>
       </c>
       <c r="N12" s="26" t="n"/>
-      <c r="O12" s="61">
-        <f>IFERROR(IF('Course Content'!E25="","—",'Course Content'!E25),"")</f>
-        <v/>
-      </c>
-      <c r="P12" s="61">
-        <f>IFERROR(IF('Course Content'!E25="","",FLOOR('Course Content'!E25/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q12" s="62">
-        <f>IFERROR(IF(P12="","",FLOOR(P12/I12,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R12" s="64">
-        <f>IFERROR(IF('Course Content'!C25="","",'Course Content'!C25),"")</f>
+      <c r="O12" s="62">
+        <f>IFERROR(IF(('Course Content'!E9="")*('Course Content'!J9="")*('Course Content'!E25="")*('Course Content'!J25=""),"—",IFERROR('Course Content'!E9*1,0)+IFERROR('Course Content'!J9*1,0)+IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="62">
+        <f>IFERROR(IF(O12="","",IF(O12="—","",FLOOR(O12/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q12" s="63">
+        <f>IFERROR(IF(P12="","",IF(P12="—","",FLOOR(P12/I12,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R12" s="66">
+        <f>IFERROR(IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,IF('Course Content'!H25&lt;&gt;"",'Course Content'!H25,IF('Course Content'!C9&lt;&gt;"",'Course Content'!C9,'Course Content'!H9))),"")</f>
         <v/>
       </c>
     </row>
@@ -5732,48 +5738,48 @@
           <t>English / Language Arts</t>
         </is>
       </c>
-      <c r="B13" s="5">
-        <f>IFERROR(IF('Course Content'!B26="","—",'Course Content'!B26),"")</f>
-        <v/>
-      </c>
-      <c r="C13" s="58" t="n"/>
-      <c r="D13" s="58" t="n"/>
-      <c r="E13" s="58" t="n"/>
-      <c r="F13" s="58" t="n"/>
-      <c r="G13" s="58" t="n"/>
-      <c r="H13" s="58" t="n"/>
+      <c r="B13" s="58">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,""),IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,""),IF('Course Content'!B26&lt;&gt;"",'Course Content'!B26,""),IF('Course Content'!G26&lt;&gt;"",'Course Content'!G26,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C13" s="59" t="n"/>
+      <c r="D13" s="59" t="n"/>
+      <c r="E13" s="59" t="n"/>
+      <c r="F13" s="59" t="n"/>
+      <c r="G13" s="59" t="n"/>
+      <c r="H13" s="59" t="n"/>
       <c r="I13" s="17">
         <f>IF(COUNTA(C13:H13)=0,$I$8,COUNTA(C13:H13))</f>
         <v/>
       </c>
       <c r="J13" s="26" t="n"/>
-      <c r="K13" s="59">
-        <f>IFERROR(IF('Course Content'!D26="","—",'Course Content'!D26),"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="59">
-        <f>IFERROR(IF('Course Content'!D26="","",FLOOR('Course Content'!D26/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="60">
-        <f>IFERROR(IF(L13="","",FLOOR(L13/I13,1)),"")</f>
+      <c r="K13" s="60">
+        <f>IFERROR(IF(('Course Content'!D10="")*('Course Content'!I10="")*('Course Content'!D26="")*('Course Content'!I26=""),"—",IFERROR('Course Content'!D10*1,0)+IFERROR('Course Content'!I10*1,0)+IFERROR('Course Content'!D26*1,0)+IFERROR('Course Content'!I26*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="60">
+        <f>IFERROR(IF(K13="","",IF(K13="—","",FLOOR(K13/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="61">
+        <f>IFERROR(IF(L13="","",IF(L13="—","",FLOOR(L13/I13,1))),"")</f>
         <v/>
       </c>
       <c r="N13" s="26" t="n"/>
-      <c r="O13" s="61">
-        <f>IFERROR(IF('Course Content'!E26="","—",'Course Content'!E26),"")</f>
-        <v/>
-      </c>
-      <c r="P13" s="61">
-        <f>IFERROR(IF('Course Content'!E26="","",FLOOR('Course Content'!E26/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q13" s="62">
-        <f>IFERROR(IF(P13="","",FLOOR(P13/I13,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R13" s="63">
-        <f>IFERROR(IF('Course Content'!C26="","",'Course Content'!C26),"")</f>
+      <c r="O13" s="62">
+        <f>IFERROR(IF(('Course Content'!E10="")*('Course Content'!J10="")*('Course Content'!E26="")*('Course Content'!J26=""),"—",IFERROR('Course Content'!E10*1,0)+IFERROR('Course Content'!J10*1,0)+IFERROR('Course Content'!E26*1,0)+IFERROR('Course Content'!J26*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="62">
+        <f>IFERROR(IF(O13="","",IF(O13="—","",FLOOR(O13/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q13" s="63">
+        <f>IFERROR(IF(P13="","",IF(P13="—","",FLOOR(P13/I13,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R13" s="64">
+        <f>IFERROR(IF('Course Content'!C26&lt;&gt;"",'Course Content'!C26,IF('Course Content'!H26&lt;&gt;"",'Course Content'!H26,IF('Course Content'!C10&lt;&gt;"",'Course Content'!C10,'Course Content'!H10))),"")</f>
         <v/>
       </c>
     </row>
@@ -5783,48 +5789,48 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B14" s="18">
-        <f>IFERROR(IF('Course Content'!B27="","—",'Course Content'!B27),"")</f>
-        <v/>
-      </c>
-      <c r="C14" s="58" t="n"/>
-      <c r="D14" s="58" t="n"/>
-      <c r="E14" s="58" t="n"/>
-      <c r="F14" s="58" t="n"/>
-      <c r="G14" s="58" t="n"/>
-      <c r="H14" s="58" t="n"/>
+      <c r="B14" s="65">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,""),IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,""),IF('Course Content'!B27&lt;&gt;"",'Course Content'!B27,""),IF('Course Content'!G27&lt;&gt;"",'Course Content'!G27,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C14" s="59" t="n"/>
+      <c r="D14" s="59" t="n"/>
+      <c r="E14" s="59" t="n"/>
+      <c r="F14" s="59" t="n"/>
+      <c r="G14" s="59" t="n"/>
+      <c r="H14" s="59" t="n"/>
       <c r="I14" s="17">
         <f>IF(COUNTA(C14:H14)=0,$I$8,COUNTA(C14:H14))</f>
         <v/>
       </c>
       <c r="J14" s="26" t="n"/>
-      <c r="K14" s="59">
-        <f>IFERROR(IF('Course Content'!D27="","—",'Course Content'!D27),"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="59">
-        <f>IFERROR(IF('Course Content'!D27="","",FLOOR('Course Content'!D27/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="60">
-        <f>IFERROR(IF(L14="","",FLOOR(L14/I14,1)),"")</f>
+      <c r="K14" s="60">
+        <f>IFERROR(IF(('Course Content'!D11="")*('Course Content'!I11="")*('Course Content'!D27="")*('Course Content'!I27=""),"—",IFERROR('Course Content'!D11*1,0)+IFERROR('Course Content'!I11*1,0)+IFERROR('Course Content'!D27*1,0)+IFERROR('Course Content'!I27*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="60">
+        <f>IFERROR(IF(K14="","",IF(K14="—","",FLOOR(K14/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="61">
+        <f>IFERROR(IF(L14="","",IF(L14="—","",FLOOR(L14/I14,1))),"")</f>
         <v/>
       </c>
       <c r="N14" s="26" t="n"/>
-      <c r="O14" s="61">
-        <f>IFERROR(IF('Course Content'!E27="","—",'Course Content'!E27),"")</f>
-        <v/>
-      </c>
-      <c r="P14" s="61">
-        <f>IFERROR(IF('Course Content'!E27="","",FLOOR('Course Content'!E27/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q14" s="62">
-        <f>IFERROR(IF(P14="","",FLOOR(P14/I14,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R14" s="64">
-        <f>IFERROR(IF('Course Content'!C27="","",'Course Content'!C27),"")</f>
+      <c r="O14" s="62">
+        <f>IFERROR(IF(('Course Content'!E11="")*('Course Content'!J11="")*('Course Content'!E27="")*('Course Content'!J27=""),"—",IFERROR('Course Content'!E11*1,0)+IFERROR('Course Content'!J11*1,0)+IFERROR('Course Content'!E27*1,0)+IFERROR('Course Content'!J27*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="62">
+        <f>IFERROR(IF(O14="","",IF(O14="—","",FLOOR(O14/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="63">
+        <f>IFERROR(IF(P14="","",IF(P14="—","",FLOOR(P14/I14,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R14" s="66">
+        <f>IFERROR(IF('Course Content'!C27&lt;&gt;"",'Course Content'!C27,IF('Course Content'!H27&lt;&gt;"",'Course Content'!H27,IF('Course Content'!C11&lt;&gt;"",'Course Content'!C11,'Course Content'!H11))),"")</f>
         <v/>
       </c>
     </row>
@@ -5834,48 +5840,48 @@
           <t>Writing / Composition</t>
         </is>
       </c>
-      <c r="B15" s="5">
-        <f>IFERROR(IF('Course Content'!B28="","—",'Course Content'!B28),"")</f>
-        <v/>
-      </c>
-      <c r="C15" s="58" t="n"/>
-      <c r="D15" s="58" t="n"/>
-      <c r="E15" s="58" t="n"/>
-      <c r="F15" s="58" t="n"/>
-      <c r="G15" s="58" t="n"/>
-      <c r="H15" s="58" t="n"/>
+      <c r="B15" s="58">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,""),IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,""),IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,""),IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C15" s="59" t="n"/>
+      <c r="D15" s="59" t="n"/>
+      <c r="E15" s="59" t="n"/>
+      <c r="F15" s="59" t="n"/>
+      <c r="G15" s="59" t="n"/>
+      <c r="H15" s="59" t="n"/>
       <c r="I15" s="17">
         <f>IF(COUNTA(C15:H15)=0,$I$8,COUNTA(C15:H15))</f>
         <v/>
       </c>
       <c r="J15" s="26" t="n"/>
-      <c r="K15" s="59">
-        <f>IFERROR(IF('Course Content'!D28="","—",'Course Content'!D28),"")</f>
-        <v/>
-      </c>
-      <c r="L15" s="59">
-        <f>IFERROR(IF('Course Content'!D28="","",FLOOR('Course Content'!D28/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M15" s="60">
-        <f>IFERROR(IF(L15="","",FLOOR(L15/I15,1)),"")</f>
+      <c r="K15" s="60">
+        <f>IFERROR(IF(('Course Content'!D12="")*('Course Content'!I12="")*('Course Content'!D28="")*('Course Content'!I28=""),"—",IFERROR('Course Content'!D12*1,0)+IFERROR('Course Content'!I12*1,0)+IFERROR('Course Content'!D28*1,0)+IFERROR('Course Content'!I28*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="60">
+        <f>IFERROR(IF(K15="","",IF(K15="—","",FLOOR(K15/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="61">
+        <f>IFERROR(IF(L15="","",IF(L15="—","",FLOOR(L15/I15,1))),"")</f>
         <v/>
       </c>
       <c r="N15" s="26" t="n"/>
-      <c r="O15" s="61">
-        <f>IFERROR(IF('Course Content'!E28="","—",'Course Content'!E28),"")</f>
-        <v/>
-      </c>
-      <c r="P15" s="61">
-        <f>IFERROR(IF('Course Content'!E28="","",FLOOR('Course Content'!E28/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q15" s="62">
-        <f>IFERROR(IF(P15="","",FLOOR(P15/I15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R15" s="63">
-        <f>IFERROR(IF('Course Content'!C28="","",'Course Content'!C28),"")</f>
+      <c r="O15" s="62">
+        <f>IFERROR(IF(('Course Content'!E12="")*('Course Content'!J12="")*('Course Content'!E28="")*('Course Content'!J28=""),"—",IFERROR('Course Content'!E12*1,0)+IFERROR('Course Content'!J12*1,0)+IFERROR('Course Content'!E28*1,0)+IFERROR('Course Content'!J28*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="62">
+        <f>IFERROR(IF(O15="","",IF(O15="—","",FLOOR(O15/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="63">
+        <f>IFERROR(IF(P15="","",IF(P15="—","",FLOOR(P15/I15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="64">
+        <f>IFERROR(IF('Course Content'!C28&lt;&gt;"",'Course Content'!C28,IF('Course Content'!H28&lt;&gt;"",'Course Content'!H28,IF('Course Content'!C12&lt;&gt;"",'Course Content'!C12,'Course Content'!H12))),"")</f>
         <v/>
       </c>
     </row>
@@ -5885,48 +5891,48 @@
           <t>Science</t>
         </is>
       </c>
-      <c r="B16" s="18">
-        <f>IFERROR(IF('Course Content'!B29="","—",'Course Content'!B29),"")</f>
-        <v/>
-      </c>
-      <c r="C16" s="58" t="n"/>
-      <c r="D16" s="58" t="n"/>
-      <c r="E16" s="58" t="n"/>
-      <c r="F16" s="58" t="n"/>
-      <c r="G16" s="58" t="n"/>
-      <c r="H16" s="58" t="n"/>
+      <c r="B16" s="65">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,""),IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,""),IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,""),IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C16" s="59" t="n"/>
+      <c r="D16" s="59" t="n"/>
+      <c r="E16" s="59" t="n"/>
+      <c r="F16" s="59" t="n"/>
+      <c r="G16" s="59" t="n"/>
+      <c r="H16" s="59" t="n"/>
       <c r="I16" s="17">
         <f>IF(COUNTA(C16:H16)=0,$I$8,COUNTA(C16:H16))</f>
         <v/>
       </c>
       <c r="J16" s="26" t="n"/>
-      <c r="K16" s="59">
-        <f>IFERROR(IF('Course Content'!D29="","—",'Course Content'!D29),"")</f>
-        <v/>
-      </c>
-      <c r="L16" s="59">
-        <f>IFERROR(IF('Course Content'!D29="","",FLOOR('Course Content'!D29/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M16" s="60">
-        <f>IFERROR(IF(L16="","",FLOOR(L16/I16,1)),"")</f>
+      <c r="K16" s="60">
+        <f>IFERROR(IF(('Course Content'!D13="")*('Course Content'!I13="")*('Course Content'!D29="")*('Course Content'!I29=""),"—",IFERROR('Course Content'!D13*1,0)+IFERROR('Course Content'!I13*1,0)+IFERROR('Course Content'!D29*1,0)+IFERROR('Course Content'!I29*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="60">
+        <f>IFERROR(IF(K16="","",IF(K16="—","",FLOOR(K16/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="61">
+        <f>IFERROR(IF(L16="","",IF(L16="—","",FLOOR(L16/I16,1))),"")</f>
         <v/>
       </c>
       <c r="N16" s="26" t="n"/>
-      <c r="O16" s="61">
-        <f>IFERROR(IF('Course Content'!E29="","—",'Course Content'!E29),"")</f>
-        <v/>
-      </c>
-      <c r="P16" s="61">
-        <f>IFERROR(IF('Course Content'!E29="","",FLOOR('Course Content'!E29/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q16" s="62">
-        <f>IFERROR(IF(P16="","",FLOOR(P16/I16,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R16" s="64">
-        <f>IFERROR(IF('Course Content'!C29="","",'Course Content'!C29),"")</f>
+      <c r="O16" s="62">
+        <f>IFERROR(IF(('Course Content'!E13="")*('Course Content'!J13="")*('Course Content'!E29="")*('Course Content'!J29=""),"—",IFERROR('Course Content'!E13*1,0)+IFERROR('Course Content'!J13*1,0)+IFERROR('Course Content'!E29*1,0)+IFERROR('Course Content'!J29*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="62">
+        <f>IFERROR(IF(O16="","",IF(O16="—","",FLOOR(O16/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q16" s="63">
+        <f>IFERROR(IF(P16="","",IF(P16="—","",FLOOR(P16/I16,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R16" s="66">
+        <f>IFERROR(IF('Course Content'!C29&lt;&gt;"",'Course Content'!C29,IF('Course Content'!H29&lt;&gt;"",'Course Content'!H29,IF('Course Content'!C13&lt;&gt;"",'Course Content'!C13,'Course Content'!H13))),"")</f>
         <v/>
       </c>
     </row>
@@ -5936,48 +5942,48 @@
           <t>Social Studies / History</t>
         </is>
       </c>
-      <c r="B17" s="5">
-        <f>IFERROR(IF('Course Content'!B30="","—",'Course Content'!B30),"")</f>
-        <v/>
-      </c>
-      <c r="C17" s="58" t="n"/>
-      <c r="D17" s="58" t="n"/>
-      <c r="E17" s="58" t="n"/>
-      <c r="F17" s="58" t="n"/>
-      <c r="G17" s="58" t="n"/>
-      <c r="H17" s="58" t="n"/>
+      <c r="B17" s="58">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,""),IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,""),IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,""),IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C17" s="59" t="n"/>
+      <c r="D17" s="59" t="n"/>
+      <c r="E17" s="59" t="n"/>
+      <c r="F17" s="59" t="n"/>
+      <c r="G17" s="59" t="n"/>
+      <c r="H17" s="59" t="n"/>
       <c r="I17" s="17">
         <f>IF(COUNTA(C17:H17)=0,$I$8,COUNTA(C17:H17))</f>
         <v/>
       </c>
       <c r="J17" s="26" t="n"/>
-      <c r="K17" s="59">
-        <f>IFERROR(IF('Course Content'!D30="","—",'Course Content'!D30),"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="59">
-        <f>IFERROR(IF('Course Content'!D30="","",FLOOR('Course Content'!D30/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M17" s="60">
-        <f>IFERROR(IF(L17="","",FLOOR(L17/I17,1)),"")</f>
+      <c r="K17" s="60">
+        <f>IFERROR(IF(('Course Content'!D14="")*('Course Content'!I14="")*('Course Content'!D30="")*('Course Content'!I30=""),"—",IFERROR('Course Content'!D14*1,0)+IFERROR('Course Content'!I14*1,0)+IFERROR('Course Content'!D30*1,0)+IFERROR('Course Content'!I30*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="60">
+        <f>IFERROR(IF(K17="","",IF(K17="—","",FLOOR(K17/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="61">
+        <f>IFERROR(IF(L17="","",IF(L17="—","",FLOOR(L17/I17,1))),"")</f>
         <v/>
       </c>
       <c r="N17" s="26" t="n"/>
-      <c r="O17" s="61">
-        <f>IFERROR(IF('Course Content'!E30="","—",'Course Content'!E30),"")</f>
-        <v/>
-      </c>
-      <c r="P17" s="61">
-        <f>IFERROR(IF('Course Content'!E30="","",FLOOR('Course Content'!E30/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q17" s="62">
-        <f>IFERROR(IF(P17="","",FLOOR(P17/I17,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R17" s="63">
-        <f>IFERROR(IF('Course Content'!C30="","",'Course Content'!C30),"")</f>
+      <c r="O17" s="62">
+        <f>IFERROR(IF(('Course Content'!E14="")*('Course Content'!J14="")*('Course Content'!E30="")*('Course Content'!J30=""),"—",IFERROR('Course Content'!E14*1,0)+IFERROR('Course Content'!J14*1,0)+IFERROR('Course Content'!E30*1,0)+IFERROR('Course Content'!J30*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="62">
+        <f>IFERROR(IF(O17="","",IF(O17="—","",FLOOR(O17/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="63">
+        <f>IFERROR(IF(P17="","",IF(P17="—","",FLOOR(P17/I17,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R17" s="64">
+        <f>IFERROR(IF('Course Content'!C30&lt;&gt;"",'Course Content'!C30,IF('Course Content'!H30&lt;&gt;"",'Course Content'!H30,IF('Course Content'!C14&lt;&gt;"",'Course Content'!C14,'Course Content'!H14))),"")</f>
         <v/>
       </c>
     </row>
@@ -5987,48 +5993,48 @@
           <t>Health</t>
         </is>
       </c>
-      <c r="B18" s="18">
-        <f>IFERROR(IF('Course Content'!B31="","—",'Course Content'!B31),"")</f>
-        <v/>
-      </c>
-      <c r="C18" s="58" t="n"/>
-      <c r="D18" s="58" t="n"/>
-      <c r="E18" s="58" t="n"/>
-      <c r="F18" s="58" t="n"/>
-      <c r="G18" s="58" t="n"/>
-      <c r="H18" s="58" t="n"/>
+      <c r="B18" s="65">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,""),IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,""),IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,""),IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C18" s="59" t="n"/>
+      <c r="D18" s="59" t="n"/>
+      <c r="E18" s="59" t="n"/>
+      <c r="F18" s="59" t="n"/>
+      <c r="G18" s="59" t="n"/>
+      <c r="H18" s="59" t="n"/>
       <c r="I18" s="17">
         <f>IF(COUNTA(C18:H18)=0,$I$8,COUNTA(C18:H18))</f>
         <v/>
       </c>
       <c r="J18" s="26" t="n"/>
-      <c r="K18" s="59">
-        <f>IFERROR(IF('Course Content'!D31="","—",'Course Content'!D31),"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="59">
-        <f>IFERROR(IF('Course Content'!D31="","",FLOOR('Course Content'!D31/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M18" s="60">
-        <f>IFERROR(IF(L18="","",FLOOR(L18/I18,1)),"")</f>
+      <c r="K18" s="60">
+        <f>IFERROR(IF(('Course Content'!D15="")*('Course Content'!I15="")*('Course Content'!D31="")*('Course Content'!I31=""),"—",IFERROR('Course Content'!D15*1,0)+IFERROR('Course Content'!I15*1,0)+IFERROR('Course Content'!D31*1,0)+IFERROR('Course Content'!I31*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="60">
+        <f>IFERROR(IF(K18="","",IF(K18="—","",FLOOR(K18/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="61">
+        <f>IFERROR(IF(L18="","",IF(L18="—","",FLOOR(L18/I18,1))),"")</f>
         <v/>
       </c>
       <c r="N18" s="26" t="n"/>
-      <c r="O18" s="61">
-        <f>IFERROR(IF('Course Content'!E31="","—",'Course Content'!E31),"")</f>
-        <v/>
-      </c>
-      <c r="P18" s="61">
-        <f>IFERROR(IF('Course Content'!E31="","",FLOOR('Course Content'!E31/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q18" s="62">
-        <f>IFERROR(IF(P18="","",FLOOR(P18/I18,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R18" s="64">
-        <f>IFERROR(IF('Course Content'!C31="","",'Course Content'!C31),"")</f>
+      <c r="O18" s="62">
+        <f>IFERROR(IF(('Course Content'!E15="")*('Course Content'!J15="")*('Course Content'!E31="")*('Course Content'!J31=""),"—",IFERROR('Course Content'!E15*1,0)+IFERROR('Course Content'!J15*1,0)+IFERROR('Course Content'!E31*1,0)+IFERROR('Course Content'!J31*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="62">
+        <f>IFERROR(IF(O18="","",IF(O18="—","",FLOOR(O18/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q18" s="63">
+        <f>IFERROR(IF(P18="","",IF(P18="—","",FLOOR(P18/I18,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R18" s="66">
+        <f>IFERROR(IF('Course Content'!C31&lt;&gt;"",'Course Content'!C31,IF('Course Content'!H31&lt;&gt;"",'Course Content'!H31,IF('Course Content'!C15&lt;&gt;"",'Course Content'!C15,'Course Content'!H15))),"")</f>
         <v/>
       </c>
     </row>
@@ -6038,48 +6044,48 @@
           <t>Physical Education</t>
         </is>
       </c>
-      <c r="B19" s="5">
-        <f>IFERROR(IF('Course Content'!B32="","—",'Course Content'!B32),"")</f>
-        <v/>
-      </c>
-      <c r="C19" s="58" t="n"/>
-      <c r="D19" s="58" t="n"/>
-      <c r="E19" s="58" t="n"/>
-      <c r="F19" s="58" t="n"/>
-      <c r="G19" s="58" t="n"/>
-      <c r="H19" s="58" t="n"/>
+      <c r="B19" s="58">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,""),IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,""),IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,""),IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C19" s="59" t="n"/>
+      <c r="D19" s="59" t="n"/>
+      <c r="E19" s="59" t="n"/>
+      <c r="F19" s="59" t="n"/>
+      <c r="G19" s="59" t="n"/>
+      <c r="H19" s="59" t="n"/>
       <c r="I19" s="17">
         <f>IF(COUNTA(C19:H19)=0,$I$8,COUNTA(C19:H19))</f>
         <v/>
       </c>
       <c r="J19" s="26" t="n"/>
-      <c r="K19" s="59">
-        <f>IFERROR(IF('Course Content'!D32="","—",'Course Content'!D32),"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="59">
-        <f>IFERROR(IF('Course Content'!D32="","",FLOOR('Course Content'!D32/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M19" s="60">
-        <f>IFERROR(IF(L19="","",FLOOR(L19/I19,1)),"")</f>
+      <c r="K19" s="60">
+        <f>IFERROR(IF(('Course Content'!D16="")*('Course Content'!I16="")*('Course Content'!D32="")*('Course Content'!I32=""),"—",IFERROR('Course Content'!D16*1,0)+IFERROR('Course Content'!I16*1,0)+IFERROR('Course Content'!D32*1,0)+IFERROR('Course Content'!I32*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="60">
+        <f>IFERROR(IF(K19="","",IF(K19="—","",FLOOR(K19/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="61">
+        <f>IFERROR(IF(L19="","",IF(L19="—","",FLOOR(L19/I19,1))),"")</f>
         <v/>
       </c>
       <c r="N19" s="26" t="n"/>
-      <c r="O19" s="61">
-        <f>IFERROR(IF('Course Content'!E32="","—",'Course Content'!E32),"")</f>
-        <v/>
-      </c>
-      <c r="P19" s="61">
-        <f>IFERROR(IF('Course Content'!E32="","",FLOOR('Course Content'!E32/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q19" s="62">
-        <f>IFERROR(IF(P19="","",FLOOR(P19/I19,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R19" s="63">
-        <f>IFERROR(IF('Course Content'!C32="","",'Course Content'!C32),"")</f>
+      <c r="O19" s="62">
+        <f>IFERROR(IF(('Course Content'!E16="")*('Course Content'!J16="")*('Course Content'!E32="")*('Course Content'!J32=""),"—",IFERROR('Course Content'!E16*1,0)+IFERROR('Course Content'!J16*1,0)+IFERROR('Course Content'!E32*1,0)+IFERROR('Course Content'!J32*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="62">
+        <f>IFERROR(IF(O19="","",IF(O19="—","",FLOOR(O19/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q19" s="63">
+        <f>IFERROR(IF(P19="","",IF(P19="—","",FLOOR(P19/I19,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R19" s="64">
+        <f>IFERROR(IF('Course Content'!C32&lt;&gt;"",'Course Content'!C32,IF('Course Content'!H32&lt;&gt;"",'Course Content'!H32,IF('Course Content'!C16&lt;&gt;"",'Course Content'!C16,'Course Content'!H16))),"")</f>
         <v/>
       </c>
     </row>
@@ -6089,48 +6095,48 @@
           <t>Art / Music</t>
         </is>
       </c>
-      <c r="B20" s="18">
-        <f>IFERROR(IF('Course Content'!B33="","—",'Course Content'!B33),"")</f>
-        <v/>
-      </c>
-      <c r="C20" s="58" t="n"/>
-      <c r="D20" s="58" t="n"/>
-      <c r="E20" s="58" t="n"/>
-      <c r="F20" s="58" t="n"/>
-      <c r="G20" s="58" t="n"/>
-      <c r="H20" s="58" t="n"/>
+      <c r="B20" s="65">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,""),IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,""),IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,""),IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C20" s="59" t="n"/>
+      <c r="D20" s="59" t="n"/>
+      <c r="E20" s="59" t="n"/>
+      <c r="F20" s="59" t="n"/>
+      <c r="G20" s="59" t="n"/>
+      <c r="H20" s="59" t="n"/>
       <c r="I20" s="17">
         <f>IF(COUNTA(C20:H20)=0,$I$8,COUNTA(C20:H20))</f>
         <v/>
       </c>
       <c r="J20" s="26" t="n"/>
-      <c r="K20" s="59">
-        <f>IFERROR(IF('Course Content'!D33="","—",'Course Content'!D33),"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="59">
-        <f>IFERROR(IF('Course Content'!D33="","",FLOOR('Course Content'!D33/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="60">
-        <f>IFERROR(IF(L20="","",FLOOR(L20/I20,1)),"")</f>
+      <c r="K20" s="60">
+        <f>IFERROR(IF(('Course Content'!D17="")*('Course Content'!I17="")*('Course Content'!D33="")*('Course Content'!I33=""),"—",IFERROR('Course Content'!D17*1,0)+IFERROR('Course Content'!I17*1,0)+IFERROR('Course Content'!D33*1,0)+IFERROR('Course Content'!I33*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="60">
+        <f>IFERROR(IF(K20="","",IF(K20="—","",FLOOR(K20/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M20" s="61">
+        <f>IFERROR(IF(L20="","",IF(L20="—","",FLOOR(L20/I20,1))),"")</f>
         <v/>
       </c>
       <c r="N20" s="26" t="n"/>
-      <c r="O20" s="61">
-        <f>IFERROR(IF('Course Content'!E33="","—",'Course Content'!E33),"")</f>
-        <v/>
-      </c>
-      <c r="P20" s="61">
-        <f>IFERROR(IF('Course Content'!E33="","",FLOOR('Course Content'!E33/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q20" s="62">
-        <f>IFERROR(IF(P20="","",FLOOR(P20/I20,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R20" s="64">
-        <f>IFERROR(IF('Course Content'!C33="","",'Course Content'!C33),"")</f>
+      <c r="O20" s="62">
+        <f>IFERROR(IF(('Course Content'!E17="")*('Course Content'!J17="")*('Course Content'!E33="")*('Course Content'!J33=""),"—",IFERROR('Course Content'!E17*1,0)+IFERROR('Course Content'!J17*1,0)+IFERROR('Course Content'!E33*1,0)+IFERROR('Course Content'!J33*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P20" s="62">
+        <f>IFERROR(IF(O20="","",IF(O20="—","",FLOOR(O20/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q20" s="63">
+        <f>IFERROR(IF(P20="","",IF(P20="—","",FLOOR(P20/I20,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R20" s="66">
+        <f>IFERROR(IF('Course Content'!C33&lt;&gt;"",'Course Content'!C33,IF('Course Content'!H33&lt;&gt;"",'Course Content'!H33,IF('Course Content'!C17&lt;&gt;"",'Course Content'!C17,'Course Content'!H17))),"")</f>
         <v/>
       </c>
     </row>
@@ -6139,48 +6145,48 @@
         <f>IF('Course Content'!A34="Elective / Other 1","Elective / Other 1",'Course Content'!A34)</f>
         <v/>
       </c>
-      <c r="B21" s="5">
-        <f>IFERROR(IF('Course Content'!B34="","—",'Course Content'!B34),"")</f>
-        <v/>
-      </c>
-      <c r="C21" s="58" t="n"/>
-      <c r="D21" s="58" t="n"/>
-      <c r="E21" s="58" t="n"/>
-      <c r="F21" s="58" t="n"/>
-      <c r="G21" s="58" t="n"/>
-      <c r="H21" s="58" t="n"/>
+      <c r="B21" s="58">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,""),IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,""),IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,""),IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C21" s="59" t="n"/>
+      <c r="D21" s="59" t="n"/>
+      <c r="E21" s="59" t="n"/>
+      <c r="F21" s="59" t="n"/>
+      <c r="G21" s="59" t="n"/>
+      <c r="H21" s="59" t="n"/>
       <c r="I21" s="17">
         <f>IF(COUNTA(C21:H21)=0,$I$8,COUNTA(C21:H21))</f>
         <v/>
       </c>
       <c r="J21" s="26" t="n"/>
-      <c r="K21" s="59">
-        <f>IFERROR(IF('Course Content'!D34="","—",'Course Content'!D34),"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="59">
-        <f>IFERROR(IF('Course Content'!D34="","",FLOOR('Course Content'!D34/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M21" s="60">
-        <f>IFERROR(IF(L21="","",FLOOR(L21/I21,1)),"")</f>
+      <c r="K21" s="60">
+        <f>IFERROR(IF(('Course Content'!D18="")*('Course Content'!I18="")*('Course Content'!D34="")*('Course Content'!I34=""),"—",IFERROR('Course Content'!D18*1,0)+IFERROR('Course Content'!I18*1,0)+IFERROR('Course Content'!D34*1,0)+IFERROR('Course Content'!I34*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="60">
+        <f>IFERROR(IF(K21="","",IF(K21="—","",FLOOR(K21/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M21" s="61">
+        <f>IFERROR(IF(L21="","",IF(L21="—","",FLOOR(L21/I21,1))),"")</f>
         <v/>
       </c>
       <c r="N21" s="26" t="n"/>
-      <c r="O21" s="61">
-        <f>IFERROR(IF('Course Content'!E34="","—",'Course Content'!E34),"")</f>
-        <v/>
-      </c>
-      <c r="P21" s="61">
-        <f>IFERROR(IF('Course Content'!E34="","",FLOOR('Course Content'!E34/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q21" s="62">
-        <f>IFERROR(IF(P21="","",FLOOR(P21/I21,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R21" s="63">
-        <f>IFERROR(IF('Course Content'!C34="","",'Course Content'!C34),"")</f>
+      <c r="O21" s="62">
+        <f>IFERROR(IF(('Course Content'!E18="")*('Course Content'!J18="")*('Course Content'!E34="")*('Course Content'!J34=""),"—",IFERROR('Course Content'!E18*1,0)+IFERROR('Course Content'!J18*1,0)+IFERROR('Course Content'!E34*1,0)+IFERROR('Course Content'!J34*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P21" s="62">
+        <f>IFERROR(IF(O21="","",IF(O21="—","",FLOOR(O21/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q21" s="63">
+        <f>IFERROR(IF(P21="","",IF(P21="—","",FLOOR(P21/I21,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R21" s="64">
+        <f>IFERROR(IF('Course Content'!C34&lt;&gt;"",'Course Content'!C34,IF('Course Content'!H34&lt;&gt;"",'Course Content'!H34,IF('Course Content'!C18&lt;&gt;"",'Course Content'!C18,'Course Content'!H18))),"")</f>
         <v/>
       </c>
     </row>
@@ -6189,48 +6195,48 @@
         <f>IF('Course Content'!A35="Elective / Other 2","Elective / Other 2",'Course Content'!A35)</f>
         <v/>
       </c>
-      <c r="B22" s="18">
-        <f>IFERROR(IF('Course Content'!B35="","—",'Course Content'!B35),"")</f>
-        <v/>
-      </c>
-      <c r="C22" s="58" t="n"/>
-      <c r="D22" s="58" t="n"/>
-      <c r="E22" s="58" t="n"/>
-      <c r="F22" s="58" t="n"/>
-      <c r="G22" s="58" t="n"/>
-      <c r="H22" s="58" t="n"/>
+      <c r="B22" s="65">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,""),IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,""),IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,""),IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C22" s="59" t="n"/>
+      <c r="D22" s="59" t="n"/>
+      <c r="E22" s="59" t="n"/>
+      <c r="F22" s="59" t="n"/>
+      <c r="G22" s="59" t="n"/>
+      <c r="H22" s="59" t="n"/>
       <c r="I22" s="17">
         <f>IF(COUNTA(C22:H22)=0,$I$8,COUNTA(C22:H22))</f>
         <v/>
       </c>
       <c r="J22" s="26" t="n"/>
-      <c r="K22" s="59">
-        <f>IFERROR(IF('Course Content'!D35="","—",'Course Content'!D35),"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="59">
-        <f>IFERROR(IF('Course Content'!D35="","",FLOOR('Course Content'!D35/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M22" s="60">
-        <f>IFERROR(IF(L22="","",FLOOR(L22/I22,1)),"")</f>
+      <c r="K22" s="60">
+        <f>IFERROR(IF(('Course Content'!D19="")*('Course Content'!I19="")*('Course Content'!D35="")*('Course Content'!I35=""),"—",IFERROR('Course Content'!D19*1,0)+IFERROR('Course Content'!I19*1,0)+IFERROR('Course Content'!D35*1,0)+IFERROR('Course Content'!I35*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="60">
+        <f>IFERROR(IF(K22="","",IF(K22="—","",FLOOR(K22/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M22" s="61">
+        <f>IFERROR(IF(L22="","",IF(L22="—","",FLOOR(L22/I22,1))),"")</f>
         <v/>
       </c>
       <c r="N22" s="26" t="n"/>
-      <c r="O22" s="61">
-        <f>IFERROR(IF('Course Content'!E35="","—",'Course Content'!E35),"")</f>
-        <v/>
-      </c>
-      <c r="P22" s="61">
-        <f>IFERROR(IF('Course Content'!E35="","",FLOOR('Course Content'!E35/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q22" s="62">
-        <f>IFERROR(IF(P22="","",FLOOR(P22/I22,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R22" s="64">
-        <f>IFERROR(IF('Course Content'!C35="","",'Course Content'!C35),"")</f>
+      <c r="O22" s="62">
+        <f>IFERROR(IF(('Course Content'!E19="")*('Course Content'!J19="")*('Course Content'!E35="")*('Course Content'!J35=""),"—",IFERROR('Course Content'!E19*1,0)+IFERROR('Course Content'!J19*1,0)+IFERROR('Course Content'!E35*1,0)+IFERROR('Course Content'!J35*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="62">
+        <f>IFERROR(IF(O22="","",IF(O22="—","",FLOOR(O22/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q22" s="63">
+        <f>IFERROR(IF(P22="","",IF(P22="—","",FLOOR(P22/I22,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R22" s="66">
+        <f>IFERROR(IF('Course Content'!C35&lt;&gt;"",'Course Content'!C35,IF('Course Content'!H35&lt;&gt;"",'Course Content'!H35,IF('Course Content'!C19&lt;&gt;"",'Course Content'!C19,'Course Content'!H19))),"")</f>
         <v/>
       </c>
     </row>
@@ -6239,48 +6245,48 @@
         <f>IF('Course Content'!A36="Elective / Other 3","Elective / Other 3",'Course Content'!A36)</f>
         <v/>
       </c>
-      <c r="B23" s="5">
-        <f>IFERROR(IF('Course Content'!B36="","—",'Course Content'!B36),"")</f>
-        <v/>
-      </c>
-      <c r="C23" s="58" t="n"/>
-      <c r="D23" s="58" t="n"/>
-      <c r="E23" s="58" t="n"/>
-      <c r="F23" s="58" t="n"/>
-      <c r="G23" s="58" t="n"/>
-      <c r="H23" s="58" t="n"/>
+      <c r="B23" s="58">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,""),IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,""),IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,""),IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C23" s="59" t="n"/>
+      <c r="D23" s="59" t="n"/>
+      <c r="E23" s="59" t="n"/>
+      <c r="F23" s="59" t="n"/>
+      <c r="G23" s="59" t="n"/>
+      <c r="H23" s="59" t="n"/>
       <c r="I23" s="17">
         <f>IF(COUNTA(C23:H23)=0,$I$8,COUNTA(C23:H23))</f>
         <v/>
       </c>
       <c r="J23" s="26" t="n"/>
-      <c r="K23" s="59">
-        <f>IFERROR(IF('Course Content'!D36="","—",'Course Content'!D36),"")</f>
-        <v/>
-      </c>
-      <c r="L23" s="59">
-        <f>IFERROR(IF('Course Content'!D36="","",FLOOR('Course Content'!D36/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M23" s="60">
-        <f>IFERROR(IF(L23="","",FLOOR(L23/I23,1)),"")</f>
+      <c r="K23" s="60">
+        <f>IFERROR(IF(('Course Content'!D20="")*('Course Content'!I20="")*('Course Content'!D36="")*('Course Content'!I36=""),"—",IFERROR('Course Content'!D20*1,0)+IFERROR('Course Content'!I20*1,0)+IFERROR('Course Content'!D36*1,0)+IFERROR('Course Content'!I36*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="60">
+        <f>IFERROR(IF(K23="","",IF(K23="—","",FLOOR(K23/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="61">
+        <f>IFERROR(IF(L23="","",IF(L23="—","",FLOOR(L23/I23,1))),"")</f>
         <v/>
       </c>
       <c r="N23" s="26" t="n"/>
-      <c r="O23" s="61">
-        <f>IFERROR(IF('Course Content'!E36="","—",'Course Content'!E36),"")</f>
-        <v/>
-      </c>
-      <c r="P23" s="61">
-        <f>IFERROR(IF('Course Content'!E36="","",FLOOR('Course Content'!E36/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q23" s="62">
-        <f>IFERROR(IF(P23="","",FLOOR(P23/I23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R23" s="63">
-        <f>IFERROR(IF('Course Content'!C36="","",'Course Content'!C36),"")</f>
+      <c r="O23" s="62">
+        <f>IFERROR(IF(('Course Content'!E20="")*('Course Content'!J20="")*('Course Content'!E36="")*('Course Content'!J36=""),"—",IFERROR('Course Content'!E20*1,0)+IFERROR('Course Content'!J20*1,0)+IFERROR('Course Content'!E36*1,0)+IFERROR('Course Content'!J36*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P23" s="62">
+        <f>IFERROR(IF(O23="","",IF(O23="—","",FLOOR(O23/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q23" s="63">
+        <f>IFERROR(IF(P23="","",IF(P23="—","",FLOOR(P23/I23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R23" s="64">
+        <f>IFERROR(IF('Course Content'!C36&lt;&gt;"",'Course Content'!C36,IF('Course Content'!H36&lt;&gt;"",'Course Content'!H36,IF('Course Content'!C20&lt;&gt;"",'Course Content'!C20,'Course Content'!H20))),"")</f>
         <v/>
       </c>
     </row>
@@ -6289,48 +6295,48 @@
         <f>IF('Course Content'!A37="Elective / Other 4","Elective / Other 4",'Course Content'!A37)</f>
         <v/>
       </c>
-      <c r="B24" s="18">
-        <f>IFERROR(IF('Course Content'!B37="","—",'Course Content'!B37),"")</f>
-        <v/>
-      </c>
-      <c r="C24" s="58" t="n"/>
-      <c r="D24" s="58" t="n"/>
-      <c r="E24" s="58" t="n"/>
-      <c r="F24" s="58" t="n"/>
-      <c r="G24" s="58" t="n"/>
-      <c r="H24" s="58" t="n"/>
+      <c r="B24" s="65">
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,""),IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,""),IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,""),IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,"")),"—")</f>
+        <v/>
+      </c>
+      <c r="C24" s="59" t="n"/>
+      <c r="D24" s="59" t="n"/>
+      <c r="E24" s="59" t="n"/>
+      <c r="F24" s="59" t="n"/>
+      <c r="G24" s="59" t="n"/>
+      <c r="H24" s="59" t="n"/>
       <c r="I24" s="17">
         <f>IF(COUNTA(C24:H24)=0,$I$8,COUNTA(C24:H24))</f>
         <v/>
       </c>
       <c r="J24" s="26" t="n"/>
-      <c r="K24" s="59">
-        <f>IFERROR(IF('Course Content'!D37="","—",'Course Content'!D37),"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="59">
-        <f>IFERROR(IF('Course Content'!D37="","",FLOOR('Course Content'!D37/'Getting Started'!C15,1)),"")</f>
-        <v/>
-      </c>
-      <c r="M24" s="60">
-        <f>IFERROR(IF(L24="","",FLOOR(L24/I24,1)),"")</f>
+      <c r="K24" s="60">
+        <f>IFERROR(IF(('Course Content'!D21="")*('Course Content'!I21="")*('Course Content'!D37="")*('Course Content'!I37=""),"—",IFERROR('Course Content'!D21*1,0)+IFERROR('Course Content'!I21*1,0)+IFERROR('Course Content'!D37*1,0)+IFERROR('Course Content'!I37*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="60">
+        <f>IFERROR(IF(K24="","",IF(K24="—","",FLOOR(K24/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M24" s="61">
+        <f>IFERROR(IF(L24="","",IF(L24="—","",FLOOR(L24/I24,1))),"")</f>
         <v/>
       </c>
       <c r="N24" s="26" t="n"/>
-      <c r="O24" s="61">
-        <f>IFERROR(IF('Course Content'!E37="","—",'Course Content'!E37),"")</f>
-        <v/>
-      </c>
-      <c r="P24" s="61">
-        <f>IFERROR(IF('Course Content'!E37="","",FLOOR('Course Content'!E37/'Getting Started'!C23,1)),"")</f>
-        <v/>
-      </c>
-      <c r="Q24" s="62">
-        <f>IFERROR(IF(P24="","",FLOOR(P24/I24,1)),"")</f>
-        <v/>
-      </c>
-      <c r="R24" s="64">
-        <f>IFERROR(IF('Course Content'!C37="","",'Course Content'!C37),"")</f>
+      <c r="O24" s="62">
+        <f>IFERROR(IF(('Course Content'!E21="")*('Course Content'!J21="")*('Course Content'!E37="")*('Course Content'!J37=""),"—",IFERROR('Course Content'!E21*1,0)+IFERROR('Course Content'!J21*1,0)+IFERROR('Course Content'!E37*1,0)+IFERROR('Course Content'!J37*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P24" s="62">
+        <f>IFERROR(IF(O24="","",IF(O24="—","",FLOOR(O24/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q24" s="63">
+        <f>IFERROR(IF(P24="","",IF(P24="—","",FLOOR(P24/I24,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R24" s="66">
+        <f>IFERROR(IF('Course Content'!C37&lt;&gt;"",'Course Content'!C37,IF('Course Content'!H37&lt;&gt;"",'Course Content'!H37,IF('Course Content'!C21&lt;&gt;"",'Course Content'!C21,'Course Content'!H21))),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Split student schedule into 4 sub-rows per subject
Each subject now has four rows: Group Slot 1, Group Slot 2, Individual
Slot 1, Individual Slot 2. Subject name is merged across all four.
Group rows use a faint rose tint and italic text to distinguish them.
A medium bottom border separates each subject group visually.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -311,7 +311,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -361,11 +361,25 @@
         <color rgb="00CE8282"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D4C4BB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D4C4BB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D4C4BB"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00A08878"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -534,8 +548,8 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -552,13 +566,34 @@
     <xf numFmtId="0" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5407,7 +5442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5630,14 +5665,14 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Bible</t>
         </is>
       </c>
       <c r="B11" s="58">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,""),IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,""),IF('Course Content'!B24&lt;&gt;"",'Course Content'!B24,""),IF('Course Content'!G24&lt;&gt;"",'Course Content'!G24,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!B8="","",'Course Content'!B8),"")</f>
         <v/>
       </c>
       <c r="C11" s="59" t="n"/>
@@ -5652,7 +5687,7 @@
       </c>
       <c r="J11" s="26" t="n"/>
       <c r="K11" s="60">
-        <f>IFERROR(IF(('Course Content'!D8="")*('Course Content'!I8="")*('Course Content'!D24="")*('Course Content'!I24=""),"—",IFERROR('Course Content'!D8*1,0)+IFERROR('Course Content'!I8*1,0)+IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!D8="","—",'Course Content'!D8),"")</f>
         <v/>
       </c>
       <c r="L11" s="60">
@@ -5665,7 +5700,7 @@
       </c>
       <c r="N11" s="26" t="n"/>
       <c r="O11" s="62">
-        <f>IFERROR(IF(('Course Content'!E8="")*('Course Content'!J8="")*('Course Content'!E24="")*('Course Content'!J24=""),"—",IFERROR('Course Content'!E8*1,0)+IFERROR('Course Content'!J8*1,0)+IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!E8="","—",'Course Content'!E8),"")</f>
         <v/>
       </c>
       <c r="P11" s="62">
@@ -5677,18 +5712,13 @@
         <v/>
       </c>
       <c r="R11" s="64">
-        <f>IFERROR(IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,IF('Course Content'!H24&lt;&gt;"",'Course Content'!H24,IF('Course Content'!C8&lt;&gt;"",'Course Content'!C8,'Course Content'!H8))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
-        </is>
-      </c>
-      <c r="B12" s="65">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,""),IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,""),IF('Course Content'!B25&lt;&gt;"",'Course Content'!B25,""),IF('Course Content'!G25&lt;&gt;"",'Course Content'!G25,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!C8="","",'Course Content'!C8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="58">
+        <f>IFERROR(IF('Course Content'!G8="","",'Course Content'!G8),"")</f>
         <v/>
       </c>
       <c r="C12" s="59" t="n"/>
@@ -5703,7 +5733,7 @@
       </c>
       <c r="J12" s="26" t="n"/>
       <c r="K12" s="60">
-        <f>IFERROR(IF(('Course Content'!D9="")*('Course Content'!I9="")*('Course Content'!D25="")*('Course Content'!I25=""),"—",IFERROR('Course Content'!D9*1,0)+IFERROR('Course Content'!I9*1,0)+IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!I8="","—",'Course Content'!I8),"")</f>
         <v/>
       </c>
       <c r="L12" s="60">
@@ -5716,7 +5746,7 @@
       </c>
       <c r="N12" s="26" t="n"/>
       <c r="O12" s="62">
-        <f>IFERROR(IF(('Course Content'!E9="")*('Course Content'!J9="")*('Course Content'!E25="")*('Course Content'!J25=""),"—",IFERROR('Course Content'!E9*1,0)+IFERROR('Course Content'!J9*1,0)+IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!J8="","—",'Course Content'!J8),"")</f>
         <v/>
       </c>
       <c r="P12" s="62">
@@ -5727,19 +5757,14 @@
         <f>IFERROR(IF(P12="","",IF(P12="—","",FLOOR(P12/I12,1))),"")</f>
         <v/>
       </c>
-      <c r="R12" s="66">
-        <f>IFERROR(IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,IF('Course Content'!H25&lt;&gt;"",'Course Content'!H25,IF('Course Content'!C9&lt;&gt;"",'Course Content'!C9,'Course Content'!H9))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B13" s="58">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,""),IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,""),IF('Course Content'!B26&lt;&gt;"",'Course Content'!B26,""),IF('Course Content'!G26&lt;&gt;"",'Course Content'!G26,"")),"—")</f>
+      <c r="R12" s="64">
+        <f>IFERROR(IF('Course Content'!H8="","",'Course Content'!H8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="B13" s="5">
+        <f>IFERROR(IF('Course Content'!B24="","",'Course Content'!B24),"")</f>
         <v/>
       </c>
       <c r="C13" s="59" t="n"/>
@@ -5754,7 +5779,7 @@
       </c>
       <c r="J13" s="26" t="n"/>
       <c r="K13" s="60">
-        <f>IFERROR(IF(('Course Content'!D10="")*('Course Content'!I10="")*('Course Content'!D26="")*('Course Content'!I26=""),"—",IFERROR('Course Content'!D10*1,0)+IFERROR('Course Content'!I10*1,0)+IFERROR('Course Content'!D26*1,0)+IFERROR('Course Content'!I26*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!D24="","—",'Course Content'!D24),"")</f>
         <v/>
       </c>
       <c r="L13" s="60">
@@ -5767,7 +5792,7 @@
       </c>
       <c r="N13" s="26" t="n"/>
       <c r="O13" s="62">
-        <f>IFERROR(IF(('Course Content'!E10="")*('Course Content'!J10="")*('Course Content'!E26="")*('Course Content'!J26=""),"—",IFERROR('Course Content'!E10*1,0)+IFERROR('Course Content'!J10*1,0)+IFERROR('Course Content'!E26*1,0)+IFERROR('Course Content'!J26*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!E24="","—",'Course Content'!E24),"")</f>
         <v/>
       </c>
       <c r="P13" s="62">
@@ -5778,70 +5803,65 @@
         <f>IFERROR(IF(P13="","",IF(P13="—","",FLOOR(P13/I13,1))),"")</f>
         <v/>
       </c>
-      <c r="R13" s="64">
-        <f>IFERROR(IF('Course Content'!C26&lt;&gt;"",'Course Content'!C26,IF('Course Content'!H26&lt;&gt;"",'Course Content'!H26,IF('Course Content'!C10&lt;&gt;"",'Course Content'!C10,'Course Content'!H10))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B14" s="65">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,""),IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,""),IF('Course Content'!B27&lt;&gt;"",'Course Content'!B27,""),IF('Course Content'!G27&lt;&gt;"",'Course Content'!G27,"")),"—")</f>
-        <v/>
-      </c>
-      <c r="C14" s="59" t="n"/>
-      <c r="D14" s="59" t="n"/>
-      <c r="E14" s="59" t="n"/>
-      <c r="F14" s="59" t="n"/>
-      <c r="G14" s="59" t="n"/>
-      <c r="H14" s="59" t="n"/>
-      <c r="I14" s="17">
+      <c r="R13" s="65">
+        <f>IFERROR(IF('Course Content'!C24="","",'Course Content'!C24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="B14" s="66">
+        <f>IFERROR(IF('Course Content'!G24="","",'Course Content'!G24),"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="67" t="n"/>
+      <c r="D14" s="67" t="n"/>
+      <c r="E14" s="67" t="n"/>
+      <c r="F14" s="67" t="n"/>
+      <c r="G14" s="67" t="n"/>
+      <c r="H14" s="67" t="n"/>
+      <c r="I14" s="68">
         <f>IF(COUNTA(C14:H14)=0,$I$8,COUNTA(C14:H14))</f>
         <v/>
       </c>
       <c r="J14" s="26" t="n"/>
-      <c r="K14" s="60">
-        <f>IFERROR(IF(('Course Content'!D11="")*('Course Content'!I11="")*('Course Content'!D27="")*('Course Content'!I27=""),"—",IFERROR('Course Content'!D11*1,0)+IFERROR('Course Content'!I11*1,0)+IFERROR('Course Content'!D27*1,0)+IFERROR('Course Content'!I27*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="60">
+      <c r="K14" s="69">
+        <f>IFERROR(IF('Course Content'!I24="","—",'Course Content'!I24),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="69">
         <f>IFERROR(IF(K14="","",IF(K14="—","",FLOOR(K14/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M14" s="61">
+      <c r="M14" s="70">
         <f>IFERROR(IF(L14="","",IF(L14="—","",FLOOR(L14/I14,1))),"")</f>
         <v/>
       </c>
       <c r="N14" s="26" t="n"/>
-      <c r="O14" s="62">
-        <f>IFERROR(IF(('Course Content'!E11="")*('Course Content'!J11="")*('Course Content'!E27="")*('Course Content'!J27=""),"—",IFERROR('Course Content'!E11*1,0)+IFERROR('Course Content'!J11*1,0)+IFERROR('Course Content'!E27*1,0)+IFERROR('Course Content'!J27*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P14" s="62">
+      <c r="O14" s="71">
+        <f>IFERROR(IF('Course Content'!J24="","—",'Course Content'!J24),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="71">
         <f>IFERROR(IF(O14="","",IF(O14="—","",FLOOR(O14/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q14" s="63">
+      <c r="Q14" s="72">
         <f>IFERROR(IF(P14="","",IF(P14="—","",FLOOR(P14/I14,1))),"")</f>
         <v/>
       </c>
-      <c r="R14" s="66">
-        <f>IFERROR(IF('Course Content'!C27&lt;&gt;"",'Course Content'!C27,IF('Course Content'!H27&lt;&gt;"",'Course Content'!H27,IF('Course Content'!C11&lt;&gt;"",'Course Content'!C11,'Course Content'!H11))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
+      <c r="R14" s="73">
+        <f>IFERROR(IF('Course Content'!H24="","",'Course Content'!H24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
       <c r="A15" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B15" s="58">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,""),IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,""),IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,""),IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!B9="","",'Course Content'!B9),"")</f>
         <v/>
       </c>
       <c r="C15" s="59" t="n"/>
@@ -5856,7 +5876,7 @@
       </c>
       <c r="J15" s="26" t="n"/>
       <c r="K15" s="60">
-        <f>IFERROR(IF(('Course Content'!D12="")*('Course Content'!I12="")*('Course Content'!D28="")*('Course Content'!I28=""),"—",IFERROR('Course Content'!D12*1,0)+IFERROR('Course Content'!I12*1,0)+IFERROR('Course Content'!D28*1,0)+IFERROR('Course Content'!I28*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!D9="","—",'Course Content'!D9),"")</f>
         <v/>
       </c>
       <c r="L15" s="60">
@@ -5869,7 +5889,7 @@
       </c>
       <c r="N15" s="26" t="n"/>
       <c r="O15" s="62">
-        <f>IFERROR(IF(('Course Content'!E12="")*('Course Content'!J12="")*('Course Content'!E28="")*('Course Content'!J28=""),"—",IFERROR('Course Content'!E12*1,0)+IFERROR('Course Content'!J12*1,0)+IFERROR('Course Content'!E28*1,0)+IFERROR('Course Content'!J28*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!E9="","—",'Course Content'!E9),"")</f>
         <v/>
       </c>
       <c r="P15" s="62">
@@ -5881,18 +5901,13 @@
         <v/>
       </c>
       <c r="R15" s="64">
-        <f>IFERROR(IF('Course Content'!C28&lt;&gt;"",'Course Content'!C28,IF('Course Content'!H28&lt;&gt;"",'Course Content'!H28,IF('Course Content'!C12&lt;&gt;"",'Course Content'!C12,'Course Content'!H12))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="31" t="inlineStr">
-        <is>
-          <t>Science</t>
-        </is>
-      </c>
-      <c r="B16" s="65">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,""),IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,""),IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,""),IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!C9="","",'Course Content'!C9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="58">
+        <f>IFERROR(IF('Course Content'!G9="","",'Course Content'!G9),"")</f>
         <v/>
       </c>
       <c r="C16" s="59" t="n"/>
@@ -5907,7 +5922,7 @@
       </c>
       <c r="J16" s="26" t="n"/>
       <c r="K16" s="60">
-        <f>IFERROR(IF(('Course Content'!D13="")*('Course Content'!I13="")*('Course Content'!D29="")*('Course Content'!I29=""),"—",IFERROR('Course Content'!D13*1,0)+IFERROR('Course Content'!I13*1,0)+IFERROR('Course Content'!D29*1,0)+IFERROR('Course Content'!I29*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!I9="","—",'Course Content'!I9),"")</f>
         <v/>
       </c>
       <c r="L16" s="60">
@@ -5920,7 +5935,7 @@
       </c>
       <c r="N16" s="26" t="n"/>
       <c r="O16" s="62">
-        <f>IFERROR(IF(('Course Content'!E13="")*('Course Content'!J13="")*('Course Content'!E29="")*('Course Content'!J29=""),"—",IFERROR('Course Content'!E13*1,0)+IFERROR('Course Content'!J13*1,0)+IFERROR('Course Content'!E29*1,0)+IFERROR('Course Content'!J29*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!J9="","—",'Course Content'!J9),"")</f>
         <v/>
       </c>
       <c r="P16" s="62">
@@ -5931,19 +5946,14 @@
         <f>IFERROR(IF(P16="","",IF(P16="—","",FLOOR(P16/I16,1))),"")</f>
         <v/>
       </c>
-      <c r="R16" s="66">
-        <f>IFERROR(IF('Course Content'!C29&lt;&gt;"",'Course Content'!C29,IF('Course Content'!H29&lt;&gt;"",'Course Content'!H29,IF('Course Content'!C13&lt;&gt;"",'Course Content'!C13,'Course Content'!H13))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
-        </is>
-      </c>
-      <c r="B17" s="58">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,""),IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,""),IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,""),IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,"")),"—")</f>
+      <c r="R16" s="64">
+        <f>IFERROR(IF('Course Content'!H9="","",'Course Content'!H9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="5">
+        <f>IFERROR(IF('Course Content'!B25="","",'Course Content'!B25),"")</f>
         <v/>
       </c>
       <c r="C17" s="59" t="n"/>
@@ -5958,7 +5968,7 @@
       </c>
       <c r="J17" s="26" t="n"/>
       <c r="K17" s="60">
-        <f>IFERROR(IF(('Course Content'!D14="")*('Course Content'!I14="")*('Course Content'!D30="")*('Course Content'!I30=""),"—",IFERROR('Course Content'!D14*1,0)+IFERROR('Course Content'!I14*1,0)+IFERROR('Course Content'!D30*1,0)+IFERROR('Course Content'!I30*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!D25="","—",'Course Content'!D25),"")</f>
         <v/>
       </c>
       <c r="L17" s="60">
@@ -5971,7 +5981,7 @@
       </c>
       <c r="N17" s="26" t="n"/>
       <c r="O17" s="62">
-        <f>IFERROR(IF(('Course Content'!E14="")*('Course Content'!J14="")*('Course Content'!E30="")*('Course Content'!J30=""),"—",IFERROR('Course Content'!E14*1,0)+IFERROR('Course Content'!J14*1,0)+IFERROR('Course Content'!E30*1,0)+IFERROR('Course Content'!J30*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!E25="","—",'Course Content'!E25),"")</f>
         <v/>
       </c>
       <c r="P17" s="62">
@@ -5982,70 +5992,65 @@
         <f>IFERROR(IF(P17="","",IF(P17="—","",FLOOR(P17/I17,1))),"")</f>
         <v/>
       </c>
-      <c r="R17" s="64">
-        <f>IFERROR(IF('Course Content'!C30&lt;&gt;"",'Course Content'!C30,IF('Course Content'!H30&lt;&gt;"",'Course Content'!H30,IF('Course Content'!C14&lt;&gt;"",'Course Content'!C14,'Course Content'!H14))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
-        </is>
-      </c>
-      <c r="B18" s="65">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,""),IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,""),IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,""),IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,"")),"—")</f>
-        <v/>
-      </c>
-      <c r="C18" s="59" t="n"/>
-      <c r="D18" s="59" t="n"/>
-      <c r="E18" s="59" t="n"/>
-      <c r="F18" s="59" t="n"/>
-      <c r="G18" s="59" t="n"/>
-      <c r="H18" s="59" t="n"/>
-      <c r="I18" s="17">
+      <c r="R17" s="65">
+        <f>IFERROR(IF('Course Content'!C25="","",'Course Content'!C25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="66">
+        <f>IFERROR(IF('Course Content'!G25="","",'Course Content'!G25),"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="67" t="n"/>
+      <c r="D18" s="67" t="n"/>
+      <c r="E18" s="67" t="n"/>
+      <c r="F18" s="67" t="n"/>
+      <c r="G18" s="67" t="n"/>
+      <c r="H18" s="67" t="n"/>
+      <c r="I18" s="68">
         <f>IF(COUNTA(C18:H18)=0,$I$8,COUNTA(C18:H18))</f>
         <v/>
       </c>
       <c r="J18" s="26" t="n"/>
-      <c r="K18" s="60">
-        <f>IFERROR(IF(('Course Content'!D15="")*('Course Content'!I15="")*('Course Content'!D31="")*('Course Content'!I31=""),"—",IFERROR('Course Content'!D15*1,0)+IFERROR('Course Content'!I15*1,0)+IFERROR('Course Content'!D31*1,0)+IFERROR('Course Content'!I31*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="60">
+      <c r="K18" s="69">
+        <f>IFERROR(IF('Course Content'!I25="","—",'Course Content'!I25),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="69">
         <f>IFERROR(IF(K18="","",IF(K18="—","",FLOOR(K18/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M18" s="61">
+      <c r="M18" s="70">
         <f>IFERROR(IF(L18="","",IF(L18="—","",FLOOR(L18/I18,1))),"")</f>
         <v/>
       </c>
       <c r="N18" s="26" t="n"/>
-      <c r="O18" s="62">
-        <f>IFERROR(IF(('Course Content'!E15="")*('Course Content'!J15="")*('Course Content'!E31="")*('Course Content'!J31=""),"—",IFERROR('Course Content'!E15*1,0)+IFERROR('Course Content'!J15*1,0)+IFERROR('Course Content'!E31*1,0)+IFERROR('Course Content'!J31*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P18" s="62">
+      <c r="O18" s="71">
+        <f>IFERROR(IF('Course Content'!J25="","—",'Course Content'!J25),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="71">
         <f>IFERROR(IF(O18="","",IF(O18="—","",FLOOR(O18/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q18" s="63">
+      <c r="Q18" s="72">
         <f>IFERROR(IF(P18="","",IF(P18="—","",FLOOR(P18/I18,1))),"")</f>
         <v/>
       </c>
-      <c r="R18" s="66">
-        <f>IFERROR(IF('Course Content'!C31&lt;&gt;"",'Course Content'!C31,IF('Course Content'!H31&lt;&gt;"",'Course Content'!H31,IF('Course Content'!C15&lt;&gt;"",'Course Content'!C15,'Course Content'!H15))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
+      <c r="R18" s="73">
+        <f>IFERROR(IF('Course Content'!H25="","",'Course Content'!H25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
       <c r="A19" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B19" s="58">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,""),IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,""),IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,""),IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!B10="","",'Course Content'!B10),"")</f>
         <v/>
       </c>
       <c r="C19" s="59" t="n"/>
@@ -6060,7 +6065,7 @@
       </c>
       <c r="J19" s="26" t="n"/>
       <c r="K19" s="60">
-        <f>IFERROR(IF(('Course Content'!D16="")*('Course Content'!I16="")*('Course Content'!D32="")*('Course Content'!I32=""),"—",IFERROR('Course Content'!D16*1,0)+IFERROR('Course Content'!I16*1,0)+IFERROR('Course Content'!D32*1,0)+IFERROR('Course Content'!I32*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!D10="","—",'Course Content'!D10),"")</f>
         <v/>
       </c>
       <c r="L19" s="60">
@@ -6073,7 +6078,7 @@
       </c>
       <c r="N19" s="26" t="n"/>
       <c r="O19" s="62">
-        <f>IFERROR(IF(('Course Content'!E16="")*('Course Content'!J16="")*('Course Content'!E32="")*('Course Content'!J32=""),"—",IFERROR('Course Content'!E16*1,0)+IFERROR('Course Content'!J16*1,0)+IFERROR('Course Content'!E32*1,0)+IFERROR('Course Content'!J32*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!E10="","—",'Course Content'!E10),"")</f>
         <v/>
       </c>
       <c r="P19" s="62">
@@ -6085,18 +6090,13 @@
         <v/>
       </c>
       <c r="R19" s="64">
-        <f>IFERROR(IF('Course Content'!C32&lt;&gt;"",'Course Content'!C32,IF('Course Content'!H32&lt;&gt;"",'Course Content'!H32,IF('Course Content'!C16&lt;&gt;"",'Course Content'!C16,'Course Content'!H16))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
-        <is>
-          <t>Art / Music</t>
-        </is>
-      </c>
-      <c r="B20" s="65">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,""),IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,""),IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,""),IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!C10="","",'Course Content'!C10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="B20" s="58">
+        <f>IFERROR(IF('Course Content'!G10="","",'Course Content'!G10),"")</f>
         <v/>
       </c>
       <c r="C20" s="59" t="n"/>
@@ -6111,7 +6111,7 @@
       </c>
       <c r="J20" s="26" t="n"/>
       <c r="K20" s="60">
-        <f>IFERROR(IF(('Course Content'!D17="")*('Course Content'!I17="")*('Course Content'!D33="")*('Course Content'!I33=""),"—",IFERROR('Course Content'!D17*1,0)+IFERROR('Course Content'!I17*1,0)+IFERROR('Course Content'!D33*1,0)+IFERROR('Course Content'!I33*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!I10="","—",'Course Content'!I10),"")</f>
         <v/>
       </c>
       <c r="L20" s="60">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="N20" s="26" t="n"/>
       <c r="O20" s="62">
-        <f>IFERROR(IF(('Course Content'!E17="")*('Course Content'!J17="")*('Course Content'!E33="")*('Course Content'!J33=""),"—",IFERROR('Course Content'!E17*1,0)+IFERROR('Course Content'!J17*1,0)+IFERROR('Course Content'!E33*1,0)+IFERROR('Course Content'!J33*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!J10="","—",'Course Content'!J10),"")</f>
         <v/>
       </c>
       <c r="P20" s="62">
@@ -6135,18 +6135,14 @@
         <f>IFERROR(IF(P20="","",IF(P20="—","",FLOOR(P20/I20,1))),"")</f>
         <v/>
       </c>
-      <c r="R20" s="66">
-        <f>IFERROR(IF('Course Content'!C33&lt;&gt;"",'Course Content'!C33,IF('Course Content'!H33&lt;&gt;"",'Course Content'!H33,IF('Course Content'!C17&lt;&gt;"",'Course Content'!C17,'Course Content'!H17))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="31">
-        <f>IF('Course Content'!A34="Elective / Other 1","Elective / Other 1",'Course Content'!A34)</f>
-        <v/>
-      </c>
-      <c r="B21" s="58">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,""),IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,""),IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,""),IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,"")),"—")</f>
+      <c r="R20" s="64">
+        <f>IFERROR(IF('Course Content'!H10="","",'Course Content'!H10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="B21" s="5">
+        <f>IFERROR(IF('Course Content'!B26="","",'Course Content'!B26),"")</f>
         <v/>
       </c>
       <c r="C21" s="59" t="n"/>
@@ -6161,7 +6157,7 @@
       </c>
       <c r="J21" s="26" t="n"/>
       <c r="K21" s="60">
-        <f>IFERROR(IF(('Course Content'!D18="")*('Course Content'!I18="")*('Course Content'!D34="")*('Course Content'!I34=""),"—",IFERROR('Course Content'!D18*1,0)+IFERROR('Course Content'!I18*1,0)+IFERROR('Course Content'!D34*1,0)+IFERROR('Course Content'!I34*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!D26="","—",'Course Content'!D26),"")</f>
         <v/>
       </c>
       <c r="L21" s="60">
@@ -6174,7 +6170,7 @@
       </c>
       <c r="N21" s="26" t="n"/>
       <c r="O21" s="62">
-        <f>IFERROR(IF(('Course Content'!E18="")*('Course Content'!J18="")*('Course Content'!E34="")*('Course Content'!J34=""),"—",IFERROR('Course Content'!E18*1,0)+IFERROR('Course Content'!J18*1,0)+IFERROR('Course Content'!E34*1,0)+IFERROR('Course Content'!J34*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!E26="","—",'Course Content'!E26),"")</f>
         <v/>
       </c>
       <c r="P21" s="62">
@@ -6185,68 +6181,65 @@
         <f>IFERROR(IF(P21="","",IF(P21="—","",FLOOR(P21/I21,1))),"")</f>
         <v/>
       </c>
-      <c r="R21" s="64">
-        <f>IFERROR(IF('Course Content'!C34&lt;&gt;"",'Course Content'!C34,IF('Course Content'!H34&lt;&gt;"",'Course Content'!H34,IF('Course Content'!C18&lt;&gt;"",'Course Content'!C18,'Course Content'!H18))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="31">
-        <f>IF('Course Content'!A35="Elective / Other 2","Elective / Other 2",'Course Content'!A35)</f>
-        <v/>
-      </c>
-      <c r="B22" s="65">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,""),IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,""),IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,""),IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,"")),"—")</f>
-        <v/>
-      </c>
-      <c r="C22" s="59" t="n"/>
-      <c r="D22" s="59" t="n"/>
-      <c r="E22" s="59" t="n"/>
-      <c r="F22" s="59" t="n"/>
-      <c r="G22" s="59" t="n"/>
-      <c r="H22" s="59" t="n"/>
-      <c r="I22" s="17">
+      <c r="R21" s="65">
+        <f>IFERROR(IF('Course Content'!C26="","",'Course Content'!C26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="66">
+        <f>IFERROR(IF('Course Content'!G26="","",'Course Content'!G26),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="67" t="n"/>
+      <c r="D22" s="67" t="n"/>
+      <c r="E22" s="67" t="n"/>
+      <c r="F22" s="67" t="n"/>
+      <c r="G22" s="67" t="n"/>
+      <c r="H22" s="67" t="n"/>
+      <c r="I22" s="68">
         <f>IF(COUNTA(C22:H22)=0,$I$8,COUNTA(C22:H22))</f>
         <v/>
       </c>
       <c r="J22" s="26" t="n"/>
-      <c r="K22" s="60">
-        <f>IFERROR(IF(('Course Content'!D19="")*('Course Content'!I19="")*('Course Content'!D35="")*('Course Content'!I35=""),"—",IFERROR('Course Content'!D19*1,0)+IFERROR('Course Content'!I19*1,0)+IFERROR('Course Content'!D35*1,0)+IFERROR('Course Content'!I35*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="60">
+      <c r="K22" s="69">
+        <f>IFERROR(IF('Course Content'!I26="","—",'Course Content'!I26),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="69">
         <f>IFERROR(IF(K22="","",IF(K22="—","",FLOOR(K22/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M22" s="61">
+      <c r="M22" s="70">
         <f>IFERROR(IF(L22="","",IF(L22="—","",FLOOR(L22/I22,1))),"")</f>
         <v/>
       </c>
       <c r="N22" s="26" t="n"/>
-      <c r="O22" s="62">
-        <f>IFERROR(IF(('Course Content'!E19="")*('Course Content'!J19="")*('Course Content'!E35="")*('Course Content'!J35=""),"—",IFERROR('Course Content'!E19*1,0)+IFERROR('Course Content'!J19*1,0)+IFERROR('Course Content'!E35*1,0)+IFERROR('Course Content'!J35*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P22" s="62">
+      <c r="O22" s="71">
+        <f>IFERROR(IF('Course Content'!J26="","—",'Course Content'!J26),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="71">
         <f>IFERROR(IF(O22="","",IF(O22="—","",FLOOR(O22/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q22" s="63">
+      <c r="Q22" s="72">
         <f>IFERROR(IF(P22="","",IF(P22="—","",FLOOR(P22/I22,1))),"")</f>
         <v/>
       </c>
-      <c r="R22" s="66">
-        <f>IFERROR(IF('Course Content'!C35&lt;&gt;"",'Course Content'!C35,IF('Course Content'!H35&lt;&gt;"",'Course Content'!H35,IF('Course Content'!C19&lt;&gt;"",'Course Content'!C19,'Course Content'!H19))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="31">
-        <f>IF('Course Content'!A36="Elective / Other 3","Elective / Other 3",'Course Content'!A36)</f>
-        <v/>
+      <c r="R22" s="73">
+        <f>IFERROR(IF('Course Content'!H26="","",'Course Content'!H26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
       </c>
       <c r="B23" s="58">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,""),IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,""),IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,""),IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!B11="","",'Course Content'!B11),"")</f>
         <v/>
       </c>
       <c r="C23" s="59" t="n"/>
@@ -6261,7 +6254,7 @@
       </c>
       <c r="J23" s="26" t="n"/>
       <c r="K23" s="60">
-        <f>IFERROR(IF(('Course Content'!D20="")*('Course Content'!I20="")*('Course Content'!D36="")*('Course Content'!I36=""),"—",IFERROR('Course Content'!D20*1,0)+IFERROR('Course Content'!I20*1,0)+IFERROR('Course Content'!D36*1,0)+IFERROR('Course Content'!I36*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!D11="","—",'Course Content'!D11),"")</f>
         <v/>
       </c>
       <c r="L23" s="60">
@@ -6274,7 +6267,7 @@
       </c>
       <c r="N23" s="26" t="n"/>
       <c r="O23" s="62">
-        <f>IFERROR(IF(('Course Content'!E20="")*('Course Content'!J20="")*('Course Content'!E36="")*('Course Content'!J36=""),"—",IFERROR('Course Content'!E20*1,0)+IFERROR('Course Content'!J20*1,0)+IFERROR('Course Content'!E36*1,0)+IFERROR('Course Content'!J36*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!E11="","—",'Course Content'!E11),"")</f>
         <v/>
       </c>
       <c r="P23" s="62">
@@ -6286,17 +6279,13 @@
         <v/>
       </c>
       <c r="R23" s="64">
-        <f>IFERROR(IF('Course Content'!C36&lt;&gt;"",'Course Content'!C36,IF('Course Content'!H36&lt;&gt;"",'Course Content'!H36,IF('Course Content'!C20&lt;&gt;"",'Course Content'!C20,'Course Content'!H20))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="31">
-        <f>IF('Course Content'!A37="Elective / Other 4","Elective / Other 4",'Course Content'!A37)</f>
-        <v/>
-      </c>
-      <c r="B24" s="65">
-        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,""),IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,""),IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,""),IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,"")),"—")</f>
+        <f>IFERROR(IF('Course Content'!C11="","",'Course Content'!C11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="58">
+        <f>IFERROR(IF('Course Content'!G11="","",'Course Content'!G11),"")</f>
         <v/>
       </c>
       <c r="C24" s="59" t="n"/>
@@ -6311,7 +6300,7 @@
       </c>
       <c r="J24" s="26" t="n"/>
       <c r="K24" s="60">
-        <f>IFERROR(IF(('Course Content'!D21="")*('Course Content'!I21="")*('Course Content'!D37="")*('Course Content'!I37=""),"—",IFERROR('Course Content'!D21*1,0)+IFERROR('Course Content'!I21*1,0)+IFERROR('Course Content'!D37*1,0)+IFERROR('Course Content'!I37*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!I11="","—",'Course Content'!I11),"")</f>
         <v/>
       </c>
       <c r="L24" s="60">
@@ -6324,7 +6313,7 @@
       </c>
       <c r="N24" s="26" t="n"/>
       <c r="O24" s="62">
-        <f>IFERROR(IF(('Course Content'!E21="")*('Course Content'!J21="")*('Course Content'!E37="")*('Course Content'!J37=""),"—",IFERROR('Course Content'!E21*1,0)+IFERROR('Course Content'!J21*1,0)+IFERROR('Course Content'!E37*1,0)+IFERROR('Course Content'!J37*1,0)),"")</f>
+        <f>IFERROR(IF('Course Content'!J11="","—",'Course Content'!J11),"")</f>
         <v/>
       </c>
       <c r="P24" s="62">
@@ -6335,18 +6324,2010 @@
         <f>IFERROR(IF(P24="","",IF(P24="—","",FLOOR(P24/I24,1))),"")</f>
         <v/>
       </c>
-      <c r="R24" s="66">
-        <f>IFERROR(IF('Course Content'!C37&lt;&gt;"",'Course Content'!C37,IF('Course Content'!H37&lt;&gt;"",'Course Content'!H37,IF('Course Content'!C21&lt;&gt;"",'Course Content'!C21,'Course Content'!H21))),"")</f>
+      <c r="R24" s="64">
+        <f>IFERROR(IF('Course Content'!H11="","",'Course Content'!H11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="5">
+        <f>IFERROR(IF('Course Content'!B27="","",'Course Content'!B27),"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="59" t="n"/>
+      <c r="D25" s="59" t="n"/>
+      <c r="E25" s="59" t="n"/>
+      <c r="F25" s="59" t="n"/>
+      <c r="G25" s="59" t="n"/>
+      <c r="H25" s="59" t="n"/>
+      <c r="I25" s="17">
+        <f>IF(COUNTA(C25:H25)=0,$I$8,COUNTA(C25:H25))</f>
+        <v/>
+      </c>
+      <c r="J25" s="26" t="n"/>
+      <c r="K25" s="60">
+        <f>IFERROR(IF('Course Content'!D27="","—",'Course Content'!D27),"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="60">
+        <f>IFERROR(IF(K25="","",IF(K25="—","",FLOOR(K25/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="61">
+        <f>IFERROR(IF(L25="","",IF(L25="—","",FLOOR(L25/I25,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="26" t="n"/>
+      <c r="O25" s="62">
+        <f>IFERROR(IF('Course Content'!E27="","—",'Course Content'!E27),"")</f>
+        <v/>
+      </c>
+      <c r="P25" s="62">
+        <f>IFERROR(IF(O25="","",IF(O25="—","",FLOOR(O25/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q25" s="63">
+        <f>IFERROR(IF(P25="","",IF(P25="—","",FLOOR(P25/I25,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R25" s="65">
+        <f>IFERROR(IF('Course Content'!C27="","",'Course Content'!C27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="66">
+        <f>IFERROR(IF('Course Content'!G27="","",'Course Content'!G27),"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="67" t="n"/>
+      <c r="D26" s="67" t="n"/>
+      <c r="E26" s="67" t="n"/>
+      <c r="F26" s="67" t="n"/>
+      <c r="G26" s="67" t="n"/>
+      <c r="H26" s="67" t="n"/>
+      <c r="I26" s="68">
+        <f>IF(COUNTA(C26:H26)=0,$I$8,COUNTA(C26:H26))</f>
+        <v/>
+      </c>
+      <c r="J26" s="26" t="n"/>
+      <c r="K26" s="69">
+        <f>IFERROR(IF('Course Content'!I27="","—",'Course Content'!I27),"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="69">
+        <f>IFERROR(IF(K26="","",IF(K26="—","",FLOOR(K26/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="70">
+        <f>IFERROR(IF(L26="","",IF(L26="—","",FLOOR(L26/I26,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="26" t="n"/>
+      <c r="O26" s="71">
+        <f>IFERROR(IF('Course Content'!J27="","—",'Course Content'!J27),"")</f>
+        <v/>
+      </c>
+      <c r="P26" s="71">
+        <f>IFERROR(IF(O26="","",IF(O26="—","",FLOOR(O26/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q26" s="72">
+        <f>IFERROR(IF(P26="","",IF(P26="—","",FLOOR(P26/I26,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R26" s="73">
+        <f>IFERROR(IF('Course Content'!H27="","",'Course Content'!H27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Writing / Composition</t>
+        </is>
+      </c>
+      <c r="B27" s="58">
+        <f>IFERROR(IF('Course Content'!B12="","",'Course Content'!B12),"")</f>
+        <v/>
+      </c>
+      <c r="C27" s="59" t="n"/>
+      <c r="D27" s="59" t="n"/>
+      <c r="E27" s="59" t="n"/>
+      <c r="F27" s="59" t="n"/>
+      <c r="G27" s="59" t="n"/>
+      <c r="H27" s="59" t="n"/>
+      <c r="I27" s="17">
+        <f>IF(COUNTA(C27:H27)=0,$I$8,COUNTA(C27:H27))</f>
+        <v/>
+      </c>
+      <c r="J27" s="26" t="n"/>
+      <c r="K27" s="60">
+        <f>IFERROR(IF('Course Content'!D12="","—",'Course Content'!D12),"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="60">
+        <f>IFERROR(IF(K27="","",IF(K27="—","",FLOOR(K27/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="61">
+        <f>IFERROR(IF(L27="","",IF(L27="—","",FLOOR(L27/I27,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="26" t="n"/>
+      <c r="O27" s="62">
+        <f>IFERROR(IF('Course Content'!E12="","—",'Course Content'!E12),"")</f>
+        <v/>
+      </c>
+      <c r="P27" s="62">
+        <f>IFERROR(IF(O27="","",IF(O27="—","",FLOOR(O27/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q27" s="63">
+        <f>IFERROR(IF(P27="","",IF(P27="—","",FLOOR(P27/I27,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R27" s="64">
+        <f>IFERROR(IF('Course Content'!C12="","",'Course Content'!C12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="58">
+        <f>IFERROR(IF('Course Content'!G12="","",'Course Content'!G12),"")</f>
+        <v/>
+      </c>
+      <c r="C28" s="59" t="n"/>
+      <c r="D28" s="59" t="n"/>
+      <c r="E28" s="59" t="n"/>
+      <c r="F28" s="59" t="n"/>
+      <c r="G28" s="59" t="n"/>
+      <c r="H28" s="59" t="n"/>
+      <c r="I28" s="17">
+        <f>IF(COUNTA(C28:H28)=0,$I$8,COUNTA(C28:H28))</f>
+        <v/>
+      </c>
+      <c r="J28" s="26" t="n"/>
+      <c r="K28" s="60">
+        <f>IFERROR(IF('Course Content'!I12="","—",'Course Content'!I12),"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="60">
+        <f>IFERROR(IF(K28="","",IF(K28="—","",FLOOR(K28/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="61">
+        <f>IFERROR(IF(L28="","",IF(L28="—","",FLOOR(L28/I28,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="26" t="n"/>
+      <c r="O28" s="62">
+        <f>IFERROR(IF('Course Content'!J12="","—",'Course Content'!J12),"")</f>
+        <v/>
+      </c>
+      <c r="P28" s="62">
+        <f>IFERROR(IF(O28="","",IF(O28="—","",FLOOR(O28/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q28" s="63">
+        <f>IFERROR(IF(P28="","",IF(P28="—","",FLOOR(P28/I28,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R28" s="64">
+        <f>IFERROR(IF('Course Content'!H12="","",'Course Content'!H12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="B29" s="5">
+        <f>IFERROR(IF('Course Content'!B28="","",'Course Content'!B28),"")</f>
+        <v/>
+      </c>
+      <c r="C29" s="59" t="n"/>
+      <c r="D29" s="59" t="n"/>
+      <c r="E29" s="59" t="n"/>
+      <c r="F29" s="59" t="n"/>
+      <c r="G29" s="59" t="n"/>
+      <c r="H29" s="59" t="n"/>
+      <c r="I29" s="17">
+        <f>IF(COUNTA(C29:H29)=0,$I$8,COUNTA(C29:H29))</f>
+        <v/>
+      </c>
+      <c r="J29" s="26" t="n"/>
+      <c r="K29" s="60">
+        <f>IFERROR(IF('Course Content'!D28="","—",'Course Content'!D28),"")</f>
+        <v/>
+      </c>
+      <c r="L29" s="60">
+        <f>IFERROR(IF(K29="","",IF(K29="—","",FLOOR(K29/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M29" s="61">
+        <f>IFERROR(IF(L29="","",IF(L29="—","",FLOOR(L29/I29,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N29" s="26" t="n"/>
+      <c r="O29" s="62">
+        <f>IFERROR(IF('Course Content'!E28="","—",'Course Content'!E28),"")</f>
+        <v/>
+      </c>
+      <c r="P29" s="62">
+        <f>IFERROR(IF(O29="","",IF(O29="—","",FLOOR(O29/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q29" s="63">
+        <f>IFERROR(IF(P29="","",IF(P29="—","",FLOOR(P29/I29,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R29" s="65">
+        <f>IFERROR(IF('Course Content'!C28="","",'Course Content'!C28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="B30" s="66">
+        <f>IFERROR(IF('Course Content'!G28="","",'Course Content'!G28),"")</f>
+        <v/>
+      </c>
+      <c r="C30" s="67" t="n"/>
+      <c r="D30" s="67" t="n"/>
+      <c r="E30" s="67" t="n"/>
+      <c r="F30" s="67" t="n"/>
+      <c r="G30" s="67" t="n"/>
+      <c r="H30" s="67" t="n"/>
+      <c r="I30" s="68">
+        <f>IF(COUNTA(C30:H30)=0,$I$8,COUNTA(C30:H30))</f>
+        <v/>
+      </c>
+      <c r="J30" s="26" t="n"/>
+      <c r="K30" s="69">
+        <f>IFERROR(IF('Course Content'!I28="","—",'Course Content'!I28),"")</f>
+        <v/>
+      </c>
+      <c r="L30" s="69">
+        <f>IFERROR(IF(K30="","",IF(K30="—","",FLOOR(K30/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M30" s="70">
+        <f>IFERROR(IF(L30="","",IF(L30="—","",FLOOR(L30/I30,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N30" s="26" t="n"/>
+      <c r="O30" s="71">
+        <f>IFERROR(IF('Course Content'!J28="","—",'Course Content'!J28),"")</f>
+        <v/>
+      </c>
+      <c r="P30" s="71">
+        <f>IFERROR(IF(O30="","",IF(O30="—","",FLOOR(O30/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q30" s="72">
+        <f>IFERROR(IF(P30="","",IF(P30="—","",FLOOR(P30/I30,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R30" s="73">
+        <f>IFERROR(IF('Course Content'!H28="","",'Course Content'!H28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="31" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="B31" s="58">
+        <f>IFERROR(IF('Course Content'!B13="","",'Course Content'!B13),"")</f>
+        <v/>
+      </c>
+      <c r="C31" s="59" t="n"/>
+      <c r="D31" s="59" t="n"/>
+      <c r="E31" s="59" t="n"/>
+      <c r="F31" s="59" t="n"/>
+      <c r="G31" s="59" t="n"/>
+      <c r="H31" s="59" t="n"/>
+      <c r="I31" s="17">
+        <f>IF(COUNTA(C31:H31)=0,$I$8,COUNTA(C31:H31))</f>
+        <v/>
+      </c>
+      <c r="J31" s="26" t="n"/>
+      <c r="K31" s="60">
+        <f>IFERROR(IF('Course Content'!D13="","—",'Course Content'!D13),"")</f>
+        <v/>
+      </c>
+      <c r="L31" s="60">
+        <f>IFERROR(IF(K31="","",IF(K31="—","",FLOOR(K31/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M31" s="61">
+        <f>IFERROR(IF(L31="","",IF(L31="—","",FLOOR(L31/I31,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N31" s="26" t="n"/>
+      <c r="O31" s="62">
+        <f>IFERROR(IF('Course Content'!E13="","—",'Course Content'!E13),"")</f>
+        <v/>
+      </c>
+      <c r="P31" s="62">
+        <f>IFERROR(IF(O31="","",IF(O31="—","",FLOOR(O31/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q31" s="63">
+        <f>IFERROR(IF(P31="","",IF(P31="—","",FLOOR(P31/I31,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R31" s="64">
+        <f>IFERROR(IF('Course Content'!C13="","",'Course Content'!C13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="58">
+        <f>IFERROR(IF('Course Content'!G13="","",'Course Content'!G13),"")</f>
+        <v/>
+      </c>
+      <c r="C32" s="59" t="n"/>
+      <c r="D32" s="59" t="n"/>
+      <c r="E32" s="59" t="n"/>
+      <c r="F32" s="59" t="n"/>
+      <c r="G32" s="59" t="n"/>
+      <c r="H32" s="59" t="n"/>
+      <c r="I32" s="17">
+        <f>IF(COUNTA(C32:H32)=0,$I$8,COUNTA(C32:H32))</f>
+        <v/>
+      </c>
+      <c r="J32" s="26" t="n"/>
+      <c r="K32" s="60">
+        <f>IFERROR(IF('Course Content'!I13="","—",'Course Content'!I13),"")</f>
+        <v/>
+      </c>
+      <c r="L32" s="60">
+        <f>IFERROR(IF(K32="","",IF(K32="—","",FLOOR(K32/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M32" s="61">
+        <f>IFERROR(IF(L32="","",IF(L32="—","",FLOOR(L32/I32,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N32" s="26" t="n"/>
+      <c r="O32" s="62">
+        <f>IFERROR(IF('Course Content'!J13="","—",'Course Content'!J13),"")</f>
+        <v/>
+      </c>
+      <c r="P32" s="62">
+        <f>IFERROR(IF(O32="","",IF(O32="—","",FLOOR(O32/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q32" s="63">
+        <f>IFERROR(IF(P32="","",IF(P32="—","",FLOOR(P32/I32,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R32" s="64">
+        <f>IFERROR(IF('Course Content'!H13="","",'Course Content'!H13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="B33" s="5">
+        <f>IFERROR(IF('Course Content'!B29="","",'Course Content'!B29),"")</f>
+        <v/>
+      </c>
+      <c r="C33" s="59" t="n"/>
+      <c r="D33" s="59" t="n"/>
+      <c r="E33" s="59" t="n"/>
+      <c r="F33" s="59" t="n"/>
+      <c r="G33" s="59" t="n"/>
+      <c r="H33" s="59" t="n"/>
+      <c r="I33" s="17">
+        <f>IF(COUNTA(C33:H33)=0,$I$8,COUNTA(C33:H33))</f>
+        <v/>
+      </c>
+      <c r="J33" s="26" t="n"/>
+      <c r="K33" s="60">
+        <f>IFERROR(IF('Course Content'!D29="","—",'Course Content'!D29),"")</f>
+        <v/>
+      </c>
+      <c r="L33" s="60">
+        <f>IFERROR(IF(K33="","",IF(K33="—","",FLOOR(K33/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M33" s="61">
+        <f>IFERROR(IF(L33="","",IF(L33="—","",FLOOR(L33/I33,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N33" s="26" t="n"/>
+      <c r="O33" s="62">
+        <f>IFERROR(IF('Course Content'!E29="","—",'Course Content'!E29),"")</f>
+        <v/>
+      </c>
+      <c r="P33" s="62">
+        <f>IFERROR(IF(O33="","",IF(O33="—","",FLOOR(O33/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q33" s="63">
+        <f>IFERROR(IF(P33="","",IF(P33="—","",FLOOR(P33/I33,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R33" s="65">
+        <f>IFERROR(IF('Course Content'!C29="","",'Course Content'!C29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="B34" s="66">
+        <f>IFERROR(IF('Course Content'!G29="","",'Course Content'!G29),"")</f>
+        <v/>
+      </c>
+      <c r="C34" s="67" t="n"/>
+      <c r="D34" s="67" t="n"/>
+      <c r="E34" s="67" t="n"/>
+      <c r="F34" s="67" t="n"/>
+      <c r="G34" s="67" t="n"/>
+      <c r="H34" s="67" t="n"/>
+      <c r="I34" s="68">
+        <f>IF(COUNTA(C34:H34)=0,$I$8,COUNTA(C34:H34))</f>
+        <v/>
+      </c>
+      <c r="J34" s="26" t="n"/>
+      <c r="K34" s="69">
+        <f>IFERROR(IF('Course Content'!I29="","—",'Course Content'!I29),"")</f>
+        <v/>
+      </c>
+      <c r="L34" s="69">
+        <f>IFERROR(IF(K34="","",IF(K34="—","",FLOOR(K34/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M34" s="70">
+        <f>IFERROR(IF(L34="","",IF(L34="—","",FLOOR(L34/I34,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="26" t="n"/>
+      <c r="O34" s="71">
+        <f>IFERROR(IF('Course Content'!J29="","—",'Course Content'!J29),"")</f>
+        <v/>
+      </c>
+      <c r="P34" s="71">
+        <f>IFERROR(IF(O34="","",IF(O34="—","",FLOOR(O34/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q34" s="72">
+        <f>IFERROR(IF(P34="","",IF(P34="—","",FLOOR(P34/I34,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R34" s="73">
+        <f>IFERROR(IF('Course Content'!H29="","",'Course Content'!H29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
+        </is>
+      </c>
+      <c r="B35" s="58">
+        <f>IFERROR(IF('Course Content'!B14="","",'Course Content'!B14),"")</f>
+        <v/>
+      </c>
+      <c r="C35" s="59" t="n"/>
+      <c r="D35" s="59" t="n"/>
+      <c r="E35" s="59" t="n"/>
+      <c r="F35" s="59" t="n"/>
+      <c r="G35" s="59" t="n"/>
+      <c r="H35" s="59" t="n"/>
+      <c r="I35" s="17">
+        <f>IF(COUNTA(C35:H35)=0,$I$8,COUNTA(C35:H35))</f>
+        <v/>
+      </c>
+      <c r="J35" s="26" t="n"/>
+      <c r="K35" s="60">
+        <f>IFERROR(IF('Course Content'!D14="","—",'Course Content'!D14),"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="60">
+        <f>IFERROR(IF(K35="","",IF(K35="—","",FLOOR(K35/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M35" s="61">
+        <f>IFERROR(IF(L35="","",IF(L35="—","",FLOOR(L35/I35,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N35" s="26" t="n"/>
+      <c r="O35" s="62">
+        <f>IFERROR(IF('Course Content'!E14="","—",'Course Content'!E14),"")</f>
+        <v/>
+      </c>
+      <c r="P35" s="62">
+        <f>IFERROR(IF(O35="","",IF(O35="—","",FLOOR(O35/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q35" s="63">
+        <f>IFERROR(IF(P35="","",IF(P35="—","",FLOOR(P35/I35,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R35" s="64">
+        <f>IFERROR(IF('Course Content'!C14="","",'Course Content'!C14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="B36" s="58">
+        <f>IFERROR(IF('Course Content'!G14="","",'Course Content'!G14),"")</f>
+        <v/>
+      </c>
+      <c r="C36" s="59" t="n"/>
+      <c r="D36" s="59" t="n"/>
+      <c r="E36" s="59" t="n"/>
+      <c r="F36" s="59" t="n"/>
+      <c r="G36" s="59" t="n"/>
+      <c r="H36" s="59" t="n"/>
+      <c r="I36" s="17">
+        <f>IF(COUNTA(C36:H36)=0,$I$8,COUNTA(C36:H36))</f>
+        <v/>
+      </c>
+      <c r="J36" s="26" t="n"/>
+      <c r="K36" s="60">
+        <f>IFERROR(IF('Course Content'!I14="","—",'Course Content'!I14),"")</f>
+        <v/>
+      </c>
+      <c r="L36" s="60">
+        <f>IFERROR(IF(K36="","",IF(K36="—","",FLOOR(K36/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M36" s="61">
+        <f>IFERROR(IF(L36="","",IF(L36="—","",FLOOR(L36/I36,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N36" s="26" t="n"/>
+      <c r="O36" s="62">
+        <f>IFERROR(IF('Course Content'!J14="","—",'Course Content'!J14),"")</f>
+        <v/>
+      </c>
+      <c r="P36" s="62">
+        <f>IFERROR(IF(O36="","",IF(O36="—","",FLOOR(O36/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q36" s="63">
+        <f>IFERROR(IF(P36="","",IF(P36="—","",FLOOR(P36/I36,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R36" s="64">
+        <f>IFERROR(IF('Course Content'!H14="","",'Course Content'!H14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="5">
+        <f>IFERROR(IF('Course Content'!B30="","",'Course Content'!B30),"")</f>
+        <v/>
+      </c>
+      <c r="C37" s="59" t="n"/>
+      <c r="D37" s="59" t="n"/>
+      <c r="E37" s="59" t="n"/>
+      <c r="F37" s="59" t="n"/>
+      <c r="G37" s="59" t="n"/>
+      <c r="H37" s="59" t="n"/>
+      <c r="I37" s="17">
+        <f>IF(COUNTA(C37:H37)=0,$I$8,COUNTA(C37:H37))</f>
+        <v/>
+      </c>
+      <c r="J37" s="26" t="n"/>
+      <c r="K37" s="60">
+        <f>IFERROR(IF('Course Content'!D30="","—",'Course Content'!D30),"")</f>
+        <v/>
+      </c>
+      <c r="L37" s="60">
+        <f>IFERROR(IF(K37="","",IF(K37="—","",FLOOR(K37/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M37" s="61">
+        <f>IFERROR(IF(L37="","",IF(L37="—","",FLOOR(L37/I37,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N37" s="26" t="n"/>
+      <c r="O37" s="62">
+        <f>IFERROR(IF('Course Content'!E30="","—",'Course Content'!E30),"")</f>
+        <v/>
+      </c>
+      <c r="P37" s="62">
+        <f>IFERROR(IF(O37="","",IF(O37="—","",FLOOR(O37/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q37" s="63">
+        <f>IFERROR(IF(P37="","",IF(P37="—","",FLOOR(P37/I37,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R37" s="65">
+        <f>IFERROR(IF('Course Content'!C30="","",'Course Content'!C30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="66">
+        <f>IFERROR(IF('Course Content'!G30="","",'Course Content'!G30),"")</f>
+        <v/>
+      </c>
+      <c r="C38" s="67" t="n"/>
+      <c r="D38" s="67" t="n"/>
+      <c r="E38" s="67" t="n"/>
+      <c r="F38" s="67" t="n"/>
+      <c r="G38" s="67" t="n"/>
+      <c r="H38" s="67" t="n"/>
+      <c r="I38" s="68">
+        <f>IF(COUNTA(C38:H38)=0,$I$8,COUNTA(C38:H38))</f>
+        <v/>
+      </c>
+      <c r="J38" s="26" t="n"/>
+      <c r="K38" s="69">
+        <f>IFERROR(IF('Course Content'!I30="","—",'Course Content'!I30),"")</f>
+        <v/>
+      </c>
+      <c r="L38" s="69">
+        <f>IFERROR(IF(K38="","",IF(K38="—","",FLOOR(K38/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M38" s="70">
+        <f>IFERROR(IF(L38="","",IF(L38="—","",FLOOR(L38/I38,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N38" s="26" t="n"/>
+      <c r="O38" s="71">
+        <f>IFERROR(IF('Course Content'!J30="","—",'Course Content'!J30),"")</f>
+        <v/>
+      </c>
+      <c r="P38" s="71">
+        <f>IFERROR(IF(O38="","",IF(O38="—","",FLOOR(O38/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q38" s="72">
+        <f>IFERROR(IF(P38="","",IF(P38="—","",FLOOR(P38/I38,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R38" s="73">
+        <f>IFERROR(IF('Course Content'!H30="","",'Course Content'!H30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B39" s="58">
+        <f>IFERROR(IF('Course Content'!B15="","",'Course Content'!B15),"")</f>
+        <v/>
+      </c>
+      <c r="C39" s="59" t="n"/>
+      <c r="D39" s="59" t="n"/>
+      <c r="E39" s="59" t="n"/>
+      <c r="F39" s="59" t="n"/>
+      <c r="G39" s="59" t="n"/>
+      <c r="H39" s="59" t="n"/>
+      <c r="I39" s="17">
+        <f>IF(COUNTA(C39:H39)=0,$I$8,COUNTA(C39:H39))</f>
+        <v/>
+      </c>
+      <c r="J39" s="26" t="n"/>
+      <c r="K39" s="60">
+        <f>IFERROR(IF('Course Content'!D15="","—",'Course Content'!D15),"")</f>
+        <v/>
+      </c>
+      <c r="L39" s="60">
+        <f>IFERROR(IF(K39="","",IF(K39="—","",FLOOR(K39/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M39" s="61">
+        <f>IFERROR(IF(L39="","",IF(L39="—","",FLOOR(L39/I39,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N39" s="26" t="n"/>
+      <c r="O39" s="62">
+        <f>IFERROR(IF('Course Content'!E15="","—",'Course Content'!E15),"")</f>
+        <v/>
+      </c>
+      <c r="P39" s="62">
+        <f>IFERROR(IF(O39="","",IF(O39="—","",FLOOR(O39/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q39" s="63">
+        <f>IFERROR(IF(P39="","",IF(P39="—","",FLOOR(P39/I39,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R39" s="64">
+        <f>IFERROR(IF('Course Content'!C15="","",'Course Content'!C15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="B40" s="58">
+        <f>IFERROR(IF('Course Content'!G15="","",'Course Content'!G15),"")</f>
+        <v/>
+      </c>
+      <c r="C40" s="59" t="n"/>
+      <c r="D40" s="59" t="n"/>
+      <c r="E40" s="59" t="n"/>
+      <c r="F40" s="59" t="n"/>
+      <c r="G40" s="59" t="n"/>
+      <c r="H40" s="59" t="n"/>
+      <c r="I40" s="17">
+        <f>IF(COUNTA(C40:H40)=0,$I$8,COUNTA(C40:H40))</f>
+        <v/>
+      </c>
+      <c r="J40" s="26" t="n"/>
+      <c r="K40" s="60">
+        <f>IFERROR(IF('Course Content'!I15="","—",'Course Content'!I15),"")</f>
+        <v/>
+      </c>
+      <c r="L40" s="60">
+        <f>IFERROR(IF(K40="","",IF(K40="—","",FLOOR(K40/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M40" s="61">
+        <f>IFERROR(IF(L40="","",IF(L40="—","",FLOOR(L40/I40,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N40" s="26" t="n"/>
+      <c r="O40" s="62">
+        <f>IFERROR(IF('Course Content'!J15="","—",'Course Content'!J15),"")</f>
+        <v/>
+      </c>
+      <c r="P40" s="62">
+        <f>IFERROR(IF(O40="","",IF(O40="—","",FLOOR(O40/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q40" s="63">
+        <f>IFERROR(IF(P40="","",IF(P40="—","",FLOOR(P40/I40,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R40" s="64">
+        <f>IFERROR(IF('Course Content'!H15="","",'Course Content'!H15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="5">
+        <f>IFERROR(IF('Course Content'!B31="","",'Course Content'!B31),"")</f>
+        <v/>
+      </c>
+      <c r="C41" s="59" t="n"/>
+      <c r="D41" s="59" t="n"/>
+      <c r="E41" s="59" t="n"/>
+      <c r="F41" s="59" t="n"/>
+      <c r="G41" s="59" t="n"/>
+      <c r="H41" s="59" t="n"/>
+      <c r="I41" s="17">
+        <f>IF(COUNTA(C41:H41)=0,$I$8,COUNTA(C41:H41))</f>
+        <v/>
+      </c>
+      <c r="J41" s="26" t="n"/>
+      <c r="K41" s="60">
+        <f>IFERROR(IF('Course Content'!D31="","—",'Course Content'!D31),"")</f>
+        <v/>
+      </c>
+      <c r="L41" s="60">
+        <f>IFERROR(IF(K41="","",IF(K41="—","",FLOOR(K41/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M41" s="61">
+        <f>IFERROR(IF(L41="","",IF(L41="—","",FLOOR(L41/I41,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N41" s="26" t="n"/>
+      <c r="O41" s="62">
+        <f>IFERROR(IF('Course Content'!E31="","—",'Course Content'!E31),"")</f>
+        <v/>
+      </c>
+      <c r="P41" s="62">
+        <f>IFERROR(IF(O41="","",IF(O41="—","",FLOOR(O41/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q41" s="63">
+        <f>IFERROR(IF(P41="","",IF(P41="—","",FLOOR(P41/I41,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R41" s="65">
+        <f>IFERROR(IF('Course Content'!C31="","",'Course Content'!C31),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="B42" s="66">
+        <f>IFERROR(IF('Course Content'!G31="","",'Course Content'!G31),"")</f>
+        <v/>
+      </c>
+      <c r="C42" s="67" t="n"/>
+      <c r="D42" s="67" t="n"/>
+      <c r="E42" s="67" t="n"/>
+      <c r="F42" s="67" t="n"/>
+      <c r="G42" s="67" t="n"/>
+      <c r="H42" s="67" t="n"/>
+      <c r="I42" s="68">
+        <f>IF(COUNTA(C42:H42)=0,$I$8,COUNTA(C42:H42))</f>
+        <v/>
+      </c>
+      <c r="J42" s="26" t="n"/>
+      <c r="K42" s="69">
+        <f>IFERROR(IF('Course Content'!I31="","—",'Course Content'!I31),"")</f>
+        <v/>
+      </c>
+      <c r="L42" s="69">
+        <f>IFERROR(IF(K42="","",IF(K42="—","",FLOOR(K42/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M42" s="70">
+        <f>IFERROR(IF(L42="","",IF(L42="—","",FLOOR(L42/I42,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N42" s="26" t="n"/>
+      <c r="O42" s="71">
+        <f>IFERROR(IF('Course Content'!J31="","—",'Course Content'!J31),"")</f>
+        <v/>
+      </c>
+      <c r="P42" s="71">
+        <f>IFERROR(IF(O42="","",IF(O42="—","",FLOOR(O42/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q42" s="72">
+        <f>IFERROR(IF(P42="","",IF(P42="—","",FLOOR(P42/I42,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R42" s="73">
+        <f>IFERROR(IF('Course Content'!H31="","",'Course Content'!H31),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
+        </is>
+      </c>
+      <c r="B43" s="58">
+        <f>IFERROR(IF('Course Content'!B16="","",'Course Content'!B16),"")</f>
+        <v/>
+      </c>
+      <c r="C43" s="59" t="n"/>
+      <c r="D43" s="59" t="n"/>
+      <c r="E43" s="59" t="n"/>
+      <c r="F43" s="59" t="n"/>
+      <c r="G43" s="59" t="n"/>
+      <c r="H43" s="59" t="n"/>
+      <c r="I43" s="17">
+        <f>IF(COUNTA(C43:H43)=0,$I$8,COUNTA(C43:H43))</f>
+        <v/>
+      </c>
+      <c r="J43" s="26" t="n"/>
+      <c r="K43" s="60">
+        <f>IFERROR(IF('Course Content'!D16="","—",'Course Content'!D16),"")</f>
+        <v/>
+      </c>
+      <c r="L43" s="60">
+        <f>IFERROR(IF(K43="","",IF(K43="—","",FLOOR(K43/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M43" s="61">
+        <f>IFERROR(IF(L43="","",IF(L43="—","",FLOOR(L43/I43,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N43" s="26" t="n"/>
+      <c r="O43" s="62">
+        <f>IFERROR(IF('Course Content'!E16="","—",'Course Content'!E16),"")</f>
+        <v/>
+      </c>
+      <c r="P43" s="62">
+        <f>IFERROR(IF(O43="","",IF(O43="—","",FLOOR(O43/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q43" s="63">
+        <f>IFERROR(IF(P43="","",IF(P43="—","",FLOOR(P43/I43,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R43" s="64">
+        <f>IFERROR(IF('Course Content'!C16="","",'Course Content'!C16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="B44" s="58">
+        <f>IFERROR(IF('Course Content'!G16="","",'Course Content'!G16),"")</f>
+        <v/>
+      </c>
+      <c r="C44" s="59" t="n"/>
+      <c r="D44" s="59" t="n"/>
+      <c r="E44" s="59" t="n"/>
+      <c r="F44" s="59" t="n"/>
+      <c r="G44" s="59" t="n"/>
+      <c r="H44" s="59" t="n"/>
+      <c r="I44" s="17">
+        <f>IF(COUNTA(C44:H44)=0,$I$8,COUNTA(C44:H44))</f>
+        <v/>
+      </c>
+      <c r="J44" s="26" t="n"/>
+      <c r="K44" s="60">
+        <f>IFERROR(IF('Course Content'!I16="","—",'Course Content'!I16),"")</f>
+        <v/>
+      </c>
+      <c r="L44" s="60">
+        <f>IFERROR(IF(K44="","",IF(K44="—","",FLOOR(K44/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M44" s="61">
+        <f>IFERROR(IF(L44="","",IF(L44="—","",FLOOR(L44/I44,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N44" s="26" t="n"/>
+      <c r="O44" s="62">
+        <f>IFERROR(IF('Course Content'!J16="","—",'Course Content'!J16),"")</f>
+        <v/>
+      </c>
+      <c r="P44" s="62">
+        <f>IFERROR(IF(O44="","",IF(O44="—","",FLOOR(O44/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q44" s="63">
+        <f>IFERROR(IF(P44="","",IF(P44="—","",FLOOR(P44/I44,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R44" s="64">
+        <f>IFERROR(IF('Course Content'!H16="","",'Course Content'!H16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="B45" s="5">
+        <f>IFERROR(IF('Course Content'!B32="","",'Course Content'!B32),"")</f>
+        <v/>
+      </c>
+      <c r="C45" s="59" t="n"/>
+      <c r="D45" s="59" t="n"/>
+      <c r="E45" s="59" t="n"/>
+      <c r="F45" s="59" t="n"/>
+      <c r="G45" s="59" t="n"/>
+      <c r="H45" s="59" t="n"/>
+      <c r="I45" s="17">
+        <f>IF(COUNTA(C45:H45)=0,$I$8,COUNTA(C45:H45))</f>
+        <v/>
+      </c>
+      <c r="J45" s="26" t="n"/>
+      <c r="K45" s="60">
+        <f>IFERROR(IF('Course Content'!D32="","—",'Course Content'!D32),"")</f>
+        <v/>
+      </c>
+      <c r="L45" s="60">
+        <f>IFERROR(IF(K45="","",IF(K45="—","",FLOOR(K45/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M45" s="61">
+        <f>IFERROR(IF(L45="","",IF(L45="—","",FLOOR(L45/I45,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N45" s="26" t="n"/>
+      <c r="O45" s="62">
+        <f>IFERROR(IF('Course Content'!E32="","—",'Course Content'!E32),"")</f>
+        <v/>
+      </c>
+      <c r="P45" s="62">
+        <f>IFERROR(IF(O45="","",IF(O45="—","",FLOOR(O45/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q45" s="63">
+        <f>IFERROR(IF(P45="","",IF(P45="—","",FLOOR(P45/I45,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R45" s="65">
+        <f>IFERROR(IF('Course Content'!C32="","",'Course Content'!C32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="B46" s="66">
+        <f>IFERROR(IF('Course Content'!G32="","",'Course Content'!G32),"")</f>
+        <v/>
+      </c>
+      <c r="C46" s="67" t="n"/>
+      <c r="D46" s="67" t="n"/>
+      <c r="E46" s="67" t="n"/>
+      <c r="F46" s="67" t="n"/>
+      <c r="G46" s="67" t="n"/>
+      <c r="H46" s="67" t="n"/>
+      <c r="I46" s="68">
+        <f>IF(COUNTA(C46:H46)=0,$I$8,COUNTA(C46:H46))</f>
+        <v/>
+      </c>
+      <c r="J46" s="26" t="n"/>
+      <c r="K46" s="69">
+        <f>IFERROR(IF('Course Content'!I32="","—",'Course Content'!I32),"")</f>
+        <v/>
+      </c>
+      <c r="L46" s="69">
+        <f>IFERROR(IF(K46="","",IF(K46="—","",FLOOR(K46/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M46" s="70">
+        <f>IFERROR(IF(L46="","",IF(L46="—","",FLOOR(L46/I46,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N46" s="26" t="n"/>
+      <c r="O46" s="71">
+        <f>IFERROR(IF('Course Content'!J32="","—",'Course Content'!J32),"")</f>
+        <v/>
+      </c>
+      <c r="P46" s="71">
+        <f>IFERROR(IF(O46="","",IF(O46="—","",FLOOR(O46/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q46" s="72">
+        <f>IFERROR(IF(P46="","",IF(P46="—","",FLOOR(P46/I46,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R46" s="73">
+        <f>IFERROR(IF('Course Content'!H32="","",'Course Content'!H32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
+        </is>
+      </c>
+      <c r="B47" s="58">
+        <f>IFERROR(IF('Course Content'!B17="","",'Course Content'!B17),"")</f>
+        <v/>
+      </c>
+      <c r="C47" s="59" t="n"/>
+      <c r="D47" s="59" t="n"/>
+      <c r="E47" s="59" t="n"/>
+      <c r="F47" s="59" t="n"/>
+      <c r="G47" s="59" t="n"/>
+      <c r="H47" s="59" t="n"/>
+      <c r="I47" s="17">
+        <f>IF(COUNTA(C47:H47)=0,$I$8,COUNTA(C47:H47))</f>
+        <v/>
+      </c>
+      <c r="J47" s="26" t="n"/>
+      <c r="K47" s="60">
+        <f>IFERROR(IF('Course Content'!D17="","—",'Course Content'!D17),"")</f>
+        <v/>
+      </c>
+      <c r="L47" s="60">
+        <f>IFERROR(IF(K47="","",IF(K47="—","",FLOOR(K47/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M47" s="61">
+        <f>IFERROR(IF(L47="","",IF(L47="—","",FLOOR(L47/I47,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N47" s="26" t="n"/>
+      <c r="O47" s="62">
+        <f>IFERROR(IF('Course Content'!E17="","—",'Course Content'!E17),"")</f>
+        <v/>
+      </c>
+      <c r="P47" s="62">
+        <f>IFERROR(IF(O47="","",IF(O47="—","",FLOOR(O47/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q47" s="63">
+        <f>IFERROR(IF(P47="","",IF(P47="—","",FLOOR(P47/I47,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R47" s="64">
+        <f>IFERROR(IF('Course Content'!C17="","",'Course Content'!C17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="B48" s="58">
+        <f>IFERROR(IF('Course Content'!G17="","",'Course Content'!G17),"")</f>
+        <v/>
+      </c>
+      <c r="C48" s="59" t="n"/>
+      <c r="D48" s="59" t="n"/>
+      <c r="E48" s="59" t="n"/>
+      <c r="F48" s="59" t="n"/>
+      <c r="G48" s="59" t="n"/>
+      <c r="H48" s="59" t="n"/>
+      <c r="I48" s="17">
+        <f>IF(COUNTA(C48:H48)=0,$I$8,COUNTA(C48:H48))</f>
+        <v/>
+      </c>
+      <c r="J48" s="26" t="n"/>
+      <c r="K48" s="60">
+        <f>IFERROR(IF('Course Content'!I17="","—",'Course Content'!I17),"")</f>
+        <v/>
+      </c>
+      <c r="L48" s="60">
+        <f>IFERROR(IF(K48="","",IF(K48="—","",FLOOR(K48/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M48" s="61">
+        <f>IFERROR(IF(L48="","",IF(L48="—","",FLOOR(L48/I48,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N48" s="26" t="n"/>
+      <c r="O48" s="62">
+        <f>IFERROR(IF('Course Content'!J17="","—",'Course Content'!J17),"")</f>
+        <v/>
+      </c>
+      <c r="P48" s="62">
+        <f>IFERROR(IF(O48="","",IF(O48="—","",FLOOR(O48/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q48" s="63">
+        <f>IFERROR(IF(P48="","",IF(P48="—","",FLOOR(P48/I48,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R48" s="64">
+        <f>IFERROR(IF('Course Content'!H17="","",'Course Content'!H17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="B49" s="5">
+        <f>IFERROR(IF('Course Content'!B33="","",'Course Content'!B33),"")</f>
+        <v/>
+      </c>
+      <c r="C49" s="59" t="n"/>
+      <c r="D49" s="59" t="n"/>
+      <c r="E49" s="59" t="n"/>
+      <c r="F49" s="59" t="n"/>
+      <c r="G49" s="59" t="n"/>
+      <c r="H49" s="59" t="n"/>
+      <c r="I49" s="17">
+        <f>IF(COUNTA(C49:H49)=0,$I$8,COUNTA(C49:H49))</f>
+        <v/>
+      </c>
+      <c r="J49" s="26" t="n"/>
+      <c r="K49" s="60">
+        <f>IFERROR(IF('Course Content'!D33="","—",'Course Content'!D33),"")</f>
+        <v/>
+      </c>
+      <c r="L49" s="60">
+        <f>IFERROR(IF(K49="","",IF(K49="—","",FLOOR(K49/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M49" s="61">
+        <f>IFERROR(IF(L49="","",IF(L49="—","",FLOOR(L49/I49,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N49" s="26" t="n"/>
+      <c r="O49" s="62">
+        <f>IFERROR(IF('Course Content'!E33="","—",'Course Content'!E33),"")</f>
+        <v/>
+      </c>
+      <c r="P49" s="62">
+        <f>IFERROR(IF(O49="","",IF(O49="—","",FLOOR(O49/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q49" s="63">
+        <f>IFERROR(IF(P49="","",IF(P49="—","",FLOOR(P49/I49,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R49" s="65">
+        <f>IFERROR(IF('Course Content'!C33="","",'Course Content'!C33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="B50" s="66">
+        <f>IFERROR(IF('Course Content'!G33="","",'Course Content'!G33),"")</f>
+        <v/>
+      </c>
+      <c r="C50" s="67" t="n"/>
+      <c r="D50" s="67" t="n"/>
+      <c r="E50" s="67" t="n"/>
+      <c r="F50" s="67" t="n"/>
+      <c r="G50" s="67" t="n"/>
+      <c r="H50" s="67" t="n"/>
+      <c r="I50" s="68">
+        <f>IF(COUNTA(C50:H50)=0,$I$8,COUNTA(C50:H50))</f>
+        <v/>
+      </c>
+      <c r="J50" s="26" t="n"/>
+      <c r="K50" s="69">
+        <f>IFERROR(IF('Course Content'!I33="","—",'Course Content'!I33),"")</f>
+        <v/>
+      </c>
+      <c r="L50" s="69">
+        <f>IFERROR(IF(K50="","",IF(K50="—","",FLOOR(K50/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M50" s="70">
+        <f>IFERROR(IF(L50="","",IF(L50="—","",FLOOR(L50/I50,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N50" s="26" t="n"/>
+      <c r="O50" s="71">
+        <f>IFERROR(IF('Course Content'!J33="","—",'Course Content'!J33),"")</f>
+        <v/>
+      </c>
+      <c r="P50" s="71">
+        <f>IFERROR(IF(O50="","",IF(O50="—","",FLOOR(O50/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q50" s="72">
+        <f>IFERROR(IF(P50="","",IF(P50="—","",FLOOR(P50/I50,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R50" s="73">
+        <f>IFERROR(IF('Course Content'!H33="","",'Course Content'!H33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="31">
+        <f>IF('Course Content'!A34="Elective / Other 1","Elective / Other 1",'Course Content'!A34)</f>
+        <v/>
+      </c>
+      <c r="B51" s="58">
+        <f>IFERROR(IF('Course Content'!B18="","",'Course Content'!B18),"")</f>
+        <v/>
+      </c>
+      <c r="C51" s="59" t="n"/>
+      <c r="D51" s="59" t="n"/>
+      <c r="E51" s="59" t="n"/>
+      <c r="F51" s="59" t="n"/>
+      <c r="G51" s="59" t="n"/>
+      <c r="H51" s="59" t="n"/>
+      <c r="I51" s="17">
+        <f>IF(COUNTA(C51:H51)=0,$I$8,COUNTA(C51:H51))</f>
+        <v/>
+      </c>
+      <c r="J51" s="26" t="n"/>
+      <c r="K51" s="60">
+        <f>IFERROR(IF('Course Content'!D18="","—",'Course Content'!D18),"")</f>
+        <v/>
+      </c>
+      <c r="L51" s="60">
+        <f>IFERROR(IF(K51="","",IF(K51="—","",FLOOR(K51/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M51" s="61">
+        <f>IFERROR(IF(L51="","",IF(L51="—","",FLOOR(L51/I51,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N51" s="26" t="n"/>
+      <c r="O51" s="62">
+        <f>IFERROR(IF('Course Content'!E18="","—",'Course Content'!E18),"")</f>
+        <v/>
+      </c>
+      <c r="P51" s="62">
+        <f>IFERROR(IF(O51="","",IF(O51="—","",FLOOR(O51/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q51" s="63">
+        <f>IFERROR(IF(P51="","",IF(P51="—","",FLOOR(P51/I51,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R51" s="64">
+        <f>IFERROR(IF('Course Content'!C18="","",'Course Content'!C18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="B52" s="58">
+        <f>IFERROR(IF('Course Content'!G18="","",'Course Content'!G18),"")</f>
+        <v/>
+      </c>
+      <c r="C52" s="59" t="n"/>
+      <c r="D52" s="59" t="n"/>
+      <c r="E52" s="59" t="n"/>
+      <c r="F52" s="59" t="n"/>
+      <c r="G52" s="59" t="n"/>
+      <c r="H52" s="59" t="n"/>
+      <c r="I52" s="17">
+        <f>IF(COUNTA(C52:H52)=0,$I$8,COUNTA(C52:H52))</f>
+        <v/>
+      </c>
+      <c r="J52" s="26" t="n"/>
+      <c r="K52" s="60">
+        <f>IFERROR(IF('Course Content'!I18="","—",'Course Content'!I18),"")</f>
+        <v/>
+      </c>
+      <c r="L52" s="60">
+        <f>IFERROR(IF(K52="","",IF(K52="—","",FLOOR(K52/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M52" s="61">
+        <f>IFERROR(IF(L52="","",IF(L52="—","",FLOOR(L52/I52,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N52" s="26" t="n"/>
+      <c r="O52" s="62">
+        <f>IFERROR(IF('Course Content'!J18="","—",'Course Content'!J18),"")</f>
+        <v/>
+      </c>
+      <c r="P52" s="62">
+        <f>IFERROR(IF(O52="","",IF(O52="—","",FLOOR(O52/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q52" s="63">
+        <f>IFERROR(IF(P52="","",IF(P52="—","",FLOOR(P52/I52,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R52" s="64">
+        <f>IFERROR(IF('Course Content'!H18="","",'Course Content'!H18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="B53" s="5">
+        <f>IFERROR(IF('Course Content'!B34="","",'Course Content'!B34),"")</f>
+        <v/>
+      </c>
+      <c r="C53" s="59" t="n"/>
+      <c r="D53" s="59" t="n"/>
+      <c r="E53" s="59" t="n"/>
+      <c r="F53" s="59" t="n"/>
+      <c r="G53" s="59" t="n"/>
+      <c r="H53" s="59" t="n"/>
+      <c r="I53" s="17">
+        <f>IF(COUNTA(C53:H53)=0,$I$8,COUNTA(C53:H53))</f>
+        <v/>
+      </c>
+      <c r="J53" s="26" t="n"/>
+      <c r="K53" s="60">
+        <f>IFERROR(IF('Course Content'!D34="","—",'Course Content'!D34),"")</f>
+        <v/>
+      </c>
+      <c r="L53" s="60">
+        <f>IFERROR(IF(K53="","",IF(K53="—","",FLOOR(K53/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M53" s="61">
+        <f>IFERROR(IF(L53="","",IF(L53="—","",FLOOR(L53/I53,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N53" s="26" t="n"/>
+      <c r="O53" s="62">
+        <f>IFERROR(IF('Course Content'!E34="","—",'Course Content'!E34),"")</f>
+        <v/>
+      </c>
+      <c r="P53" s="62">
+        <f>IFERROR(IF(O53="","",IF(O53="—","",FLOOR(O53/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q53" s="63">
+        <f>IFERROR(IF(P53="","",IF(P53="—","",FLOOR(P53/I53,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R53" s="65">
+        <f>IFERROR(IF('Course Content'!C34="","",'Course Content'!C34),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="B54" s="66">
+        <f>IFERROR(IF('Course Content'!G34="","",'Course Content'!G34),"")</f>
+        <v/>
+      </c>
+      <c r="C54" s="67" t="n"/>
+      <c r="D54" s="67" t="n"/>
+      <c r="E54" s="67" t="n"/>
+      <c r="F54" s="67" t="n"/>
+      <c r="G54" s="67" t="n"/>
+      <c r="H54" s="67" t="n"/>
+      <c r="I54" s="68">
+        <f>IF(COUNTA(C54:H54)=0,$I$8,COUNTA(C54:H54))</f>
+        <v/>
+      </c>
+      <c r="J54" s="26" t="n"/>
+      <c r="K54" s="69">
+        <f>IFERROR(IF('Course Content'!I34="","—",'Course Content'!I34),"")</f>
+        <v/>
+      </c>
+      <c r="L54" s="69">
+        <f>IFERROR(IF(K54="","",IF(K54="—","",FLOOR(K54/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M54" s="70">
+        <f>IFERROR(IF(L54="","",IF(L54="—","",FLOOR(L54/I54,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N54" s="26" t="n"/>
+      <c r="O54" s="71">
+        <f>IFERROR(IF('Course Content'!J34="","—",'Course Content'!J34),"")</f>
+        <v/>
+      </c>
+      <c r="P54" s="71">
+        <f>IFERROR(IF(O54="","",IF(O54="—","",FLOOR(O54/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q54" s="72">
+        <f>IFERROR(IF(P54="","",IF(P54="—","",FLOOR(P54/I54,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R54" s="73">
+        <f>IFERROR(IF('Course Content'!H34="","",'Course Content'!H34),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="31">
+        <f>IF('Course Content'!A35="Elective / Other 2","Elective / Other 2",'Course Content'!A35)</f>
+        <v/>
+      </c>
+      <c r="B55" s="58">
+        <f>IFERROR(IF('Course Content'!B19="","",'Course Content'!B19),"")</f>
+        <v/>
+      </c>
+      <c r="C55" s="59" t="n"/>
+      <c r="D55" s="59" t="n"/>
+      <c r="E55" s="59" t="n"/>
+      <c r="F55" s="59" t="n"/>
+      <c r="G55" s="59" t="n"/>
+      <c r="H55" s="59" t="n"/>
+      <c r="I55" s="17">
+        <f>IF(COUNTA(C55:H55)=0,$I$8,COUNTA(C55:H55))</f>
+        <v/>
+      </c>
+      <c r="J55" s="26" t="n"/>
+      <c r="K55" s="60">
+        <f>IFERROR(IF('Course Content'!D19="","—",'Course Content'!D19),"")</f>
+        <v/>
+      </c>
+      <c r="L55" s="60">
+        <f>IFERROR(IF(K55="","",IF(K55="—","",FLOOR(K55/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M55" s="61">
+        <f>IFERROR(IF(L55="","",IF(L55="—","",FLOOR(L55/I55,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N55" s="26" t="n"/>
+      <c r="O55" s="62">
+        <f>IFERROR(IF('Course Content'!E19="","—",'Course Content'!E19),"")</f>
+        <v/>
+      </c>
+      <c r="P55" s="62">
+        <f>IFERROR(IF(O55="","",IF(O55="—","",FLOOR(O55/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q55" s="63">
+        <f>IFERROR(IF(P55="","",IF(P55="—","",FLOOR(P55/I55,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R55" s="64">
+        <f>IFERROR(IF('Course Content'!C19="","",'Course Content'!C19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="58">
+        <f>IFERROR(IF('Course Content'!G19="","",'Course Content'!G19),"")</f>
+        <v/>
+      </c>
+      <c r="C56" s="59" t="n"/>
+      <c r="D56" s="59" t="n"/>
+      <c r="E56" s="59" t="n"/>
+      <c r="F56" s="59" t="n"/>
+      <c r="G56" s="59" t="n"/>
+      <c r="H56" s="59" t="n"/>
+      <c r="I56" s="17">
+        <f>IF(COUNTA(C56:H56)=0,$I$8,COUNTA(C56:H56))</f>
+        <v/>
+      </c>
+      <c r="J56" s="26" t="n"/>
+      <c r="K56" s="60">
+        <f>IFERROR(IF('Course Content'!I19="","—",'Course Content'!I19),"")</f>
+        <v/>
+      </c>
+      <c r="L56" s="60">
+        <f>IFERROR(IF(K56="","",IF(K56="—","",FLOOR(K56/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M56" s="61">
+        <f>IFERROR(IF(L56="","",IF(L56="—","",FLOOR(L56/I56,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N56" s="26" t="n"/>
+      <c r="O56" s="62">
+        <f>IFERROR(IF('Course Content'!J19="","—",'Course Content'!J19),"")</f>
+        <v/>
+      </c>
+      <c r="P56" s="62">
+        <f>IFERROR(IF(O56="","",IF(O56="—","",FLOOR(O56/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q56" s="63">
+        <f>IFERROR(IF(P56="","",IF(P56="—","",FLOOR(P56/I56,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R56" s="64">
+        <f>IFERROR(IF('Course Content'!H19="","",'Course Content'!H19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="5">
+        <f>IFERROR(IF('Course Content'!B35="","",'Course Content'!B35),"")</f>
+        <v/>
+      </c>
+      <c r="C57" s="59" t="n"/>
+      <c r="D57" s="59" t="n"/>
+      <c r="E57" s="59" t="n"/>
+      <c r="F57" s="59" t="n"/>
+      <c r="G57" s="59" t="n"/>
+      <c r="H57" s="59" t="n"/>
+      <c r="I57" s="17">
+        <f>IF(COUNTA(C57:H57)=0,$I$8,COUNTA(C57:H57))</f>
+        <v/>
+      </c>
+      <c r="J57" s="26" t="n"/>
+      <c r="K57" s="60">
+        <f>IFERROR(IF('Course Content'!D35="","—",'Course Content'!D35),"")</f>
+        <v/>
+      </c>
+      <c r="L57" s="60">
+        <f>IFERROR(IF(K57="","",IF(K57="—","",FLOOR(K57/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M57" s="61">
+        <f>IFERROR(IF(L57="","",IF(L57="—","",FLOOR(L57/I57,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N57" s="26" t="n"/>
+      <c r="O57" s="62">
+        <f>IFERROR(IF('Course Content'!E35="","—",'Course Content'!E35),"")</f>
+        <v/>
+      </c>
+      <c r="P57" s="62">
+        <f>IFERROR(IF(O57="","",IF(O57="—","",FLOOR(O57/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q57" s="63">
+        <f>IFERROR(IF(P57="","",IF(P57="—","",FLOOR(P57/I57,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R57" s="65">
+        <f>IFERROR(IF('Course Content'!C35="","",'Course Content'!C35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="66">
+        <f>IFERROR(IF('Course Content'!G35="","",'Course Content'!G35),"")</f>
+        <v/>
+      </c>
+      <c r="C58" s="67" t="n"/>
+      <c r="D58" s="67" t="n"/>
+      <c r="E58" s="67" t="n"/>
+      <c r="F58" s="67" t="n"/>
+      <c r="G58" s="67" t="n"/>
+      <c r="H58" s="67" t="n"/>
+      <c r="I58" s="68">
+        <f>IF(COUNTA(C58:H58)=0,$I$8,COUNTA(C58:H58))</f>
+        <v/>
+      </c>
+      <c r="J58" s="26" t="n"/>
+      <c r="K58" s="69">
+        <f>IFERROR(IF('Course Content'!I35="","—",'Course Content'!I35),"")</f>
+        <v/>
+      </c>
+      <c r="L58" s="69">
+        <f>IFERROR(IF(K58="","",IF(K58="—","",FLOOR(K58/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M58" s="70">
+        <f>IFERROR(IF(L58="","",IF(L58="—","",FLOOR(L58/I58,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N58" s="26" t="n"/>
+      <c r="O58" s="71">
+        <f>IFERROR(IF('Course Content'!J35="","—",'Course Content'!J35),"")</f>
+        <v/>
+      </c>
+      <c r="P58" s="71">
+        <f>IFERROR(IF(O58="","",IF(O58="—","",FLOOR(O58/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q58" s="72">
+        <f>IFERROR(IF(P58="","",IF(P58="—","",FLOOR(P58/I58,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R58" s="73">
+        <f>IFERROR(IF('Course Content'!H35="","",'Course Content'!H35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="31">
+        <f>IF('Course Content'!A36="Elective / Other 3","Elective / Other 3",'Course Content'!A36)</f>
+        <v/>
+      </c>
+      <c r="B59" s="58">
+        <f>IFERROR(IF('Course Content'!B20="","",'Course Content'!B20),"")</f>
+        <v/>
+      </c>
+      <c r="C59" s="59" t="n"/>
+      <c r="D59" s="59" t="n"/>
+      <c r="E59" s="59" t="n"/>
+      <c r="F59" s="59" t="n"/>
+      <c r="G59" s="59" t="n"/>
+      <c r="H59" s="59" t="n"/>
+      <c r="I59" s="17">
+        <f>IF(COUNTA(C59:H59)=0,$I$8,COUNTA(C59:H59))</f>
+        <v/>
+      </c>
+      <c r="J59" s="26" t="n"/>
+      <c r="K59" s="60">
+        <f>IFERROR(IF('Course Content'!D20="","—",'Course Content'!D20),"")</f>
+        <v/>
+      </c>
+      <c r="L59" s="60">
+        <f>IFERROR(IF(K59="","",IF(K59="—","",FLOOR(K59/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M59" s="61">
+        <f>IFERROR(IF(L59="","",IF(L59="—","",FLOOR(L59/I59,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N59" s="26" t="n"/>
+      <c r="O59" s="62">
+        <f>IFERROR(IF('Course Content'!E20="","—",'Course Content'!E20),"")</f>
+        <v/>
+      </c>
+      <c r="P59" s="62">
+        <f>IFERROR(IF(O59="","",IF(O59="—","",FLOOR(O59/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q59" s="63">
+        <f>IFERROR(IF(P59="","",IF(P59="—","",FLOOR(P59/I59,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R59" s="64">
+        <f>IFERROR(IF('Course Content'!C20="","",'Course Content'!C20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="B60" s="58">
+        <f>IFERROR(IF('Course Content'!G20="","",'Course Content'!G20),"")</f>
+        <v/>
+      </c>
+      <c r="C60" s="59" t="n"/>
+      <c r="D60" s="59" t="n"/>
+      <c r="E60" s="59" t="n"/>
+      <c r="F60" s="59" t="n"/>
+      <c r="G60" s="59" t="n"/>
+      <c r="H60" s="59" t="n"/>
+      <c r="I60" s="17">
+        <f>IF(COUNTA(C60:H60)=0,$I$8,COUNTA(C60:H60))</f>
+        <v/>
+      </c>
+      <c r="J60" s="26" t="n"/>
+      <c r="K60" s="60">
+        <f>IFERROR(IF('Course Content'!I20="","—",'Course Content'!I20),"")</f>
+        <v/>
+      </c>
+      <c r="L60" s="60">
+        <f>IFERROR(IF(K60="","",IF(K60="—","",FLOOR(K60/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M60" s="61">
+        <f>IFERROR(IF(L60="","",IF(L60="—","",FLOOR(L60/I60,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N60" s="26" t="n"/>
+      <c r="O60" s="62">
+        <f>IFERROR(IF('Course Content'!J20="","—",'Course Content'!J20),"")</f>
+        <v/>
+      </c>
+      <c r="P60" s="62">
+        <f>IFERROR(IF(O60="","",IF(O60="—","",FLOOR(O60/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q60" s="63">
+        <f>IFERROR(IF(P60="","",IF(P60="—","",FLOOR(P60/I60,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R60" s="64">
+        <f>IFERROR(IF('Course Content'!H20="","",'Course Content'!H20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="B61" s="5">
+        <f>IFERROR(IF('Course Content'!B36="","",'Course Content'!B36),"")</f>
+        <v/>
+      </c>
+      <c r="C61" s="59" t="n"/>
+      <c r="D61" s="59" t="n"/>
+      <c r="E61" s="59" t="n"/>
+      <c r="F61" s="59" t="n"/>
+      <c r="G61" s="59" t="n"/>
+      <c r="H61" s="59" t="n"/>
+      <c r="I61" s="17">
+        <f>IF(COUNTA(C61:H61)=0,$I$8,COUNTA(C61:H61))</f>
+        <v/>
+      </c>
+      <c r="J61" s="26" t="n"/>
+      <c r="K61" s="60">
+        <f>IFERROR(IF('Course Content'!D36="","—",'Course Content'!D36),"")</f>
+        <v/>
+      </c>
+      <c r="L61" s="60">
+        <f>IFERROR(IF(K61="","",IF(K61="—","",FLOOR(K61/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M61" s="61">
+        <f>IFERROR(IF(L61="","",IF(L61="—","",FLOOR(L61/I61,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N61" s="26" t="n"/>
+      <c r="O61" s="62">
+        <f>IFERROR(IF('Course Content'!E36="","—",'Course Content'!E36),"")</f>
+        <v/>
+      </c>
+      <c r="P61" s="62">
+        <f>IFERROR(IF(O61="","",IF(O61="—","",FLOOR(O61/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q61" s="63">
+        <f>IFERROR(IF(P61="","",IF(P61="—","",FLOOR(P61/I61,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R61" s="65">
+        <f>IFERROR(IF('Course Content'!C36="","",'Course Content'!C36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="B62" s="66">
+        <f>IFERROR(IF('Course Content'!G36="","",'Course Content'!G36),"")</f>
+        <v/>
+      </c>
+      <c r="C62" s="67" t="n"/>
+      <c r="D62" s="67" t="n"/>
+      <c r="E62" s="67" t="n"/>
+      <c r="F62" s="67" t="n"/>
+      <c r="G62" s="67" t="n"/>
+      <c r="H62" s="67" t="n"/>
+      <c r="I62" s="68">
+        <f>IF(COUNTA(C62:H62)=0,$I$8,COUNTA(C62:H62))</f>
+        <v/>
+      </c>
+      <c r="J62" s="26" t="n"/>
+      <c r="K62" s="69">
+        <f>IFERROR(IF('Course Content'!I36="","—",'Course Content'!I36),"")</f>
+        <v/>
+      </c>
+      <c r="L62" s="69">
+        <f>IFERROR(IF(K62="","",IF(K62="—","",FLOOR(K62/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M62" s="70">
+        <f>IFERROR(IF(L62="","",IF(L62="—","",FLOOR(L62/I62,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N62" s="26" t="n"/>
+      <c r="O62" s="71">
+        <f>IFERROR(IF('Course Content'!J36="","—",'Course Content'!J36),"")</f>
+        <v/>
+      </c>
+      <c r="P62" s="71">
+        <f>IFERROR(IF(O62="","",IF(O62="—","",FLOOR(O62/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q62" s="72">
+        <f>IFERROR(IF(P62="","",IF(P62="—","",FLOOR(P62/I62,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R62" s="73">
+        <f>IFERROR(IF('Course Content'!H36="","",'Course Content'!H36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="31">
+        <f>IF('Course Content'!A37="Elective / Other 4","Elective / Other 4",'Course Content'!A37)</f>
+        <v/>
+      </c>
+      <c r="B63" s="58">
+        <f>IFERROR(IF('Course Content'!B21="","",'Course Content'!B21),"")</f>
+        <v/>
+      </c>
+      <c r="C63" s="59" t="n"/>
+      <c r="D63" s="59" t="n"/>
+      <c r="E63" s="59" t="n"/>
+      <c r="F63" s="59" t="n"/>
+      <c r="G63" s="59" t="n"/>
+      <c r="H63" s="59" t="n"/>
+      <c r="I63" s="17">
+        <f>IF(COUNTA(C63:H63)=0,$I$8,COUNTA(C63:H63))</f>
+        <v/>
+      </c>
+      <c r="J63" s="26" t="n"/>
+      <c r="K63" s="60">
+        <f>IFERROR(IF('Course Content'!D21="","—",'Course Content'!D21),"")</f>
+        <v/>
+      </c>
+      <c r="L63" s="60">
+        <f>IFERROR(IF(K63="","",IF(K63="—","",FLOOR(K63/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M63" s="61">
+        <f>IFERROR(IF(L63="","",IF(L63="—","",FLOOR(L63/I63,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N63" s="26" t="n"/>
+      <c r="O63" s="62">
+        <f>IFERROR(IF('Course Content'!E21="","—",'Course Content'!E21),"")</f>
+        <v/>
+      </c>
+      <c r="P63" s="62">
+        <f>IFERROR(IF(O63="","",IF(O63="—","",FLOOR(O63/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q63" s="63">
+        <f>IFERROR(IF(P63="","",IF(P63="—","",FLOOR(P63/I63,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R63" s="64">
+        <f>IFERROR(IF('Course Content'!C21="","",'Course Content'!C21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="58">
+        <f>IFERROR(IF('Course Content'!G21="","",'Course Content'!G21),"")</f>
+        <v/>
+      </c>
+      <c r="C64" s="59" t="n"/>
+      <c r="D64" s="59" t="n"/>
+      <c r="E64" s="59" t="n"/>
+      <c r="F64" s="59" t="n"/>
+      <c r="G64" s="59" t="n"/>
+      <c r="H64" s="59" t="n"/>
+      <c r="I64" s="17">
+        <f>IF(COUNTA(C64:H64)=0,$I$8,COUNTA(C64:H64))</f>
+        <v/>
+      </c>
+      <c r="J64" s="26" t="n"/>
+      <c r="K64" s="60">
+        <f>IFERROR(IF('Course Content'!I21="","—",'Course Content'!I21),"")</f>
+        <v/>
+      </c>
+      <c r="L64" s="60">
+        <f>IFERROR(IF(K64="","",IF(K64="—","",FLOOR(K64/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M64" s="61">
+        <f>IFERROR(IF(L64="","",IF(L64="—","",FLOOR(L64/I64,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N64" s="26" t="n"/>
+      <c r="O64" s="62">
+        <f>IFERROR(IF('Course Content'!J21="","—",'Course Content'!J21),"")</f>
+        <v/>
+      </c>
+      <c r="P64" s="62">
+        <f>IFERROR(IF(O64="","",IF(O64="—","",FLOOR(O64/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q64" s="63">
+        <f>IFERROR(IF(P64="","",IF(P64="—","",FLOOR(P64/I64,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R64" s="64">
+        <f>IFERROR(IF('Course Content'!H21="","",'Course Content'!H21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="5">
+        <f>IFERROR(IF('Course Content'!B37="","",'Course Content'!B37),"")</f>
+        <v/>
+      </c>
+      <c r="C65" s="59" t="n"/>
+      <c r="D65" s="59" t="n"/>
+      <c r="E65" s="59" t="n"/>
+      <c r="F65" s="59" t="n"/>
+      <c r="G65" s="59" t="n"/>
+      <c r="H65" s="59" t="n"/>
+      <c r="I65" s="17">
+        <f>IF(COUNTA(C65:H65)=0,$I$8,COUNTA(C65:H65))</f>
+        <v/>
+      </c>
+      <c r="J65" s="26" t="n"/>
+      <c r="K65" s="60">
+        <f>IFERROR(IF('Course Content'!D37="","—",'Course Content'!D37),"")</f>
+        <v/>
+      </c>
+      <c r="L65" s="60">
+        <f>IFERROR(IF(K65="","",IF(K65="—","",FLOOR(K65/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M65" s="61">
+        <f>IFERROR(IF(L65="","",IF(L65="—","",FLOOR(L65/I65,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N65" s="26" t="n"/>
+      <c r="O65" s="62">
+        <f>IFERROR(IF('Course Content'!E37="","—",'Course Content'!E37),"")</f>
+        <v/>
+      </c>
+      <c r="P65" s="62">
+        <f>IFERROR(IF(O65="","",IF(O65="—","",FLOOR(O65/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q65" s="63">
+        <f>IFERROR(IF(P65="","",IF(P65="—","",FLOOR(P65/I65,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R65" s="65">
+        <f>IFERROR(IF('Course Content'!C37="","",'Course Content'!C37),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="66">
+        <f>IFERROR(IF('Course Content'!G37="","",'Course Content'!G37),"")</f>
+        <v/>
+      </c>
+      <c r="C66" s="67" t="n"/>
+      <c r="D66" s="67" t="n"/>
+      <c r="E66" s="67" t="n"/>
+      <c r="F66" s="67" t="n"/>
+      <c r="G66" s="67" t="n"/>
+      <c r="H66" s="67" t="n"/>
+      <c r="I66" s="68">
+        <f>IF(COUNTA(C66:H66)=0,$I$8,COUNTA(C66:H66))</f>
+        <v/>
+      </c>
+      <c r="J66" s="26" t="n"/>
+      <c r="K66" s="69">
+        <f>IFERROR(IF('Course Content'!I37="","—",'Course Content'!I37),"")</f>
+        <v/>
+      </c>
+      <c r="L66" s="69">
+        <f>IFERROR(IF(K66="","",IF(K66="—","",FLOOR(K66/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M66" s="70">
+        <f>IFERROR(IF(L66="","",IF(L66="—","",FLOOR(L66/I66,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N66" s="26" t="n"/>
+      <c r="O66" s="71">
+        <f>IFERROR(IF('Course Content'!J37="","—",'Course Content'!J37),"")</f>
+        <v/>
+      </c>
+      <c r="P66" s="71">
+        <f>IFERROR(IF(O66="","",IF(O66="—","",FLOOR(O66/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q66" s="72">
+        <f>IFERROR(IF(P66="","",IF(P66="—","",FLOOR(P66/I66,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R66" s="73">
+        <f>IFERROR(IF('Course Content'!H37="","",'Course Content'!H37),"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="19">
+    <mergeCell ref="A11:A14"/>
     <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A6:R6"/>
+    <mergeCell ref="A55:A58"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A27:A30"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A63:A66"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="A31:A34"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="A39:A42"/>
     <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A59:A62"/>
+    <mergeCell ref="A35:A38"/>
     <mergeCell ref="K4:R4"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A6:R6"/>
+    <mergeCell ref="A51:A54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert to 1 row per subject; fix Course Content freeze pane
Student schedule back to 14 rows (1 per subject). Curriculum column
shows the first non-blank title without text wrapping so row heights
stay uniform. Totals still sum all 4 sources (Group Slot 1 & 2 +
Individual Slot 1 & 2). Fixed CC freeze pane to lock at first data row
so the Group Studies header is always visible when scrolling.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -311,7 +311,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -361,25 +361,11 @@
         <color rgb="00CE8282"/>
       </bottom>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D4C4BB"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D4C4BB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D4C4BB"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="00A08878"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -548,9 +534,6 @@
     <xf numFmtId="0" fontId="22" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -566,34 +549,10 @@
     <xf numFmtId="0" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5442,7 +5401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R66"/>
+  <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5665,2669 +5624,723 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Bible</t>
         </is>
       </c>
-      <c r="B11" s="58">
-        <f>IFERROR(IF('Course Content'!B8="","",'Course Content'!B8),"")</f>
-        <v/>
-      </c>
-      <c r="C11" s="59" t="n"/>
-      <c r="D11" s="59" t="n"/>
-      <c r="E11" s="59" t="n"/>
-      <c r="F11" s="59" t="n"/>
-      <c r="G11" s="59" t="n"/>
-      <c r="H11" s="59" t="n"/>
+      <c r="B11" s="5">
+        <f>IFERROR(IF('Course Content'!B24&lt;&gt;"",'Course Content'!B24,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,IF('Course Content'!G24&lt;&gt;"",'Course Content'!G24,IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="58" t="n"/>
+      <c r="E11" s="58" t="n"/>
+      <c r="F11" s="58" t="n"/>
+      <c r="G11" s="58" t="n"/>
+      <c r="H11" s="58" t="n"/>
       <c r="I11" s="17">
         <f>IF(COUNTA(C11:H11)=0,$I$8,COUNTA(C11:H11))</f>
         <v/>
       </c>
       <c r="J11" s="26" t="n"/>
-      <c r="K11" s="60">
-        <f>IFERROR(IF('Course Content'!D8="","—",'Course Content'!D8),"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="60">
+      <c r="K11" s="59">
+        <f>IFERROR(IF(('Course Content'!D8="")*('Course Content'!I8="")*('Course Content'!D24="")*('Course Content'!I24=""),"—",IFERROR('Course Content'!D8*1,0)+IFERROR('Course Content'!I8*1,0)+IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="59">
         <f>IFERROR(IF(K11="","",IF(K11="—","",FLOOR(K11/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M11" s="61">
+      <c r="M11" s="60">
         <f>IFERROR(IF(L11="","",IF(L11="—","",FLOOR(L11/I11,1))),"")</f>
         <v/>
       </c>
       <c r="N11" s="26" t="n"/>
-      <c r="O11" s="62">
-        <f>IFERROR(IF('Course Content'!E8="","—",'Course Content'!E8),"")</f>
-        <v/>
-      </c>
-      <c r="P11" s="62">
+      <c r="O11" s="61">
+        <f>IFERROR(IF(('Course Content'!E8="")*('Course Content'!J8="")*('Course Content'!E24="")*('Course Content'!J24=""),"—",IFERROR('Course Content'!E8*1,0)+IFERROR('Course Content'!J8*1,0)+IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="61">
         <f>IFERROR(IF(O11="","",IF(O11="—","",FLOOR(O11/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q11" s="63">
+      <c r="Q11" s="62">
         <f>IFERROR(IF(P11="","",IF(P11="—","",FLOOR(P11/I11,1))),"")</f>
         <v/>
       </c>
-      <c r="R11" s="64">
-        <f>IFERROR(IF('Course Content'!C8="","",'Course Content'!C8),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="58">
-        <f>IFERROR(IF('Course Content'!G8="","",'Course Content'!G8),"")</f>
-        <v/>
-      </c>
-      <c r="C12" s="59" t="n"/>
-      <c r="D12" s="59" t="n"/>
-      <c r="E12" s="59" t="n"/>
-      <c r="F12" s="59" t="n"/>
-      <c r="G12" s="59" t="n"/>
-      <c r="H12" s="59" t="n"/>
+      <c r="R11" s="63">
+        <f>IFERROR(IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,IF('Course Content'!H24&lt;&gt;"",'Course Content'!H24,IF('Course Content'!C8&lt;&gt;"",'Course Content'!C8,'Course Content'!H8))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>Math</t>
+        </is>
+      </c>
+      <c r="B12" s="18">
+        <f>IFERROR(IF('Course Content'!B25&lt;&gt;"",'Course Content'!B25,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,IF('Course Content'!G25&lt;&gt;"",'Course Content'!G25,IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C12" s="58" t="n"/>
+      <c r="D12" s="58" t="n"/>
+      <c r="E12" s="58" t="n"/>
+      <c r="F12" s="58" t="n"/>
+      <c r="G12" s="58" t="n"/>
+      <c r="H12" s="58" t="n"/>
       <c r="I12" s="17">
         <f>IF(COUNTA(C12:H12)=0,$I$8,COUNTA(C12:H12))</f>
         <v/>
       </c>
       <c r="J12" s="26" t="n"/>
-      <c r="K12" s="60">
-        <f>IFERROR(IF('Course Content'!I8="","—",'Course Content'!I8),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="60">
+      <c r="K12" s="59">
+        <f>IFERROR(IF(('Course Content'!D9="")*('Course Content'!I9="")*('Course Content'!D25="")*('Course Content'!I25=""),"—",IFERROR('Course Content'!D9*1,0)+IFERROR('Course Content'!I9*1,0)+IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="59">
         <f>IFERROR(IF(K12="","",IF(K12="—","",FLOOR(K12/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M12" s="61">
+      <c r="M12" s="60">
         <f>IFERROR(IF(L12="","",IF(L12="—","",FLOOR(L12/I12,1))),"")</f>
         <v/>
       </c>
       <c r="N12" s="26" t="n"/>
-      <c r="O12" s="62">
-        <f>IFERROR(IF('Course Content'!J8="","—",'Course Content'!J8),"")</f>
-        <v/>
-      </c>
-      <c r="P12" s="62">
+      <c r="O12" s="61">
+        <f>IFERROR(IF(('Course Content'!E9="")*('Course Content'!J9="")*('Course Content'!E25="")*('Course Content'!J25=""),"—",IFERROR('Course Content'!E9*1,0)+IFERROR('Course Content'!J9*1,0)+IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="61">
         <f>IFERROR(IF(O12="","",IF(O12="—","",FLOOR(O12/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q12" s="63">
+      <c r="Q12" s="62">
         <f>IFERROR(IF(P12="","",IF(P12="—","",FLOOR(P12/I12,1))),"")</f>
         <v/>
       </c>
       <c r="R12" s="64">
-        <f>IFERROR(IF('Course Content'!H8="","",'Course Content'!H8),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
+        <f>IFERROR(IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,IF('Course Content'!H25&lt;&gt;"",'Course Content'!H25,IF('Course Content'!C9&lt;&gt;"",'Course Content'!C9,'Course Content'!H9))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
+        </is>
+      </c>
       <c r="B13" s="5">
-        <f>IFERROR(IF('Course Content'!B24="","",'Course Content'!B24),"")</f>
-        <v/>
-      </c>
-      <c r="C13" s="59" t="n"/>
-      <c r="D13" s="59" t="n"/>
-      <c r="E13" s="59" t="n"/>
-      <c r="F13" s="59" t="n"/>
-      <c r="G13" s="59" t="n"/>
-      <c r="H13" s="59" t="n"/>
+        <f>IFERROR(IF('Course Content'!B26&lt;&gt;"",'Course Content'!B26,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,IF('Course Content'!G26&lt;&gt;"",'Course Content'!G26,IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C13" s="58" t="n"/>
+      <c r="D13" s="58" t="n"/>
+      <c r="E13" s="58" t="n"/>
+      <c r="F13" s="58" t="n"/>
+      <c r="G13" s="58" t="n"/>
+      <c r="H13" s="58" t="n"/>
       <c r="I13" s="17">
         <f>IF(COUNTA(C13:H13)=0,$I$8,COUNTA(C13:H13))</f>
         <v/>
       </c>
       <c r="J13" s="26" t="n"/>
-      <c r="K13" s="60">
-        <f>IFERROR(IF('Course Content'!D24="","—",'Course Content'!D24),"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="60">
+      <c r="K13" s="59">
+        <f>IFERROR(IF(('Course Content'!D10="")*('Course Content'!I10="")*('Course Content'!D26="")*('Course Content'!I26=""),"—",IFERROR('Course Content'!D10*1,0)+IFERROR('Course Content'!I10*1,0)+IFERROR('Course Content'!D26*1,0)+IFERROR('Course Content'!I26*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="59">
         <f>IFERROR(IF(K13="","",IF(K13="—","",FLOOR(K13/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M13" s="61">
+      <c r="M13" s="60">
         <f>IFERROR(IF(L13="","",IF(L13="—","",FLOOR(L13/I13,1))),"")</f>
         <v/>
       </c>
       <c r="N13" s="26" t="n"/>
-      <c r="O13" s="62">
-        <f>IFERROR(IF('Course Content'!E24="","—",'Course Content'!E24),"")</f>
-        <v/>
-      </c>
-      <c r="P13" s="62">
+      <c r="O13" s="61">
+        <f>IFERROR(IF(('Course Content'!E10="")*('Course Content'!J10="")*('Course Content'!E26="")*('Course Content'!J26=""),"—",IFERROR('Course Content'!E10*1,0)+IFERROR('Course Content'!J10*1,0)+IFERROR('Course Content'!E26*1,0)+IFERROR('Course Content'!J26*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="61">
         <f>IFERROR(IF(O13="","",IF(O13="—","",FLOOR(O13/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q13" s="63">
+      <c r="Q13" s="62">
         <f>IFERROR(IF(P13="","",IF(P13="—","",FLOOR(P13/I13,1))),"")</f>
         <v/>
       </c>
-      <c r="R13" s="65">
-        <f>IFERROR(IF('Course Content'!C24="","",'Course Content'!C24),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="66">
-        <f>IFERROR(IF('Course Content'!G24="","",'Course Content'!G24),"")</f>
-        <v/>
-      </c>
-      <c r="C14" s="67" t="n"/>
-      <c r="D14" s="67" t="n"/>
-      <c r="E14" s="67" t="n"/>
-      <c r="F14" s="67" t="n"/>
-      <c r="G14" s="67" t="n"/>
-      <c r="H14" s="67" t="n"/>
-      <c r="I14" s="68">
+      <c r="R13" s="63">
+        <f>IFERROR(IF('Course Content'!C26&lt;&gt;"",'Course Content'!C26,IF('Course Content'!H26&lt;&gt;"",'Course Content'!H26,IF('Course Content'!C10&lt;&gt;"",'Course Content'!C10,'Course Content'!H10))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B14" s="18">
+        <f>IFERROR(IF('Course Content'!B27&lt;&gt;"",'Course Content'!B27,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,IF('Course Content'!G27&lt;&gt;"",'Course Content'!G27,IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C14" s="58" t="n"/>
+      <c r="D14" s="58" t="n"/>
+      <c r="E14" s="58" t="n"/>
+      <c r="F14" s="58" t="n"/>
+      <c r="G14" s="58" t="n"/>
+      <c r="H14" s="58" t="n"/>
+      <c r="I14" s="17">
         <f>IF(COUNTA(C14:H14)=0,$I$8,COUNTA(C14:H14))</f>
         <v/>
       </c>
       <c r="J14" s="26" t="n"/>
-      <c r="K14" s="69">
-        <f>IFERROR(IF('Course Content'!I24="","—",'Course Content'!I24),"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="69">
+      <c r="K14" s="59">
+        <f>IFERROR(IF(('Course Content'!D11="")*('Course Content'!I11="")*('Course Content'!D27="")*('Course Content'!I27=""),"—",IFERROR('Course Content'!D11*1,0)+IFERROR('Course Content'!I11*1,0)+IFERROR('Course Content'!D27*1,0)+IFERROR('Course Content'!I27*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="59">
         <f>IFERROR(IF(K14="","",IF(K14="—","",FLOOR(K14/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M14" s="70">
+      <c r="M14" s="60">
         <f>IFERROR(IF(L14="","",IF(L14="—","",FLOOR(L14/I14,1))),"")</f>
         <v/>
       </c>
       <c r="N14" s="26" t="n"/>
-      <c r="O14" s="71">
-        <f>IFERROR(IF('Course Content'!J24="","—",'Course Content'!J24),"")</f>
-        <v/>
-      </c>
-      <c r="P14" s="71">
+      <c r="O14" s="61">
+        <f>IFERROR(IF(('Course Content'!E11="")*('Course Content'!J11="")*('Course Content'!E27="")*('Course Content'!J27=""),"—",IFERROR('Course Content'!E11*1,0)+IFERROR('Course Content'!J11*1,0)+IFERROR('Course Content'!E27*1,0)+IFERROR('Course Content'!J27*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="61">
         <f>IFERROR(IF(O14="","",IF(O14="—","",FLOOR(O14/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q14" s="72">
+      <c r="Q14" s="62">
         <f>IFERROR(IF(P14="","",IF(P14="—","",FLOOR(P14/I14,1))),"")</f>
         <v/>
       </c>
-      <c r="R14" s="73">
-        <f>IFERROR(IF('Course Content'!H24="","",'Course Content'!H24),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
+      <c r="R14" s="64">
+        <f>IFERROR(IF('Course Content'!C27&lt;&gt;"",'Course Content'!C27,IF('Course Content'!H27&lt;&gt;"",'Course Content'!H27,IF('Course Content'!C11&lt;&gt;"",'Course Content'!C11,'Course Content'!H11))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="31" t="inlineStr">
         <is>
-          <t>Math</t>
-        </is>
-      </c>
-      <c r="B15" s="58">
-        <f>IFERROR(IF('Course Content'!B9="","",'Course Content'!B9),"")</f>
-        <v/>
-      </c>
-      <c r="C15" s="59" t="n"/>
-      <c r="D15" s="59" t="n"/>
-      <c r="E15" s="59" t="n"/>
-      <c r="F15" s="59" t="n"/>
-      <c r="G15" s="59" t="n"/>
-      <c r="H15" s="59" t="n"/>
+          <t>Writing / Composition</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>IFERROR(IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="n"/>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="58" t="n"/>
+      <c r="H15" s="58" t="n"/>
       <c r="I15" s="17">
         <f>IF(COUNTA(C15:H15)=0,$I$8,COUNTA(C15:H15))</f>
         <v/>
       </c>
       <c r="J15" s="26" t="n"/>
-      <c r="K15" s="60">
-        <f>IFERROR(IF('Course Content'!D9="","—",'Course Content'!D9),"")</f>
-        <v/>
-      </c>
-      <c r="L15" s="60">
+      <c r="K15" s="59">
+        <f>IFERROR(IF(('Course Content'!D12="")*('Course Content'!I12="")*('Course Content'!D28="")*('Course Content'!I28=""),"—",IFERROR('Course Content'!D12*1,0)+IFERROR('Course Content'!I12*1,0)+IFERROR('Course Content'!D28*1,0)+IFERROR('Course Content'!I28*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="59">
         <f>IFERROR(IF(K15="","",IF(K15="—","",FLOOR(K15/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M15" s="61">
+      <c r="M15" s="60">
         <f>IFERROR(IF(L15="","",IF(L15="—","",FLOOR(L15/I15,1))),"")</f>
         <v/>
       </c>
       <c r="N15" s="26" t="n"/>
-      <c r="O15" s="62">
-        <f>IFERROR(IF('Course Content'!E9="","—",'Course Content'!E9),"")</f>
-        <v/>
-      </c>
-      <c r="P15" s="62">
+      <c r="O15" s="61">
+        <f>IFERROR(IF(('Course Content'!E12="")*('Course Content'!J12="")*('Course Content'!E28="")*('Course Content'!J28=""),"—",IFERROR('Course Content'!E12*1,0)+IFERROR('Course Content'!J12*1,0)+IFERROR('Course Content'!E28*1,0)+IFERROR('Course Content'!J28*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="61">
         <f>IFERROR(IF(O15="","",IF(O15="—","",FLOOR(O15/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q15" s="63">
+      <c r="Q15" s="62">
         <f>IFERROR(IF(P15="","",IF(P15="—","",FLOOR(P15/I15,1))),"")</f>
         <v/>
       </c>
-      <c r="R15" s="64">
-        <f>IFERROR(IF('Course Content'!C9="","",'Course Content'!C9),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="58">
-        <f>IFERROR(IF('Course Content'!G9="","",'Course Content'!G9),"")</f>
-        <v/>
-      </c>
-      <c r="C16" s="59" t="n"/>
-      <c r="D16" s="59" t="n"/>
-      <c r="E16" s="59" t="n"/>
-      <c r="F16" s="59" t="n"/>
-      <c r="G16" s="59" t="n"/>
-      <c r="H16" s="59" t="n"/>
+      <c r="R15" s="63">
+        <f>IFERROR(IF('Course Content'!C28&lt;&gt;"",'Course Content'!C28,IF('Course Content'!H28&lt;&gt;"",'Course Content'!H28,IF('Course Content'!C12&lt;&gt;"",'Course Content'!C12,'Course Content'!H12))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="B16" s="18">
+        <f>IFERROR(IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="n"/>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="58" t="n"/>
       <c r="I16" s="17">
         <f>IF(COUNTA(C16:H16)=0,$I$8,COUNTA(C16:H16))</f>
         <v/>
       </c>
       <c r="J16" s="26" t="n"/>
-      <c r="K16" s="60">
-        <f>IFERROR(IF('Course Content'!I9="","—",'Course Content'!I9),"")</f>
-        <v/>
-      </c>
-      <c r="L16" s="60">
+      <c r="K16" s="59">
+        <f>IFERROR(IF(('Course Content'!D13="")*('Course Content'!I13="")*('Course Content'!D29="")*('Course Content'!I29=""),"—",IFERROR('Course Content'!D13*1,0)+IFERROR('Course Content'!I13*1,0)+IFERROR('Course Content'!D29*1,0)+IFERROR('Course Content'!I29*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="59">
         <f>IFERROR(IF(K16="","",IF(K16="—","",FLOOR(K16/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M16" s="61">
+      <c r="M16" s="60">
         <f>IFERROR(IF(L16="","",IF(L16="—","",FLOOR(L16/I16,1))),"")</f>
         <v/>
       </c>
       <c r="N16" s="26" t="n"/>
-      <c r="O16" s="62">
-        <f>IFERROR(IF('Course Content'!J9="","—",'Course Content'!J9),"")</f>
-        <v/>
-      </c>
-      <c r="P16" s="62">
+      <c r="O16" s="61">
+        <f>IFERROR(IF(('Course Content'!E13="")*('Course Content'!J13="")*('Course Content'!E29="")*('Course Content'!J29=""),"—",IFERROR('Course Content'!E13*1,0)+IFERROR('Course Content'!J13*1,0)+IFERROR('Course Content'!E29*1,0)+IFERROR('Course Content'!J29*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="61">
         <f>IFERROR(IF(O16="","",IF(O16="—","",FLOOR(O16/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q16" s="63">
+      <c r="Q16" s="62">
         <f>IFERROR(IF(P16="","",IF(P16="—","",FLOOR(P16/I16,1))),"")</f>
         <v/>
       </c>
       <c r="R16" s="64">
-        <f>IFERROR(IF('Course Content'!H9="","",'Course Content'!H9),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
+        <f>IFERROR(IF('Course Content'!C29&lt;&gt;"",'Course Content'!C29,IF('Course Content'!H29&lt;&gt;"",'Course Content'!H29,IF('Course Content'!C13&lt;&gt;"",'Course Content'!C13,'Course Content'!H13))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
+        </is>
+      </c>
       <c r="B17" s="5">
-        <f>IFERROR(IF('Course Content'!B25="","",'Course Content'!B25),"")</f>
-        <v/>
-      </c>
-      <c r="C17" s="59" t="n"/>
-      <c r="D17" s="59" t="n"/>
-      <c r="E17" s="59" t="n"/>
-      <c r="F17" s="59" t="n"/>
-      <c r="G17" s="59" t="n"/>
-      <c r="H17" s="59" t="n"/>
+        <f>IFERROR(IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C17" s="58" t="n"/>
+      <c r="D17" s="58" t="n"/>
+      <c r="E17" s="58" t="n"/>
+      <c r="F17" s="58" t="n"/>
+      <c r="G17" s="58" t="n"/>
+      <c r="H17" s="58" t="n"/>
       <c r="I17" s="17">
         <f>IF(COUNTA(C17:H17)=0,$I$8,COUNTA(C17:H17))</f>
         <v/>
       </c>
       <c r="J17" s="26" t="n"/>
-      <c r="K17" s="60">
-        <f>IFERROR(IF('Course Content'!D25="","—",'Course Content'!D25),"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="60">
+      <c r="K17" s="59">
+        <f>IFERROR(IF(('Course Content'!D14="")*('Course Content'!I14="")*('Course Content'!D30="")*('Course Content'!I30=""),"—",IFERROR('Course Content'!D14*1,0)+IFERROR('Course Content'!I14*1,0)+IFERROR('Course Content'!D30*1,0)+IFERROR('Course Content'!I30*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="59">
         <f>IFERROR(IF(K17="","",IF(K17="—","",FLOOR(K17/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M17" s="61">
+      <c r="M17" s="60">
         <f>IFERROR(IF(L17="","",IF(L17="—","",FLOOR(L17/I17,1))),"")</f>
         <v/>
       </c>
       <c r="N17" s="26" t="n"/>
-      <c r="O17" s="62">
-        <f>IFERROR(IF('Course Content'!E25="","—",'Course Content'!E25),"")</f>
-        <v/>
-      </c>
-      <c r="P17" s="62">
+      <c r="O17" s="61">
+        <f>IFERROR(IF(('Course Content'!E14="")*('Course Content'!J14="")*('Course Content'!E30="")*('Course Content'!J30=""),"—",IFERROR('Course Content'!E14*1,0)+IFERROR('Course Content'!J14*1,0)+IFERROR('Course Content'!E30*1,0)+IFERROR('Course Content'!J30*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="61">
         <f>IFERROR(IF(O17="","",IF(O17="—","",FLOOR(O17/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q17" s="63">
+      <c r="Q17" s="62">
         <f>IFERROR(IF(P17="","",IF(P17="—","",FLOOR(P17/I17,1))),"")</f>
         <v/>
       </c>
-      <c r="R17" s="65">
-        <f>IFERROR(IF('Course Content'!C25="","",'Course Content'!C25),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="66">
-        <f>IFERROR(IF('Course Content'!G25="","",'Course Content'!G25),"")</f>
-        <v/>
-      </c>
-      <c r="C18" s="67" t="n"/>
-      <c r="D18" s="67" t="n"/>
-      <c r="E18" s="67" t="n"/>
-      <c r="F18" s="67" t="n"/>
-      <c r="G18" s="67" t="n"/>
-      <c r="H18" s="67" t="n"/>
-      <c r="I18" s="68">
+      <c r="R17" s="63">
+        <f>IFERROR(IF('Course Content'!C30&lt;&gt;"",'Course Content'!C30,IF('Course Content'!H30&lt;&gt;"",'Course Content'!H30,IF('Course Content'!C14&lt;&gt;"",'Course Content'!C14,'Course Content'!H14))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B18" s="18">
+        <f>IFERROR(IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C18" s="58" t="n"/>
+      <c r="D18" s="58" t="n"/>
+      <c r="E18" s="58" t="n"/>
+      <c r="F18" s="58" t="n"/>
+      <c r="G18" s="58" t="n"/>
+      <c r="H18" s="58" t="n"/>
+      <c r="I18" s="17">
         <f>IF(COUNTA(C18:H18)=0,$I$8,COUNTA(C18:H18))</f>
         <v/>
       </c>
       <c r="J18" s="26" t="n"/>
-      <c r="K18" s="69">
-        <f>IFERROR(IF('Course Content'!I25="","—",'Course Content'!I25),"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="69">
+      <c r="K18" s="59">
+        <f>IFERROR(IF(('Course Content'!D15="")*('Course Content'!I15="")*('Course Content'!D31="")*('Course Content'!I31=""),"—",IFERROR('Course Content'!D15*1,0)+IFERROR('Course Content'!I15*1,0)+IFERROR('Course Content'!D31*1,0)+IFERROR('Course Content'!I31*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="59">
         <f>IFERROR(IF(K18="","",IF(K18="—","",FLOOR(K18/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M18" s="70">
+      <c r="M18" s="60">
         <f>IFERROR(IF(L18="","",IF(L18="—","",FLOOR(L18/I18,1))),"")</f>
         <v/>
       </c>
       <c r="N18" s="26" t="n"/>
-      <c r="O18" s="71">
-        <f>IFERROR(IF('Course Content'!J25="","—",'Course Content'!J25),"")</f>
-        <v/>
-      </c>
-      <c r="P18" s="71">
+      <c r="O18" s="61">
+        <f>IFERROR(IF(('Course Content'!E15="")*('Course Content'!J15="")*('Course Content'!E31="")*('Course Content'!J31=""),"—",IFERROR('Course Content'!E15*1,0)+IFERROR('Course Content'!J15*1,0)+IFERROR('Course Content'!E31*1,0)+IFERROR('Course Content'!J31*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="61">
         <f>IFERROR(IF(O18="","",IF(O18="—","",FLOOR(O18/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q18" s="72">
+      <c r="Q18" s="62">
         <f>IFERROR(IF(P18="","",IF(P18="—","",FLOOR(P18/I18,1))),"")</f>
         <v/>
       </c>
-      <c r="R18" s="73">
-        <f>IFERROR(IF('Course Content'!H25="","",'Course Content'!H25),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
+      <c r="R18" s="64">
+        <f>IFERROR(IF('Course Content'!C31&lt;&gt;"",'Course Content'!C31,IF('Course Content'!H31&lt;&gt;"",'Course Content'!H31,IF('Course Content'!C15&lt;&gt;"",'Course Content'!C15,'Course Content'!H15))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
       <c r="A19" s="31" t="inlineStr">
         <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B19" s="58">
-        <f>IFERROR(IF('Course Content'!B10="","",'Course Content'!B10),"")</f>
-        <v/>
-      </c>
-      <c r="C19" s="59" t="n"/>
-      <c r="D19" s="59" t="n"/>
-      <c r="E19" s="59" t="n"/>
-      <c r="F19" s="59" t="n"/>
-      <c r="G19" s="59" t="n"/>
-      <c r="H19" s="59" t="n"/>
+          <t>Physical Education</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>IFERROR(IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C19" s="58" t="n"/>
+      <c r="D19" s="58" t="n"/>
+      <c r="E19" s="58" t="n"/>
+      <c r="F19" s="58" t="n"/>
+      <c r="G19" s="58" t="n"/>
+      <c r="H19" s="58" t="n"/>
       <c r="I19" s="17">
         <f>IF(COUNTA(C19:H19)=0,$I$8,COUNTA(C19:H19))</f>
         <v/>
       </c>
       <c r="J19" s="26" t="n"/>
-      <c r="K19" s="60">
-        <f>IFERROR(IF('Course Content'!D10="","—",'Course Content'!D10),"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="60">
+      <c r="K19" s="59">
+        <f>IFERROR(IF(('Course Content'!D16="")*('Course Content'!I16="")*('Course Content'!D32="")*('Course Content'!I32=""),"—",IFERROR('Course Content'!D16*1,0)+IFERROR('Course Content'!I16*1,0)+IFERROR('Course Content'!D32*1,0)+IFERROR('Course Content'!I32*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="59">
         <f>IFERROR(IF(K19="","",IF(K19="—","",FLOOR(K19/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M19" s="61">
+      <c r="M19" s="60">
         <f>IFERROR(IF(L19="","",IF(L19="—","",FLOOR(L19/I19,1))),"")</f>
         <v/>
       </c>
       <c r="N19" s="26" t="n"/>
-      <c r="O19" s="62">
-        <f>IFERROR(IF('Course Content'!E10="","—",'Course Content'!E10),"")</f>
-        <v/>
-      </c>
-      <c r="P19" s="62">
+      <c r="O19" s="61">
+        <f>IFERROR(IF(('Course Content'!E16="")*('Course Content'!J16="")*('Course Content'!E32="")*('Course Content'!J32=""),"—",IFERROR('Course Content'!E16*1,0)+IFERROR('Course Content'!J16*1,0)+IFERROR('Course Content'!E32*1,0)+IFERROR('Course Content'!J32*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="61">
         <f>IFERROR(IF(O19="","",IF(O19="—","",FLOOR(O19/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q19" s="63">
+      <c r="Q19" s="62">
         <f>IFERROR(IF(P19="","",IF(P19="—","",FLOOR(P19/I19,1))),"")</f>
         <v/>
       </c>
-      <c r="R19" s="64">
-        <f>IFERROR(IF('Course Content'!C10="","",'Course Content'!C10),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="B20" s="58">
-        <f>IFERROR(IF('Course Content'!G10="","",'Course Content'!G10),"")</f>
-        <v/>
-      </c>
-      <c r="C20" s="59" t="n"/>
-      <c r="D20" s="59" t="n"/>
-      <c r="E20" s="59" t="n"/>
-      <c r="F20" s="59" t="n"/>
-      <c r="G20" s="59" t="n"/>
-      <c r="H20" s="59" t="n"/>
+      <c r="R19" s="63">
+        <f>IFERROR(IF('Course Content'!C32&lt;&gt;"",'Course Content'!C32,IF('Course Content'!H32&lt;&gt;"",'Course Content'!H32,IF('Course Content'!C16&lt;&gt;"",'Course Content'!C16,'Course Content'!H16))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>IFERROR(IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C20" s="58" t="n"/>
+      <c r="D20" s="58" t="n"/>
+      <c r="E20" s="58" t="n"/>
+      <c r="F20" s="58" t="n"/>
+      <c r="G20" s="58" t="n"/>
+      <c r="H20" s="58" t="n"/>
       <c r="I20" s="17">
         <f>IF(COUNTA(C20:H20)=0,$I$8,COUNTA(C20:H20))</f>
         <v/>
       </c>
       <c r="J20" s="26" t="n"/>
-      <c r="K20" s="60">
-        <f>IFERROR(IF('Course Content'!I10="","—",'Course Content'!I10),"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="60">
+      <c r="K20" s="59">
+        <f>IFERROR(IF(('Course Content'!D17="")*('Course Content'!I17="")*('Course Content'!D33="")*('Course Content'!I33=""),"—",IFERROR('Course Content'!D17*1,0)+IFERROR('Course Content'!I17*1,0)+IFERROR('Course Content'!D33*1,0)+IFERROR('Course Content'!I33*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="59">
         <f>IFERROR(IF(K20="","",IF(K20="—","",FLOOR(K20/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M20" s="61">
+      <c r="M20" s="60">
         <f>IFERROR(IF(L20="","",IF(L20="—","",FLOOR(L20/I20,1))),"")</f>
         <v/>
       </c>
       <c r="N20" s="26" t="n"/>
-      <c r="O20" s="62">
-        <f>IFERROR(IF('Course Content'!J10="","—",'Course Content'!J10),"")</f>
-        <v/>
-      </c>
-      <c r="P20" s="62">
+      <c r="O20" s="61">
+        <f>IFERROR(IF(('Course Content'!E17="")*('Course Content'!J17="")*('Course Content'!E33="")*('Course Content'!J33=""),"—",IFERROR('Course Content'!E17*1,0)+IFERROR('Course Content'!J17*1,0)+IFERROR('Course Content'!E33*1,0)+IFERROR('Course Content'!J33*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P20" s="61">
         <f>IFERROR(IF(O20="","",IF(O20="—","",FLOOR(O20/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q20" s="63">
+      <c r="Q20" s="62">
         <f>IFERROR(IF(P20="","",IF(P20="—","",FLOOR(P20/I20,1))),"")</f>
         <v/>
       </c>
       <c r="R20" s="64">
-        <f>IFERROR(IF('Course Content'!H10="","",'Course Content'!H10),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
+        <f>IFERROR(IF('Course Content'!C33&lt;&gt;"",'Course Content'!C33,IF('Course Content'!H33&lt;&gt;"",'Course Content'!H33,IF('Course Content'!C17&lt;&gt;"",'Course Content'!C17,'Course Content'!H17))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="31">
+        <f>IF('Course Content'!A34="Elective / Other 1","Elective / Other 1",'Course Content'!A34)</f>
+        <v/>
+      </c>
       <c r="B21" s="5">
-        <f>IFERROR(IF('Course Content'!B26="","",'Course Content'!B26),"")</f>
-        <v/>
-      </c>
-      <c r="C21" s="59" t="n"/>
-      <c r="D21" s="59" t="n"/>
-      <c r="E21" s="59" t="n"/>
-      <c r="F21" s="59" t="n"/>
-      <c r="G21" s="59" t="n"/>
-      <c r="H21" s="59" t="n"/>
+        <f>IFERROR(IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C21" s="58" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="58" t="n"/>
+      <c r="F21" s="58" t="n"/>
+      <c r="G21" s="58" t="n"/>
+      <c r="H21" s="58" t="n"/>
       <c r="I21" s="17">
         <f>IF(COUNTA(C21:H21)=0,$I$8,COUNTA(C21:H21))</f>
         <v/>
       </c>
       <c r="J21" s="26" t="n"/>
-      <c r="K21" s="60">
-        <f>IFERROR(IF('Course Content'!D26="","—",'Course Content'!D26),"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="60">
+      <c r="K21" s="59">
+        <f>IFERROR(IF(('Course Content'!D18="")*('Course Content'!I18="")*('Course Content'!D34="")*('Course Content'!I34=""),"—",IFERROR('Course Content'!D18*1,0)+IFERROR('Course Content'!I18*1,0)+IFERROR('Course Content'!D34*1,0)+IFERROR('Course Content'!I34*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="59">
         <f>IFERROR(IF(K21="","",IF(K21="—","",FLOOR(K21/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M21" s="61">
+      <c r="M21" s="60">
         <f>IFERROR(IF(L21="","",IF(L21="—","",FLOOR(L21/I21,1))),"")</f>
         <v/>
       </c>
       <c r="N21" s="26" t="n"/>
-      <c r="O21" s="62">
-        <f>IFERROR(IF('Course Content'!E26="","—",'Course Content'!E26),"")</f>
-        <v/>
-      </c>
-      <c r="P21" s="62">
+      <c r="O21" s="61">
+        <f>IFERROR(IF(('Course Content'!E18="")*('Course Content'!J18="")*('Course Content'!E34="")*('Course Content'!J34=""),"—",IFERROR('Course Content'!E18*1,0)+IFERROR('Course Content'!J18*1,0)+IFERROR('Course Content'!E34*1,0)+IFERROR('Course Content'!J34*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P21" s="61">
         <f>IFERROR(IF(O21="","",IF(O21="—","",FLOOR(O21/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q21" s="63">
+      <c r="Q21" s="62">
         <f>IFERROR(IF(P21="","",IF(P21="—","",FLOOR(P21/I21,1))),"")</f>
         <v/>
       </c>
-      <c r="R21" s="65">
-        <f>IFERROR(IF('Course Content'!C26="","",'Course Content'!C26),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="B22" s="66">
-        <f>IFERROR(IF('Course Content'!G26="","",'Course Content'!G26),"")</f>
-        <v/>
-      </c>
-      <c r="C22" s="67" t="n"/>
-      <c r="D22" s="67" t="n"/>
-      <c r="E22" s="67" t="n"/>
-      <c r="F22" s="67" t="n"/>
-      <c r="G22" s="67" t="n"/>
-      <c r="H22" s="67" t="n"/>
-      <c r="I22" s="68">
+      <c r="R21" s="63">
+        <f>IFERROR(IF('Course Content'!C34&lt;&gt;"",'Course Content'!C34,IF('Course Content'!H34&lt;&gt;"",'Course Content'!H34,IF('Course Content'!C18&lt;&gt;"",'Course Content'!C18,'Course Content'!H18))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="31">
+        <f>IF('Course Content'!A35="Elective / Other 2","Elective / Other 2",'Course Content'!A35)</f>
+        <v/>
+      </c>
+      <c r="B22" s="18">
+        <f>IFERROR(IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C22" s="58" t="n"/>
+      <c r="D22" s="58" t="n"/>
+      <c r="E22" s="58" t="n"/>
+      <c r="F22" s="58" t="n"/>
+      <c r="G22" s="58" t="n"/>
+      <c r="H22" s="58" t="n"/>
+      <c r="I22" s="17">
         <f>IF(COUNTA(C22:H22)=0,$I$8,COUNTA(C22:H22))</f>
         <v/>
       </c>
       <c r="J22" s="26" t="n"/>
-      <c r="K22" s="69">
-        <f>IFERROR(IF('Course Content'!I26="","—",'Course Content'!I26),"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="69">
+      <c r="K22" s="59">
+        <f>IFERROR(IF(('Course Content'!D19="")*('Course Content'!I19="")*('Course Content'!D35="")*('Course Content'!I35=""),"—",IFERROR('Course Content'!D19*1,0)+IFERROR('Course Content'!I19*1,0)+IFERROR('Course Content'!D35*1,0)+IFERROR('Course Content'!I35*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="59">
         <f>IFERROR(IF(K22="","",IF(K22="—","",FLOOR(K22/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M22" s="70">
+      <c r="M22" s="60">
         <f>IFERROR(IF(L22="","",IF(L22="—","",FLOOR(L22/I22,1))),"")</f>
         <v/>
       </c>
       <c r="N22" s="26" t="n"/>
-      <c r="O22" s="71">
-        <f>IFERROR(IF('Course Content'!J26="","—",'Course Content'!J26),"")</f>
-        <v/>
-      </c>
-      <c r="P22" s="71">
+      <c r="O22" s="61">
+        <f>IFERROR(IF(('Course Content'!E19="")*('Course Content'!J19="")*('Course Content'!E35="")*('Course Content'!J35=""),"—",IFERROR('Course Content'!E19*1,0)+IFERROR('Course Content'!J19*1,0)+IFERROR('Course Content'!E35*1,0)+IFERROR('Course Content'!J35*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="61">
         <f>IFERROR(IF(O22="","",IF(O22="—","",FLOOR(O22/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q22" s="72">
+      <c r="Q22" s="62">
         <f>IFERROR(IF(P22="","",IF(P22="—","",FLOOR(P22/I22,1))),"")</f>
         <v/>
       </c>
-      <c r="R22" s="73">
-        <f>IFERROR(IF('Course Content'!H26="","",'Course Content'!H26),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B23" s="58">
-        <f>IFERROR(IF('Course Content'!B11="","",'Course Content'!B11),"")</f>
-        <v/>
-      </c>
-      <c r="C23" s="59" t="n"/>
-      <c r="D23" s="59" t="n"/>
-      <c r="E23" s="59" t="n"/>
-      <c r="F23" s="59" t="n"/>
-      <c r="G23" s="59" t="n"/>
-      <c r="H23" s="59" t="n"/>
+      <c r="R22" s="64">
+        <f>IFERROR(IF('Course Content'!C35&lt;&gt;"",'Course Content'!C35,IF('Course Content'!H35&lt;&gt;"",'Course Content'!H35,IF('Course Content'!C19&lt;&gt;"",'Course Content'!C19,'Course Content'!H19))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="31">
+        <f>IF('Course Content'!A36="Elective / Other 3","Elective / Other 3",'Course Content'!A36)</f>
+        <v/>
+      </c>
+      <c r="B23" s="5">
+        <f>IFERROR(IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C23" s="58" t="n"/>
+      <c r="D23" s="58" t="n"/>
+      <c r="E23" s="58" t="n"/>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="58" t="n"/>
+      <c r="H23" s="58" t="n"/>
       <c r="I23" s="17">
         <f>IF(COUNTA(C23:H23)=0,$I$8,COUNTA(C23:H23))</f>
         <v/>
       </c>
       <c r="J23" s="26" t="n"/>
-      <c r="K23" s="60">
-        <f>IFERROR(IF('Course Content'!D11="","—",'Course Content'!D11),"")</f>
-        <v/>
-      </c>
-      <c r="L23" s="60">
+      <c r="K23" s="59">
+        <f>IFERROR(IF(('Course Content'!D20="")*('Course Content'!I20="")*('Course Content'!D36="")*('Course Content'!I36=""),"—",IFERROR('Course Content'!D20*1,0)+IFERROR('Course Content'!I20*1,0)+IFERROR('Course Content'!D36*1,0)+IFERROR('Course Content'!I36*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="59">
         <f>IFERROR(IF(K23="","",IF(K23="—","",FLOOR(K23/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M23" s="61">
+      <c r="M23" s="60">
         <f>IFERROR(IF(L23="","",IF(L23="—","",FLOOR(L23/I23,1))),"")</f>
         <v/>
       </c>
       <c r="N23" s="26" t="n"/>
-      <c r="O23" s="62">
-        <f>IFERROR(IF('Course Content'!E11="","—",'Course Content'!E11),"")</f>
-        <v/>
-      </c>
-      <c r="P23" s="62">
+      <c r="O23" s="61">
+        <f>IFERROR(IF(('Course Content'!E20="")*('Course Content'!J20="")*('Course Content'!E36="")*('Course Content'!J36=""),"—",IFERROR('Course Content'!E20*1,0)+IFERROR('Course Content'!J20*1,0)+IFERROR('Course Content'!E36*1,0)+IFERROR('Course Content'!J36*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P23" s="61">
         <f>IFERROR(IF(O23="","",IF(O23="—","",FLOOR(O23/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q23" s="63">
+      <c r="Q23" s="62">
         <f>IFERROR(IF(P23="","",IF(P23="—","",FLOOR(P23/I23,1))),"")</f>
         <v/>
       </c>
-      <c r="R23" s="64">
-        <f>IFERROR(IF('Course Content'!C11="","",'Course Content'!C11),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="B24" s="58">
-        <f>IFERROR(IF('Course Content'!G11="","",'Course Content'!G11),"")</f>
-        <v/>
-      </c>
-      <c r="C24" s="59" t="n"/>
-      <c r="D24" s="59" t="n"/>
-      <c r="E24" s="59" t="n"/>
-      <c r="F24" s="59" t="n"/>
-      <c r="G24" s="59" t="n"/>
-      <c r="H24" s="59" t="n"/>
+      <c r="R23" s="63">
+        <f>IFERROR(IF('Course Content'!C36&lt;&gt;"",'Course Content'!C36,IF('Course Content'!H36&lt;&gt;"",'Course Content'!H36,IF('Course Content'!C20&lt;&gt;"",'Course Content'!C20,'Course Content'!H20))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="31">
+        <f>IF('Course Content'!A37="Elective / Other 4","Elective / Other 4",'Course Content'!A37)</f>
+        <v/>
+      </c>
+      <c r="B24" s="18">
+        <f>IFERROR(IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C24" s="58" t="n"/>
+      <c r="D24" s="58" t="n"/>
+      <c r="E24" s="58" t="n"/>
+      <c r="F24" s="58" t="n"/>
+      <c r="G24" s="58" t="n"/>
+      <c r="H24" s="58" t="n"/>
       <c r="I24" s="17">
         <f>IF(COUNTA(C24:H24)=0,$I$8,COUNTA(C24:H24))</f>
         <v/>
       </c>
       <c r="J24" s="26" t="n"/>
-      <c r="K24" s="60">
-        <f>IFERROR(IF('Course Content'!I11="","—",'Course Content'!I11),"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="60">
+      <c r="K24" s="59">
+        <f>IFERROR(IF(('Course Content'!D21="")*('Course Content'!I21="")*('Course Content'!D37="")*('Course Content'!I37=""),"—",IFERROR('Course Content'!D21*1,0)+IFERROR('Course Content'!I21*1,0)+IFERROR('Course Content'!D37*1,0)+IFERROR('Course Content'!I37*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="59">
         <f>IFERROR(IF(K24="","",IF(K24="—","",FLOOR(K24/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M24" s="61">
+      <c r="M24" s="60">
         <f>IFERROR(IF(L24="","",IF(L24="—","",FLOOR(L24/I24,1))),"")</f>
         <v/>
       </c>
       <c r="N24" s="26" t="n"/>
-      <c r="O24" s="62">
-        <f>IFERROR(IF('Course Content'!J11="","—",'Course Content'!J11),"")</f>
-        <v/>
-      </c>
-      <c r="P24" s="62">
+      <c r="O24" s="61">
+        <f>IFERROR(IF(('Course Content'!E21="")*('Course Content'!J21="")*('Course Content'!E37="")*('Course Content'!J37=""),"—",IFERROR('Course Content'!E21*1,0)+IFERROR('Course Content'!J21*1,0)+IFERROR('Course Content'!E37*1,0)+IFERROR('Course Content'!J37*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P24" s="61">
         <f>IFERROR(IF(O24="","",IF(O24="—","",FLOOR(O24/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q24" s="63">
+      <c r="Q24" s="62">
         <f>IFERROR(IF(P24="","",IF(P24="—","",FLOOR(P24/I24,1))),"")</f>
         <v/>
       </c>
       <c r="R24" s="64">
-        <f>IFERROR(IF('Course Content'!H11="","",'Course Content'!H11),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="B25" s="5">
-        <f>IFERROR(IF('Course Content'!B27="","",'Course Content'!B27),"")</f>
-        <v/>
-      </c>
-      <c r="C25" s="59" t="n"/>
-      <c r="D25" s="59" t="n"/>
-      <c r="E25" s="59" t="n"/>
-      <c r="F25" s="59" t="n"/>
-      <c r="G25" s="59" t="n"/>
-      <c r="H25" s="59" t="n"/>
-      <c r="I25" s="17">
-        <f>IF(COUNTA(C25:H25)=0,$I$8,COUNTA(C25:H25))</f>
-        <v/>
-      </c>
-      <c r="J25" s="26" t="n"/>
-      <c r="K25" s="60">
-        <f>IFERROR(IF('Course Content'!D27="","—",'Course Content'!D27),"")</f>
-        <v/>
-      </c>
-      <c r="L25" s="60">
-        <f>IFERROR(IF(K25="","",IF(K25="—","",FLOOR(K25/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M25" s="61">
-        <f>IFERROR(IF(L25="","",IF(L25="—","",FLOOR(L25/I25,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N25" s="26" t="n"/>
-      <c r="O25" s="62">
-        <f>IFERROR(IF('Course Content'!E27="","—",'Course Content'!E27),"")</f>
-        <v/>
-      </c>
-      <c r="P25" s="62">
-        <f>IFERROR(IF(O25="","",IF(O25="—","",FLOOR(O25/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q25" s="63">
-        <f>IFERROR(IF(P25="","",IF(P25="—","",FLOOR(P25/I25,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R25" s="65">
-        <f>IFERROR(IF('Course Content'!C27="","",'Course Content'!C27),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="B26" s="66">
-        <f>IFERROR(IF('Course Content'!G27="","",'Course Content'!G27),"")</f>
-        <v/>
-      </c>
-      <c r="C26" s="67" t="n"/>
-      <c r="D26" s="67" t="n"/>
-      <c r="E26" s="67" t="n"/>
-      <c r="F26" s="67" t="n"/>
-      <c r="G26" s="67" t="n"/>
-      <c r="H26" s="67" t="n"/>
-      <c r="I26" s="68">
-        <f>IF(COUNTA(C26:H26)=0,$I$8,COUNTA(C26:H26))</f>
-        <v/>
-      </c>
-      <c r="J26" s="26" t="n"/>
-      <c r="K26" s="69">
-        <f>IFERROR(IF('Course Content'!I27="","—",'Course Content'!I27),"")</f>
-        <v/>
-      </c>
-      <c r="L26" s="69">
-        <f>IFERROR(IF(K26="","",IF(K26="—","",FLOOR(K26/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M26" s="70">
-        <f>IFERROR(IF(L26="","",IF(L26="—","",FLOOR(L26/I26,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N26" s="26" t="n"/>
-      <c r="O26" s="71">
-        <f>IFERROR(IF('Course Content'!J27="","—",'Course Content'!J27),"")</f>
-        <v/>
-      </c>
-      <c r="P26" s="71">
-        <f>IFERROR(IF(O26="","",IF(O26="—","",FLOOR(O26/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q26" s="72">
-        <f>IFERROR(IF(P26="","",IF(P26="—","",FLOOR(P26/I26,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R26" s="73">
-        <f>IFERROR(IF('Course Content'!H27="","",'Course Content'!H27),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t>Writing / Composition</t>
-        </is>
-      </c>
-      <c r="B27" s="58">
-        <f>IFERROR(IF('Course Content'!B12="","",'Course Content'!B12),"")</f>
-        <v/>
-      </c>
-      <c r="C27" s="59" t="n"/>
-      <c r="D27" s="59" t="n"/>
-      <c r="E27" s="59" t="n"/>
-      <c r="F27" s="59" t="n"/>
-      <c r="G27" s="59" t="n"/>
-      <c r="H27" s="59" t="n"/>
-      <c r="I27" s="17">
-        <f>IF(COUNTA(C27:H27)=0,$I$8,COUNTA(C27:H27))</f>
-        <v/>
-      </c>
-      <c r="J27" s="26" t="n"/>
-      <c r="K27" s="60">
-        <f>IFERROR(IF('Course Content'!D12="","—",'Course Content'!D12),"")</f>
-        <v/>
-      </c>
-      <c r="L27" s="60">
-        <f>IFERROR(IF(K27="","",IF(K27="—","",FLOOR(K27/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="61">
-        <f>IFERROR(IF(L27="","",IF(L27="—","",FLOOR(L27/I27,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N27" s="26" t="n"/>
-      <c r="O27" s="62">
-        <f>IFERROR(IF('Course Content'!E12="","—",'Course Content'!E12),"")</f>
-        <v/>
-      </c>
-      <c r="P27" s="62">
-        <f>IFERROR(IF(O27="","",IF(O27="—","",FLOOR(O27/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q27" s="63">
-        <f>IFERROR(IF(P27="","",IF(P27="—","",FLOOR(P27/I27,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R27" s="64">
-        <f>IFERROR(IF('Course Content'!C12="","",'Course Content'!C12),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="B28" s="58">
-        <f>IFERROR(IF('Course Content'!G12="","",'Course Content'!G12),"")</f>
-        <v/>
-      </c>
-      <c r="C28" s="59" t="n"/>
-      <c r="D28" s="59" t="n"/>
-      <c r="E28" s="59" t="n"/>
-      <c r="F28" s="59" t="n"/>
-      <c r="G28" s="59" t="n"/>
-      <c r="H28" s="59" t="n"/>
-      <c r="I28" s="17">
-        <f>IF(COUNTA(C28:H28)=0,$I$8,COUNTA(C28:H28))</f>
-        <v/>
-      </c>
-      <c r="J28" s="26" t="n"/>
-      <c r="K28" s="60">
-        <f>IFERROR(IF('Course Content'!I12="","—",'Course Content'!I12),"")</f>
-        <v/>
-      </c>
-      <c r="L28" s="60">
-        <f>IFERROR(IF(K28="","",IF(K28="—","",FLOOR(K28/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="61">
-        <f>IFERROR(IF(L28="","",IF(L28="—","",FLOOR(L28/I28,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N28" s="26" t="n"/>
-      <c r="O28" s="62">
-        <f>IFERROR(IF('Course Content'!J12="","—",'Course Content'!J12),"")</f>
-        <v/>
-      </c>
-      <c r="P28" s="62">
-        <f>IFERROR(IF(O28="","",IF(O28="—","",FLOOR(O28/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q28" s="63">
-        <f>IFERROR(IF(P28="","",IF(P28="—","",FLOOR(P28/I28,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R28" s="64">
-        <f>IFERROR(IF('Course Content'!H12="","",'Course Content'!H12),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="5">
-        <f>IFERROR(IF('Course Content'!B28="","",'Course Content'!B28),"")</f>
-        <v/>
-      </c>
-      <c r="C29" s="59" t="n"/>
-      <c r="D29" s="59" t="n"/>
-      <c r="E29" s="59" t="n"/>
-      <c r="F29" s="59" t="n"/>
-      <c r="G29" s="59" t="n"/>
-      <c r="H29" s="59" t="n"/>
-      <c r="I29" s="17">
-        <f>IF(COUNTA(C29:H29)=0,$I$8,COUNTA(C29:H29))</f>
-        <v/>
-      </c>
-      <c r="J29" s="26" t="n"/>
-      <c r="K29" s="60">
-        <f>IFERROR(IF('Course Content'!D28="","—",'Course Content'!D28),"")</f>
-        <v/>
-      </c>
-      <c r="L29" s="60">
-        <f>IFERROR(IF(K29="","",IF(K29="—","",FLOOR(K29/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="61">
-        <f>IFERROR(IF(L29="","",IF(L29="—","",FLOOR(L29/I29,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N29" s="26" t="n"/>
-      <c r="O29" s="62">
-        <f>IFERROR(IF('Course Content'!E28="","—",'Course Content'!E28),"")</f>
-        <v/>
-      </c>
-      <c r="P29" s="62">
-        <f>IFERROR(IF(O29="","",IF(O29="—","",FLOOR(O29/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q29" s="63">
-        <f>IFERROR(IF(P29="","",IF(P29="—","",FLOOR(P29/I29,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R29" s="65">
-        <f>IFERROR(IF('Course Content'!C28="","",'Course Content'!C28),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="B30" s="66">
-        <f>IFERROR(IF('Course Content'!G28="","",'Course Content'!G28),"")</f>
-        <v/>
-      </c>
-      <c r="C30" s="67" t="n"/>
-      <c r="D30" s="67" t="n"/>
-      <c r="E30" s="67" t="n"/>
-      <c r="F30" s="67" t="n"/>
-      <c r="G30" s="67" t="n"/>
-      <c r="H30" s="67" t="n"/>
-      <c r="I30" s="68">
-        <f>IF(COUNTA(C30:H30)=0,$I$8,COUNTA(C30:H30))</f>
-        <v/>
-      </c>
-      <c r="J30" s="26" t="n"/>
-      <c r="K30" s="69">
-        <f>IFERROR(IF('Course Content'!I28="","—",'Course Content'!I28),"")</f>
-        <v/>
-      </c>
-      <c r="L30" s="69">
-        <f>IFERROR(IF(K30="","",IF(K30="—","",FLOOR(K30/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="70">
-        <f>IFERROR(IF(L30="","",IF(L30="—","",FLOOR(L30/I30,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N30" s="26" t="n"/>
-      <c r="O30" s="71">
-        <f>IFERROR(IF('Course Content'!J28="","—",'Course Content'!J28),"")</f>
-        <v/>
-      </c>
-      <c r="P30" s="71">
-        <f>IFERROR(IF(O30="","",IF(O30="—","",FLOOR(O30/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q30" s="72">
-        <f>IFERROR(IF(P30="","",IF(P30="—","",FLOOR(P30/I30,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R30" s="73">
-        <f>IFERROR(IF('Course Content'!H28="","",'Course Content'!H28),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="31" t="inlineStr">
-        <is>
-          <t>Science</t>
-        </is>
-      </c>
-      <c r="B31" s="58">
-        <f>IFERROR(IF('Course Content'!B13="","",'Course Content'!B13),"")</f>
-        <v/>
-      </c>
-      <c r="C31" s="59" t="n"/>
-      <c r="D31" s="59" t="n"/>
-      <c r="E31" s="59" t="n"/>
-      <c r="F31" s="59" t="n"/>
-      <c r="G31" s="59" t="n"/>
-      <c r="H31" s="59" t="n"/>
-      <c r="I31" s="17">
-        <f>IF(COUNTA(C31:H31)=0,$I$8,COUNTA(C31:H31))</f>
-        <v/>
-      </c>
-      <c r="J31" s="26" t="n"/>
-      <c r="K31" s="60">
-        <f>IFERROR(IF('Course Content'!D13="","—",'Course Content'!D13),"")</f>
-        <v/>
-      </c>
-      <c r="L31" s="60">
-        <f>IFERROR(IF(K31="","",IF(K31="—","",FLOOR(K31/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M31" s="61">
-        <f>IFERROR(IF(L31="","",IF(L31="—","",FLOOR(L31/I31,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N31" s="26" t="n"/>
-      <c r="O31" s="62">
-        <f>IFERROR(IF('Course Content'!E13="","—",'Course Content'!E13),"")</f>
-        <v/>
-      </c>
-      <c r="P31" s="62">
-        <f>IFERROR(IF(O31="","",IF(O31="—","",FLOOR(O31/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q31" s="63">
-        <f>IFERROR(IF(P31="","",IF(P31="—","",FLOOR(P31/I31,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R31" s="64">
-        <f>IFERROR(IF('Course Content'!C13="","",'Course Content'!C13),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="58">
-        <f>IFERROR(IF('Course Content'!G13="","",'Course Content'!G13),"")</f>
-        <v/>
-      </c>
-      <c r="C32" s="59" t="n"/>
-      <c r="D32" s="59" t="n"/>
-      <c r="E32" s="59" t="n"/>
-      <c r="F32" s="59" t="n"/>
-      <c r="G32" s="59" t="n"/>
-      <c r="H32" s="59" t="n"/>
-      <c r="I32" s="17">
-        <f>IF(COUNTA(C32:H32)=0,$I$8,COUNTA(C32:H32))</f>
-        <v/>
-      </c>
-      <c r="J32" s="26" t="n"/>
-      <c r="K32" s="60">
-        <f>IFERROR(IF('Course Content'!I13="","—",'Course Content'!I13),"")</f>
-        <v/>
-      </c>
-      <c r="L32" s="60">
-        <f>IFERROR(IF(K32="","",IF(K32="—","",FLOOR(K32/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="61">
-        <f>IFERROR(IF(L32="","",IF(L32="—","",FLOOR(L32/I32,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N32" s="26" t="n"/>
-      <c r="O32" s="62">
-        <f>IFERROR(IF('Course Content'!J13="","—",'Course Content'!J13),"")</f>
-        <v/>
-      </c>
-      <c r="P32" s="62">
-        <f>IFERROR(IF(O32="","",IF(O32="—","",FLOOR(O32/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q32" s="63">
-        <f>IFERROR(IF(P32="","",IF(P32="—","",FLOOR(P32/I32,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R32" s="64">
-        <f>IFERROR(IF('Course Content'!H13="","",'Course Content'!H13),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="B33" s="5">
-        <f>IFERROR(IF('Course Content'!B29="","",'Course Content'!B29),"")</f>
-        <v/>
-      </c>
-      <c r="C33" s="59" t="n"/>
-      <c r="D33" s="59" t="n"/>
-      <c r="E33" s="59" t="n"/>
-      <c r="F33" s="59" t="n"/>
-      <c r="G33" s="59" t="n"/>
-      <c r="H33" s="59" t="n"/>
-      <c r="I33" s="17">
-        <f>IF(COUNTA(C33:H33)=0,$I$8,COUNTA(C33:H33))</f>
-        <v/>
-      </c>
-      <c r="J33" s="26" t="n"/>
-      <c r="K33" s="60">
-        <f>IFERROR(IF('Course Content'!D29="","—",'Course Content'!D29),"")</f>
-        <v/>
-      </c>
-      <c r="L33" s="60">
-        <f>IFERROR(IF(K33="","",IF(K33="—","",FLOOR(K33/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="61">
-        <f>IFERROR(IF(L33="","",IF(L33="—","",FLOOR(L33/I33,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N33" s="26" t="n"/>
-      <c r="O33" s="62">
-        <f>IFERROR(IF('Course Content'!E29="","—",'Course Content'!E29),"")</f>
-        <v/>
-      </c>
-      <c r="P33" s="62">
-        <f>IFERROR(IF(O33="","",IF(O33="—","",FLOOR(O33/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q33" s="63">
-        <f>IFERROR(IF(P33="","",IF(P33="—","",FLOOR(P33/I33,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R33" s="65">
-        <f>IFERROR(IF('Course Content'!C29="","",'Course Content'!C29),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="B34" s="66">
-        <f>IFERROR(IF('Course Content'!G29="","",'Course Content'!G29),"")</f>
-        <v/>
-      </c>
-      <c r="C34" s="67" t="n"/>
-      <c r="D34" s="67" t="n"/>
-      <c r="E34" s="67" t="n"/>
-      <c r="F34" s="67" t="n"/>
-      <c r="G34" s="67" t="n"/>
-      <c r="H34" s="67" t="n"/>
-      <c r="I34" s="68">
-        <f>IF(COUNTA(C34:H34)=0,$I$8,COUNTA(C34:H34))</f>
-        <v/>
-      </c>
-      <c r="J34" s="26" t="n"/>
-      <c r="K34" s="69">
-        <f>IFERROR(IF('Course Content'!I29="","—",'Course Content'!I29),"")</f>
-        <v/>
-      </c>
-      <c r="L34" s="69">
-        <f>IFERROR(IF(K34="","",IF(K34="—","",FLOOR(K34/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M34" s="70">
-        <f>IFERROR(IF(L34="","",IF(L34="—","",FLOOR(L34/I34,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N34" s="26" t="n"/>
-      <c r="O34" s="71">
-        <f>IFERROR(IF('Course Content'!J29="","—",'Course Content'!J29),"")</f>
-        <v/>
-      </c>
-      <c r="P34" s="71">
-        <f>IFERROR(IF(O34="","",IF(O34="—","",FLOOR(O34/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q34" s="72">
-        <f>IFERROR(IF(P34="","",IF(P34="—","",FLOOR(P34/I34,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R34" s="73">
-        <f>IFERROR(IF('Course Content'!H29="","",'Course Content'!H29),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
-        </is>
-      </c>
-      <c r="B35" s="58">
-        <f>IFERROR(IF('Course Content'!B14="","",'Course Content'!B14),"")</f>
-        <v/>
-      </c>
-      <c r="C35" s="59" t="n"/>
-      <c r="D35" s="59" t="n"/>
-      <c r="E35" s="59" t="n"/>
-      <c r="F35" s="59" t="n"/>
-      <c r="G35" s="59" t="n"/>
-      <c r="H35" s="59" t="n"/>
-      <c r="I35" s="17">
-        <f>IF(COUNTA(C35:H35)=0,$I$8,COUNTA(C35:H35))</f>
-        <v/>
-      </c>
-      <c r="J35" s="26" t="n"/>
-      <c r="K35" s="60">
-        <f>IFERROR(IF('Course Content'!D14="","—",'Course Content'!D14),"")</f>
-        <v/>
-      </c>
-      <c r="L35" s="60">
-        <f>IFERROR(IF(K35="","",IF(K35="—","",FLOOR(K35/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M35" s="61">
-        <f>IFERROR(IF(L35="","",IF(L35="—","",FLOOR(L35/I35,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N35" s="26" t="n"/>
-      <c r="O35" s="62">
-        <f>IFERROR(IF('Course Content'!E14="","—",'Course Content'!E14),"")</f>
-        <v/>
-      </c>
-      <c r="P35" s="62">
-        <f>IFERROR(IF(O35="","",IF(O35="—","",FLOOR(O35/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q35" s="63">
-        <f>IFERROR(IF(P35="","",IF(P35="—","",FLOOR(P35/I35,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R35" s="64">
-        <f>IFERROR(IF('Course Content'!C14="","",'Course Content'!C14),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="58">
-        <f>IFERROR(IF('Course Content'!G14="","",'Course Content'!G14),"")</f>
-        <v/>
-      </c>
-      <c r="C36" s="59" t="n"/>
-      <c r="D36" s="59" t="n"/>
-      <c r="E36" s="59" t="n"/>
-      <c r="F36" s="59" t="n"/>
-      <c r="G36" s="59" t="n"/>
-      <c r="H36" s="59" t="n"/>
-      <c r="I36" s="17">
-        <f>IF(COUNTA(C36:H36)=0,$I$8,COUNTA(C36:H36))</f>
-        <v/>
-      </c>
-      <c r="J36" s="26" t="n"/>
-      <c r="K36" s="60">
-        <f>IFERROR(IF('Course Content'!I14="","—",'Course Content'!I14),"")</f>
-        <v/>
-      </c>
-      <c r="L36" s="60">
-        <f>IFERROR(IF(K36="","",IF(K36="—","",FLOOR(K36/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M36" s="61">
-        <f>IFERROR(IF(L36="","",IF(L36="—","",FLOOR(L36/I36,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N36" s="26" t="n"/>
-      <c r="O36" s="62">
-        <f>IFERROR(IF('Course Content'!J14="","—",'Course Content'!J14),"")</f>
-        <v/>
-      </c>
-      <c r="P36" s="62">
-        <f>IFERROR(IF(O36="","",IF(O36="—","",FLOOR(O36/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q36" s="63">
-        <f>IFERROR(IF(P36="","",IF(P36="—","",FLOOR(P36/I36,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R36" s="64">
-        <f>IFERROR(IF('Course Content'!H14="","",'Course Content'!H14),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="5">
-        <f>IFERROR(IF('Course Content'!B30="","",'Course Content'!B30),"")</f>
-        <v/>
-      </c>
-      <c r="C37" s="59" t="n"/>
-      <c r="D37" s="59" t="n"/>
-      <c r="E37" s="59" t="n"/>
-      <c r="F37" s="59" t="n"/>
-      <c r="G37" s="59" t="n"/>
-      <c r="H37" s="59" t="n"/>
-      <c r="I37" s="17">
-        <f>IF(COUNTA(C37:H37)=0,$I$8,COUNTA(C37:H37))</f>
-        <v/>
-      </c>
-      <c r="J37" s="26" t="n"/>
-      <c r="K37" s="60">
-        <f>IFERROR(IF('Course Content'!D30="","—",'Course Content'!D30),"")</f>
-        <v/>
-      </c>
-      <c r="L37" s="60">
-        <f>IFERROR(IF(K37="","",IF(K37="—","",FLOOR(K37/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M37" s="61">
-        <f>IFERROR(IF(L37="","",IF(L37="—","",FLOOR(L37/I37,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N37" s="26" t="n"/>
-      <c r="O37" s="62">
-        <f>IFERROR(IF('Course Content'!E30="","—",'Course Content'!E30),"")</f>
-        <v/>
-      </c>
-      <c r="P37" s="62">
-        <f>IFERROR(IF(O37="","",IF(O37="—","",FLOOR(O37/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q37" s="63">
-        <f>IFERROR(IF(P37="","",IF(P37="—","",FLOOR(P37/I37,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R37" s="65">
-        <f>IFERROR(IF('Course Content'!C30="","",'Course Content'!C30),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="66">
-        <f>IFERROR(IF('Course Content'!G30="","",'Course Content'!G30),"")</f>
-        <v/>
-      </c>
-      <c r="C38" s="67" t="n"/>
-      <c r="D38" s="67" t="n"/>
-      <c r="E38" s="67" t="n"/>
-      <c r="F38" s="67" t="n"/>
-      <c r="G38" s="67" t="n"/>
-      <c r="H38" s="67" t="n"/>
-      <c r="I38" s="68">
-        <f>IF(COUNTA(C38:H38)=0,$I$8,COUNTA(C38:H38))</f>
-        <v/>
-      </c>
-      <c r="J38" s="26" t="n"/>
-      <c r="K38" s="69">
-        <f>IFERROR(IF('Course Content'!I30="","—",'Course Content'!I30),"")</f>
-        <v/>
-      </c>
-      <c r="L38" s="69">
-        <f>IFERROR(IF(K38="","",IF(K38="—","",FLOOR(K38/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M38" s="70">
-        <f>IFERROR(IF(L38="","",IF(L38="—","",FLOOR(L38/I38,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N38" s="26" t="n"/>
-      <c r="O38" s="71">
-        <f>IFERROR(IF('Course Content'!J30="","—",'Course Content'!J30),"")</f>
-        <v/>
-      </c>
-      <c r="P38" s="71">
-        <f>IFERROR(IF(O38="","",IF(O38="—","",FLOOR(O38/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q38" s="72">
-        <f>IFERROR(IF(P38="","",IF(P38="—","",FLOOR(P38/I38,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R38" s="73">
-        <f>IFERROR(IF('Course Content'!H30="","",'Course Content'!H30),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
-        </is>
-      </c>
-      <c r="B39" s="58">
-        <f>IFERROR(IF('Course Content'!B15="","",'Course Content'!B15),"")</f>
-        <v/>
-      </c>
-      <c r="C39" s="59" t="n"/>
-      <c r="D39" s="59" t="n"/>
-      <c r="E39" s="59" t="n"/>
-      <c r="F39" s="59" t="n"/>
-      <c r="G39" s="59" t="n"/>
-      <c r="H39" s="59" t="n"/>
-      <c r="I39" s="17">
-        <f>IF(COUNTA(C39:H39)=0,$I$8,COUNTA(C39:H39))</f>
-        <v/>
-      </c>
-      <c r="J39" s="26" t="n"/>
-      <c r="K39" s="60">
-        <f>IFERROR(IF('Course Content'!D15="","—",'Course Content'!D15),"")</f>
-        <v/>
-      </c>
-      <c r="L39" s="60">
-        <f>IFERROR(IF(K39="","",IF(K39="—","",FLOOR(K39/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M39" s="61">
-        <f>IFERROR(IF(L39="","",IF(L39="—","",FLOOR(L39/I39,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N39" s="26" t="n"/>
-      <c r="O39" s="62">
-        <f>IFERROR(IF('Course Content'!E15="","—",'Course Content'!E15),"")</f>
-        <v/>
-      </c>
-      <c r="P39" s="62">
-        <f>IFERROR(IF(O39="","",IF(O39="—","",FLOOR(O39/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q39" s="63">
-        <f>IFERROR(IF(P39="","",IF(P39="—","",FLOOR(P39/I39,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R39" s="64">
-        <f>IFERROR(IF('Course Content'!C15="","",'Course Content'!C15),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="58">
-        <f>IFERROR(IF('Course Content'!G15="","",'Course Content'!G15),"")</f>
-        <v/>
-      </c>
-      <c r="C40" s="59" t="n"/>
-      <c r="D40" s="59" t="n"/>
-      <c r="E40" s="59" t="n"/>
-      <c r="F40" s="59" t="n"/>
-      <c r="G40" s="59" t="n"/>
-      <c r="H40" s="59" t="n"/>
-      <c r="I40" s="17">
-        <f>IF(COUNTA(C40:H40)=0,$I$8,COUNTA(C40:H40))</f>
-        <v/>
-      </c>
-      <c r="J40" s="26" t="n"/>
-      <c r="K40" s="60">
-        <f>IFERROR(IF('Course Content'!I15="","—",'Course Content'!I15),"")</f>
-        <v/>
-      </c>
-      <c r="L40" s="60">
-        <f>IFERROR(IF(K40="","",IF(K40="—","",FLOOR(K40/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M40" s="61">
-        <f>IFERROR(IF(L40="","",IF(L40="—","",FLOOR(L40/I40,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N40" s="26" t="n"/>
-      <c r="O40" s="62">
-        <f>IFERROR(IF('Course Content'!J15="","—",'Course Content'!J15),"")</f>
-        <v/>
-      </c>
-      <c r="P40" s="62">
-        <f>IFERROR(IF(O40="","",IF(O40="—","",FLOOR(O40/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q40" s="63">
-        <f>IFERROR(IF(P40="","",IF(P40="—","",FLOOR(P40/I40,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R40" s="64">
-        <f>IFERROR(IF('Course Content'!H15="","",'Course Content'!H15),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="5">
-        <f>IFERROR(IF('Course Content'!B31="","",'Course Content'!B31),"")</f>
-        <v/>
-      </c>
-      <c r="C41" s="59" t="n"/>
-      <c r="D41" s="59" t="n"/>
-      <c r="E41" s="59" t="n"/>
-      <c r="F41" s="59" t="n"/>
-      <c r="G41" s="59" t="n"/>
-      <c r="H41" s="59" t="n"/>
-      <c r="I41" s="17">
-        <f>IF(COUNTA(C41:H41)=0,$I$8,COUNTA(C41:H41))</f>
-        <v/>
-      </c>
-      <c r="J41" s="26" t="n"/>
-      <c r="K41" s="60">
-        <f>IFERROR(IF('Course Content'!D31="","—",'Course Content'!D31),"")</f>
-        <v/>
-      </c>
-      <c r="L41" s="60">
-        <f>IFERROR(IF(K41="","",IF(K41="—","",FLOOR(K41/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M41" s="61">
-        <f>IFERROR(IF(L41="","",IF(L41="—","",FLOOR(L41/I41,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N41" s="26" t="n"/>
-      <c r="O41" s="62">
-        <f>IFERROR(IF('Course Content'!E31="","—",'Course Content'!E31),"")</f>
-        <v/>
-      </c>
-      <c r="P41" s="62">
-        <f>IFERROR(IF(O41="","",IF(O41="—","",FLOOR(O41/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q41" s="63">
-        <f>IFERROR(IF(P41="","",IF(P41="—","",FLOOR(P41/I41,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R41" s="65">
-        <f>IFERROR(IF('Course Content'!C31="","",'Course Content'!C31),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="B42" s="66">
-        <f>IFERROR(IF('Course Content'!G31="","",'Course Content'!G31),"")</f>
-        <v/>
-      </c>
-      <c r="C42" s="67" t="n"/>
-      <c r="D42" s="67" t="n"/>
-      <c r="E42" s="67" t="n"/>
-      <c r="F42" s="67" t="n"/>
-      <c r="G42" s="67" t="n"/>
-      <c r="H42" s="67" t="n"/>
-      <c r="I42" s="68">
-        <f>IF(COUNTA(C42:H42)=0,$I$8,COUNTA(C42:H42))</f>
-        <v/>
-      </c>
-      <c r="J42" s="26" t="n"/>
-      <c r="K42" s="69">
-        <f>IFERROR(IF('Course Content'!I31="","—",'Course Content'!I31),"")</f>
-        <v/>
-      </c>
-      <c r="L42" s="69">
-        <f>IFERROR(IF(K42="","",IF(K42="—","",FLOOR(K42/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M42" s="70">
-        <f>IFERROR(IF(L42="","",IF(L42="—","",FLOOR(L42/I42,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N42" s="26" t="n"/>
-      <c r="O42" s="71">
-        <f>IFERROR(IF('Course Content'!J31="","—",'Course Content'!J31),"")</f>
-        <v/>
-      </c>
-      <c r="P42" s="71">
-        <f>IFERROR(IF(O42="","",IF(O42="—","",FLOOR(O42/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q42" s="72">
-        <f>IFERROR(IF(P42="","",IF(P42="—","",FLOOR(P42/I42,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R42" s="73">
-        <f>IFERROR(IF('Course Content'!H31="","",'Course Content'!H31),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="31" t="inlineStr">
-        <is>
-          <t>Physical Education</t>
-        </is>
-      </c>
-      <c r="B43" s="58">
-        <f>IFERROR(IF('Course Content'!B16="","",'Course Content'!B16),"")</f>
-        <v/>
-      </c>
-      <c r="C43" s="59" t="n"/>
-      <c r="D43" s="59" t="n"/>
-      <c r="E43" s="59" t="n"/>
-      <c r="F43" s="59" t="n"/>
-      <c r="G43" s="59" t="n"/>
-      <c r="H43" s="59" t="n"/>
-      <c r="I43" s="17">
-        <f>IF(COUNTA(C43:H43)=0,$I$8,COUNTA(C43:H43))</f>
-        <v/>
-      </c>
-      <c r="J43" s="26" t="n"/>
-      <c r="K43" s="60">
-        <f>IFERROR(IF('Course Content'!D16="","—",'Course Content'!D16),"")</f>
-        <v/>
-      </c>
-      <c r="L43" s="60">
-        <f>IFERROR(IF(K43="","",IF(K43="—","",FLOOR(K43/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M43" s="61">
-        <f>IFERROR(IF(L43="","",IF(L43="—","",FLOOR(L43/I43,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N43" s="26" t="n"/>
-      <c r="O43" s="62">
-        <f>IFERROR(IF('Course Content'!E16="","—",'Course Content'!E16),"")</f>
-        <v/>
-      </c>
-      <c r="P43" s="62">
-        <f>IFERROR(IF(O43="","",IF(O43="—","",FLOOR(O43/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q43" s="63">
-        <f>IFERROR(IF(P43="","",IF(P43="—","",FLOOR(P43/I43,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R43" s="64">
-        <f>IFERROR(IF('Course Content'!C16="","",'Course Content'!C16),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="B44" s="58">
-        <f>IFERROR(IF('Course Content'!G16="","",'Course Content'!G16),"")</f>
-        <v/>
-      </c>
-      <c r="C44" s="59" t="n"/>
-      <c r="D44" s="59" t="n"/>
-      <c r="E44" s="59" t="n"/>
-      <c r="F44" s="59" t="n"/>
-      <c r="G44" s="59" t="n"/>
-      <c r="H44" s="59" t="n"/>
-      <c r="I44" s="17">
-        <f>IF(COUNTA(C44:H44)=0,$I$8,COUNTA(C44:H44))</f>
-        <v/>
-      </c>
-      <c r="J44" s="26" t="n"/>
-      <c r="K44" s="60">
-        <f>IFERROR(IF('Course Content'!I16="","—",'Course Content'!I16),"")</f>
-        <v/>
-      </c>
-      <c r="L44" s="60">
-        <f>IFERROR(IF(K44="","",IF(K44="—","",FLOOR(K44/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M44" s="61">
-        <f>IFERROR(IF(L44="","",IF(L44="—","",FLOOR(L44/I44,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N44" s="26" t="n"/>
-      <c r="O44" s="62">
-        <f>IFERROR(IF('Course Content'!J16="","—",'Course Content'!J16),"")</f>
-        <v/>
-      </c>
-      <c r="P44" s="62">
-        <f>IFERROR(IF(O44="","",IF(O44="—","",FLOOR(O44/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q44" s="63">
-        <f>IFERROR(IF(P44="","",IF(P44="—","",FLOOR(P44/I44,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R44" s="64">
-        <f>IFERROR(IF('Course Content'!H16="","",'Course Content'!H16),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="B45" s="5">
-        <f>IFERROR(IF('Course Content'!B32="","",'Course Content'!B32),"")</f>
-        <v/>
-      </c>
-      <c r="C45" s="59" t="n"/>
-      <c r="D45" s="59" t="n"/>
-      <c r="E45" s="59" t="n"/>
-      <c r="F45" s="59" t="n"/>
-      <c r="G45" s="59" t="n"/>
-      <c r="H45" s="59" t="n"/>
-      <c r="I45" s="17">
-        <f>IF(COUNTA(C45:H45)=0,$I$8,COUNTA(C45:H45))</f>
-        <v/>
-      </c>
-      <c r="J45" s="26" t="n"/>
-      <c r="K45" s="60">
-        <f>IFERROR(IF('Course Content'!D32="","—",'Course Content'!D32),"")</f>
-        <v/>
-      </c>
-      <c r="L45" s="60">
-        <f>IFERROR(IF(K45="","",IF(K45="—","",FLOOR(K45/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M45" s="61">
-        <f>IFERROR(IF(L45="","",IF(L45="—","",FLOOR(L45/I45,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N45" s="26" t="n"/>
-      <c r="O45" s="62">
-        <f>IFERROR(IF('Course Content'!E32="","—",'Course Content'!E32),"")</f>
-        <v/>
-      </c>
-      <c r="P45" s="62">
-        <f>IFERROR(IF(O45="","",IF(O45="—","",FLOOR(O45/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q45" s="63">
-        <f>IFERROR(IF(P45="","",IF(P45="—","",FLOOR(P45/I45,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R45" s="65">
-        <f>IFERROR(IF('Course Content'!C32="","",'Course Content'!C32),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="66">
-        <f>IFERROR(IF('Course Content'!G32="","",'Course Content'!G32),"")</f>
-        <v/>
-      </c>
-      <c r="C46" s="67" t="n"/>
-      <c r="D46" s="67" t="n"/>
-      <c r="E46" s="67" t="n"/>
-      <c r="F46" s="67" t="n"/>
-      <c r="G46" s="67" t="n"/>
-      <c r="H46" s="67" t="n"/>
-      <c r="I46" s="68">
-        <f>IF(COUNTA(C46:H46)=0,$I$8,COUNTA(C46:H46))</f>
-        <v/>
-      </c>
-      <c r="J46" s="26" t="n"/>
-      <c r="K46" s="69">
-        <f>IFERROR(IF('Course Content'!I32="","—",'Course Content'!I32),"")</f>
-        <v/>
-      </c>
-      <c r="L46" s="69">
-        <f>IFERROR(IF(K46="","",IF(K46="—","",FLOOR(K46/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M46" s="70">
-        <f>IFERROR(IF(L46="","",IF(L46="—","",FLOOR(L46/I46,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N46" s="26" t="n"/>
-      <c r="O46" s="71">
-        <f>IFERROR(IF('Course Content'!J32="","—",'Course Content'!J32),"")</f>
-        <v/>
-      </c>
-      <c r="P46" s="71">
-        <f>IFERROR(IF(O46="","",IF(O46="—","",FLOOR(O46/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q46" s="72">
-        <f>IFERROR(IF(P46="","",IF(P46="—","",FLOOR(P46/I46,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R46" s="73">
-        <f>IFERROR(IF('Course Content'!H32="","",'Course Content'!H32),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="31" t="inlineStr">
-        <is>
-          <t>Art / Music</t>
-        </is>
-      </c>
-      <c r="B47" s="58">
-        <f>IFERROR(IF('Course Content'!B17="","",'Course Content'!B17),"")</f>
-        <v/>
-      </c>
-      <c r="C47" s="59" t="n"/>
-      <c r="D47" s="59" t="n"/>
-      <c r="E47" s="59" t="n"/>
-      <c r="F47" s="59" t="n"/>
-      <c r="G47" s="59" t="n"/>
-      <c r="H47" s="59" t="n"/>
-      <c r="I47" s="17">
-        <f>IF(COUNTA(C47:H47)=0,$I$8,COUNTA(C47:H47))</f>
-        <v/>
-      </c>
-      <c r="J47" s="26" t="n"/>
-      <c r="K47" s="60">
-        <f>IFERROR(IF('Course Content'!D17="","—",'Course Content'!D17),"")</f>
-        <v/>
-      </c>
-      <c r="L47" s="60">
-        <f>IFERROR(IF(K47="","",IF(K47="—","",FLOOR(K47/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M47" s="61">
-        <f>IFERROR(IF(L47="","",IF(L47="—","",FLOOR(L47/I47,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N47" s="26" t="n"/>
-      <c r="O47" s="62">
-        <f>IFERROR(IF('Course Content'!E17="","—",'Course Content'!E17),"")</f>
-        <v/>
-      </c>
-      <c r="P47" s="62">
-        <f>IFERROR(IF(O47="","",IF(O47="—","",FLOOR(O47/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q47" s="63">
-        <f>IFERROR(IF(P47="","",IF(P47="—","",FLOOR(P47/I47,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R47" s="64">
-        <f>IFERROR(IF('Course Content'!C17="","",'Course Content'!C17),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="B48" s="58">
-        <f>IFERROR(IF('Course Content'!G17="","",'Course Content'!G17),"")</f>
-        <v/>
-      </c>
-      <c r="C48" s="59" t="n"/>
-      <c r="D48" s="59" t="n"/>
-      <c r="E48" s="59" t="n"/>
-      <c r="F48" s="59" t="n"/>
-      <c r="G48" s="59" t="n"/>
-      <c r="H48" s="59" t="n"/>
-      <c r="I48" s="17">
-        <f>IF(COUNTA(C48:H48)=0,$I$8,COUNTA(C48:H48))</f>
-        <v/>
-      </c>
-      <c r="J48" s="26" t="n"/>
-      <c r="K48" s="60">
-        <f>IFERROR(IF('Course Content'!I17="","—",'Course Content'!I17),"")</f>
-        <v/>
-      </c>
-      <c r="L48" s="60">
-        <f>IFERROR(IF(K48="","",IF(K48="—","",FLOOR(K48/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M48" s="61">
-        <f>IFERROR(IF(L48="","",IF(L48="—","",FLOOR(L48/I48,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N48" s="26" t="n"/>
-      <c r="O48" s="62">
-        <f>IFERROR(IF('Course Content'!J17="","—",'Course Content'!J17),"")</f>
-        <v/>
-      </c>
-      <c r="P48" s="62">
-        <f>IFERROR(IF(O48="","",IF(O48="—","",FLOOR(O48/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q48" s="63">
-        <f>IFERROR(IF(P48="","",IF(P48="—","",FLOOR(P48/I48,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R48" s="64">
-        <f>IFERROR(IF('Course Content'!H17="","",'Course Content'!H17),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="B49" s="5">
-        <f>IFERROR(IF('Course Content'!B33="","",'Course Content'!B33),"")</f>
-        <v/>
-      </c>
-      <c r="C49" s="59" t="n"/>
-      <c r="D49" s="59" t="n"/>
-      <c r="E49" s="59" t="n"/>
-      <c r="F49" s="59" t="n"/>
-      <c r="G49" s="59" t="n"/>
-      <c r="H49" s="59" t="n"/>
-      <c r="I49" s="17">
-        <f>IF(COUNTA(C49:H49)=0,$I$8,COUNTA(C49:H49))</f>
-        <v/>
-      </c>
-      <c r="J49" s="26" t="n"/>
-      <c r="K49" s="60">
-        <f>IFERROR(IF('Course Content'!D33="","—",'Course Content'!D33),"")</f>
-        <v/>
-      </c>
-      <c r="L49" s="60">
-        <f>IFERROR(IF(K49="","",IF(K49="—","",FLOOR(K49/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M49" s="61">
-        <f>IFERROR(IF(L49="","",IF(L49="—","",FLOOR(L49/I49,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N49" s="26" t="n"/>
-      <c r="O49" s="62">
-        <f>IFERROR(IF('Course Content'!E33="","—",'Course Content'!E33),"")</f>
-        <v/>
-      </c>
-      <c r="P49" s="62">
-        <f>IFERROR(IF(O49="","",IF(O49="—","",FLOOR(O49/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q49" s="63">
-        <f>IFERROR(IF(P49="","",IF(P49="—","",FLOOR(P49/I49,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R49" s="65">
-        <f>IFERROR(IF('Course Content'!C33="","",'Course Content'!C33),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="B50" s="66">
-        <f>IFERROR(IF('Course Content'!G33="","",'Course Content'!G33),"")</f>
-        <v/>
-      </c>
-      <c r="C50" s="67" t="n"/>
-      <c r="D50" s="67" t="n"/>
-      <c r="E50" s="67" t="n"/>
-      <c r="F50" s="67" t="n"/>
-      <c r="G50" s="67" t="n"/>
-      <c r="H50" s="67" t="n"/>
-      <c r="I50" s="68">
-        <f>IF(COUNTA(C50:H50)=0,$I$8,COUNTA(C50:H50))</f>
-        <v/>
-      </c>
-      <c r="J50" s="26" t="n"/>
-      <c r="K50" s="69">
-        <f>IFERROR(IF('Course Content'!I33="","—",'Course Content'!I33),"")</f>
-        <v/>
-      </c>
-      <c r="L50" s="69">
-        <f>IFERROR(IF(K50="","",IF(K50="—","",FLOOR(K50/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M50" s="70">
-        <f>IFERROR(IF(L50="","",IF(L50="—","",FLOOR(L50/I50,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N50" s="26" t="n"/>
-      <c r="O50" s="71">
-        <f>IFERROR(IF('Course Content'!J33="","—",'Course Content'!J33),"")</f>
-        <v/>
-      </c>
-      <c r="P50" s="71">
-        <f>IFERROR(IF(O50="","",IF(O50="—","",FLOOR(O50/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q50" s="72">
-        <f>IFERROR(IF(P50="","",IF(P50="—","",FLOOR(P50/I50,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R50" s="73">
-        <f>IFERROR(IF('Course Content'!H33="","",'Course Content'!H33),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="31">
-        <f>IF('Course Content'!A34="Elective / Other 1","Elective / Other 1",'Course Content'!A34)</f>
-        <v/>
-      </c>
-      <c r="B51" s="58">
-        <f>IFERROR(IF('Course Content'!B18="","",'Course Content'!B18),"")</f>
-        <v/>
-      </c>
-      <c r="C51" s="59" t="n"/>
-      <c r="D51" s="59" t="n"/>
-      <c r="E51" s="59" t="n"/>
-      <c r="F51" s="59" t="n"/>
-      <c r="G51" s="59" t="n"/>
-      <c r="H51" s="59" t="n"/>
-      <c r="I51" s="17">
-        <f>IF(COUNTA(C51:H51)=0,$I$8,COUNTA(C51:H51))</f>
-        <v/>
-      </c>
-      <c r="J51" s="26" t="n"/>
-      <c r="K51" s="60">
-        <f>IFERROR(IF('Course Content'!D18="","—",'Course Content'!D18),"")</f>
-        <v/>
-      </c>
-      <c r="L51" s="60">
-        <f>IFERROR(IF(K51="","",IF(K51="—","",FLOOR(K51/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M51" s="61">
-        <f>IFERROR(IF(L51="","",IF(L51="—","",FLOOR(L51/I51,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N51" s="26" t="n"/>
-      <c r="O51" s="62">
-        <f>IFERROR(IF('Course Content'!E18="","—",'Course Content'!E18),"")</f>
-        <v/>
-      </c>
-      <c r="P51" s="62">
-        <f>IFERROR(IF(O51="","",IF(O51="—","",FLOOR(O51/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q51" s="63">
-        <f>IFERROR(IF(P51="","",IF(P51="—","",FLOOR(P51/I51,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R51" s="64">
-        <f>IFERROR(IF('Course Content'!C18="","",'Course Content'!C18),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="20" customHeight="1">
-      <c r="B52" s="58">
-        <f>IFERROR(IF('Course Content'!G18="","",'Course Content'!G18),"")</f>
-        <v/>
-      </c>
-      <c r="C52" s="59" t="n"/>
-      <c r="D52" s="59" t="n"/>
-      <c r="E52" s="59" t="n"/>
-      <c r="F52" s="59" t="n"/>
-      <c r="G52" s="59" t="n"/>
-      <c r="H52" s="59" t="n"/>
-      <c r="I52" s="17">
-        <f>IF(COUNTA(C52:H52)=0,$I$8,COUNTA(C52:H52))</f>
-        <v/>
-      </c>
-      <c r="J52" s="26" t="n"/>
-      <c r="K52" s="60">
-        <f>IFERROR(IF('Course Content'!I18="","—",'Course Content'!I18),"")</f>
-        <v/>
-      </c>
-      <c r="L52" s="60">
-        <f>IFERROR(IF(K52="","",IF(K52="—","",FLOOR(K52/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M52" s="61">
-        <f>IFERROR(IF(L52="","",IF(L52="—","",FLOOR(L52/I52,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N52" s="26" t="n"/>
-      <c r="O52" s="62">
-        <f>IFERROR(IF('Course Content'!J18="","—",'Course Content'!J18),"")</f>
-        <v/>
-      </c>
-      <c r="P52" s="62">
-        <f>IFERROR(IF(O52="","",IF(O52="—","",FLOOR(O52/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q52" s="63">
-        <f>IFERROR(IF(P52="","",IF(P52="—","",FLOOR(P52/I52,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R52" s="64">
-        <f>IFERROR(IF('Course Content'!H18="","",'Course Content'!H18),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="5">
-        <f>IFERROR(IF('Course Content'!B34="","",'Course Content'!B34),"")</f>
-        <v/>
-      </c>
-      <c r="C53" s="59" t="n"/>
-      <c r="D53" s="59" t="n"/>
-      <c r="E53" s="59" t="n"/>
-      <c r="F53" s="59" t="n"/>
-      <c r="G53" s="59" t="n"/>
-      <c r="H53" s="59" t="n"/>
-      <c r="I53" s="17">
-        <f>IF(COUNTA(C53:H53)=0,$I$8,COUNTA(C53:H53))</f>
-        <v/>
-      </c>
-      <c r="J53" s="26" t="n"/>
-      <c r="K53" s="60">
-        <f>IFERROR(IF('Course Content'!D34="","—",'Course Content'!D34),"")</f>
-        <v/>
-      </c>
-      <c r="L53" s="60">
-        <f>IFERROR(IF(K53="","",IF(K53="—","",FLOOR(K53/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M53" s="61">
-        <f>IFERROR(IF(L53="","",IF(L53="—","",FLOOR(L53/I53,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N53" s="26" t="n"/>
-      <c r="O53" s="62">
-        <f>IFERROR(IF('Course Content'!E34="","—",'Course Content'!E34),"")</f>
-        <v/>
-      </c>
-      <c r="P53" s="62">
-        <f>IFERROR(IF(O53="","",IF(O53="—","",FLOOR(O53/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q53" s="63">
-        <f>IFERROR(IF(P53="","",IF(P53="—","",FLOOR(P53/I53,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R53" s="65">
-        <f>IFERROR(IF('Course Content'!C34="","",'Course Content'!C34),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" ht="20" customHeight="1">
-      <c r="B54" s="66">
-        <f>IFERROR(IF('Course Content'!G34="","",'Course Content'!G34),"")</f>
-        <v/>
-      </c>
-      <c r="C54" s="67" t="n"/>
-      <c r="D54" s="67" t="n"/>
-      <c r="E54" s="67" t="n"/>
-      <c r="F54" s="67" t="n"/>
-      <c r="G54" s="67" t="n"/>
-      <c r="H54" s="67" t="n"/>
-      <c r="I54" s="68">
-        <f>IF(COUNTA(C54:H54)=0,$I$8,COUNTA(C54:H54))</f>
-        <v/>
-      </c>
-      <c r="J54" s="26" t="n"/>
-      <c r="K54" s="69">
-        <f>IFERROR(IF('Course Content'!I34="","—",'Course Content'!I34),"")</f>
-        <v/>
-      </c>
-      <c r="L54" s="69">
-        <f>IFERROR(IF(K54="","",IF(K54="—","",FLOOR(K54/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M54" s="70">
-        <f>IFERROR(IF(L54="","",IF(L54="—","",FLOOR(L54/I54,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N54" s="26" t="n"/>
-      <c r="O54" s="71">
-        <f>IFERROR(IF('Course Content'!J34="","—",'Course Content'!J34),"")</f>
-        <v/>
-      </c>
-      <c r="P54" s="71">
-        <f>IFERROR(IF(O54="","",IF(O54="—","",FLOOR(O54/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q54" s="72">
-        <f>IFERROR(IF(P54="","",IF(P54="—","",FLOOR(P54/I54,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R54" s="73">
-        <f>IFERROR(IF('Course Content'!H34="","",'Course Content'!H34),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="31">
-        <f>IF('Course Content'!A35="Elective / Other 2","Elective / Other 2",'Course Content'!A35)</f>
-        <v/>
-      </c>
-      <c r="B55" s="58">
-        <f>IFERROR(IF('Course Content'!B19="","",'Course Content'!B19),"")</f>
-        <v/>
-      </c>
-      <c r="C55" s="59" t="n"/>
-      <c r="D55" s="59" t="n"/>
-      <c r="E55" s="59" t="n"/>
-      <c r="F55" s="59" t="n"/>
-      <c r="G55" s="59" t="n"/>
-      <c r="H55" s="59" t="n"/>
-      <c r="I55" s="17">
-        <f>IF(COUNTA(C55:H55)=0,$I$8,COUNTA(C55:H55))</f>
-        <v/>
-      </c>
-      <c r="J55" s="26" t="n"/>
-      <c r="K55" s="60">
-        <f>IFERROR(IF('Course Content'!D19="","—",'Course Content'!D19),"")</f>
-        <v/>
-      </c>
-      <c r="L55" s="60">
-        <f>IFERROR(IF(K55="","",IF(K55="—","",FLOOR(K55/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M55" s="61">
-        <f>IFERROR(IF(L55="","",IF(L55="—","",FLOOR(L55/I55,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N55" s="26" t="n"/>
-      <c r="O55" s="62">
-        <f>IFERROR(IF('Course Content'!E19="","—",'Course Content'!E19),"")</f>
-        <v/>
-      </c>
-      <c r="P55" s="62">
-        <f>IFERROR(IF(O55="","",IF(O55="—","",FLOOR(O55/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q55" s="63">
-        <f>IFERROR(IF(P55="","",IF(P55="—","",FLOOR(P55/I55,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R55" s="64">
-        <f>IFERROR(IF('Course Content'!C19="","",'Course Content'!C19),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="B56" s="58">
-        <f>IFERROR(IF('Course Content'!G19="","",'Course Content'!G19),"")</f>
-        <v/>
-      </c>
-      <c r="C56" s="59" t="n"/>
-      <c r="D56" s="59" t="n"/>
-      <c r="E56" s="59" t="n"/>
-      <c r="F56" s="59" t="n"/>
-      <c r="G56" s="59" t="n"/>
-      <c r="H56" s="59" t="n"/>
-      <c r="I56" s="17">
-        <f>IF(COUNTA(C56:H56)=0,$I$8,COUNTA(C56:H56))</f>
-        <v/>
-      </c>
-      <c r="J56" s="26" t="n"/>
-      <c r="K56" s="60">
-        <f>IFERROR(IF('Course Content'!I19="","—",'Course Content'!I19),"")</f>
-        <v/>
-      </c>
-      <c r="L56" s="60">
-        <f>IFERROR(IF(K56="","",IF(K56="—","",FLOOR(K56/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M56" s="61">
-        <f>IFERROR(IF(L56="","",IF(L56="—","",FLOOR(L56/I56,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N56" s="26" t="n"/>
-      <c r="O56" s="62">
-        <f>IFERROR(IF('Course Content'!J19="","—",'Course Content'!J19),"")</f>
-        <v/>
-      </c>
-      <c r="P56" s="62">
-        <f>IFERROR(IF(O56="","",IF(O56="—","",FLOOR(O56/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q56" s="63">
-        <f>IFERROR(IF(P56="","",IF(P56="—","",FLOOR(P56/I56,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R56" s="64">
-        <f>IFERROR(IF('Course Content'!H19="","",'Course Content'!H19),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" ht="20" customHeight="1">
-      <c r="B57" s="5">
-        <f>IFERROR(IF('Course Content'!B35="","",'Course Content'!B35),"")</f>
-        <v/>
-      </c>
-      <c r="C57" s="59" t="n"/>
-      <c r="D57" s="59" t="n"/>
-      <c r="E57" s="59" t="n"/>
-      <c r="F57" s="59" t="n"/>
-      <c r="G57" s="59" t="n"/>
-      <c r="H57" s="59" t="n"/>
-      <c r="I57" s="17">
-        <f>IF(COUNTA(C57:H57)=0,$I$8,COUNTA(C57:H57))</f>
-        <v/>
-      </c>
-      <c r="J57" s="26" t="n"/>
-      <c r="K57" s="60">
-        <f>IFERROR(IF('Course Content'!D35="","—",'Course Content'!D35),"")</f>
-        <v/>
-      </c>
-      <c r="L57" s="60">
-        <f>IFERROR(IF(K57="","",IF(K57="—","",FLOOR(K57/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M57" s="61">
-        <f>IFERROR(IF(L57="","",IF(L57="—","",FLOOR(L57/I57,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N57" s="26" t="n"/>
-      <c r="O57" s="62">
-        <f>IFERROR(IF('Course Content'!E35="","—",'Course Content'!E35),"")</f>
-        <v/>
-      </c>
-      <c r="P57" s="62">
-        <f>IFERROR(IF(O57="","",IF(O57="—","",FLOOR(O57/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q57" s="63">
-        <f>IFERROR(IF(P57="","",IF(P57="—","",FLOOR(P57/I57,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R57" s="65">
-        <f>IFERROR(IF('Course Content'!C35="","",'Course Content'!C35),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="20" customHeight="1">
-      <c r="B58" s="66">
-        <f>IFERROR(IF('Course Content'!G35="","",'Course Content'!G35),"")</f>
-        <v/>
-      </c>
-      <c r="C58" s="67" t="n"/>
-      <c r="D58" s="67" t="n"/>
-      <c r="E58" s="67" t="n"/>
-      <c r="F58" s="67" t="n"/>
-      <c r="G58" s="67" t="n"/>
-      <c r="H58" s="67" t="n"/>
-      <c r="I58" s="68">
-        <f>IF(COUNTA(C58:H58)=0,$I$8,COUNTA(C58:H58))</f>
-        <v/>
-      </c>
-      <c r="J58" s="26" t="n"/>
-      <c r="K58" s="69">
-        <f>IFERROR(IF('Course Content'!I35="","—",'Course Content'!I35),"")</f>
-        <v/>
-      </c>
-      <c r="L58" s="69">
-        <f>IFERROR(IF(K58="","",IF(K58="—","",FLOOR(K58/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M58" s="70">
-        <f>IFERROR(IF(L58="","",IF(L58="—","",FLOOR(L58/I58,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N58" s="26" t="n"/>
-      <c r="O58" s="71">
-        <f>IFERROR(IF('Course Content'!J35="","—",'Course Content'!J35),"")</f>
-        <v/>
-      </c>
-      <c r="P58" s="71">
-        <f>IFERROR(IF(O58="","",IF(O58="—","",FLOOR(O58/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q58" s="72">
-        <f>IFERROR(IF(P58="","",IF(P58="—","",FLOOR(P58/I58,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R58" s="73">
-        <f>IFERROR(IF('Course Content'!H35="","",'Course Content'!H35),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" ht="20" customHeight="1">
-      <c r="A59" s="31">
-        <f>IF('Course Content'!A36="Elective / Other 3","Elective / Other 3",'Course Content'!A36)</f>
-        <v/>
-      </c>
-      <c r="B59" s="58">
-        <f>IFERROR(IF('Course Content'!B20="","",'Course Content'!B20),"")</f>
-        <v/>
-      </c>
-      <c r="C59" s="59" t="n"/>
-      <c r="D59" s="59" t="n"/>
-      <c r="E59" s="59" t="n"/>
-      <c r="F59" s="59" t="n"/>
-      <c r="G59" s="59" t="n"/>
-      <c r="H59" s="59" t="n"/>
-      <c r="I59" s="17">
-        <f>IF(COUNTA(C59:H59)=0,$I$8,COUNTA(C59:H59))</f>
-        <v/>
-      </c>
-      <c r="J59" s="26" t="n"/>
-      <c r="K59" s="60">
-        <f>IFERROR(IF('Course Content'!D20="","—",'Course Content'!D20),"")</f>
-        <v/>
-      </c>
-      <c r="L59" s="60">
-        <f>IFERROR(IF(K59="","",IF(K59="—","",FLOOR(K59/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M59" s="61">
-        <f>IFERROR(IF(L59="","",IF(L59="—","",FLOOR(L59/I59,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N59" s="26" t="n"/>
-      <c r="O59" s="62">
-        <f>IFERROR(IF('Course Content'!E20="","—",'Course Content'!E20),"")</f>
-        <v/>
-      </c>
-      <c r="P59" s="62">
-        <f>IFERROR(IF(O59="","",IF(O59="—","",FLOOR(O59/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q59" s="63">
-        <f>IFERROR(IF(P59="","",IF(P59="—","",FLOOR(P59/I59,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R59" s="64">
-        <f>IFERROR(IF('Course Content'!C20="","",'Course Content'!C20),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="20" customHeight="1">
-      <c r="B60" s="58">
-        <f>IFERROR(IF('Course Content'!G20="","",'Course Content'!G20),"")</f>
-        <v/>
-      </c>
-      <c r="C60" s="59" t="n"/>
-      <c r="D60" s="59" t="n"/>
-      <c r="E60" s="59" t="n"/>
-      <c r="F60" s="59" t="n"/>
-      <c r="G60" s="59" t="n"/>
-      <c r="H60" s="59" t="n"/>
-      <c r="I60" s="17">
-        <f>IF(COUNTA(C60:H60)=0,$I$8,COUNTA(C60:H60))</f>
-        <v/>
-      </c>
-      <c r="J60" s="26" t="n"/>
-      <c r="K60" s="60">
-        <f>IFERROR(IF('Course Content'!I20="","—",'Course Content'!I20),"")</f>
-        <v/>
-      </c>
-      <c r="L60" s="60">
-        <f>IFERROR(IF(K60="","",IF(K60="—","",FLOOR(K60/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M60" s="61">
-        <f>IFERROR(IF(L60="","",IF(L60="—","",FLOOR(L60/I60,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N60" s="26" t="n"/>
-      <c r="O60" s="62">
-        <f>IFERROR(IF('Course Content'!J20="","—",'Course Content'!J20),"")</f>
-        <v/>
-      </c>
-      <c r="P60" s="62">
-        <f>IFERROR(IF(O60="","",IF(O60="—","",FLOOR(O60/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q60" s="63">
-        <f>IFERROR(IF(P60="","",IF(P60="—","",FLOOR(P60/I60,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R60" s="64">
-        <f>IFERROR(IF('Course Content'!H20="","",'Course Content'!H20),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="B61" s="5">
-        <f>IFERROR(IF('Course Content'!B36="","",'Course Content'!B36),"")</f>
-        <v/>
-      </c>
-      <c r="C61" s="59" t="n"/>
-      <c r="D61" s="59" t="n"/>
-      <c r="E61" s="59" t="n"/>
-      <c r="F61" s="59" t="n"/>
-      <c r="G61" s="59" t="n"/>
-      <c r="H61" s="59" t="n"/>
-      <c r="I61" s="17">
-        <f>IF(COUNTA(C61:H61)=0,$I$8,COUNTA(C61:H61))</f>
-        <v/>
-      </c>
-      <c r="J61" s="26" t="n"/>
-      <c r="K61" s="60">
-        <f>IFERROR(IF('Course Content'!D36="","—",'Course Content'!D36),"")</f>
-        <v/>
-      </c>
-      <c r="L61" s="60">
-        <f>IFERROR(IF(K61="","",IF(K61="—","",FLOOR(K61/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M61" s="61">
-        <f>IFERROR(IF(L61="","",IF(L61="—","",FLOOR(L61/I61,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N61" s="26" t="n"/>
-      <c r="O61" s="62">
-        <f>IFERROR(IF('Course Content'!E36="","—",'Course Content'!E36),"")</f>
-        <v/>
-      </c>
-      <c r="P61" s="62">
-        <f>IFERROR(IF(O61="","",IF(O61="—","",FLOOR(O61/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q61" s="63">
-        <f>IFERROR(IF(P61="","",IF(P61="—","",FLOOR(P61/I61,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R61" s="65">
-        <f>IFERROR(IF('Course Content'!C36="","",'Course Content'!C36),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="B62" s="66">
-        <f>IFERROR(IF('Course Content'!G36="","",'Course Content'!G36),"")</f>
-        <v/>
-      </c>
-      <c r="C62" s="67" t="n"/>
-      <c r="D62" s="67" t="n"/>
-      <c r="E62" s="67" t="n"/>
-      <c r="F62" s="67" t="n"/>
-      <c r="G62" s="67" t="n"/>
-      <c r="H62" s="67" t="n"/>
-      <c r="I62" s="68">
-        <f>IF(COUNTA(C62:H62)=0,$I$8,COUNTA(C62:H62))</f>
-        <v/>
-      </c>
-      <c r="J62" s="26" t="n"/>
-      <c r="K62" s="69">
-        <f>IFERROR(IF('Course Content'!I36="","—",'Course Content'!I36),"")</f>
-        <v/>
-      </c>
-      <c r="L62" s="69">
-        <f>IFERROR(IF(K62="","",IF(K62="—","",FLOOR(K62/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M62" s="70">
-        <f>IFERROR(IF(L62="","",IF(L62="—","",FLOOR(L62/I62,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N62" s="26" t="n"/>
-      <c r="O62" s="71">
-        <f>IFERROR(IF('Course Content'!J36="","—",'Course Content'!J36),"")</f>
-        <v/>
-      </c>
-      <c r="P62" s="71">
-        <f>IFERROR(IF(O62="","",IF(O62="—","",FLOOR(O62/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q62" s="72">
-        <f>IFERROR(IF(P62="","",IF(P62="—","",FLOOR(P62/I62,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R62" s="73">
-        <f>IFERROR(IF('Course Content'!H36="","",'Course Content'!H36),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="20" customHeight="1">
-      <c r="A63" s="31">
-        <f>IF('Course Content'!A37="Elective / Other 4","Elective / Other 4",'Course Content'!A37)</f>
-        <v/>
-      </c>
-      <c r="B63" s="58">
-        <f>IFERROR(IF('Course Content'!B21="","",'Course Content'!B21),"")</f>
-        <v/>
-      </c>
-      <c r="C63" s="59" t="n"/>
-      <c r="D63" s="59" t="n"/>
-      <c r="E63" s="59" t="n"/>
-      <c r="F63" s="59" t="n"/>
-      <c r="G63" s="59" t="n"/>
-      <c r="H63" s="59" t="n"/>
-      <c r="I63" s="17">
-        <f>IF(COUNTA(C63:H63)=0,$I$8,COUNTA(C63:H63))</f>
-        <v/>
-      </c>
-      <c r="J63" s="26" t="n"/>
-      <c r="K63" s="60">
-        <f>IFERROR(IF('Course Content'!D21="","—",'Course Content'!D21),"")</f>
-        <v/>
-      </c>
-      <c r="L63" s="60">
-        <f>IFERROR(IF(K63="","",IF(K63="—","",FLOOR(K63/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M63" s="61">
-        <f>IFERROR(IF(L63="","",IF(L63="—","",FLOOR(L63/I63,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N63" s="26" t="n"/>
-      <c r="O63" s="62">
-        <f>IFERROR(IF('Course Content'!E21="","—",'Course Content'!E21),"")</f>
-        <v/>
-      </c>
-      <c r="P63" s="62">
-        <f>IFERROR(IF(O63="","",IF(O63="—","",FLOOR(O63/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q63" s="63">
-        <f>IFERROR(IF(P63="","",IF(P63="—","",FLOOR(P63/I63,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R63" s="64">
-        <f>IFERROR(IF('Course Content'!C21="","",'Course Content'!C21),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="20" customHeight="1">
-      <c r="B64" s="58">
-        <f>IFERROR(IF('Course Content'!G21="","",'Course Content'!G21),"")</f>
-        <v/>
-      </c>
-      <c r="C64" s="59" t="n"/>
-      <c r="D64" s="59" t="n"/>
-      <c r="E64" s="59" t="n"/>
-      <c r="F64" s="59" t="n"/>
-      <c r="G64" s="59" t="n"/>
-      <c r="H64" s="59" t="n"/>
-      <c r="I64" s="17">
-        <f>IF(COUNTA(C64:H64)=0,$I$8,COUNTA(C64:H64))</f>
-        <v/>
-      </c>
-      <c r="J64" s="26" t="n"/>
-      <c r="K64" s="60">
-        <f>IFERROR(IF('Course Content'!I21="","—",'Course Content'!I21),"")</f>
-        <v/>
-      </c>
-      <c r="L64" s="60">
-        <f>IFERROR(IF(K64="","",IF(K64="—","",FLOOR(K64/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M64" s="61">
-        <f>IFERROR(IF(L64="","",IF(L64="—","",FLOOR(L64/I64,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N64" s="26" t="n"/>
-      <c r="O64" s="62">
-        <f>IFERROR(IF('Course Content'!J21="","—",'Course Content'!J21),"")</f>
-        <v/>
-      </c>
-      <c r="P64" s="62">
-        <f>IFERROR(IF(O64="","",IF(O64="—","",FLOOR(O64/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q64" s="63">
-        <f>IFERROR(IF(P64="","",IF(P64="—","",FLOOR(P64/I64,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R64" s="64">
-        <f>IFERROR(IF('Course Content'!H21="","",'Course Content'!H21),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" ht="20" customHeight="1">
-      <c r="B65" s="5">
-        <f>IFERROR(IF('Course Content'!B37="","",'Course Content'!B37),"")</f>
-        <v/>
-      </c>
-      <c r="C65" s="59" t="n"/>
-      <c r="D65" s="59" t="n"/>
-      <c r="E65" s="59" t="n"/>
-      <c r="F65" s="59" t="n"/>
-      <c r="G65" s="59" t="n"/>
-      <c r="H65" s="59" t="n"/>
-      <c r="I65" s="17">
-        <f>IF(COUNTA(C65:H65)=0,$I$8,COUNTA(C65:H65))</f>
-        <v/>
-      </c>
-      <c r="J65" s="26" t="n"/>
-      <c r="K65" s="60">
-        <f>IFERROR(IF('Course Content'!D37="","—",'Course Content'!D37),"")</f>
-        <v/>
-      </c>
-      <c r="L65" s="60">
-        <f>IFERROR(IF(K65="","",IF(K65="—","",FLOOR(K65/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M65" s="61">
-        <f>IFERROR(IF(L65="","",IF(L65="—","",FLOOR(L65/I65,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N65" s="26" t="n"/>
-      <c r="O65" s="62">
-        <f>IFERROR(IF('Course Content'!E37="","—",'Course Content'!E37),"")</f>
-        <v/>
-      </c>
-      <c r="P65" s="62">
-        <f>IFERROR(IF(O65="","",IF(O65="—","",FLOOR(O65/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q65" s="63">
-        <f>IFERROR(IF(P65="","",IF(P65="—","",FLOOR(P65/I65,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R65" s="65">
-        <f>IFERROR(IF('Course Content'!C37="","",'Course Content'!C37),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="B66" s="66">
-        <f>IFERROR(IF('Course Content'!G37="","",'Course Content'!G37),"")</f>
-        <v/>
-      </c>
-      <c r="C66" s="67" t="n"/>
-      <c r="D66" s="67" t="n"/>
-      <c r="E66" s="67" t="n"/>
-      <c r="F66" s="67" t="n"/>
-      <c r="G66" s="67" t="n"/>
-      <c r="H66" s="67" t="n"/>
-      <c r="I66" s="68">
-        <f>IF(COUNTA(C66:H66)=0,$I$8,COUNTA(C66:H66))</f>
-        <v/>
-      </c>
-      <c r="J66" s="26" t="n"/>
-      <c r="K66" s="69">
-        <f>IFERROR(IF('Course Content'!I37="","—",'Course Content'!I37),"")</f>
-        <v/>
-      </c>
-      <c r="L66" s="69">
-        <f>IFERROR(IF(K66="","",IF(K66="—","",FLOOR(K66/'Getting Started'!C15,1))),"")</f>
-        <v/>
-      </c>
-      <c r="M66" s="70">
-        <f>IFERROR(IF(L66="","",IF(L66="—","",FLOOR(L66/I66,1))),"")</f>
-        <v/>
-      </c>
-      <c r="N66" s="26" t="n"/>
-      <c r="O66" s="71">
-        <f>IFERROR(IF('Course Content'!J37="","—",'Course Content'!J37),"")</f>
-        <v/>
-      </c>
-      <c r="P66" s="71">
-        <f>IFERROR(IF(O66="","",IF(O66="—","",FLOOR(O66/'Getting Started'!C23,1))),"")</f>
-        <v/>
-      </c>
-      <c r="Q66" s="72">
-        <f>IFERROR(IF(P66="","",IF(P66="—","",FLOOR(P66/I66,1))),"")</f>
-        <v/>
-      </c>
-      <c r="R66" s="73">
-        <f>IFERROR(IF('Course Content'!H37="","",'Course Content'!H37),"")</f>
+        <f>IFERROR(IF('Course Content'!C37&lt;&gt;"",'Course Content'!C37,IF('Course Content'!H37&lt;&gt;"",'Course Content'!H37,IF('Course Content'!C21&lt;&gt;"",'Course Content'!C21,'Course Content'!H21))),"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A11:A14"/>
+  <mergeCells count="5">
     <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="K4:R4"/>
+    <mergeCell ref="A4:I4"/>
     <mergeCell ref="A6:R6"/>
-    <mergeCell ref="A55:A58"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="A27:A30"/>
-    <mergeCell ref="A23:A26"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A63:A66"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A43:A46"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A15:A18"/>
-    <mergeCell ref="A59:A62"/>
-    <mergeCell ref="A35:A38"/>
-    <mergeCell ref="K4:R4"/>
-    <mergeCell ref="A51:A54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Expand to 8 Other slots, replacing 4 Elective/Other slots
Gives families room to use overflow rows for extra curricula per
subject (e.g. "Bible — Free Reading") as well as true electives.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -311,7 +311,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -348,6 +348,50 @@
       </bottom>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D4C4BB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D4C4BB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D4C4BB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D4C4BB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D4C4BB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D4C4BB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D4C4BB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D4C4BB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="00CE8282"/>
       </left>
@@ -365,7 +409,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -470,6 +514,8 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -519,7 +565,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1487,7 +1533,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J181"/>
+  <dimension ref="A1:J185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1841,7 +1887,7 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B18" s="5" t="n"/>
@@ -1865,7 +1911,7 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B19" s="5" t="n"/>
@@ -1889,7 +1935,7 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B20" s="5" t="n"/>
@@ -1913,7 +1959,7 @@
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B21" s="5" t="n"/>
@@ -1934,12 +1980,44 @@
       <c r="I21" s="33" t="n"/>
       <c r="J21" s="33" t="n"/>
     </row>
-    <row r="22" ht="8" customHeight="1"/>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="32" t="n"/>
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I22" s="32" t="n"/>
+      <c r="J22" s="32" t="n"/>
+    </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="35">
         <f>IF('Getting Started'!B29&lt;&gt;"","  "&amp;UPPER('Getting Started'!B29)&amp;"   ·   "&amp;'Getting Started'!F29,"  STUDENT 1")</f>
         <v/>
       </c>
+      <c r="B23" s="36" t="n"/>
+      <c r="C23" s="36" t="n"/>
+      <c r="D23" s="36" t="n"/>
+      <c r="E23" s="36" t="n"/>
+      <c r="F23" s="36" t="n"/>
+      <c r="G23" s="36" t="n"/>
+      <c r="H23" s="36" t="n"/>
+      <c r="I23" s="36" t="n"/>
+      <c r="J23" s="37" t="n"/>
     </row>
     <row r="24" outlineLevel="1" ht="20" customHeight="1">
       <c r="A24" s="31" t="inlineStr">
@@ -2184,7 +2262,7 @@
     <row r="34" outlineLevel="1" ht="20" customHeight="1">
       <c r="A34" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B34" s="5" t="n"/>
@@ -2208,7 +2286,7 @@
     <row r="35" outlineLevel="1" ht="20" customHeight="1">
       <c r="A35" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B35" s="5" t="n"/>
@@ -2232,7 +2310,7 @@
     <row r="36" outlineLevel="1" ht="20" customHeight="1">
       <c r="A36" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B36" s="5" t="n"/>
@@ -2256,7 +2334,7 @@
     <row r="37" outlineLevel="1" ht="20" customHeight="1">
       <c r="A37" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B37" s="5" t="n"/>
@@ -2277,12 +2355,44 @@
       <c r="I37" s="33" t="n"/>
       <c r="J37" s="33" t="n"/>
     </row>
-    <row r="38" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="36">
+    <row r="38" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A38" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D38" s="32" t="n"/>
+      <c r="E38" s="32" t="n"/>
+      <c r="F38" s="26" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I38" s="32" t="n"/>
+      <c r="J38" s="32" t="n"/>
+    </row>
+    <row r="39" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A39" s="38">
         <f>IF('Getting Started'!B30&lt;&gt;"","  "&amp;UPPER('Getting Started'!B30)&amp;"   ·   "&amp;'Getting Started'!F30,"  STUDENT 2")</f>
         <v/>
       </c>
+      <c r="B39" s="36" t="n"/>
+      <c r="C39" s="36" t="n"/>
+      <c r="D39" s="36" t="n"/>
+      <c r="E39" s="36" t="n"/>
+      <c r="F39" s="36" t="n"/>
+      <c r="G39" s="36" t="n"/>
+      <c r="H39" s="36" t="n"/>
+      <c r="I39" s="36" t="n"/>
+      <c r="J39" s="37" t="n"/>
     </row>
     <row r="40" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A40" s="31" t="inlineStr">
@@ -2527,7 +2637,7 @@
     <row r="50" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A50" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B50" s="5" t="n"/>
@@ -2551,7 +2661,7 @@
     <row r="51" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A51" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B51" s="5" t="n"/>
@@ -2575,7 +2685,7 @@
     <row r="52" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A52" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B52" s="5" t="n"/>
@@ -2599,7 +2709,7 @@
     <row r="53" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A53" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B53" s="5" t="n"/>
@@ -2620,12 +2730,44 @@
       <c r="I53" s="33" t="n"/>
       <c r="J53" s="33" t="n"/>
     </row>
-    <row r="54" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="37">
+    <row r="54" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A54" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n"/>
+      <c r="C54" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D54" s="32" t="n"/>
+      <c r="E54" s="32" t="n"/>
+      <c r="F54" s="26" t="n"/>
+      <c r="G54" s="5" t="n"/>
+      <c r="H54" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I54" s="32" t="n"/>
+      <c r="J54" s="32" t="n"/>
+    </row>
+    <row r="55" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A55" s="39">
         <f>IF('Getting Started'!B31&lt;&gt;"","  "&amp;UPPER('Getting Started'!B31)&amp;"   ·   "&amp;'Getting Started'!F31,"  STUDENT 3")</f>
         <v/>
       </c>
+      <c r="B55" s="36" t="n"/>
+      <c r="C55" s="36" t="n"/>
+      <c r="D55" s="36" t="n"/>
+      <c r="E55" s="36" t="n"/>
+      <c r="F55" s="36" t="n"/>
+      <c r="G55" s="36" t="n"/>
+      <c r="H55" s="36" t="n"/>
+      <c r="I55" s="36" t="n"/>
+      <c r="J55" s="37" t="n"/>
     </row>
     <row r="56" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A56" s="31" t="inlineStr">
@@ -2870,7 +3012,7 @@
     <row r="66" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A66" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B66" s="5" t="n"/>
@@ -2894,7 +3036,7 @@
     <row r="67" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A67" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B67" s="5" t="n"/>
@@ -2918,7 +3060,7 @@
     <row r="68" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A68" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B68" s="5" t="n"/>
@@ -2942,7 +3084,7 @@
     <row r="69" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A69" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B69" s="5" t="n"/>
@@ -2963,12 +3105,44 @@
       <c r="I69" s="33" t="n"/>
       <c r="J69" s="33" t="n"/>
     </row>
-    <row r="70" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="71" ht="26" customHeight="1">
-      <c r="A71" s="38">
+    <row r="70" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A70" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="n"/>
+      <c r="C70" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D70" s="32" t="n"/>
+      <c r="E70" s="32" t="n"/>
+      <c r="F70" s="26" t="n"/>
+      <c r="G70" s="5" t="n"/>
+      <c r="H70" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I70" s="32" t="n"/>
+      <c r="J70" s="32" t="n"/>
+    </row>
+    <row r="71" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A71" s="40">
         <f>IF('Getting Started'!B32&lt;&gt;"","  "&amp;UPPER('Getting Started'!B32)&amp;"   ·   "&amp;'Getting Started'!F32,"  STUDENT 4")</f>
         <v/>
       </c>
+      <c r="B71" s="36" t="n"/>
+      <c r="C71" s="36" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="36" t="n"/>
+      <c r="F71" s="36" t="n"/>
+      <c r="G71" s="36" t="n"/>
+      <c r="H71" s="36" t="n"/>
+      <c r="I71" s="36" t="n"/>
+      <c r="J71" s="37" t="n"/>
     </row>
     <row r="72" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A72" s="31" t="inlineStr">
@@ -3213,7 +3387,7 @@
     <row r="82" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A82" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B82" s="5" t="n"/>
@@ -3237,7 +3411,7 @@
     <row r="83" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A83" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B83" s="5" t="n"/>
@@ -3261,7 +3435,7 @@
     <row r="84" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A84" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B84" s="5" t="n"/>
@@ -3285,7 +3459,7 @@
     <row r="85" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A85" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B85" s="5" t="n"/>
@@ -3306,12 +3480,44 @@
       <c r="I85" s="33" t="n"/>
       <c r="J85" s="33" t="n"/>
     </row>
-    <row r="86" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="87" ht="26" customHeight="1">
-      <c r="A87" s="39">
+    <row r="86" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A86" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="n"/>
+      <c r="C86" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D86" s="32" t="n"/>
+      <c r="E86" s="32" t="n"/>
+      <c r="F86" s="26" t="n"/>
+      <c r="G86" s="5" t="n"/>
+      <c r="H86" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I86" s="32" t="n"/>
+      <c r="J86" s="32" t="n"/>
+    </row>
+    <row r="87" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A87" s="41">
         <f>IF('Getting Started'!B33&lt;&gt;"","  "&amp;UPPER('Getting Started'!B33)&amp;"   ·   "&amp;'Getting Started'!F33,"  STUDENT 5")</f>
         <v/>
       </c>
+      <c r="B87" s="36" t="n"/>
+      <c r="C87" s="36" t="n"/>
+      <c r="D87" s="36" t="n"/>
+      <c r="E87" s="36" t="n"/>
+      <c r="F87" s="36" t="n"/>
+      <c r="G87" s="36" t="n"/>
+      <c r="H87" s="36" t="n"/>
+      <c r="I87" s="36" t="n"/>
+      <c r="J87" s="37" t="n"/>
     </row>
     <row r="88" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A88" s="31" t="inlineStr">
@@ -3556,7 +3762,7 @@
     <row r="98" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A98" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B98" s="5" t="n"/>
@@ -3580,7 +3786,7 @@
     <row r="99" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A99" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B99" s="5" t="n"/>
@@ -3604,7 +3810,7 @@
     <row r="100" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A100" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B100" s="5" t="n"/>
@@ -3628,7 +3834,7 @@
     <row r="101" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A101" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B101" s="5" t="n"/>
@@ -3649,12 +3855,44 @@
       <c r="I101" s="33" t="n"/>
       <c r="J101" s="33" t="n"/>
     </row>
-    <row r="102" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="103" ht="26" customHeight="1">
-      <c r="A103" s="40">
+    <row r="102" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A102" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="n"/>
+      <c r="C102" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D102" s="32" t="n"/>
+      <c r="E102" s="32" t="n"/>
+      <c r="F102" s="26" t="n"/>
+      <c r="G102" s="5" t="n"/>
+      <c r="H102" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I102" s="32" t="n"/>
+      <c r="J102" s="32" t="n"/>
+    </row>
+    <row r="103" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A103" s="42">
         <f>IF('Getting Started'!B34&lt;&gt;"","  "&amp;UPPER('Getting Started'!B34)&amp;"   ·   "&amp;'Getting Started'!F34,"  STUDENT 6")</f>
         <v/>
       </c>
+      <c r="B103" s="36" t="n"/>
+      <c r="C103" s="36" t="n"/>
+      <c r="D103" s="36" t="n"/>
+      <c r="E103" s="36" t="n"/>
+      <c r="F103" s="36" t="n"/>
+      <c r="G103" s="36" t="n"/>
+      <c r="H103" s="36" t="n"/>
+      <c r="I103" s="36" t="n"/>
+      <c r="J103" s="37" t="n"/>
     </row>
     <row r="104" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A104" s="31" t="inlineStr">
@@ -3899,7 +4137,7 @@
     <row r="114" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A114" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B114" s="5" t="n"/>
@@ -3923,7 +4161,7 @@
     <row r="115" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A115" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B115" s="5" t="n"/>
@@ -3947,7 +4185,7 @@
     <row r="116" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A116" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B116" s="5" t="n"/>
@@ -3971,7 +4209,7 @@
     <row r="117" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A117" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B117" s="5" t="n"/>
@@ -3992,12 +4230,44 @@
       <c r="I117" s="33" t="n"/>
       <c r="J117" s="33" t="n"/>
     </row>
-    <row r="118" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="119" ht="26" customHeight="1">
-      <c r="A119" s="41">
+    <row r="118" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A118" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B118" s="5" t="n"/>
+      <c r="C118" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D118" s="32" t="n"/>
+      <c r="E118" s="32" t="n"/>
+      <c r="F118" s="26" t="n"/>
+      <c r="G118" s="5" t="n"/>
+      <c r="H118" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I118" s="32" t="n"/>
+      <c r="J118" s="32" t="n"/>
+    </row>
+    <row r="119" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A119" s="43">
         <f>IF('Getting Started'!B35&lt;&gt;"","  "&amp;UPPER('Getting Started'!B35)&amp;"   ·   "&amp;'Getting Started'!F35,"  STUDENT 7")</f>
         <v/>
       </c>
+      <c r="B119" s="36" t="n"/>
+      <c r="C119" s="36" t="n"/>
+      <c r="D119" s="36" t="n"/>
+      <c r="E119" s="36" t="n"/>
+      <c r="F119" s="36" t="n"/>
+      <c r="G119" s="36" t="n"/>
+      <c r="H119" s="36" t="n"/>
+      <c r="I119" s="36" t="n"/>
+      <c r="J119" s="37" t="n"/>
     </row>
     <row r="120" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A120" s="31" t="inlineStr">
@@ -4242,7 +4512,7 @@
     <row r="130" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A130" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B130" s="5" t="n"/>
@@ -4266,7 +4536,7 @@
     <row r="131" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A131" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B131" s="5" t="n"/>
@@ -4290,7 +4560,7 @@
     <row r="132" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A132" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B132" s="5" t="n"/>
@@ -4314,7 +4584,7 @@
     <row r="133" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A133" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B133" s="5" t="n"/>
@@ -4335,12 +4605,44 @@
       <c r="I133" s="33" t="n"/>
       <c r="J133" s="33" t="n"/>
     </row>
-    <row r="134" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="135" ht="26" customHeight="1">
-      <c r="A135" s="42">
+    <row r="134" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A134" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="n"/>
+      <c r="C134" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D134" s="32" t="n"/>
+      <c r="E134" s="32" t="n"/>
+      <c r="F134" s="26" t="n"/>
+      <c r="G134" s="5" t="n"/>
+      <c r="H134" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I134" s="32" t="n"/>
+      <c r="J134" s="32" t="n"/>
+    </row>
+    <row r="135" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A135" s="44">
         <f>IF('Getting Started'!B36&lt;&gt;"","  "&amp;UPPER('Getting Started'!B36)&amp;"   ·   "&amp;'Getting Started'!F36,"  STUDENT 8")</f>
         <v/>
       </c>
+      <c r="B135" s="36" t="n"/>
+      <c r="C135" s="36" t="n"/>
+      <c r="D135" s="36" t="n"/>
+      <c r="E135" s="36" t="n"/>
+      <c r="F135" s="36" t="n"/>
+      <c r="G135" s="36" t="n"/>
+      <c r="H135" s="36" t="n"/>
+      <c r="I135" s="36" t="n"/>
+      <c r="J135" s="37" t="n"/>
     </row>
     <row r="136" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A136" s="31" t="inlineStr">
@@ -4585,7 +4887,7 @@
     <row r="146" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A146" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B146" s="5" t="n"/>
@@ -4609,7 +4911,7 @@
     <row r="147" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A147" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B147" s="5" t="n"/>
@@ -4633,7 +4935,7 @@
     <row r="148" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A148" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B148" s="5" t="n"/>
@@ -4657,7 +4959,7 @@
     <row r="149" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A149" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B149" s="5" t="n"/>
@@ -4678,12 +4980,44 @@
       <c r="I149" s="33" t="n"/>
       <c r="J149" s="33" t="n"/>
     </row>
-    <row r="150" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="151" ht="26" customHeight="1">
-      <c r="A151" s="43">
+    <row r="150" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A150" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="n"/>
+      <c r="C150" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D150" s="32" t="n"/>
+      <c r="E150" s="32" t="n"/>
+      <c r="F150" s="26" t="n"/>
+      <c r="G150" s="5" t="n"/>
+      <c r="H150" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I150" s="32" t="n"/>
+      <c r="J150" s="32" t="n"/>
+    </row>
+    <row r="151" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A151" s="45">
         <f>IF('Getting Started'!B37&lt;&gt;"","  "&amp;UPPER('Getting Started'!B37)&amp;"   ·   "&amp;'Getting Started'!F37,"  STUDENT 9")</f>
         <v/>
       </c>
+      <c r="B151" s="36" t="n"/>
+      <c r="C151" s="36" t="n"/>
+      <c r="D151" s="36" t="n"/>
+      <c r="E151" s="36" t="n"/>
+      <c r="F151" s="36" t="n"/>
+      <c r="G151" s="36" t="n"/>
+      <c r="H151" s="36" t="n"/>
+      <c r="I151" s="36" t="n"/>
+      <c r="J151" s="37" t="n"/>
     </row>
     <row r="152" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A152" s="31" t="inlineStr">
@@ -4928,7 +5262,7 @@
     <row r="162" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A162" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B162" s="5" t="n"/>
@@ -4952,7 +5286,7 @@
     <row r="163" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A163" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B163" s="5" t="n"/>
@@ -4976,7 +5310,7 @@
     <row r="164" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A164" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B164" s="5" t="n"/>
@@ -5000,7 +5334,7 @@
     <row r="165" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A165" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B165" s="5" t="n"/>
@@ -5021,12 +5355,44 @@
       <c r="I165" s="33" t="n"/>
       <c r="J165" s="33" t="n"/>
     </row>
-    <row r="166" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="167" ht="26" customHeight="1">
-      <c r="A167" s="44">
+    <row r="166" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A166" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="n"/>
+      <c r="C166" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D166" s="32" t="n"/>
+      <c r="E166" s="32" t="n"/>
+      <c r="F166" s="26" t="n"/>
+      <c r="G166" s="5" t="n"/>
+      <c r="H166" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I166" s="32" t="n"/>
+      <c r="J166" s="32" t="n"/>
+    </row>
+    <row r="167" hidden="1" outlineLevel="1" ht="26" customHeight="1">
+      <c r="A167" s="46">
         <f>IF('Getting Started'!B38&lt;&gt;"","  "&amp;UPPER('Getting Started'!B38)&amp;"   ·   "&amp;'Getting Started'!F38,"  STUDENT 10")</f>
         <v/>
       </c>
+      <c r="B167" s="36" t="n"/>
+      <c r="C167" s="36" t="n"/>
+      <c r="D167" s="36" t="n"/>
+      <c r="E167" s="36" t="n"/>
+      <c r="F167" s="36" t="n"/>
+      <c r="G167" s="36" t="n"/>
+      <c r="H167" s="36" t="n"/>
+      <c r="I167" s="36" t="n"/>
+      <c r="J167" s="37" t="n"/>
     </row>
     <row r="168" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A168" s="31" t="inlineStr">
@@ -5271,7 +5637,7 @@
     <row r="178" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A178" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 1</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B178" s="5" t="n"/>
@@ -5295,7 +5661,7 @@
     <row r="179" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A179" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 2</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B179" s="5" t="n"/>
@@ -5319,7 +5685,7 @@
     <row r="180" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A180" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 3</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B180" s="5" t="n"/>
@@ -5343,7 +5709,7 @@
     <row r="181" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A181" s="34" t="inlineStr">
         <is>
-          <t>Elective / Other 4</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B181" s="5" t="n"/>
@@ -5364,7 +5730,103 @@
       <c r="I181" s="33" t="n"/>
       <c r="J181" s="33" t="n"/>
     </row>
-    <row r="182" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="182" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A182" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="n"/>
+      <c r="C182" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D182" s="32" t="n"/>
+      <c r="E182" s="32" t="n"/>
+      <c r="F182" s="26" t="n"/>
+      <c r="G182" s="5" t="n"/>
+      <c r="H182" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I182" s="32" t="n"/>
+      <c r="J182" s="32" t="n"/>
+    </row>
+    <row r="183" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A183" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="n"/>
+      <c r="C183" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D183" s="33" t="n"/>
+      <c r="E183" s="33" t="n"/>
+      <c r="F183" s="26" t="n"/>
+      <c r="G183" s="5" t="n"/>
+      <c r="H183" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I183" s="33" t="n"/>
+      <c r="J183" s="33" t="n"/>
+    </row>
+    <row r="184" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A184" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
+        </is>
+      </c>
+      <c r="B184" s="5" t="n"/>
+      <c r="C184" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D184" s="32" t="n"/>
+      <c r="E184" s="32" t="n"/>
+      <c r="F184" s="26" t="n"/>
+      <c r="G184" s="5" t="n"/>
+      <c r="H184" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I184" s="32" t="n"/>
+      <c r="J184" s="32" t="n"/>
+    </row>
+    <row r="185" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A185" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="n"/>
+      <c r="C185" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D185" s="33" t="n"/>
+      <c r="E185" s="33" t="n"/>
+      <c r="F185" s="26" t="n"/>
+      <c r="G185" s="5" t="n"/>
+      <c r="H185" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I185" s="33" t="n"/>
+      <c r="J185" s="33" t="n"/>
+    </row>
+    <row r="186" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="A5:A6"/>
@@ -5386,7 +5848,7 @@
     <mergeCell ref="A71:J71"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C56 C57 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67 C68 C69 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C83 C84 C85 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C104 C105 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C120 C121 C122 C123 C124 C125 C126 C127 C128 C129 C130 C131 C132 C133 C136 C137 C138 C139 C140 C141 C142 C143 C144 C145 C146 C147 C148 C149 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C162 C163 C164 C165 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H120 H121 H122 H123 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H146 H147 H148 H149 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C83 C84 C85 C86 C87 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C102 C103 C104 C105 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C118 C119 C120 C121 C122 C123 C124 C125 C126 C127 C128 C129 C130 C131 C132 C133 C134 C135 C136 C137 C138 C139 C140 C141 C142 C143 C144 C145 C146 C147 C148 C149 C150 C151 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C162 C163 C164 C165 C166 C167 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 C182 C183 C184 C185 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 H103 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H122 H123 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H146 H147 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H166 H167 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H182 H183 H184 H185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"pages,lessons,chapters,units,assignments,projects"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5401,7 +5863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5425,40 +5887,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="45">
+      <c r="A1" s="47">
         <f>IF('Getting Started'!B29="","Student 1",'Getting Started'!B29)</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="46">
+      <c r="A2" s="48">
         <f>IFERROR("Grade: "&amp;'Getting Started'!F29&amp;"   ·   School Year: "&amp;'Getting Started'!C6,"")</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="47">
+      <c r="A4" s="49">
         <f>IFERROR("SEM 1   "&amp;TEXT('Getting Started'!C10,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C11,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C15&amp;" school wks)","SEMESTER 1")</f>
         <v/>
       </c>
       <c r="J4" s="26" t="n"/>
-      <c r="K4" s="48">
+      <c r="K4" s="50">
         <f>IFERROR("SEM 2   "&amp;TEXT('Getting Started'!C18,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C19,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C23&amp;" school wks)","SEMESTER 2")</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1"/>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="49" t="inlineStr">
+      <c r="A6" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">  SCHOOL DAYS  ·  Mark each day this student attends</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="50" t="inlineStr"/>
-      <c r="B7" s="51" t="inlineStr">
+      <c r="A7" s="52" t="inlineStr"/>
+      <c r="B7" s="53" t="inlineStr">
         <is>
           <t>Typical school week  →</t>
         </is>
@@ -5499,25 +5961,25 @@
         </is>
       </c>
       <c r="J7" s="26" t="n"/>
-      <c r="K7" s="52" t="n"/>
-      <c r="L7" s="52" t="n"/>
-      <c r="M7" s="52" t="n"/>
-      <c r="N7" s="52" t="n"/>
-      <c r="O7" s="52" t="n"/>
-      <c r="P7" s="52" t="n"/>
-      <c r="Q7" s="52" t="n"/>
-      <c r="R7" s="52" t="n"/>
+      <c r="K7" s="54" t="n"/>
+      <c r="L7" s="54" t="n"/>
+      <c r="M7" s="54" t="n"/>
+      <c r="N7" s="54" t="n"/>
+      <c r="O7" s="54" t="n"/>
+      <c r="P7" s="54" t="n"/>
+      <c r="Q7" s="54" t="n"/>
+      <c r="R7" s="54" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="26" t="n"/>
       <c r="B8" s="26" t="n"/>
-      <c r="C8" s="53" t="n"/>
-      <c r="D8" s="53" t="n"/>
-      <c r="E8" s="53" t="n"/>
-      <c r="F8" s="53" t="n"/>
-      <c r="G8" s="53" t="n"/>
-      <c r="H8" s="53" t="n"/>
-      <c r="I8" s="54">
+      <c r="C8" s="55" t="n"/>
+      <c r="D8" s="55" t="n"/>
+      <c r="E8" s="55" t="n"/>
+      <c r="F8" s="55" t="n"/>
+      <c r="G8" s="55" t="n"/>
+      <c r="H8" s="55" t="n"/>
+      <c r="I8" s="56">
         <f>MAX(1,COUNTA(C8:H8))</f>
         <v/>
       </c>
@@ -5533,91 +5995,91 @@
     </row>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="55" t="inlineStr">
+      <c r="A10" s="57" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="B10" s="55" t="inlineStr">
+      <c r="B10" s="57" t="inlineStr">
         <is>
           <t>Curriculum / Book</t>
         </is>
       </c>
-      <c r="C10" s="55" t="inlineStr">
+      <c r="C10" s="57" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D10" s="55" t="inlineStr">
+      <c r="D10" s="57" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="E10" s="55" t="inlineStr">
+      <c r="E10" s="57" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="F10" s="55" t="inlineStr">
+      <c r="F10" s="57" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="G10" s="55" t="inlineStr">
+      <c r="G10" s="57" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="H10" s="55" t="inlineStr">
+      <c r="H10" s="57" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="I10" s="55" t="inlineStr">
+      <c r="I10" s="57" t="inlineStr">
         <is>
           <t>Days
 /Wk</t>
         </is>
       </c>
       <c r="J10" s="26" t="n"/>
-      <c r="K10" s="56" t="inlineStr">
+      <c r="K10" s="58" t="inlineStr">
         <is>
           <t>S1
 Total</t>
         </is>
       </c>
-      <c r="L10" s="56" t="inlineStr">
+      <c r="L10" s="58" t="inlineStr">
         <is>
           <t>S1
 /Wk</t>
         </is>
       </c>
-      <c r="M10" s="56" t="inlineStr">
+      <c r="M10" s="58" t="inlineStr">
         <is>
           <t>S1
 /Day</t>
         </is>
       </c>
       <c r="N10" s="26" t="n"/>
-      <c r="O10" s="57" t="inlineStr">
+      <c r="O10" s="59" t="inlineStr">
         <is>
           <t>S2
 Total</t>
         </is>
       </c>
-      <c r="P10" s="57" t="inlineStr">
+      <c r="P10" s="59" t="inlineStr">
         <is>
           <t>S2
 /Wk</t>
         </is>
       </c>
-      <c r="Q10" s="57" t="inlineStr">
+      <c r="Q10" s="59" t="inlineStr">
         <is>
           <t>S2
 /Day</t>
         </is>
       </c>
-      <c r="R10" s="55" t="inlineStr">
+      <c r="R10" s="57" t="inlineStr">
         <is>
           <t>Unit
 Type</t>
@@ -5634,43 +6096,43 @@
         <f>IFERROR(IF('Course Content'!B24&lt;&gt;"",'Course Content'!B24,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,IF('Course Content'!G24&lt;&gt;"",'Course Content'!G24,IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C11" s="58" t="n"/>
-      <c r="D11" s="58" t="n"/>
-      <c r="E11" s="58" t="n"/>
-      <c r="F11" s="58" t="n"/>
-      <c r="G11" s="58" t="n"/>
-      <c r="H11" s="58" t="n"/>
+      <c r="C11" s="60" t="n"/>
+      <c r="D11" s="60" t="n"/>
+      <c r="E11" s="60" t="n"/>
+      <c r="F11" s="60" t="n"/>
+      <c r="G11" s="60" t="n"/>
+      <c r="H11" s="60" t="n"/>
       <c r="I11" s="17">
         <f>IF(COUNTA(C11:H11)=0,$I$8,COUNTA(C11:H11))</f>
         <v/>
       </c>
       <c r="J11" s="26" t="n"/>
-      <c r="K11" s="59">
+      <c r="K11" s="61">
         <f>IFERROR(IF(('Course Content'!D8="")*('Course Content'!I8="")*('Course Content'!D24="")*('Course Content'!I24=""),"—",IFERROR('Course Content'!D8*1,0)+IFERROR('Course Content'!I8*1,0)+IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L11" s="59">
+      <c r="L11" s="61">
         <f>IFERROR(IF(K11="","",IF(K11="—","",FLOOR(K11/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M11" s="60">
+      <c r="M11" s="62">
         <f>IFERROR(IF(L11="","",IF(L11="—","",FLOOR(L11/I11,1))),"")</f>
         <v/>
       </c>
       <c r="N11" s="26" t="n"/>
-      <c r="O11" s="61">
+      <c r="O11" s="63">
         <f>IFERROR(IF(('Course Content'!E8="")*('Course Content'!J8="")*('Course Content'!E24="")*('Course Content'!J24=""),"—",IFERROR('Course Content'!E8*1,0)+IFERROR('Course Content'!J8*1,0)+IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P11" s="61">
+      <c r="P11" s="63">
         <f>IFERROR(IF(O11="","",IF(O11="—","",FLOOR(O11/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q11" s="62">
+      <c r="Q11" s="64">
         <f>IFERROR(IF(P11="","",IF(P11="—","",FLOOR(P11/I11,1))),"")</f>
         <v/>
       </c>
-      <c r="R11" s="63">
+      <c r="R11" s="65">
         <f>IFERROR(IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,IF('Course Content'!H24&lt;&gt;"",'Course Content'!H24,IF('Course Content'!C8&lt;&gt;"",'Course Content'!C8,'Course Content'!H8))),"")</f>
         <v/>
       </c>
@@ -5685,43 +6147,43 @@
         <f>IFERROR(IF('Course Content'!B25&lt;&gt;"",'Course Content'!B25,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,IF('Course Content'!G25&lt;&gt;"",'Course Content'!G25,IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C12" s="58" t="n"/>
-      <c r="D12" s="58" t="n"/>
-      <c r="E12" s="58" t="n"/>
-      <c r="F12" s="58" t="n"/>
-      <c r="G12" s="58" t="n"/>
-      <c r="H12" s="58" t="n"/>
+      <c r="C12" s="60" t="n"/>
+      <c r="D12" s="60" t="n"/>
+      <c r="E12" s="60" t="n"/>
+      <c r="F12" s="60" t="n"/>
+      <c r="G12" s="60" t="n"/>
+      <c r="H12" s="60" t="n"/>
       <c r="I12" s="17">
         <f>IF(COUNTA(C12:H12)=0,$I$8,COUNTA(C12:H12))</f>
         <v/>
       </c>
       <c r="J12" s="26" t="n"/>
-      <c r="K12" s="59">
+      <c r="K12" s="61">
         <f>IFERROR(IF(('Course Content'!D9="")*('Course Content'!I9="")*('Course Content'!D25="")*('Course Content'!I25=""),"—",IFERROR('Course Content'!D9*1,0)+IFERROR('Course Content'!I9*1,0)+IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L12" s="59">
+      <c r="L12" s="61">
         <f>IFERROR(IF(K12="","",IF(K12="—","",FLOOR(K12/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M12" s="60">
+      <c r="M12" s="62">
         <f>IFERROR(IF(L12="","",IF(L12="—","",FLOOR(L12/I12,1))),"")</f>
         <v/>
       </c>
       <c r="N12" s="26" t="n"/>
-      <c r="O12" s="61">
+      <c r="O12" s="63">
         <f>IFERROR(IF(('Course Content'!E9="")*('Course Content'!J9="")*('Course Content'!E25="")*('Course Content'!J25=""),"—",IFERROR('Course Content'!E9*1,0)+IFERROR('Course Content'!J9*1,0)+IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P12" s="61">
+      <c r="P12" s="63">
         <f>IFERROR(IF(O12="","",IF(O12="—","",FLOOR(O12/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q12" s="62">
+      <c r="Q12" s="64">
         <f>IFERROR(IF(P12="","",IF(P12="—","",FLOOR(P12/I12,1))),"")</f>
         <v/>
       </c>
-      <c r="R12" s="64">
+      <c r="R12" s="66">
         <f>IFERROR(IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,IF('Course Content'!H25&lt;&gt;"",'Course Content'!H25,IF('Course Content'!C9&lt;&gt;"",'Course Content'!C9,'Course Content'!H9))),"")</f>
         <v/>
       </c>
@@ -5736,43 +6198,43 @@
         <f>IFERROR(IF('Course Content'!B26&lt;&gt;"",'Course Content'!B26,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,IF('Course Content'!G26&lt;&gt;"",'Course Content'!G26,IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C13" s="58" t="n"/>
-      <c r="D13" s="58" t="n"/>
-      <c r="E13" s="58" t="n"/>
-      <c r="F13" s="58" t="n"/>
-      <c r="G13" s="58" t="n"/>
-      <c r="H13" s="58" t="n"/>
+      <c r="C13" s="60" t="n"/>
+      <c r="D13" s="60" t="n"/>
+      <c r="E13" s="60" t="n"/>
+      <c r="F13" s="60" t="n"/>
+      <c r="G13" s="60" t="n"/>
+      <c r="H13" s="60" t="n"/>
       <c r="I13" s="17">
         <f>IF(COUNTA(C13:H13)=0,$I$8,COUNTA(C13:H13))</f>
         <v/>
       </c>
       <c r="J13" s="26" t="n"/>
-      <c r="K13" s="59">
+      <c r="K13" s="61">
         <f>IFERROR(IF(('Course Content'!D10="")*('Course Content'!I10="")*('Course Content'!D26="")*('Course Content'!I26=""),"—",IFERROR('Course Content'!D10*1,0)+IFERROR('Course Content'!I10*1,0)+IFERROR('Course Content'!D26*1,0)+IFERROR('Course Content'!I26*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L13" s="59">
+      <c r="L13" s="61">
         <f>IFERROR(IF(K13="","",IF(K13="—","",FLOOR(K13/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M13" s="60">
+      <c r="M13" s="62">
         <f>IFERROR(IF(L13="","",IF(L13="—","",FLOOR(L13/I13,1))),"")</f>
         <v/>
       </c>
       <c r="N13" s="26" t="n"/>
-      <c r="O13" s="61">
+      <c r="O13" s="63">
         <f>IFERROR(IF(('Course Content'!E10="")*('Course Content'!J10="")*('Course Content'!E26="")*('Course Content'!J26=""),"—",IFERROR('Course Content'!E10*1,0)+IFERROR('Course Content'!J10*1,0)+IFERROR('Course Content'!E26*1,0)+IFERROR('Course Content'!J26*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P13" s="61">
+      <c r="P13" s="63">
         <f>IFERROR(IF(O13="","",IF(O13="—","",FLOOR(O13/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q13" s="62">
+      <c r="Q13" s="64">
         <f>IFERROR(IF(P13="","",IF(P13="—","",FLOOR(P13/I13,1))),"")</f>
         <v/>
       </c>
-      <c r="R13" s="63">
+      <c r="R13" s="65">
         <f>IFERROR(IF('Course Content'!C26&lt;&gt;"",'Course Content'!C26,IF('Course Content'!H26&lt;&gt;"",'Course Content'!H26,IF('Course Content'!C10&lt;&gt;"",'Course Content'!C10,'Course Content'!H10))),"")</f>
         <v/>
       </c>
@@ -5787,43 +6249,43 @@
         <f>IFERROR(IF('Course Content'!B27&lt;&gt;"",'Course Content'!B27,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,IF('Course Content'!G27&lt;&gt;"",'Course Content'!G27,IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C14" s="58" t="n"/>
-      <c r="D14" s="58" t="n"/>
-      <c r="E14" s="58" t="n"/>
-      <c r="F14" s="58" t="n"/>
-      <c r="G14" s="58" t="n"/>
-      <c r="H14" s="58" t="n"/>
+      <c r="C14" s="60" t="n"/>
+      <c r="D14" s="60" t="n"/>
+      <c r="E14" s="60" t="n"/>
+      <c r="F14" s="60" t="n"/>
+      <c r="G14" s="60" t="n"/>
+      <c r="H14" s="60" t="n"/>
       <c r="I14" s="17">
         <f>IF(COUNTA(C14:H14)=0,$I$8,COUNTA(C14:H14))</f>
         <v/>
       </c>
       <c r="J14" s="26" t="n"/>
-      <c r="K14" s="59">
+      <c r="K14" s="61">
         <f>IFERROR(IF(('Course Content'!D11="")*('Course Content'!I11="")*('Course Content'!D27="")*('Course Content'!I27=""),"—",IFERROR('Course Content'!D11*1,0)+IFERROR('Course Content'!I11*1,0)+IFERROR('Course Content'!D27*1,0)+IFERROR('Course Content'!I27*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L14" s="59">
+      <c r="L14" s="61">
         <f>IFERROR(IF(K14="","",IF(K14="—","",FLOOR(K14/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M14" s="60">
+      <c r="M14" s="62">
         <f>IFERROR(IF(L14="","",IF(L14="—","",FLOOR(L14/I14,1))),"")</f>
         <v/>
       </c>
       <c r="N14" s="26" t="n"/>
-      <c r="O14" s="61">
+      <c r="O14" s="63">
         <f>IFERROR(IF(('Course Content'!E11="")*('Course Content'!J11="")*('Course Content'!E27="")*('Course Content'!J27=""),"—",IFERROR('Course Content'!E11*1,0)+IFERROR('Course Content'!J11*1,0)+IFERROR('Course Content'!E27*1,0)+IFERROR('Course Content'!J27*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P14" s="61">
+      <c r="P14" s="63">
         <f>IFERROR(IF(O14="","",IF(O14="—","",FLOOR(O14/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q14" s="62">
+      <c r="Q14" s="64">
         <f>IFERROR(IF(P14="","",IF(P14="—","",FLOOR(P14/I14,1))),"")</f>
         <v/>
       </c>
-      <c r="R14" s="64">
+      <c r="R14" s="66">
         <f>IFERROR(IF('Course Content'!C27&lt;&gt;"",'Course Content'!C27,IF('Course Content'!H27&lt;&gt;"",'Course Content'!H27,IF('Course Content'!C11&lt;&gt;"",'Course Content'!C11,'Course Content'!H11))),"")</f>
         <v/>
       </c>
@@ -5838,43 +6300,43 @@
         <f>IFERROR(IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C15" s="58" t="n"/>
-      <c r="D15" s="58" t="n"/>
-      <c r="E15" s="58" t="n"/>
-      <c r="F15" s="58" t="n"/>
-      <c r="G15" s="58" t="n"/>
-      <c r="H15" s="58" t="n"/>
+      <c r="C15" s="60" t="n"/>
+      <c r="D15" s="60" t="n"/>
+      <c r="E15" s="60" t="n"/>
+      <c r="F15" s="60" t="n"/>
+      <c r="G15" s="60" t="n"/>
+      <c r="H15" s="60" t="n"/>
       <c r="I15" s="17">
         <f>IF(COUNTA(C15:H15)=0,$I$8,COUNTA(C15:H15))</f>
         <v/>
       </c>
       <c r="J15" s="26" t="n"/>
-      <c r="K15" s="59">
+      <c r="K15" s="61">
         <f>IFERROR(IF(('Course Content'!D12="")*('Course Content'!I12="")*('Course Content'!D28="")*('Course Content'!I28=""),"—",IFERROR('Course Content'!D12*1,0)+IFERROR('Course Content'!I12*1,0)+IFERROR('Course Content'!D28*1,0)+IFERROR('Course Content'!I28*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L15" s="59">
+      <c r="L15" s="61">
         <f>IFERROR(IF(K15="","",IF(K15="—","",FLOOR(K15/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M15" s="60">
+      <c r="M15" s="62">
         <f>IFERROR(IF(L15="","",IF(L15="—","",FLOOR(L15/I15,1))),"")</f>
         <v/>
       </c>
       <c r="N15" s="26" t="n"/>
-      <c r="O15" s="61">
+      <c r="O15" s="63">
         <f>IFERROR(IF(('Course Content'!E12="")*('Course Content'!J12="")*('Course Content'!E28="")*('Course Content'!J28=""),"—",IFERROR('Course Content'!E12*1,0)+IFERROR('Course Content'!J12*1,0)+IFERROR('Course Content'!E28*1,0)+IFERROR('Course Content'!J28*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P15" s="61">
+      <c r="P15" s="63">
         <f>IFERROR(IF(O15="","",IF(O15="—","",FLOOR(O15/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q15" s="62">
+      <c r="Q15" s="64">
         <f>IFERROR(IF(P15="","",IF(P15="—","",FLOOR(P15/I15,1))),"")</f>
         <v/>
       </c>
-      <c r="R15" s="63">
+      <c r="R15" s="65">
         <f>IFERROR(IF('Course Content'!C28&lt;&gt;"",'Course Content'!C28,IF('Course Content'!H28&lt;&gt;"",'Course Content'!H28,IF('Course Content'!C12&lt;&gt;"",'Course Content'!C12,'Course Content'!H12))),"")</f>
         <v/>
       </c>
@@ -5889,43 +6351,43 @@
         <f>IFERROR(IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C16" s="58" t="n"/>
-      <c r="D16" s="58" t="n"/>
-      <c r="E16" s="58" t="n"/>
-      <c r="F16" s="58" t="n"/>
-      <c r="G16" s="58" t="n"/>
-      <c r="H16" s="58" t="n"/>
+      <c r="C16" s="60" t="n"/>
+      <c r="D16" s="60" t="n"/>
+      <c r="E16" s="60" t="n"/>
+      <c r="F16" s="60" t="n"/>
+      <c r="G16" s="60" t="n"/>
+      <c r="H16" s="60" t="n"/>
       <c r="I16" s="17">
         <f>IF(COUNTA(C16:H16)=0,$I$8,COUNTA(C16:H16))</f>
         <v/>
       </c>
       <c r="J16" s="26" t="n"/>
-      <c r="K16" s="59">
+      <c r="K16" s="61">
         <f>IFERROR(IF(('Course Content'!D13="")*('Course Content'!I13="")*('Course Content'!D29="")*('Course Content'!I29=""),"—",IFERROR('Course Content'!D13*1,0)+IFERROR('Course Content'!I13*1,0)+IFERROR('Course Content'!D29*1,0)+IFERROR('Course Content'!I29*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L16" s="59">
+      <c r="L16" s="61">
         <f>IFERROR(IF(K16="","",IF(K16="—","",FLOOR(K16/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M16" s="60">
+      <c r="M16" s="62">
         <f>IFERROR(IF(L16="","",IF(L16="—","",FLOOR(L16/I16,1))),"")</f>
         <v/>
       </c>
       <c r="N16" s="26" t="n"/>
-      <c r="O16" s="61">
+      <c r="O16" s="63">
         <f>IFERROR(IF(('Course Content'!E13="")*('Course Content'!J13="")*('Course Content'!E29="")*('Course Content'!J29=""),"—",IFERROR('Course Content'!E13*1,0)+IFERROR('Course Content'!J13*1,0)+IFERROR('Course Content'!E29*1,0)+IFERROR('Course Content'!J29*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P16" s="61">
+      <c r="P16" s="63">
         <f>IFERROR(IF(O16="","",IF(O16="—","",FLOOR(O16/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q16" s="62">
+      <c r="Q16" s="64">
         <f>IFERROR(IF(P16="","",IF(P16="—","",FLOOR(P16/I16,1))),"")</f>
         <v/>
       </c>
-      <c r="R16" s="64">
+      <c r="R16" s="66">
         <f>IFERROR(IF('Course Content'!C29&lt;&gt;"",'Course Content'!C29,IF('Course Content'!H29&lt;&gt;"",'Course Content'!H29,IF('Course Content'!C13&lt;&gt;"",'Course Content'!C13,'Course Content'!H13))),"")</f>
         <v/>
       </c>
@@ -5940,43 +6402,43 @@
         <f>IFERROR(IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C17" s="58" t="n"/>
-      <c r="D17" s="58" t="n"/>
-      <c r="E17" s="58" t="n"/>
-      <c r="F17" s="58" t="n"/>
-      <c r="G17" s="58" t="n"/>
-      <c r="H17" s="58" t="n"/>
+      <c r="C17" s="60" t="n"/>
+      <c r="D17" s="60" t="n"/>
+      <c r="E17" s="60" t="n"/>
+      <c r="F17" s="60" t="n"/>
+      <c r="G17" s="60" t="n"/>
+      <c r="H17" s="60" t="n"/>
       <c r="I17" s="17">
         <f>IF(COUNTA(C17:H17)=0,$I$8,COUNTA(C17:H17))</f>
         <v/>
       </c>
       <c r="J17" s="26" t="n"/>
-      <c r="K17" s="59">
+      <c r="K17" s="61">
         <f>IFERROR(IF(('Course Content'!D14="")*('Course Content'!I14="")*('Course Content'!D30="")*('Course Content'!I30=""),"—",IFERROR('Course Content'!D14*1,0)+IFERROR('Course Content'!I14*1,0)+IFERROR('Course Content'!D30*1,0)+IFERROR('Course Content'!I30*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L17" s="59">
+      <c r="L17" s="61">
         <f>IFERROR(IF(K17="","",IF(K17="—","",FLOOR(K17/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M17" s="60">
+      <c r="M17" s="62">
         <f>IFERROR(IF(L17="","",IF(L17="—","",FLOOR(L17/I17,1))),"")</f>
         <v/>
       </c>
       <c r="N17" s="26" t="n"/>
-      <c r="O17" s="61">
+      <c r="O17" s="63">
         <f>IFERROR(IF(('Course Content'!E14="")*('Course Content'!J14="")*('Course Content'!E30="")*('Course Content'!J30=""),"—",IFERROR('Course Content'!E14*1,0)+IFERROR('Course Content'!J14*1,0)+IFERROR('Course Content'!E30*1,0)+IFERROR('Course Content'!J30*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P17" s="61">
+      <c r="P17" s="63">
         <f>IFERROR(IF(O17="","",IF(O17="—","",FLOOR(O17/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q17" s="62">
+      <c r="Q17" s="64">
         <f>IFERROR(IF(P17="","",IF(P17="—","",FLOOR(P17/I17,1))),"")</f>
         <v/>
       </c>
-      <c r="R17" s="63">
+      <c r="R17" s="65">
         <f>IFERROR(IF('Course Content'!C30&lt;&gt;"",'Course Content'!C30,IF('Course Content'!H30&lt;&gt;"",'Course Content'!H30,IF('Course Content'!C14&lt;&gt;"",'Course Content'!C14,'Course Content'!H14))),"")</f>
         <v/>
       </c>
@@ -5991,43 +6453,43 @@
         <f>IFERROR(IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C18" s="58" t="n"/>
-      <c r="D18" s="58" t="n"/>
-      <c r="E18" s="58" t="n"/>
-      <c r="F18" s="58" t="n"/>
-      <c r="G18" s="58" t="n"/>
-      <c r="H18" s="58" t="n"/>
+      <c r="C18" s="60" t="n"/>
+      <c r="D18" s="60" t="n"/>
+      <c r="E18" s="60" t="n"/>
+      <c r="F18" s="60" t="n"/>
+      <c r="G18" s="60" t="n"/>
+      <c r="H18" s="60" t="n"/>
       <c r="I18" s="17">
         <f>IF(COUNTA(C18:H18)=0,$I$8,COUNTA(C18:H18))</f>
         <v/>
       </c>
       <c r="J18" s="26" t="n"/>
-      <c r="K18" s="59">
+      <c r="K18" s="61">
         <f>IFERROR(IF(('Course Content'!D15="")*('Course Content'!I15="")*('Course Content'!D31="")*('Course Content'!I31=""),"—",IFERROR('Course Content'!D15*1,0)+IFERROR('Course Content'!I15*1,0)+IFERROR('Course Content'!D31*1,0)+IFERROR('Course Content'!I31*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L18" s="59">
+      <c r="L18" s="61">
         <f>IFERROR(IF(K18="","",IF(K18="—","",FLOOR(K18/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M18" s="60">
+      <c r="M18" s="62">
         <f>IFERROR(IF(L18="","",IF(L18="—","",FLOOR(L18/I18,1))),"")</f>
         <v/>
       </c>
       <c r="N18" s="26" t="n"/>
-      <c r="O18" s="61">
+      <c r="O18" s="63">
         <f>IFERROR(IF(('Course Content'!E15="")*('Course Content'!J15="")*('Course Content'!E31="")*('Course Content'!J31=""),"—",IFERROR('Course Content'!E15*1,0)+IFERROR('Course Content'!J15*1,0)+IFERROR('Course Content'!E31*1,0)+IFERROR('Course Content'!J31*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P18" s="61">
+      <c r="P18" s="63">
         <f>IFERROR(IF(O18="","",IF(O18="—","",FLOOR(O18/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q18" s="62">
+      <c r="Q18" s="64">
         <f>IFERROR(IF(P18="","",IF(P18="—","",FLOOR(P18/I18,1))),"")</f>
         <v/>
       </c>
-      <c r="R18" s="64">
+      <c r="R18" s="66">
         <f>IFERROR(IF('Course Content'!C31&lt;&gt;"",'Course Content'!C31,IF('Course Content'!H31&lt;&gt;"",'Course Content'!H31,IF('Course Content'!C15&lt;&gt;"",'Course Content'!C15,'Course Content'!H15))),"")</f>
         <v/>
       </c>
@@ -6042,43 +6504,43 @@
         <f>IFERROR(IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C19" s="58" t="n"/>
-      <c r="D19" s="58" t="n"/>
-      <c r="E19" s="58" t="n"/>
-      <c r="F19" s="58" t="n"/>
-      <c r="G19" s="58" t="n"/>
-      <c r="H19" s="58" t="n"/>
+      <c r="C19" s="60" t="n"/>
+      <c r="D19" s="60" t="n"/>
+      <c r="E19" s="60" t="n"/>
+      <c r="F19" s="60" t="n"/>
+      <c r="G19" s="60" t="n"/>
+      <c r="H19" s="60" t="n"/>
       <c r="I19" s="17">
         <f>IF(COUNTA(C19:H19)=0,$I$8,COUNTA(C19:H19))</f>
         <v/>
       </c>
       <c r="J19" s="26" t="n"/>
-      <c r="K19" s="59">
+      <c r="K19" s="61">
         <f>IFERROR(IF(('Course Content'!D16="")*('Course Content'!I16="")*('Course Content'!D32="")*('Course Content'!I32=""),"—",IFERROR('Course Content'!D16*1,0)+IFERROR('Course Content'!I16*1,0)+IFERROR('Course Content'!D32*1,0)+IFERROR('Course Content'!I32*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L19" s="59">
+      <c r="L19" s="61">
         <f>IFERROR(IF(K19="","",IF(K19="—","",FLOOR(K19/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M19" s="60">
+      <c r="M19" s="62">
         <f>IFERROR(IF(L19="","",IF(L19="—","",FLOOR(L19/I19,1))),"")</f>
         <v/>
       </c>
       <c r="N19" s="26" t="n"/>
-      <c r="O19" s="61">
+      <c r="O19" s="63">
         <f>IFERROR(IF(('Course Content'!E16="")*('Course Content'!J16="")*('Course Content'!E32="")*('Course Content'!J32=""),"—",IFERROR('Course Content'!E16*1,0)+IFERROR('Course Content'!J16*1,0)+IFERROR('Course Content'!E32*1,0)+IFERROR('Course Content'!J32*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P19" s="61">
+      <c r="P19" s="63">
         <f>IFERROR(IF(O19="","",IF(O19="—","",FLOOR(O19/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q19" s="62">
+      <c r="Q19" s="64">
         <f>IFERROR(IF(P19="","",IF(P19="—","",FLOOR(P19/I19,1))),"")</f>
         <v/>
       </c>
-      <c r="R19" s="63">
+      <c r="R19" s="65">
         <f>IFERROR(IF('Course Content'!C32&lt;&gt;"",'Course Content'!C32,IF('Course Content'!H32&lt;&gt;"",'Course Content'!H32,IF('Course Content'!C16&lt;&gt;"",'Course Content'!C16,'Course Content'!H16))),"")</f>
         <v/>
       </c>
@@ -6093,244 +6555,444 @@
         <f>IFERROR(IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C20" s="58" t="n"/>
-      <c r="D20" s="58" t="n"/>
-      <c r="E20" s="58" t="n"/>
-      <c r="F20" s="58" t="n"/>
-      <c r="G20" s="58" t="n"/>
-      <c r="H20" s="58" t="n"/>
+      <c r="C20" s="60" t="n"/>
+      <c r="D20" s="60" t="n"/>
+      <c r="E20" s="60" t="n"/>
+      <c r="F20" s="60" t="n"/>
+      <c r="G20" s="60" t="n"/>
+      <c r="H20" s="60" t="n"/>
       <c r="I20" s="17">
         <f>IF(COUNTA(C20:H20)=0,$I$8,COUNTA(C20:H20))</f>
         <v/>
       </c>
       <c r="J20" s="26" t="n"/>
-      <c r="K20" s="59">
+      <c r="K20" s="61">
         <f>IFERROR(IF(('Course Content'!D17="")*('Course Content'!I17="")*('Course Content'!D33="")*('Course Content'!I33=""),"—",IFERROR('Course Content'!D17*1,0)+IFERROR('Course Content'!I17*1,0)+IFERROR('Course Content'!D33*1,0)+IFERROR('Course Content'!I33*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L20" s="59">
+      <c r="L20" s="61">
         <f>IFERROR(IF(K20="","",IF(K20="—","",FLOOR(K20/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M20" s="60">
+      <c r="M20" s="62">
         <f>IFERROR(IF(L20="","",IF(L20="—","",FLOOR(L20/I20,1))),"")</f>
         <v/>
       </c>
       <c r="N20" s="26" t="n"/>
-      <c r="O20" s="61">
+      <c r="O20" s="63">
         <f>IFERROR(IF(('Course Content'!E17="")*('Course Content'!J17="")*('Course Content'!E33="")*('Course Content'!J33=""),"—",IFERROR('Course Content'!E17*1,0)+IFERROR('Course Content'!J17*1,0)+IFERROR('Course Content'!E33*1,0)+IFERROR('Course Content'!J33*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P20" s="61">
+      <c r="P20" s="63">
         <f>IFERROR(IF(O20="","",IF(O20="—","",FLOOR(O20/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q20" s="62">
+      <c r="Q20" s="64">
         <f>IFERROR(IF(P20="","",IF(P20="—","",FLOOR(P20/I20,1))),"")</f>
         <v/>
       </c>
-      <c r="R20" s="64">
+      <c r="R20" s="66">
         <f>IFERROR(IF('Course Content'!C33&lt;&gt;"",'Course Content'!C33,IF('Course Content'!H33&lt;&gt;"",'Course Content'!H33,IF('Course Content'!C17&lt;&gt;"",'Course Content'!C17,'Course Content'!H17))),"")</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="31">
-        <f>IF('Course Content'!A34="Elective / Other 1","Elective / Other 1",'Course Content'!A34)</f>
+        <f>IF('Course Content'!A34="Other 1","Other 1",'Course Content'!A34)</f>
         <v/>
       </c>
       <c r="B21" s="5">
         <f>IFERROR(IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C21" s="58" t="n"/>
-      <c r="D21" s="58" t="n"/>
-      <c r="E21" s="58" t="n"/>
-      <c r="F21" s="58" t="n"/>
-      <c r="G21" s="58" t="n"/>
-      <c r="H21" s="58" t="n"/>
+      <c r="C21" s="60" t="n"/>
+      <c r="D21" s="60" t="n"/>
+      <c r="E21" s="60" t="n"/>
+      <c r="F21" s="60" t="n"/>
+      <c r="G21" s="60" t="n"/>
+      <c r="H21" s="60" t="n"/>
       <c r="I21" s="17">
         <f>IF(COUNTA(C21:H21)=0,$I$8,COUNTA(C21:H21))</f>
         <v/>
       </c>
       <c r="J21" s="26" t="n"/>
-      <c r="K21" s="59">
+      <c r="K21" s="61">
         <f>IFERROR(IF(('Course Content'!D18="")*('Course Content'!I18="")*('Course Content'!D34="")*('Course Content'!I34=""),"—",IFERROR('Course Content'!D18*1,0)+IFERROR('Course Content'!I18*1,0)+IFERROR('Course Content'!D34*1,0)+IFERROR('Course Content'!I34*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L21" s="59">
+      <c r="L21" s="61">
         <f>IFERROR(IF(K21="","",IF(K21="—","",FLOOR(K21/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M21" s="60">
+      <c r="M21" s="62">
         <f>IFERROR(IF(L21="","",IF(L21="—","",FLOOR(L21/I21,1))),"")</f>
         <v/>
       </c>
       <c r="N21" s="26" t="n"/>
-      <c r="O21" s="61">
+      <c r="O21" s="63">
         <f>IFERROR(IF(('Course Content'!E18="")*('Course Content'!J18="")*('Course Content'!E34="")*('Course Content'!J34=""),"—",IFERROR('Course Content'!E18*1,0)+IFERROR('Course Content'!J18*1,0)+IFERROR('Course Content'!E34*1,0)+IFERROR('Course Content'!J34*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P21" s="61">
+      <c r="P21" s="63">
         <f>IFERROR(IF(O21="","",IF(O21="—","",FLOOR(O21/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q21" s="62">
+      <c r="Q21" s="64">
         <f>IFERROR(IF(P21="","",IF(P21="—","",FLOOR(P21/I21,1))),"")</f>
         <v/>
       </c>
-      <c r="R21" s="63">
+      <c r="R21" s="65">
         <f>IFERROR(IF('Course Content'!C34&lt;&gt;"",'Course Content'!C34,IF('Course Content'!H34&lt;&gt;"",'Course Content'!H34,IF('Course Content'!C18&lt;&gt;"",'Course Content'!C18,'Course Content'!H18))),"")</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="31">
-        <f>IF('Course Content'!A35="Elective / Other 2","Elective / Other 2",'Course Content'!A35)</f>
+        <f>IF('Course Content'!A35="Other 2","Other 2",'Course Content'!A35)</f>
         <v/>
       </c>
       <c r="B22" s="18">
         <f>IFERROR(IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C22" s="58" t="n"/>
-      <c r="D22" s="58" t="n"/>
-      <c r="E22" s="58" t="n"/>
-      <c r="F22" s="58" t="n"/>
-      <c r="G22" s="58" t="n"/>
-      <c r="H22" s="58" t="n"/>
+      <c r="C22" s="60" t="n"/>
+      <c r="D22" s="60" t="n"/>
+      <c r="E22" s="60" t="n"/>
+      <c r="F22" s="60" t="n"/>
+      <c r="G22" s="60" t="n"/>
+      <c r="H22" s="60" t="n"/>
       <c r="I22" s="17">
         <f>IF(COUNTA(C22:H22)=0,$I$8,COUNTA(C22:H22))</f>
         <v/>
       </c>
       <c r="J22" s="26" t="n"/>
-      <c r="K22" s="59">
+      <c r="K22" s="61">
         <f>IFERROR(IF(('Course Content'!D19="")*('Course Content'!I19="")*('Course Content'!D35="")*('Course Content'!I35=""),"—",IFERROR('Course Content'!D19*1,0)+IFERROR('Course Content'!I19*1,0)+IFERROR('Course Content'!D35*1,0)+IFERROR('Course Content'!I35*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L22" s="59">
+      <c r="L22" s="61">
         <f>IFERROR(IF(K22="","",IF(K22="—","",FLOOR(K22/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M22" s="60">
+      <c r="M22" s="62">
         <f>IFERROR(IF(L22="","",IF(L22="—","",FLOOR(L22/I22,1))),"")</f>
         <v/>
       </c>
       <c r="N22" s="26" t="n"/>
-      <c r="O22" s="61">
+      <c r="O22" s="63">
         <f>IFERROR(IF(('Course Content'!E19="")*('Course Content'!J19="")*('Course Content'!E35="")*('Course Content'!J35=""),"—",IFERROR('Course Content'!E19*1,0)+IFERROR('Course Content'!J19*1,0)+IFERROR('Course Content'!E35*1,0)+IFERROR('Course Content'!J35*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P22" s="61">
+      <c r="P22" s="63">
         <f>IFERROR(IF(O22="","",IF(O22="—","",FLOOR(O22/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q22" s="62">
+      <c r="Q22" s="64">
         <f>IFERROR(IF(P22="","",IF(P22="—","",FLOOR(P22/I22,1))),"")</f>
         <v/>
       </c>
-      <c r="R22" s="64">
+      <c r="R22" s="66">
         <f>IFERROR(IF('Course Content'!C35&lt;&gt;"",'Course Content'!C35,IF('Course Content'!H35&lt;&gt;"",'Course Content'!H35,IF('Course Content'!C19&lt;&gt;"",'Course Content'!C19,'Course Content'!H19))),"")</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="31">
-        <f>IF('Course Content'!A36="Elective / Other 3","Elective / Other 3",'Course Content'!A36)</f>
+        <f>IF('Course Content'!A36="Other 3","Other 3",'Course Content'!A36)</f>
         <v/>
       </c>
       <c r="B23" s="5">
         <f>IFERROR(IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C23" s="58" t="n"/>
-      <c r="D23" s="58" t="n"/>
-      <c r="E23" s="58" t="n"/>
-      <c r="F23" s="58" t="n"/>
-      <c r="G23" s="58" t="n"/>
-      <c r="H23" s="58" t="n"/>
+      <c r="C23" s="60" t="n"/>
+      <c r="D23" s="60" t="n"/>
+      <c r="E23" s="60" t="n"/>
+      <c r="F23" s="60" t="n"/>
+      <c r="G23" s="60" t="n"/>
+      <c r="H23" s="60" t="n"/>
       <c r="I23" s="17">
         <f>IF(COUNTA(C23:H23)=0,$I$8,COUNTA(C23:H23))</f>
         <v/>
       </c>
       <c r="J23" s="26" t="n"/>
-      <c r="K23" s="59">
+      <c r="K23" s="61">
         <f>IFERROR(IF(('Course Content'!D20="")*('Course Content'!I20="")*('Course Content'!D36="")*('Course Content'!I36=""),"—",IFERROR('Course Content'!D20*1,0)+IFERROR('Course Content'!I20*1,0)+IFERROR('Course Content'!D36*1,0)+IFERROR('Course Content'!I36*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L23" s="59">
+      <c r="L23" s="61">
         <f>IFERROR(IF(K23="","",IF(K23="—","",FLOOR(K23/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M23" s="60">
+      <c r="M23" s="62">
         <f>IFERROR(IF(L23="","",IF(L23="—","",FLOOR(L23/I23,1))),"")</f>
         <v/>
       </c>
       <c r="N23" s="26" t="n"/>
-      <c r="O23" s="61">
+      <c r="O23" s="63">
         <f>IFERROR(IF(('Course Content'!E20="")*('Course Content'!J20="")*('Course Content'!E36="")*('Course Content'!J36=""),"—",IFERROR('Course Content'!E20*1,0)+IFERROR('Course Content'!J20*1,0)+IFERROR('Course Content'!E36*1,0)+IFERROR('Course Content'!J36*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P23" s="61">
+      <c r="P23" s="63">
         <f>IFERROR(IF(O23="","",IF(O23="—","",FLOOR(O23/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q23" s="62">
+      <c r="Q23" s="64">
         <f>IFERROR(IF(P23="","",IF(P23="—","",FLOOR(P23/I23,1))),"")</f>
         <v/>
       </c>
-      <c r="R23" s="63">
+      <c r="R23" s="65">
         <f>IFERROR(IF('Course Content'!C36&lt;&gt;"",'Course Content'!C36,IF('Course Content'!H36&lt;&gt;"",'Course Content'!H36,IF('Course Content'!C20&lt;&gt;"",'Course Content'!C20,'Course Content'!H20))),"")</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="31">
-        <f>IF('Course Content'!A37="Elective / Other 4","Elective / Other 4",'Course Content'!A37)</f>
+        <f>IF('Course Content'!A37="Other 4","Other 4",'Course Content'!A37)</f>
         <v/>
       </c>
       <c r="B24" s="18">
         <f>IFERROR(IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,"—")))),"—")</f>
         <v/>
       </c>
-      <c r="C24" s="58" t="n"/>
-      <c r="D24" s="58" t="n"/>
-      <c r="E24" s="58" t="n"/>
-      <c r="F24" s="58" t="n"/>
-      <c r="G24" s="58" t="n"/>
-      <c r="H24" s="58" t="n"/>
+      <c r="C24" s="60" t="n"/>
+      <c r="D24" s="60" t="n"/>
+      <c r="E24" s="60" t="n"/>
+      <c r="F24" s="60" t="n"/>
+      <c r="G24" s="60" t="n"/>
+      <c r="H24" s="60" t="n"/>
       <c r="I24" s="17">
         <f>IF(COUNTA(C24:H24)=0,$I$8,COUNTA(C24:H24))</f>
         <v/>
       </c>
       <c r="J24" s="26" t="n"/>
-      <c r="K24" s="59">
+      <c r="K24" s="61">
         <f>IFERROR(IF(('Course Content'!D21="")*('Course Content'!I21="")*('Course Content'!D37="")*('Course Content'!I37=""),"—",IFERROR('Course Content'!D21*1,0)+IFERROR('Course Content'!I21*1,0)+IFERROR('Course Content'!D37*1,0)+IFERROR('Course Content'!I37*1,0)),"")</f>
         <v/>
       </c>
-      <c r="L24" s="59">
+      <c r="L24" s="61">
         <f>IFERROR(IF(K24="","",IF(K24="—","",FLOOR(K24/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M24" s="60">
+      <c r="M24" s="62">
         <f>IFERROR(IF(L24="","",IF(L24="—","",FLOOR(L24/I24,1))),"")</f>
         <v/>
       </c>
       <c r="N24" s="26" t="n"/>
-      <c r="O24" s="61">
+      <c r="O24" s="63">
         <f>IFERROR(IF(('Course Content'!E21="")*('Course Content'!J21="")*('Course Content'!E37="")*('Course Content'!J37=""),"—",IFERROR('Course Content'!E21*1,0)+IFERROR('Course Content'!J21*1,0)+IFERROR('Course Content'!E37*1,0)+IFERROR('Course Content'!J37*1,0)),"")</f>
         <v/>
       </c>
-      <c r="P24" s="61">
+      <c r="P24" s="63">
         <f>IFERROR(IF(O24="","",IF(O24="—","",FLOOR(O24/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q24" s="62">
+      <c r="Q24" s="64">
         <f>IFERROR(IF(P24="","",IF(P24="—","",FLOOR(P24/I24,1))),"")</f>
         <v/>
       </c>
-      <c r="R24" s="64">
+      <c r="R24" s="66">
         <f>IFERROR(IF('Course Content'!C37&lt;&gt;"",'Course Content'!C37,IF('Course Content'!H37&lt;&gt;"",'Course Content'!H37,IF('Course Content'!C21&lt;&gt;"",'Course Content'!C21,'Course Content'!H21))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="31">
+        <f>IF('Course Content'!A38="Other 5","Other 5",'Course Content'!A38)</f>
+        <v/>
+      </c>
+      <c r="B25" s="5">
+        <f>IFERROR(IF('Course Content'!B38&lt;&gt;"",'Course Content'!B38,IF('Course Content'!B22&lt;&gt;"","[Grp] "&amp;'Course Content'!B22,IF('Course Content'!G38&lt;&gt;"",'Course Content'!G38,IF('Course Content'!G22&lt;&gt;"","[Grp] "&amp;'Course Content'!G22,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C25" s="60" t="n"/>
+      <c r="D25" s="60" t="n"/>
+      <c r="E25" s="60" t="n"/>
+      <c r="F25" s="60" t="n"/>
+      <c r="G25" s="60" t="n"/>
+      <c r="H25" s="60" t="n"/>
+      <c r="I25" s="17">
+        <f>IF(COUNTA(C25:H25)=0,$I$8,COUNTA(C25:H25))</f>
+        <v/>
+      </c>
+      <c r="J25" s="26" t="n"/>
+      <c r="K25" s="61">
+        <f>IFERROR(IF(('Course Content'!D22="")*('Course Content'!I22="")*('Course Content'!D38="")*('Course Content'!I38=""),"—",IFERROR('Course Content'!D22*1,0)+IFERROR('Course Content'!I22*1,0)+IFERROR('Course Content'!D38*1,0)+IFERROR('Course Content'!I38*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="61">
+        <f>IFERROR(IF(K25="","",IF(K25="—","",FLOOR(K25/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="62">
+        <f>IFERROR(IF(L25="","",IF(L25="—","",FLOOR(L25/I25,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="26" t="n"/>
+      <c r="O25" s="63">
+        <f>IFERROR(IF(('Course Content'!E22="")*('Course Content'!J22="")*('Course Content'!E38="")*('Course Content'!J38=""),"—",IFERROR('Course Content'!E22*1,0)+IFERROR('Course Content'!J22*1,0)+IFERROR('Course Content'!E38*1,0)+IFERROR('Course Content'!J38*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P25" s="63">
+        <f>IFERROR(IF(O25="","",IF(O25="—","",FLOOR(O25/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q25" s="64">
+        <f>IFERROR(IF(P25="","",IF(P25="—","",FLOOR(P25/I25,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R25" s="65">
+        <f>IFERROR(IF('Course Content'!C38&lt;&gt;"",'Course Content'!C38,IF('Course Content'!H38&lt;&gt;"",'Course Content'!H38,IF('Course Content'!C22&lt;&gt;"",'Course Content'!C22,'Course Content'!H22))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="31">
+        <f>IF('Course Content'!A39="Other 6","Other 6",'Course Content'!A39)</f>
+        <v/>
+      </c>
+      <c r="B26" s="18">
+        <f>IFERROR(IF('Course Content'!B39&lt;&gt;"",'Course Content'!B39,IF('Course Content'!B23&lt;&gt;"","[Grp] "&amp;'Course Content'!B23,IF('Course Content'!G39&lt;&gt;"",'Course Content'!G39,IF('Course Content'!G23&lt;&gt;"","[Grp] "&amp;'Course Content'!G23,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C26" s="60" t="n"/>
+      <c r="D26" s="60" t="n"/>
+      <c r="E26" s="60" t="n"/>
+      <c r="F26" s="60" t="n"/>
+      <c r="G26" s="60" t="n"/>
+      <c r="H26" s="60" t="n"/>
+      <c r="I26" s="17">
+        <f>IF(COUNTA(C26:H26)=0,$I$8,COUNTA(C26:H26))</f>
+        <v/>
+      </c>
+      <c r="J26" s="26" t="n"/>
+      <c r="K26" s="61">
+        <f>IFERROR(IF(('Course Content'!D23="")*('Course Content'!I23="")*('Course Content'!D39="")*('Course Content'!I39=""),"—",IFERROR('Course Content'!D23*1,0)+IFERROR('Course Content'!I23*1,0)+IFERROR('Course Content'!D39*1,0)+IFERROR('Course Content'!I39*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="61">
+        <f>IFERROR(IF(K26="","",IF(K26="—","",FLOOR(K26/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="62">
+        <f>IFERROR(IF(L26="","",IF(L26="—","",FLOOR(L26/I26,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="26" t="n"/>
+      <c r="O26" s="63">
+        <f>IFERROR(IF(('Course Content'!E23="")*('Course Content'!J23="")*('Course Content'!E39="")*('Course Content'!J39=""),"—",IFERROR('Course Content'!E23*1,0)+IFERROR('Course Content'!J23*1,0)+IFERROR('Course Content'!E39*1,0)+IFERROR('Course Content'!J39*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P26" s="63">
+        <f>IFERROR(IF(O26="","",IF(O26="—","",FLOOR(O26/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q26" s="64">
+        <f>IFERROR(IF(P26="","",IF(P26="—","",FLOOR(P26/I26,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R26" s="66">
+        <f>IFERROR(IF('Course Content'!C39&lt;&gt;"",'Course Content'!C39,IF('Course Content'!H39&lt;&gt;"",'Course Content'!H39,IF('Course Content'!C23&lt;&gt;"",'Course Content'!C23,'Course Content'!H23))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="31">
+        <f>IF('Course Content'!A40="Other 7","Other 7",'Course Content'!A40)</f>
+        <v/>
+      </c>
+      <c r="B27" s="5">
+        <f>IFERROR(IF('Course Content'!B40&lt;&gt;"",'Course Content'!B40,IF('Course Content'!B24&lt;&gt;"","[Grp] "&amp;'Course Content'!B24,IF('Course Content'!G40&lt;&gt;"",'Course Content'!G40,IF('Course Content'!G24&lt;&gt;"","[Grp] "&amp;'Course Content'!G24,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C27" s="60" t="n"/>
+      <c r="D27" s="60" t="n"/>
+      <c r="E27" s="60" t="n"/>
+      <c r="F27" s="60" t="n"/>
+      <c r="G27" s="60" t="n"/>
+      <c r="H27" s="60" t="n"/>
+      <c r="I27" s="17">
+        <f>IF(COUNTA(C27:H27)=0,$I$8,COUNTA(C27:H27))</f>
+        <v/>
+      </c>
+      <c r="J27" s="26" t="n"/>
+      <c r="K27" s="61">
+        <f>IFERROR(IF(('Course Content'!D24="")*('Course Content'!I24="")*('Course Content'!D40="")*('Course Content'!I40=""),"—",IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)+IFERROR('Course Content'!D40*1,0)+IFERROR('Course Content'!I40*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="61">
+        <f>IFERROR(IF(K27="","",IF(K27="—","",FLOOR(K27/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="62">
+        <f>IFERROR(IF(L27="","",IF(L27="—","",FLOOR(L27/I27,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="26" t="n"/>
+      <c r="O27" s="63">
+        <f>IFERROR(IF(('Course Content'!E24="")*('Course Content'!J24="")*('Course Content'!E40="")*('Course Content'!J40=""),"—",IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)+IFERROR('Course Content'!E40*1,0)+IFERROR('Course Content'!J40*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P27" s="63">
+        <f>IFERROR(IF(O27="","",IF(O27="—","",FLOOR(O27/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q27" s="64">
+        <f>IFERROR(IF(P27="","",IF(P27="—","",FLOOR(P27/I27,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R27" s="65">
+        <f>IFERROR(IF('Course Content'!C40&lt;&gt;"",'Course Content'!C40,IF('Course Content'!H40&lt;&gt;"",'Course Content'!H40,IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,'Course Content'!H24))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="31">
+        <f>IF('Course Content'!A41="Other 8","Other 8",'Course Content'!A41)</f>
+        <v/>
+      </c>
+      <c r="B28" s="18">
+        <f>IFERROR(IF('Course Content'!B41&lt;&gt;"",'Course Content'!B41,IF('Course Content'!B25&lt;&gt;"","[Grp] "&amp;'Course Content'!B25,IF('Course Content'!G41&lt;&gt;"",'Course Content'!G41,IF('Course Content'!G25&lt;&gt;"","[Grp] "&amp;'Course Content'!G25,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C28" s="60" t="n"/>
+      <c r="D28" s="60" t="n"/>
+      <c r="E28" s="60" t="n"/>
+      <c r="F28" s="60" t="n"/>
+      <c r="G28" s="60" t="n"/>
+      <c r="H28" s="60" t="n"/>
+      <c r="I28" s="17">
+        <f>IF(COUNTA(C28:H28)=0,$I$8,COUNTA(C28:H28))</f>
+        <v/>
+      </c>
+      <c r="J28" s="26" t="n"/>
+      <c r="K28" s="61">
+        <f>IFERROR(IF(('Course Content'!D25="")*('Course Content'!I25="")*('Course Content'!D41="")*('Course Content'!I41=""),"—",IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)+IFERROR('Course Content'!D41*1,0)+IFERROR('Course Content'!I41*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="61">
+        <f>IFERROR(IF(K28="","",IF(K28="—","",FLOOR(K28/'Getting Started'!C15,1))),"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="62">
+        <f>IFERROR(IF(L28="","",IF(L28="—","",FLOOR(L28/I28,1))),"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="26" t="n"/>
+      <c r="O28" s="63">
+        <f>IFERROR(IF(('Course Content'!E25="")*('Course Content'!J25="")*('Course Content'!E41="")*('Course Content'!J41=""),"—",IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)+IFERROR('Course Content'!E41*1,0)+IFERROR('Course Content'!J41*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P28" s="63">
+        <f>IFERROR(IF(O28="","",IF(O28="—","",FLOOR(O28/'Getting Started'!C23,1))),"")</f>
+        <v/>
+      </c>
+      <c r="Q28" s="64">
+        <f>IFERROR(IF(P28="","",IF(P28="—","",FLOOR(P28/I28,1))),"")</f>
+        <v/>
+      </c>
+      <c r="R28" s="66">
+        <f>IFERROR(IF('Course Content'!C41&lt;&gt;"",'Course Content'!C41,IF('Course Content'!H41&lt;&gt;"",'Course Content'!H41,IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,'Course Content'!H25))),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix CC_ROWS_PER_STUDENT to be dynamic based on NUM_SUBJECTS
Was hardcoded at 16 (for 14 subjects); now 18 subjects caused student
sections to overlap. Changed to NUM_SUBJECTS + 2 so it always matches.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -1533,7 +1533,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J185"/>
+  <dimension ref="A1:J221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2379,25 +2379,34 @@
       <c r="I38" s="32" t="n"/>
       <c r="J38" s="32" t="n"/>
     </row>
-    <row r="39" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A39" s="38">
-        <f>IF('Getting Started'!B30&lt;&gt;"","  "&amp;UPPER('Getting Started'!B30)&amp;"   ·   "&amp;'Getting Started'!F30,"  STUDENT 2")</f>
-        <v/>
-      </c>
-      <c r="B39" s="36" t="n"/>
-      <c r="C39" s="36" t="n"/>
-      <c r="D39" s="36" t="n"/>
-      <c r="E39" s="36" t="n"/>
-      <c r="F39" s="36" t="n"/>
-      <c r="G39" s="36" t="n"/>
-      <c r="H39" s="36" t="n"/>
-      <c r="I39" s="36" t="n"/>
-      <c r="J39" s="37" t="n"/>
-    </row>
-    <row r="40" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A40" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+    <row r="39" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D39" s="33" t="n"/>
+      <c r="E39" s="33" t="n"/>
+      <c r="F39" s="26" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I39" s="33" t="n"/>
+      <c r="J39" s="33" t="n"/>
+    </row>
+    <row r="40" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A40" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B40" s="5" t="n"/>
@@ -2418,10 +2427,10 @@
       <c r="I40" s="32" t="n"/>
       <c r="J40" s="32" t="n"/>
     </row>
-    <row r="41" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A41" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+    <row r="41" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A41" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B41" s="5" t="n"/>
@@ -2442,58 +2451,17 @@
       <c r="I41" s="33" t="n"/>
       <c r="J41" s="33" t="n"/>
     </row>
-    <row r="42" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A42" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D42" s="32" t="n"/>
-      <c r="E42" s="32" t="n"/>
-      <c r="F42" s="26" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I42" s="32" t="n"/>
-      <c r="J42" s="32" t="n"/>
-    </row>
-    <row r="43" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A43" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n"/>
-      <c r="C43" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D43" s="33" t="n"/>
-      <c r="E43" s="33" t="n"/>
-      <c r="F43" s="26" t="n"/>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I43" s="33" t="n"/>
-      <c r="J43" s="33" t="n"/>
+    <row r="42" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="38">
+        <f>IF('Getting Started'!B30&lt;&gt;"","  "&amp;UPPER('Getting Started'!B30)&amp;"   ·   "&amp;'Getting Started'!F30,"  STUDENT 2")</f>
+        <v/>
+      </c>
     </row>
     <row r="44" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A44" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B44" s="5" t="n"/>
@@ -2517,7 +2485,7 @@
     <row r="45" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A45" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B45" s="5" t="n"/>
@@ -2541,7 +2509,7 @@
     <row r="46" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A46" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B46" s="5" t="n"/>
@@ -2565,7 +2533,7 @@
     <row r="47" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A47" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B47" s="5" t="n"/>
@@ -2589,7 +2557,7 @@
     <row r="48" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A48" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B48" s="5" t="n"/>
@@ -2613,7 +2581,7 @@
     <row r="49" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B49" s="5" t="n"/>
@@ -2635,9 +2603,9 @@
       <c r="J49" s="33" t="n"/>
     </row>
     <row r="50" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A50" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A50" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B50" s="5" t="n"/>
@@ -2659,9 +2627,9 @@
       <c r="J50" s="32" t="n"/>
     </row>
     <row r="51" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A51" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A51" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B51" s="5" t="n"/>
@@ -2683,9 +2651,9 @@
       <c r="J51" s="33" t="n"/>
     </row>
     <row r="52" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A52" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A52" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B52" s="5" t="n"/>
@@ -2707,9 +2675,9 @@
       <c r="J52" s="32" t="n"/>
     </row>
     <row r="53" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A53" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A53" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B53" s="5" t="n"/>
@@ -2733,7 +2701,7 @@
     <row r="54" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B54" s="5" t="n"/>
@@ -2754,25 +2722,34 @@
       <c r="I54" s="32" t="n"/>
       <c r="J54" s="32" t="n"/>
     </row>
-    <row r="55" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A55" s="39">
-        <f>IF('Getting Started'!B31&lt;&gt;"","  "&amp;UPPER('Getting Started'!B31)&amp;"   ·   "&amp;'Getting Started'!F31,"  STUDENT 3")</f>
-        <v/>
-      </c>
-      <c r="B55" s="36" t="n"/>
-      <c r="C55" s="36" t="n"/>
-      <c r="D55" s="36" t="n"/>
-      <c r="E55" s="36" t="n"/>
-      <c r="F55" s="36" t="n"/>
-      <c r="G55" s="36" t="n"/>
-      <c r="H55" s="36" t="n"/>
-      <c r="I55" s="36" t="n"/>
-      <c r="J55" s="37" t="n"/>
+    <row r="55" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A55" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n"/>
+      <c r="C55" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D55" s="33" t="n"/>
+      <c r="E55" s="33" t="n"/>
+      <c r="F55" s="26" t="n"/>
+      <c r="G55" s="5" t="n"/>
+      <c r="H55" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I55" s="33" t="n"/>
+      <c r="J55" s="33" t="n"/>
     </row>
     <row r="56" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A56" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A56" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B56" s="5" t="n"/>
@@ -2794,9 +2771,9 @@
       <c r="J56" s="32" t="n"/>
     </row>
     <row r="57" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A57" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A57" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B57" s="5" t="n"/>
@@ -2818,9 +2795,9 @@
       <c r="J57" s="33" t="n"/>
     </row>
     <row r="58" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A58" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
+      <c r="A58" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
         </is>
       </c>
       <c r="B58" s="5" t="n"/>
@@ -2842,9 +2819,9 @@
       <c r="J58" s="32" t="n"/>
     </row>
     <row r="59" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A59" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
+      <c r="A59" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
         </is>
       </c>
       <c r="B59" s="5" t="n"/>
@@ -2866,9 +2843,9 @@
       <c r="J59" s="33" t="n"/>
     </row>
     <row r="60" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A60" s="31" t="inlineStr">
-        <is>
-          <t>Writing / Composition</t>
+      <c r="A60" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B60" s="5" t="n"/>
@@ -2890,9 +2867,9 @@
       <c r="J60" s="32" t="n"/>
     </row>
     <row r="61" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A61" s="31" t="inlineStr">
-        <is>
-          <t>Science</t>
+      <c r="A61" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B61" s="5" t="n"/>
@@ -2913,58 +2890,17 @@
       <c r="I61" s="33" t="n"/>
       <c r="J61" s="33" t="n"/>
     </row>
-    <row r="62" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A62" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="n"/>
-      <c r="C62" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D62" s="32" t="n"/>
-      <c r="E62" s="32" t="n"/>
-      <c r="F62" s="26" t="n"/>
-      <c r="G62" s="5" t="n"/>
-      <c r="H62" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I62" s="32" t="n"/>
-      <c r="J62" s="32" t="n"/>
-    </row>
-    <row r="63" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A63" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="n"/>
-      <c r="C63" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D63" s="33" t="n"/>
-      <c r="E63" s="33" t="n"/>
-      <c r="F63" s="26" t="n"/>
-      <c r="G63" s="5" t="n"/>
-      <c r="H63" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I63" s="33" t="n"/>
-      <c r="J63" s="33" t="n"/>
+    <row r="62" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="63" ht="26" customHeight="1">
+      <c r="A63" s="39">
+        <f>IF('Getting Started'!B31&lt;&gt;"","  "&amp;UPPER('Getting Started'!B31)&amp;"   ·   "&amp;'Getting Started'!F31,"  STUDENT 3")</f>
+        <v/>
+      </c>
     </row>
     <row r="64" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A64" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B64" s="5" t="n"/>
@@ -2988,7 +2924,7 @@
     <row r="65" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A65" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B65" s="5" t="n"/>
@@ -3010,9 +2946,9 @@
       <c r="J65" s="33" t="n"/>
     </row>
     <row r="66" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A66" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B66" s="5" t="n"/>
@@ -3034,9 +2970,9 @@
       <c r="J66" s="32" t="n"/>
     </row>
     <row r="67" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A67" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A67" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B67" s="5" t="n"/>
@@ -3058,9 +2994,9 @@
       <c r="J67" s="33" t="n"/>
     </row>
     <row r="68" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A68" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B68" s="5" t="n"/>
@@ -3082,9 +3018,9 @@
       <c r="J68" s="32" t="n"/>
     </row>
     <row r="69" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A69" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t>Science</t>
         </is>
       </c>
       <c r="B69" s="5" t="n"/>
@@ -3106,9 +3042,9 @@
       <c r="J69" s="33" t="n"/>
     </row>
     <row r="70" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A70" s="34" t="inlineStr">
-        <is>
-          <t>Other 5</t>
+      <c r="A70" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B70" s="5" t="n"/>
@@ -3129,25 +3065,34 @@
       <c r="I70" s="32" t="n"/>
       <c r="J70" s="32" t="n"/>
     </row>
-    <row r="71" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A71" s="40">
-        <f>IF('Getting Started'!B32&lt;&gt;"","  "&amp;UPPER('Getting Started'!B32)&amp;"   ·   "&amp;'Getting Started'!F32,"  STUDENT 4")</f>
-        <v/>
-      </c>
-      <c r="B71" s="36" t="n"/>
-      <c r="C71" s="36" t="n"/>
-      <c r="D71" s="36" t="n"/>
-      <c r="E71" s="36" t="n"/>
-      <c r="F71" s="36" t="n"/>
-      <c r="G71" s="36" t="n"/>
-      <c r="H71" s="36" t="n"/>
-      <c r="I71" s="36" t="n"/>
-      <c r="J71" s="37" t="n"/>
+    <row r="71" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A71" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="n"/>
+      <c r="C71" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D71" s="33" t="n"/>
+      <c r="E71" s="33" t="n"/>
+      <c r="F71" s="26" t="n"/>
+      <c r="G71" s="5" t="n"/>
+      <c r="H71" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I71" s="33" t="n"/>
+      <c r="J71" s="33" t="n"/>
     </row>
     <row r="72" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Bible</t>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B72" s="5" t="n"/>
@@ -3171,7 +3116,7 @@
     <row r="73" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B73" s="5" t="n"/>
@@ -3193,9 +3138,9 @@
       <c r="J73" s="33" t="n"/>
     </row>
     <row r="74" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A74" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
+      <c r="A74" s="34" t="inlineStr">
+        <is>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B74" s="5" t="n"/>
@@ -3217,9 +3162,9 @@
       <c r="J74" s="32" t="n"/>
     </row>
     <row r="75" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A75" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
+      <c r="A75" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B75" s="5" t="n"/>
@@ -3241,9 +3186,9 @@
       <c r="J75" s="33" t="n"/>
     </row>
     <row r="76" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A76" s="31" t="inlineStr">
-        <is>
-          <t>Writing / Composition</t>
+      <c r="A76" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B76" s="5" t="n"/>
@@ -3265,9 +3210,9 @@
       <c r="J76" s="32" t="n"/>
     </row>
     <row r="77" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A77" s="31" t="inlineStr">
-        <is>
-          <t>Science</t>
+      <c r="A77" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B77" s="5" t="n"/>
@@ -3289,9 +3234,9 @@
       <c r="J77" s="33" t="n"/>
     </row>
     <row r="78" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A78" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
+      <c r="A78" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
         </is>
       </c>
       <c r="B78" s="5" t="n"/>
@@ -3313,9 +3258,9 @@
       <c r="J78" s="32" t="n"/>
     </row>
     <row r="79" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A79" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
+      <c r="A79" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
         </is>
       </c>
       <c r="B79" s="5" t="n"/>
@@ -3337,9 +3282,9 @@
       <c r="J79" s="33" t="n"/>
     </row>
     <row r="80" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A80" s="31" t="inlineStr">
-        <is>
-          <t>Physical Education</t>
+      <c r="A80" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B80" s="5" t="n"/>
@@ -3361,9 +3306,9 @@
       <c r="J80" s="32" t="n"/>
     </row>
     <row r="81" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A81" s="31" t="inlineStr">
-        <is>
-          <t>Art / Music</t>
+      <c r="A81" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B81" s="5" t="n"/>
@@ -3384,58 +3329,17 @@
       <c r="I81" s="33" t="n"/>
       <c r="J81" s="33" t="n"/>
     </row>
-    <row r="82" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A82" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="n"/>
-      <c r="C82" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D82" s="32" t="n"/>
-      <c r="E82" s="32" t="n"/>
-      <c r="F82" s="26" t="n"/>
-      <c r="G82" s="5" t="n"/>
-      <c r="H82" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I82" s="32" t="n"/>
-      <c r="J82" s="32" t="n"/>
-    </row>
-    <row r="83" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A83" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
-        </is>
-      </c>
-      <c r="B83" s="5" t="n"/>
-      <c r="C83" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D83" s="33" t="n"/>
-      <c r="E83" s="33" t="n"/>
-      <c r="F83" s="26" t="n"/>
-      <c r="G83" s="5" t="n"/>
-      <c r="H83" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I83" s="33" t="n"/>
-      <c r="J83" s="33" t="n"/>
+    <row r="82" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="83" ht="26" customHeight="1">
+      <c r="A83" s="40">
+        <f>IF('Getting Started'!B32&lt;&gt;"","  "&amp;UPPER('Getting Started'!B32)&amp;"   ·   "&amp;'Getting Started'!F32,"  STUDENT 4")</f>
+        <v/>
+      </c>
     </row>
     <row r="84" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A84" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A84" s="31" t="inlineStr">
+        <is>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B84" s="5" t="n"/>
@@ -3457,9 +3361,9 @@
       <c r="J84" s="32" t="n"/>
     </row>
     <row r="85" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A85" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A85" s="31" t="inlineStr">
+        <is>
+          <t>Math</t>
         </is>
       </c>
       <c r="B85" s="5" t="n"/>
@@ -3481,9 +3385,9 @@
       <c r="J85" s="33" t="n"/>
     </row>
     <row r="86" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A86" s="34" t="inlineStr">
-        <is>
-          <t>Other 5</t>
+      <c r="A86" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B86" s="5" t="n"/>
@@ -3504,25 +3408,34 @@
       <c r="I86" s="32" t="n"/>
       <c r="J86" s="32" t="n"/>
     </row>
-    <row r="87" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A87" s="41">
-        <f>IF('Getting Started'!B33&lt;&gt;"","  "&amp;UPPER('Getting Started'!B33)&amp;"   ·   "&amp;'Getting Started'!F33,"  STUDENT 5")</f>
-        <v/>
-      </c>
-      <c r="B87" s="36" t="n"/>
-      <c r="C87" s="36" t="n"/>
-      <c r="D87" s="36" t="n"/>
-      <c r="E87" s="36" t="n"/>
-      <c r="F87" s="36" t="n"/>
-      <c r="G87" s="36" t="n"/>
-      <c r="H87" s="36" t="n"/>
-      <c r="I87" s="36" t="n"/>
-      <c r="J87" s="37" t="n"/>
+    <row r="87" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A87" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="n"/>
+      <c r="C87" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D87" s="33" t="n"/>
+      <c r="E87" s="33" t="n"/>
+      <c r="F87" s="26" t="n"/>
+      <c r="G87" s="5" t="n"/>
+      <c r="H87" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I87" s="33" t="n"/>
+      <c r="J87" s="33" t="n"/>
     </row>
     <row r="88" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>Bible</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B88" s="5" t="n"/>
@@ -3546,7 +3459,7 @@
     <row r="89" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B89" s="5" t="n"/>
@@ -3570,7 +3483,7 @@
     <row r="90" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>English / Language Arts</t>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B90" s="5" t="n"/>
@@ -3594,7 +3507,7 @@
     <row r="91" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B91" s="5" t="n"/>
@@ -3618,7 +3531,7 @@
     <row r="92" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A92" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B92" s="5" t="n"/>
@@ -3642,7 +3555,7 @@
     <row r="93" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A93" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B93" s="5" t="n"/>
@@ -3664,9 +3577,9 @@
       <c r="J93" s="33" t="n"/>
     </row>
     <row r="94" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A94" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
+      <c r="A94" s="34" t="inlineStr">
+        <is>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B94" s="5" t="n"/>
@@ -3688,9 +3601,9 @@
       <c r="J94" s="32" t="n"/>
     </row>
     <row r="95" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A95" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
+      <c r="A95" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B95" s="5" t="n"/>
@@ -3712,9 +3625,9 @@
       <c r="J95" s="33" t="n"/>
     </row>
     <row r="96" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A96" s="31" t="inlineStr">
-        <is>
-          <t>Physical Education</t>
+      <c r="A96" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B96" s="5" t="n"/>
@@ -3736,9 +3649,9 @@
       <c r="J96" s="32" t="n"/>
     </row>
     <row r="97" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A97" s="31" t="inlineStr">
-        <is>
-          <t>Art / Music</t>
+      <c r="A97" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B97" s="5" t="n"/>
@@ -3762,7 +3675,7 @@
     <row r="98" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A98" s="34" t="inlineStr">
         <is>
-          <t>Other 1</t>
+          <t>Other 5</t>
         </is>
       </c>
       <c r="B98" s="5" t="n"/>
@@ -3786,7 +3699,7 @@
     <row r="99" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A99" s="34" t="inlineStr">
         <is>
-          <t>Other 2</t>
+          <t>Other 6</t>
         </is>
       </c>
       <c r="B99" s="5" t="n"/>
@@ -3810,7 +3723,7 @@
     <row r="100" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A100" s="34" t="inlineStr">
         <is>
-          <t>Other 3</t>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B100" s="5" t="n"/>
@@ -3834,7 +3747,7 @@
     <row r="101" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A101" s="34" t="inlineStr">
         <is>
-          <t>Other 4</t>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B101" s="5" t="n"/>
@@ -3855,44 +3768,12 @@
       <c r="I101" s="33" t="n"/>
       <c r="J101" s="33" t="n"/>
     </row>
-    <row r="102" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A102" s="34" t="inlineStr">
-        <is>
-          <t>Other 5</t>
-        </is>
-      </c>
-      <c r="B102" s="5" t="n"/>
-      <c r="C102" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D102" s="32" t="n"/>
-      <c r="E102" s="32" t="n"/>
-      <c r="F102" s="26" t="n"/>
-      <c r="G102" s="5" t="n"/>
-      <c r="H102" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I102" s="32" t="n"/>
-      <c r="J102" s="32" t="n"/>
-    </row>
-    <row r="103" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A103" s="42">
-        <f>IF('Getting Started'!B34&lt;&gt;"","  "&amp;UPPER('Getting Started'!B34)&amp;"   ·   "&amp;'Getting Started'!F34,"  STUDENT 6")</f>
-        <v/>
-      </c>
-      <c r="B103" s="36" t="n"/>
-      <c r="C103" s="36" t="n"/>
-      <c r="D103" s="36" t="n"/>
-      <c r="E103" s="36" t="n"/>
-      <c r="F103" s="36" t="n"/>
-      <c r="G103" s="36" t="n"/>
-      <c r="H103" s="36" t="n"/>
-      <c r="I103" s="36" t="n"/>
-      <c r="J103" s="37" t="n"/>
+    <row r="102" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="103" ht="26" customHeight="1">
+      <c r="A103" s="41">
+        <f>IF('Getting Started'!B33&lt;&gt;"","  "&amp;UPPER('Getting Started'!B33)&amp;"   ·   "&amp;'Getting Started'!F33,"  STUDENT 5")</f>
+        <v/>
+      </c>
     </row>
     <row r="104" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A104" s="31" t="inlineStr">
@@ -4254,25 +4135,34 @@
       <c r="I118" s="32" t="n"/>
       <c r="J118" s="32" t="n"/>
     </row>
-    <row r="119" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A119" s="43">
-        <f>IF('Getting Started'!B35&lt;&gt;"","  "&amp;UPPER('Getting Started'!B35)&amp;"   ·   "&amp;'Getting Started'!F35,"  STUDENT 7")</f>
-        <v/>
-      </c>
-      <c r="B119" s="36" t="n"/>
-      <c r="C119" s="36" t="n"/>
-      <c r="D119" s="36" t="n"/>
-      <c r="E119" s="36" t="n"/>
-      <c r="F119" s="36" t="n"/>
-      <c r="G119" s="36" t="n"/>
-      <c r="H119" s="36" t="n"/>
-      <c r="I119" s="36" t="n"/>
-      <c r="J119" s="37" t="n"/>
+    <row r="119" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A119" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="n"/>
+      <c r="C119" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D119" s="33" t="n"/>
+      <c r="E119" s="33" t="n"/>
+      <c r="F119" s="26" t="n"/>
+      <c r="G119" s="5" t="n"/>
+      <c r="H119" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I119" s="33" t="n"/>
+      <c r="J119" s="33" t="n"/>
     </row>
     <row r="120" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A120" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A120" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B120" s="5" t="n"/>
@@ -4294,9 +4184,9 @@
       <c r="J120" s="32" t="n"/>
     </row>
     <row r="121" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A121" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A121" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B121" s="5" t="n"/>
@@ -4317,58 +4207,17 @@
       <c r="I121" s="33" t="n"/>
       <c r="J121" s="33" t="n"/>
     </row>
-    <row r="122" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A122" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B122" s="5" t="n"/>
-      <c r="C122" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D122" s="32" t="n"/>
-      <c r="E122" s="32" t="n"/>
-      <c r="F122" s="26" t="n"/>
-      <c r="G122" s="5" t="n"/>
-      <c r="H122" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I122" s="32" t="n"/>
-      <c r="J122" s="32" t="n"/>
-    </row>
-    <row r="123" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A123" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B123" s="5" t="n"/>
-      <c r="C123" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D123" s="33" t="n"/>
-      <c r="E123" s="33" t="n"/>
-      <c r="F123" s="26" t="n"/>
-      <c r="G123" s="5" t="n"/>
-      <c r="H123" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I123" s="33" t="n"/>
-      <c r="J123" s="33" t="n"/>
+    <row r="122" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="123" ht="26" customHeight="1">
+      <c r="A123" s="42">
+        <f>IF('Getting Started'!B34&lt;&gt;"","  "&amp;UPPER('Getting Started'!B34)&amp;"   ·   "&amp;'Getting Started'!F34,"  STUDENT 6")</f>
+        <v/>
+      </c>
     </row>
     <row r="124" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A124" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B124" s="5" t="n"/>
@@ -4392,7 +4241,7 @@
     <row r="125" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A125" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B125" s="5" t="n"/>
@@ -4416,7 +4265,7 @@
     <row r="126" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A126" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B126" s="5" t="n"/>
@@ -4440,7 +4289,7 @@
     <row r="127" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A127" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B127" s="5" t="n"/>
@@ -4464,7 +4313,7 @@
     <row r="128" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A128" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B128" s="5" t="n"/>
@@ -4488,7 +4337,7 @@
     <row r="129" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A129" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B129" s="5" t="n"/>
@@ -4510,9 +4359,9 @@
       <c r="J129" s="33" t="n"/>
     </row>
     <row r="130" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A130" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A130" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B130" s="5" t="n"/>
@@ -4534,9 +4383,9 @@
       <c r="J130" s="32" t="n"/>
     </row>
     <row r="131" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A131" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A131" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B131" s="5" t="n"/>
@@ -4558,9 +4407,9 @@
       <c r="J131" s="33" t="n"/>
     </row>
     <row r="132" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A132" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A132" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B132" s="5" t="n"/>
@@ -4582,9 +4431,9 @@
       <c r="J132" s="32" t="n"/>
     </row>
     <row r="133" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A133" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A133" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B133" s="5" t="n"/>
@@ -4608,7 +4457,7 @@
     <row r="134" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A134" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B134" s="5" t="n"/>
@@ -4629,25 +4478,34 @@
       <c r="I134" s="32" t="n"/>
       <c r="J134" s="32" t="n"/>
     </row>
-    <row r="135" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A135" s="44">
-        <f>IF('Getting Started'!B36&lt;&gt;"","  "&amp;UPPER('Getting Started'!B36)&amp;"   ·   "&amp;'Getting Started'!F36,"  STUDENT 8")</f>
-        <v/>
-      </c>
-      <c r="B135" s="36" t="n"/>
-      <c r="C135" s="36" t="n"/>
-      <c r="D135" s="36" t="n"/>
-      <c r="E135" s="36" t="n"/>
-      <c r="F135" s="36" t="n"/>
-      <c r="G135" s="36" t="n"/>
-      <c r="H135" s="36" t="n"/>
-      <c r="I135" s="36" t="n"/>
-      <c r="J135" s="37" t="n"/>
+    <row r="135" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A135" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="n"/>
+      <c r="C135" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D135" s="33" t="n"/>
+      <c r="E135" s="33" t="n"/>
+      <c r="F135" s="26" t="n"/>
+      <c r="G135" s="5" t="n"/>
+      <c r="H135" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I135" s="33" t="n"/>
+      <c r="J135" s="33" t="n"/>
     </row>
     <row r="136" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A136" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A136" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B136" s="5" t="n"/>
@@ -4669,9 +4527,9 @@
       <c r="J136" s="32" t="n"/>
     </row>
     <row r="137" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A137" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A137" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B137" s="5" t="n"/>
@@ -4693,9 +4551,9 @@
       <c r="J137" s="33" t="n"/>
     </row>
     <row r="138" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A138" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
+      <c r="A138" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
         </is>
       </c>
       <c r="B138" s="5" t="n"/>
@@ -4717,9 +4575,9 @@
       <c r="J138" s="32" t="n"/>
     </row>
     <row r="139" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A139" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
+      <c r="A139" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
         </is>
       </c>
       <c r="B139" s="5" t="n"/>
@@ -4741,9 +4599,9 @@
       <c r="J139" s="33" t="n"/>
     </row>
     <row r="140" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A140" s="31" t="inlineStr">
-        <is>
-          <t>Writing / Composition</t>
+      <c r="A140" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B140" s="5" t="n"/>
@@ -4765,9 +4623,9 @@
       <c r="J140" s="32" t="n"/>
     </row>
     <row r="141" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A141" s="31" t="inlineStr">
-        <is>
-          <t>Science</t>
+      <c r="A141" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B141" s="5" t="n"/>
@@ -4788,58 +4646,17 @@
       <c r="I141" s="33" t="n"/>
       <c r="J141" s="33" t="n"/>
     </row>
-    <row r="142" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A142" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
-        </is>
-      </c>
-      <c r="B142" s="5" t="n"/>
-      <c r="C142" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D142" s="32" t="n"/>
-      <c r="E142" s="32" t="n"/>
-      <c r="F142" s="26" t="n"/>
-      <c r="G142" s="5" t="n"/>
-      <c r="H142" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I142" s="32" t="n"/>
-      <c r="J142" s="32" t="n"/>
-    </row>
-    <row r="143" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A143" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
-        </is>
-      </c>
-      <c r="B143" s="5" t="n"/>
-      <c r="C143" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D143" s="33" t="n"/>
-      <c r="E143" s="33" t="n"/>
-      <c r="F143" s="26" t="n"/>
-      <c r="G143" s="5" t="n"/>
-      <c r="H143" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I143" s="33" t="n"/>
-      <c r="J143" s="33" t="n"/>
+    <row r="142" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="143" ht="26" customHeight="1">
+      <c r="A143" s="43">
+        <f>IF('Getting Started'!B35&lt;&gt;"","  "&amp;UPPER('Getting Started'!B35)&amp;"   ·   "&amp;'Getting Started'!F35,"  STUDENT 7")</f>
+        <v/>
+      </c>
     </row>
     <row r="144" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A144" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B144" s="5" t="n"/>
@@ -4863,7 +4680,7 @@
     <row r="145" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A145" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B145" s="5" t="n"/>
@@ -4885,9 +4702,9 @@
       <c r="J145" s="33" t="n"/>
     </row>
     <row r="146" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A146" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A146" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B146" s="5" t="n"/>
@@ -4909,9 +4726,9 @@
       <c r="J146" s="32" t="n"/>
     </row>
     <row r="147" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A147" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A147" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B147" s="5" t="n"/>
@@ -4933,9 +4750,9 @@
       <c r="J147" s="33" t="n"/>
     </row>
     <row r="148" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A148" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A148" s="31" t="inlineStr">
+        <is>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B148" s="5" t="n"/>
@@ -4957,9 +4774,9 @@
       <c r="J148" s="32" t="n"/>
     </row>
     <row r="149" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A149" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A149" s="31" t="inlineStr">
+        <is>
+          <t>Science</t>
         </is>
       </c>
       <c r="B149" s="5" t="n"/>
@@ -4981,9 +4798,9 @@
       <c r="J149" s="33" t="n"/>
     </row>
     <row r="150" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A150" s="34" t="inlineStr">
-        <is>
-          <t>Other 5</t>
+      <c r="A150" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B150" s="5" t="n"/>
@@ -5004,25 +4821,34 @@
       <c r="I150" s="32" t="n"/>
       <c r="J150" s="32" t="n"/>
     </row>
-    <row r="151" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A151" s="45">
-        <f>IF('Getting Started'!B37&lt;&gt;"","  "&amp;UPPER('Getting Started'!B37)&amp;"   ·   "&amp;'Getting Started'!F37,"  STUDENT 9")</f>
-        <v/>
-      </c>
-      <c r="B151" s="36" t="n"/>
-      <c r="C151" s="36" t="n"/>
-      <c r="D151" s="36" t="n"/>
-      <c r="E151" s="36" t="n"/>
-      <c r="F151" s="36" t="n"/>
-      <c r="G151" s="36" t="n"/>
-      <c r="H151" s="36" t="n"/>
-      <c r="I151" s="36" t="n"/>
-      <c r="J151" s="37" t="n"/>
+    <row r="151" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A151" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="n"/>
+      <c r="C151" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D151" s="33" t="n"/>
+      <c r="E151" s="33" t="n"/>
+      <c r="F151" s="26" t="n"/>
+      <c r="G151" s="5" t="n"/>
+      <c r="H151" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I151" s="33" t="n"/>
+      <c r="J151" s="33" t="n"/>
     </row>
     <row r="152" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A152" s="31" t="inlineStr">
         <is>
-          <t>Bible</t>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B152" s="5" t="n"/>
@@ -5046,7 +4872,7 @@
     <row r="153" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A153" s="31" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B153" s="5" t="n"/>
@@ -5068,9 +4894,9 @@
       <c r="J153" s="33" t="n"/>
     </row>
     <row r="154" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A154" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
+      <c r="A154" s="34" t="inlineStr">
+        <is>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B154" s="5" t="n"/>
@@ -5092,9 +4918,9 @@
       <c r="J154" s="32" t="n"/>
     </row>
     <row r="155" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A155" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
+      <c r="A155" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B155" s="5" t="n"/>
@@ -5116,9 +4942,9 @@
       <c r="J155" s="33" t="n"/>
     </row>
     <row r="156" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A156" s="31" t="inlineStr">
-        <is>
-          <t>Writing / Composition</t>
+      <c r="A156" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B156" s="5" t="n"/>
@@ -5140,9 +4966,9 @@
       <c r="J156" s="32" t="n"/>
     </row>
     <row r="157" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A157" s="31" t="inlineStr">
-        <is>
-          <t>Science</t>
+      <c r="A157" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B157" s="5" t="n"/>
@@ -5164,9 +4990,9 @@
       <c r="J157" s="33" t="n"/>
     </row>
     <row r="158" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A158" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
+      <c r="A158" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
         </is>
       </c>
       <c r="B158" s="5" t="n"/>
@@ -5188,9 +5014,9 @@
       <c r="J158" s="32" t="n"/>
     </row>
     <row r="159" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A159" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
+      <c r="A159" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
         </is>
       </c>
       <c r="B159" s="5" t="n"/>
@@ -5212,9 +5038,9 @@
       <c r="J159" s="33" t="n"/>
     </row>
     <row r="160" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A160" s="31" t="inlineStr">
-        <is>
-          <t>Physical Education</t>
+      <c r="A160" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B160" s="5" t="n"/>
@@ -5236,9 +5062,9 @@
       <c r="J160" s="32" t="n"/>
     </row>
     <row r="161" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A161" s="31" t="inlineStr">
-        <is>
-          <t>Art / Music</t>
+      <c r="A161" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B161" s="5" t="n"/>
@@ -5259,58 +5085,17 @@
       <c r="I161" s="33" t="n"/>
       <c r="J161" s="33" t="n"/>
     </row>
-    <row r="162" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A162" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
-        </is>
-      </c>
-      <c r="B162" s="5" t="n"/>
-      <c r="C162" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D162" s="32" t="n"/>
-      <c r="E162" s="32" t="n"/>
-      <c r="F162" s="26" t="n"/>
-      <c r="G162" s="5" t="n"/>
-      <c r="H162" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I162" s="32" t="n"/>
-      <c r="J162" s="32" t="n"/>
-    </row>
-    <row r="163" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A163" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
-        </is>
-      </c>
-      <c r="B163" s="5" t="n"/>
-      <c r="C163" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D163" s="33" t="n"/>
-      <c r="E163" s="33" t="n"/>
-      <c r="F163" s="26" t="n"/>
-      <c r="G163" s="5" t="n"/>
-      <c r="H163" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I163" s="33" t="n"/>
-      <c r="J163" s="33" t="n"/>
+    <row r="162" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="163" ht="26" customHeight="1">
+      <c r="A163" s="44">
+        <f>IF('Getting Started'!B36&lt;&gt;"","  "&amp;UPPER('Getting Started'!B36)&amp;"   ·   "&amp;'Getting Started'!F36,"  STUDENT 8")</f>
+        <v/>
+      </c>
     </row>
     <row r="164" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A164" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A164" s="31" t="inlineStr">
+        <is>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B164" s="5" t="n"/>
@@ -5332,9 +5117,9 @@
       <c r="J164" s="32" t="n"/>
     </row>
     <row r="165" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A165" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A165" s="31" t="inlineStr">
+        <is>
+          <t>Math</t>
         </is>
       </c>
       <c r="B165" s="5" t="n"/>
@@ -5356,9 +5141,9 @@
       <c r="J165" s="33" t="n"/>
     </row>
     <row r="166" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A166" s="34" t="inlineStr">
-        <is>
-          <t>Other 5</t>
+      <c r="A166" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B166" s="5" t="n"/>
@@ -5379,25 +5164,34 @@
       <c r="I166" s="32" t="n"/>
       <c r="J166" s="32" t="n"/>
     </row>
-    <row r="167" hidden="1" outlineLevel="1" ht="26" customHeight="1">
-      <c r="A167" s="46">
-        <f>IF('Getting Started'!B38&lt;&gt;"","  "&amp;UPPER('Getting Started'!B38)&amp;"   ·   "&amp;'Getting Started'!F38,"  STUDENT 10")</f>
-        <v/>
-      </c>
-      <c r="B167" s="36" t="n"/>
-      <c r="C167" s="36" t="n"/>
-      <c r="D167" s="36" t="n"/>
-      <c r="E167" s="36" t="n"/>
-      <c r="F167" s="36" t="n"/>
-      <c r="G167" s="36" t="n"/>
-      <c r="H167" s="36" t="n"/>
-      <c r="I167" s="36" t="n"/>
-      <c r="J167" s="37" t="n"/>
+    <row r="167" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A167" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="n"/>
+      <c r="C167" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D167" s="33" t="n"/>
+      <c r="E167" s="33" t="n"/>
+      <c r="F167" s="26" t="n"/>
+      <c r="G167" s="5" t="n"/>
+      <c r="H167" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I167" s="33" t="n"/>
+      <c r="J167" s="33" t="n"/>
     </row>
     <row r="168" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A168" s="31" t="inlineStr">
         <is>
-          <t>Bible</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B168" s="5" t="n"/>
@@ -5421,7 +5215,7 @@
     <row r="169" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A169" s="31" t="inlineStr">
         <is>
-          <t>Math</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B169" s="5" t="n"/>
@@ -5445,7 +5239,7 @@
     <row r="170" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A170" s="31" t="inlineStr">
         <is>
-          <t>English / Language Arts</t>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B170" s="5" t="n"/>
@@ -5469,7 +5263,7 @@
     <row r="171" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A171" s="31" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B171" s="5" t="n"/>
@@ -5493,7 +5287,7 @@
     <row r="172" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A172" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B172" s="5" t="n"/>
@@ -5517,7 +5311,7 @@
     <row r="173" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A173" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B173" s="5" t="n"/>
@@ -5539,9 +5333,9 @@
       <c r="J173" s="33" t="n"/>
     </row>
     <row r="174" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A174" s="31" t="inlineStr">
-        <is>
-          <t>Social Studies / History</t>
+      <c r="A174" s="34" t="inlineStr">
+        <is>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B174" s="5" t="n"/>
@@ -5563,9 +5357,9 @@
       <c r="J174" s="32" t="n"/>
     </row>
     <row r="175" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A175" s="31" t="inlineStr">
-        <is>
-          <t>Health</t>
+      <c r="A175" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B175" s="5" t="n"/>
@@ -5587,9 +5381,9 @@
       <c r="J175" s="33" t="n"/>
     </row>
     <row r="176" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A176" s="31" t="inlineStr">
-        <is>
-          <t>Physical Education</t>
+      <c r="A176" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B176" s="5" t="n"/>
@@ -5611,9 +5405,9 @@
       <c r="J176" s="32" t="n"/>
     </row>
     <row r="177" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A177" s="31" t="inlineStr">
-        <is>
-          <t>Art / Music</t>
+      <c r="A177" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B177" s="5" t="n"/>
@@ -5637,7 +5431,7 @@
     <row r="178" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A178" s="34" t="inlineStr">
         <is>
-          <t>Other 1</t>
+          <t>Other 5</t>
         </is>
       </c>
       <c r="B178" s="5" t="n"/>
@@ -5661,7 +5455,7 @@
     <row r="179" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A179" s="34" t="inlineStr">
         <is>
-          <t>Other 2</t>
+          <t>Other 6</t>
         </is>
       </c>
       <c r="B179" s="5" t="n"/>
@@ -5685,7 +5479,7 @@
     <row r="180" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A180" s="34" t="inlineStr">
         <is>
-          <t>Other 3</t>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B180" s="5" t="n"/>
@@ -5709,7 +5503,7 @@
     <row r="181" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A181" s="34" t="inlineStr">
         <is>
-          <t>Other 4</t>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B181" s="5" t="n"/>
@@ -5730,58 +5524,17 @@
       <c r="I181" s="33" t="n"/>
       <c r="J181" s="33" t="n"/>
     </row>
-    <row r="182" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A182" s="34" t="inlineStr">
-        <is>
-          <t>Other 5</t>
-        </is>
-      </c>
-      <c r="B182" s="5" t="n"/>
-      <c r="C182" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D182" s="32" t="n"/>
-      <c r="E182" s="32" t="n"/>
-      <c r="F182" s="26" t="n"/>
-      <c r="G182" s="5" t="n"/>
-      <c r="H182" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I182" s="32" t="n"/>
-      <c r="J182" s="32" t="n"/>
-    </row>
-    <row r="183" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A183" s="34" t="inlineStr">
-        <is>
-          <t>Other 6</t>
-        </is>
-      </c>
-      <c r="B183" s="5" t="n"/>
-      <c r="C183" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D183" s="33" t="n"/>
-      <c r="E183" s="33" t="n"/>
-      <c r="F183" s="26" t="n"/>
-      <c r="G183" s="5" t="n"/>
-      <c r="H183" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I183" s="33" t="n"/>
-      <c r="J183" s="33" t="n"/>
+    <row r="182" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="183" ht="26" customHeight="1">
+      <c r="A183" s="45">
+        <f>IF('Getting Started'!B37&lt;&gt;"","  "&amp;UPPER('Getting Started'!B37)&amp;"   ·   "&amp;'Getting Started'!F37,"  STUDENT 9")</f>
+        <v/>
+      </c>
     </row>
     <row r="184" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A184" s="34" t="inlineStr">
-        <is>
-          <t>Other 7</t>
+      <c r="A184" s="31" t="inlineStr">
+        <is>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B184" s="5" t="n"/>
@@ -5803,9 +5556,9 @@
       <c r="J184" s="32" t="n"/>
     </row>
     <row r="185" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A185" s="34" t="inlineStr">
-        <is>
-          <t>Other 8</t>
+      <c r="A185" s="31" t="inlineStr">
+        <is>
+          <t>Math</t>
         </is>
       </c>
       <c r="B185" s="5" t="n"/>
@@ -5826,29 +5579,852 @@
       <c r="I185" s="33" t="n"/>
       <c r="J185" s="33" t="n"/>
     </row>
-    <row r="186" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="186" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A186" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
+        </is>
+      </c>
+      <c r="B186" s="5" t="n"/>
+      <c r="C186" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D186" s="32" t="n"/>
+      <c r="E186" s="32" t="n"/>
+      <c r="F186" s="26" t="n"/>
+      <c r="G186" s="5" t="n"/>
+      <c r="H186" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I186" s="32" t="n"/>
+      <c r="J186" s="32" t="n"/>
+    </row>
+    <row r="187" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A187" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="n"/>
+      <c r="C187" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D187" s="33" t="n"/>
+      <c r="E187" s="33" t="n"/>
+      <c r="F187" s="26" t="n"/>
+      <c r="G187" s="5" t="n"/>
+      <c r="H187" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I187" s="33" t="n"/>
+      <c r="J187" s="33" t="n"/>
+    </row>
+    <row r="188" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A188" s="31" t="inlineStr">
+        <is>
+          <t>Writing / Composition</t>
+        </is>
+      </c>
+      <c r="B188" s="5" t="n"/>
+      <c r="C188" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D188" s="32" t="n"/>
+      <c r="E188" s="32" t="n"/>
+      <c r="F188" s="26" t="n"/>
+      <c r="G188" s="5" t="n"/>
+      <c r="H188" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I188" s="32" t="n"/>
+      <c r="J188" s="32" t="n"/>
+    </row>
+    <row r="189" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A189" s="31" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="n"/>
+      <c r="C189" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D189" s="33" t="n"/>
+      <c r="E189" s="33" t="n"/>
+      <c r="F189" s="26" t="n"/>
+      <c r="G189" s="5" t="n"/>
+      <c r="H189" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I189" s="33" t="n"/>
+      <c r="J189" s="33" t="n"/>
+    </row>
+    <row r="190" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A190" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
+        </is>
+      </c>
+      <c r="B190" s="5" t="n"/>
+      <c r="C190" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D190" s="32" t="n"/>
+      <c r="E190" s="32" t="n"/>
+      <c r="F190" s="26" t="n"/>
+      <c r="G190" s="5" t="n"/>
+      <c r="H190" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I190" s="32" t="n"/>
+      <c r="J190" s="32" t="n"/>
+    </row>
+    <row r="191" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A191" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="n"/>
+      <c r="C191" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D191" s="33" t="n"/>
+      <c r="E191" s="33" t="n"/>
+      <c r="F191" s="26" t="n"/>
+      <c r="G191" s="5" t="n"/>
+      <c r="H191" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I191" s="33" t="n"/>
+      <c r="J191" s="33" t="n"/>
+    </row>
+    <row r="192" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A192" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
+        </is>
+      </c>
+      <c r="B192" s="5" t="n"/>
+      <c r="C192" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D192" s="32" t="n"/>
+      <c r="E192" s="32" t="n"/>
+      <c r="F192" s="26" t="n"/>
+      <c r="G192" s="5" t="n"/>
+      <c r="H192" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I192" s="32" t="n"/>
+      <c r="J192" s="32" t="n"/>
+    </row>
+    <row r="193" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A193" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="n"/>
+      <c r="C193" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D193" s="33" t="n"/>
+      <c r="E193" s="33" t="n"/>
+      <c r="F193" s="26" t="n"/>
+      <c r="G193" s="5" t="n"/>
+      <c r="H193" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I193" s="33" t="n"/>
+      <c r="J193" s="33" t="n"/>
+    </row>
+    <row r="194" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A194" s="34" t="inlineStr">
+        <is>
+          <t>Other 1</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="n"/>
+      <c r="C194" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D194" s="32" t="n"/>
+      <c r="E194" s="32" t="n"/>
+      <c r="F194" s="26" t="n"/>
+      <c r="G194" s="5" t="n"/>
+      <c r="H194" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I194" s="32" t="n"/>
+      <c r="J194" s="32" t="n"/>
+    </row>
+    <row r="195" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A195" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
+        </is>
+      </c>
+      <c r="B195" s="5" t="n"/>
+      <c r="C195" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D195" s="33" t="n"/>
+      <c r="E195" s="33" t="n"/>
+      <c r="F195" s="26" t="n"/>
+      <c r="G195" s="5" t="n"/>
+      <c r="H195" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I195" s="33" t="n"/>
+      <c r="J195" s="33" t="n"/>
+    </row>
+    <row r="196" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A196" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
+        </is>
+      </c>
+      <c r="B196" s="5" t="n"/>
+      <c r="C196" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D196" s="32" t="n"/>
+      <c r="E196" s="32" t="n"/>
+      <c r="F196" s="26" t="n"/>
+      <c r="G196" s="5" t="n"/>
+      <c r="H196" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I196" s="32" t="n"/>
+      <c r="J196" s="32" t="n"/>
+    </row>
+    <row r="197" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A197" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
+        </is>
+      </c>
+      <c r="B197" s="5" t="n"/>
+      <c r="C197" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D197" s="33" t="n"/>
+      <c r="E197" s="33" t="n"/>
+      <c r="F197" s="26" t="n"/>
+      <c r="G197" s="5" t="n"/>
+      <c r="H197" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I197" s="33" t="n"/>
+      <c r="J197" s="33" t="n"/>
+    </row>
+    <row r="198" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A198" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B198" s="5" t="n"/>
+      <c r="C198" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D198" s="32" t="n"/>
+      <c r="E198" s="32" t="n"/>
+      <c r="F198" s="26" t="n"/>
+      <c r="G198" s="5" t="n"/>
+      <c r="H198" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I198" s="32" t="n"/>
+      <c r="J198" s="32" t="n"/>
+    </row>
+    <row r="199" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A199" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B199" s="5" t="n"/>
+      <c r="C199" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D199" s="33" t="n"/>
+      <c r="E199" s="33" t="n"/>
+      <c r="F199" s="26" t="n"/>
+      <c r="G199" s="5" t="n"/>
+      <c r="H199" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I199" s="33" t="n"/>
+      <c r="J199" s="33" t="n"/>
+    </row>
+    <row r="200" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A200" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
+        </is>
+      </c>
+      <c r="B200" s="5" t="n"/>
+      <c r="C200" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D200" s="32" t="n"/>
+      <c r="E200" s="32" t="n"/>
+      <c r="F200" s="26" t="n"/>
+      <c r="G200" s="5" t="n"/>
+      <c r="H200" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I200" s="32" t="n"/>
+      <c r="J200" s="32" t="n"/>
+    </row>
+    <row r="201" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A201" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
+        </is>
+      </c>
+      <c r="B201" s="5" t="n"/>
+      <c r="C201" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D201" s="33" t="n"/>
+      <c r="E201" s="33" t="n"/>
+      <c r="F201" s="26" t="n"/>
+      <c r="G201" s="5" t="n"/>
+      <c r="H201" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I201" s="33" t="n"/>
+      <c r="J201" s="33" t="n"/>
+    </row>
+    <row r="202" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="203" ht="26" customHeight="1">
+      <c r="A203" s="46">
+        <f>IF('Getting Started'!B38&lt;&gt;"","  "&amp;UPPER('Getting Started'!B38)&amp;"   ·   "&amp;'Getting Started'!F38,"  STUDENT 10")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="204" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A204" s="31" t="inlineStr">
+        <is>
+          <t>Bible</t>
+        </is>
+      </c>
+      <c r="B204" s="5" t="n"/>
+      <c r="C204" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D204" s="32" t="n"/>
+      <c r="E204" s="32" t="n"/>
+      <c r="F204" s="26" t="n"/>
+      <c r="G204" s="5" t="n"/>
+      <c r="H204" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I204" s="32" t="n"/>
+      <c r="J204" s="32" t="n"/>
+    </row>
+    <row r="205" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A205" s="31" t="inlineStr">
+        <is>
+          <t>Math</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="n"/>
+      <c r="C205" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D205" s="33" t="n"/>
+      <c r="E205" s="33" t="n"/>
+      <c r="F205" s="26" t="n"/>
+      <c r="G205" s="5" t="n"/>
+      <c r="H205" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I205" s="33" t="n"/>
+      <c r="J205" s="33" t="n"/>
+    </row>
+    <row r="206" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A206" s="31" t="inlineStr">
+        <is>
+          <t>English / Language Arts</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="n"/>
+      <c r="C206" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D206" s="32" t="n"/>
+      <c r="E206" s="32" t="n"/>
+      <c r="F206" s="26" t="n"/>
+      <c r="G206" s="5" t="n"/>
+      <c r="H206" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I206" s="32" t="n"/>
+      <c r="J206" s="32" t="n"/>
+    </row>
+    <row r="207" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A207" s="31" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="n"/>
+      <c r="C207" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D207" s="33" t="n"/>
+      <c r="E207" s="33" t="n"/>
+      <c r="F207" s="26" t="n"/>
+      <c r="G207" s="5" t="n"/>
+      <c r="H207" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I207" s="33" t="n"/>
+      <c r="J207" s="33" t="n"/>
+    </row>
+    <row r="208" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A208" s="31" t="inlineStr">
+        <is>
+          <t>Writing / Composition</t>
+        </is>
+      </c>
+      <c r="B208" s="5" t="n"/>
+      <c r="C208" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D208" s="32" t="n"/>
+      <c r="E208" s="32" t="n"/>
+      <c r="F208" s="26" t="n"/>
+      <c r="G208" s="5" t="n"/>
+      <c r="H208" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I208" s="32" t="n"/>
+      <c r="J208" s="32" t="n"/>
+    </row>
+    <row r="209" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A209" s="31" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="n"/>
+      <c r="C209" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D209" s="33" t="n"/>
+      <c r="E209" s="33" t="n"/>
+      <c r="F209" s="26" t="n"/>
+      <c r="G209" s="5" t="n"/>
+      <c r="H209" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I209" s="33" t="n"/>
+      <c r="J209" s="33" t="n"/>
+    </row>
+    <row r="210" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A210" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
+        </is>
+      </c>
+      <c r="B210" s="5" t="n"/>
+      <c r="C210" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D210" s="32" t="n"/>
+      <c r="E210" s="32" t="n"/>
+      <c r="F210" s="26" t="n"/>
+      <c r="G210" s="5" t="n"/>
+      <c r="H210" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I210" s="32" t="n"/>
+      <c r="J210" s="32" t="n"/>
+    </row>
+    <row r="211" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A211" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B211" s="5" t="n"/>
+      <c r="C211" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D211" s="33" t="n"/>
+      <c r="E211" s="33" t="n"/>
+      <c r="F211" s="26" t="n"/>
+      <c r="G211" s="5" t="n"/>
+      <c r="H211" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I211" s="33" t="n"/>
+      <c r="J211" s="33" t="n"/>
+    </row>
+    <row r="212" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A212" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
+        </is>
+      </c>
+      <c r="B212" s="5" t="n"/>
+      <c r="C212" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D212" s="32" t="n"/>
+      <c r="E212" s="32" t="n"/>
+      <c r="F212" s="26" t="n"/>
+      <c r="G212" s="5" t="n"/>
+      <c r="H212" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I212" s="32" t="n"/>
+      <c r="J212" s="32" t="n"/>
+    </row>
+    <row r="213" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A213" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
+        </is>
+      </c>
+      <c r="B213" s="5" t="n"/>
+      <c r="C213" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D213" s="33" t="n"/>
+      <c r="E213" s="33" t="n"/>
+      <c r="F213" s="26" t="n"/>
+      <c r="G213" s="5" t="n"/>
+      <c r="H213" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I213" s="33" t="n"/>
+      <c r="J213" s="33" t="n"/>
+    </row>
+    <row r="214" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A214" s="34" t="inlineStr">
+        <is>
+          <t>Other 1</t>
+        </is>
+      </c>
+      <c r="B214" s="5" t="n"/>
+      <c r="C214" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D214" s="32" t="n"/>
+      <c r="E214" s="32" t="n"/>
+      <c r="F214" s="26" t="n"/>
+      <c r="G214" s="5" t="n"/>
+      <c r="H214" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I214" s="32" t="n"/>
+      <c r="J214" s="32" t="n"/>
+    </row>
+    <row r="215" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A215" s="34" t="inlineStr">
+        <is>
+          <t>Other 2</t>
+        </is>
+      </c>
+      <c r="B215" s="5" t="n"/>
+      <c r="C215" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D215" s="33" t="n"/>
+      <c r="E215" s="33" t="n"/>
+      <c r="F215" s="26" t="n"/>
+      <c r="G215" s="5" t="n"/>
+      <c r="H215" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I215" s="33" t="n"/>
+      <c r="J215" s="33" t="n"/>
+    </row>
+    <row r="216" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A216" s="34" t="inlineStr">
+        <is>
+          <t>Other 3</t>
+        </is>
+      </c>
+      <c r="B216" s="5" t="n"/>
+      <c r="C216" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D216" s="32" t="n"/>
+      <c r="E216" s="32" t="n"/>
+      <c r="F216" s="26" t="n"/>
+      <c r="G216" s="5" t="n"/>
+      <c r="H216" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I216" s="32" t="n"/>
+      <c r="J216" s="32" t="n"/>
+    </row>
+    <row r="217" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A217" s="34" t="inlineStr">
+        <is>
+          <t>Other 4</t>
+        </is>
+      </c>
+      <c r="B217" s="5" t="n"/>
+      <c r="C217" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D217" s="33" t="n"/>
+      <c r="E217" s="33" t="n"/>
+      <c r="F217" s="26" t="n"/>
+      <c r="G217" s="5" t="n"/>
+      <c r="H217" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I217" s="33" t="n"/>
+      <c r="J217" s="33" t="n"/>
+    </row>
+    <row r="218" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A218" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B218" s="5" t="n"/>
+      <c r="C218" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D218" s="32" t="n"/>
+      <c r="E218" s="32" t="n"/>
+      <c r="F218" s="26" t="n"/>
+      <c r="G218" s="5" t="n"/>
+      <c r="H218" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I218" s="32" t="n"/>
+      <c r="J218" s="32" t="n"/>
+    </row>
+    <row r="219" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A219" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B219" s="5" t="n"/>
+      <c r="C219" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D219" s="33" t="n"/>
+      <c r="E219" s="33" t="n"/>
+      <c r="F219" s="26" t="n"/>
+      <c r="G219" s="5" t="n"/>
+      <c r="H219" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I219" s="33" t="n"/>
+      <c r="J219" s="33" t="n"/>
+    </row>
+    <row r="220" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A220" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
+        </is>
+      </c>
+      <c r="B220" s="5" t="n"/>
+      <c r="C220" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D220" s="32" t="n"/>
+      <c r="E220" s="32" t="n"/>
+      <c r="F220" s="26" t="n"/>
+      <c r="G220" s="5" t="n"/>
+      <c r="H220" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I220" s="32" t="n"/>
+      <c r="J220" s="32" t="n"/>
+    </row>
+    <row r="221" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A221" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
+        </is>
+      </c>
+      <c r="B221" s="5" t="n"/>
+      <c r="C221" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D221" s="33" t="n"/>
+      <c r="E221" s="33" t="n"/>
+      <c r="F221" s="26" t="n"/>
+      <c r="G221" s="5" t="n"/>
+      <c r="H221" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I221" s="33" t="n"/>
+      <c r="J221" s="33" t="n"/>
+    </row>
+    <row r="222" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A203:J203"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A23:J23"/>
     <mergeCell ref="A103:J103"/>
-    <mergeCell ref="A119:J119"/>
-    <mergeCell ref="A135:J135"/>
-    <mergeCell ref="A167:J167"/>
-    <mergeCell ref="A39:J39"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="A87:J87"/>
+    <mergeCell ref="A123:J123"/>
+    <mergeCell ref="A143:J143"/>
+    <mergeCell ref="A83:J83"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A7:J7"/>
+    <mergeCell ref="A43:J43"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A163:J163"/>
+    <mergeCell ref="A183:J183"/>
     <mergeCell ref="G5:J5"/>
-    <mergeCell ref="A151:J151"/>
-    <mergeCell ref="A71:J71"/>
+    <mergeCell ref="A63:J63"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C58 C59 C60 C61 C62 C63 C64 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C83 C84 C85 C86 C87 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C102 C103 C104 C105 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C118 C119 C120 C121 C122 C123 C124 C125 C126 C127 C128 C129 C130 C131 C132 C133 C134 C135 C136 C137 C138 C139 C140 C141 C142 C143 C144 C145 C146 C147 C148 C149 C150 C151 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C162 C163 C164 C165 C166 C167 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 C182 C183 C184 C185 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 H103 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H122 H123 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H146 H147 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H166 H167 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H182 H183 H184 H185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C58 C59 C60 C61 C64 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C84 C85 C86 C87 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C104 C105 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C118 C119 C120 C121 C124 C125 C126 C127 C128 C129 C130 C131 C132 C133 C134 C135 C136 C137 C138 C139 C140 C141 C144 C145 C146 C147 C148 C149 C150 C151 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C164 C165 C166 C167 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 C184 C185 C186 C187 C188 C189 C190 C191 C192 C193 C194 C195 C196 C197 C198 C199 C200 C201 C204 C205 C206 C207 C208 C209 C210 C211 C212 C213 C214 C215 C216 C217 C218 C219 C220 C221 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H144 H145 H146 H147 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H164 H165 H166 H167 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H184 H185 H186 H187 H188 H189 H190 H191 H192 H193 H194 H195 H196 H197 H198 H199 H200 H201 H204 H205 H206 H207 H208 H209 H210 H211 H212 H213 H214 H215 H216 H217 H218 H219 H220 H221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"pages,lessons,chapters,units,assignments,projects"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix CC_STUDENT_FIRST collision with group rows for Other 7 & 8
CC_STUDENT_FIRST was hardcoded at 23. With 18 subjects the group section
spans rows 8-25, so student rows overlapped group rows 24-25 (Other 7/8).
Made CC_STUDENT_FIRST dynamic: CC_GROUP_DATA_START + NUM_SUBJECTS + 1 = 27.
Student sections now start at row 27, group section ends at row 25.
Verified all CC and student-sheet formula references are collision-free.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -311,7 +311,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -348,50 +348,6 @@
       </bottom>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00D4C4BB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00D4C4BB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D4C4BB"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00D4C4BB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D4C4BB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00D4C4BB"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D4C4BB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D4C4BB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="00CE8282"/>
       </left>
@@ -409,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -514,8 +470,6 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -565,7 +519,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1533,7 +1487,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J221"/>
+  <dimension ref="A1:J225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2004,25 +1958,34 @@
       <c r="I22" s="32" t="n"/>
       <c r="J22" s="32" t="n"/>
     </row>
-    <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="35">
-        <f>IF('Getting Started'!B29&lt;&gt;"","  "&amp;UPPER('Getting Started'!B29)&amp;"   ·   "&amp;'Getting Started'!F29,"  STUDENT 1")</f>
-        <v/>
-      </c>
-      <c r="B23" s="36" t="n"/>
-      <c r="C23" s="36" t="n"/>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="36" t="n"/>
-      <c r="F23" s="36" t="n"/>
-      <c r="G23" s="36" t="n"/>
-      <c r="H23" s="36" t="n"/>
-      <c r="I23" s="36" t="n"/>
-      <c r="J23" s="37" t="n"/>
-    </row>
-    <row r="24" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="33" t="n"/>
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I23" s="33" t="n"/>
+      <c r="J23" s="33" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B24" s="5" t="n"/>
@@ -2043,10 +2006,10 @@
       <c r="I24" s="32" t="n"/>
       <c r="J24" s="32" t="n"/>
     </row>
-    <row r="25" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B25" s="5" t="n"/>
@@ -2067,58 +2030,17 @@
       <c r="I25" s="33" t="n"/>
       <c r="J25" s="33" t="n"/>
     </row>
-    <row r="26" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="26" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I26" s="32" t="n"/>
-      <c r="J26" s="32" t="n"/>
-    </row>
-    <row r="27" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D27" s="33" t="n"/>
-      <c r="E27" s="33" t="n"/>
-      <c r="F27" s="26" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I27" s="33" t="n"/>
-      <c r="J27" s="33" t="n"/>
+    <row r="26" ht="8" customHeight="1"/>
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="35">
+        <f>IF('Getting Started'!B29&lt;&gt;"","  "&amp;UPPER('Getting Started'!B29)&amp;"   ·   "&amp;'Getting Started'!F29,"  STUDENT 1")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" outlineLevel="1" ht="20" customHeight="1">
       <c r="A28" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B28" s="5" t="n"/>
@@ -2142,7 +2064,7 @@
     <row r="29" outlineLevel="1" ht="20" customHeight="1">
       <c r="A29" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B29" s="5" t="n"/>
@@ -2166,7 +2088,7 @@
     <row r="30" outlineLevel="1" ht="20" customHeight="1">
       <c r="A30" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B30" s="5" t="n"/>
@@ -2190,7 +2112,7 @@
     <row r="31" outlineLevel="1" ht="20" customHeight="1">
       <c r="A31" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B31" s="5" t="n"/>
@@ -2214,7 +2136,7 @@
     <row r="32" outlineLevel="1" ht="20" customHeight="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B32" s="5" t="n"/>
@@ -2238,7 +2160,7 @@
     <row r="33" outlineLevel="1" ht="20" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B33" s="5" t="n"/>
@@ -2260,9 +2182,9 @@
       <c r="J33" s="33" t="n"/>
     </row>
     <row r="34" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A34" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B34" s="5" t="n"/>
@@ -2284,9 +2206,9 @@
       <c r="J34" s="32" t="n"/>
     </row>
     <row r="35" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A35" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B35" s="5" t="n"/>
@@ -2308,9 +2230,9 @@
       <c r="J35" s="33" t="n"/>
     </row>
     <row r="36" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A36" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B36" s="5" t="n"/>
@@ -2332,9 +2254,9 @@
       <c r="J36" s="32" t="n"/>
     </row>
     <row r="37" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A37" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A37" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B37" s="5" t="n"/>
@@ -2358,7 +2280,7 @@
     <row r="38" outlineLevel="1" ht="20" customHeight="1">
       <c r="A38" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B38" s="5" t="n"/>
@@ -2382,7 +2304,7 @@
     <row r="39" outlineLevel="1" ht="20" customHeight="1">
       <c r="A39" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B39" s="5" t="n"/>
@@ -2406,7 +2328,7 @@
     <row r="40" outlineLevel="1" ht="20" customHeight="1">
       <c r="A40" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B40" s="5" t="n"/>
@@ -2430,7 +2352,7 @@
     <row r="41" outlineLevel="1" ht="20" customHeight="1">
       <c r="A41" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B41" s="5" t="n"/>
@@ -2451,17 +2373,58 @@
       <c r="I41" s="33" t="n"/>
       <c r="J41" s="33" t="n"/>
     </row>
-    <row r="42" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="38">
-        <f>IF('Getting Started'!B30&lt;&gt;"","  "&amp;UPPER('Getting Started'!B30)&amp;"   ·   "&amp;'Getting Started'!F30,"  STUDENT 2")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A44" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+    <row r="42" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A42" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n"/>
+      <c r="C42" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="26" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I42" s="32" t="n"/>
+      <c r="J42" s="32" t="n"/>
+    </row>
+    <row r="43" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A43" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n"/>
+      <c r="C43" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D43" s="33" t="n"/>
+      <c r="E43" s="33" t="n"/>
+      <c r="F43" s="26" t="n"/>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I43" s="33" t="n"/>
+      <c r="J43" s="33" t="n"/>
+    </row>
+    <row r="44" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A44" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B44" s="5" t="n"/>
@@ -2482,10 +2445,10 @@
       <c r="I44" s="32" t="n"/>
       <c r="J44" s="32" t="n"/>
     </row>
-    <row r="45" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A45" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+    <row r="45" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A45" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B45" s="5" t="n"/>
@@ -2506,58 +2469,17 @@
       <c r="I45" s="33" t="n"/>
       <c r="J45" s="33" t="n"/>
     </row>
-    <row r="46" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A46" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B46" s="5" t="n"/>
-      <c r="C46" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D46" s="32" t="n"/>
-      <c r="E46" s="32" t="n"/>
-      <c r="F46" s="26" t="n"/>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I46" s="32" t="n"/>
-      <c r="J46" s="32" t="n"/>
-    </row>
-    <row r="47" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A47" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="n"/>
-      <c r="C47" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D47" s="33" t="n"/>
-      <c r="E47" s="33" t="n"/>
-      <c r="F47" s="26" t="n"/>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I47" s="33" t="n"/>
-      <c r="J47" s="33" t="n"/>
+    <row r="46" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="47" ht="26" customHeight="1">
+      <c r="A47" s="36">
+        <f>IF('Getting Started'!B30&lt;&gt;"","  "&amp;UPPER('Getting Started'!B30)&amp;"   ·   "&amp;'Getting Started'!F30,"  STUDENT 2")</f>
+        <v/>
+      </c>
     </row>
     <row r="48" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A48" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B48" s="5" t="n"/>
@@ -2581,7 +2503,7 @@
     <row r="49" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A49" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B49" s="5" t="n"/>
@@ -2605,7 +2527,7 @@
     <row r="50" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A50" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B50" s="5" t="n"/>
@@ -2629,7 +2551,7 @@
     <row r="51" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A51" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B51" s="5" t="n"/>
@@ -2653,7 +2575,7 @@
     <row r="52" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A52" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B52" s="5" t="n"/>
@@ -2677,7 +2599,7 @@
     <row r="53" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A53" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B53" s="5" t="n"/>
@@ -2699,9 +2621,9 @@
       <c r="J53" s="33" t="n"/>
     </row>
     <row r="54" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A54" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A54" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B54" s="5" t="n"/>
@@ -2723,9 +2645,9 @@
       <c r="J54" s="32" t="n"/>
     </row>
     <row r="55" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A55" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A55" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B55" s="5" t="n"/>
@@ -2747,9 +2669,9 @@
       <c r="J55" s="33" t="n"/>
     </row>
     <row r="56" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A56" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A56" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B56" s="5" t="n"/>
@@ -2771,9 +2693,9 @@
       <c r="J56" s="32" t="n"/>
     </row>
     <row r="57" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A57" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A57" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B57" s="5" t="n"/>
@@ -2797,7 +2719,7 @@
     <row r="58" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A58" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B58" s="5" t="n"/>
@@ -2821,7 +2743,7 @@
     <row r="59" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A59" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B59" s="5" t="n"/>
@@ -2845,7 +2767,7 @@
     <row r="60" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A60" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B60" s="5" t="n"/>
@@ -2869,7 +2791,7 @@
     <row r="61" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A61" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B61" s="5" t="n"/>
@@ -2890,17 +2812,58 @@
       <c r="I61" s="33" t="n"/>
       <c r="J61" s="33" t="n"/>
     </row>
-    <row r="62" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="39">
-        <f>IF('Getting Started'!B31&lt;&gt;"","  "&amp;UPPER('Getting Started'!B31)&amp;"   ·   "&amp;'Getting Started'!F31,"  STUDENT 3")</f>
-        <v/>
-      </c>
+    <row r="62" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A62" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D62" s="32" t="n"/>
+      <c r="E62" s="32" t="n"/>
+      <c r="F62" s="26" t="n"/>
+      <c r="G62" s="5" t="n"/>
+      <c r="H62" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I62" s="32" t="n"/>
+      <c r="J62" s="32" t="n"/>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A63" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n"/>
+      <c r="C63" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D63" s="33" t="n"/>
+      <c r="E63" s="33" t="n"/>
+      <c r="F63" s="26" t="n"/>
+      <c r="G63" s="5" t="n"/>
+      <c r="H63" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I63" s="33" t="n"/>
+      <c r="J63" s="33" t="n"/>
     </row>
     <row r="64" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A64" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A64" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B64" s="5" t="n"/>
@@ -2922,9 +2885,9 @@
       <c r="J64" s="32" t="n"/>
     </row>
     <row r="65" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A65" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A65" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B65" s="5" t="n"/>
@@ -2945,58 +2908,17 @@
       <c r="I65" s="33" t="n"/>
       <c r="J65" s="33" t="n"/>
     </row>
-    <row r="66" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A66" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="n"/>
-      <c r="C66" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D66" s="32" t="n"/>
-      <c r="E66" s="32" t="n"/>
-      <c r="F66" s="26" t="n"/>
-      <c r="G66" s="5" t="n"/>
-      <c r="H66" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I66" s="32" t="n"/>
-      <c r="J66" s="32" t="n"/>
-    </row>
-    <row r="67" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A67" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="n"/>
-      <c r="C67" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D67" s="33" t="n"/>
-      <c r="E67" s="33" t="n"/>
-      <c r="F67" s="26" t="n"/>
-      <c r="G67" s="5" t="n"/>
-      <c r="H67" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I67" s="33" t="n"/>
-      <c r="J67" s="33" t="n"/>
+    <row r="66" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="67" ht="26" customHeight="1">
+      <c r="A67" s="37">
+        <f>IF('Getting Started'!B31&lt;&gt;"","  "&amp;UPPER('Getting Started'!B31)&amp;"   ·   "&amp;'Getting Started'!F31,"  STUDENT 3")</f>
+        <v/>
+      </c>
     </row>
     <row r="68" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A68" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B68" s="5" t="n"/>
@@ -3020,7 +2942,7 @@
     <row r="69" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A69" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B69" s="5" t="n"/>
@@ -3044,7 +2966,7 @@
     <row r="70" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A70" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B70" s="5" t="n"/>
@@ -3068,7 +2990,7 @@
     <row r="71" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A71" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B71" s="5" t="n"/>
@@ -3092,7 +3014,7 @@
     <row r="72" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A72" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B72" s="5" t="n"/>
@@ -3116,7 +3038,7 @@
     <row r="73" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A73" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B73" s="5" t="n"/>
@@ -3138,9 +3060,9 @@
       <c r="J73" s="33" t="n"/>
     </row>
     <row r="74" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A74" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B74" s="5" t="n"/>
@@ -3162,9 +3084,9 @@
       <c r="J74" s="32" t="n"/>
     </row>
     <row r="75" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A75" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A75" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B75" s="5" t="n"/>
@@ -3186,9 +3108,9 @@
       <c r="J75" s="33" t="n"/>
     </row>
     <row r="76" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A76" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A76" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B76" s="5" t="n"/>
@@ -3210,9 +3132,9 @@
       <c r="J76" s="32" t="n"/>
     </row>
     <row r="77" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A77" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A77" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B77" s="5" t="n"/>
@@ -3236,7 +3158,7 @@
     <row r="78" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A78" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B78" s="5" t="n"/>
@@ -3260,7 +3182,7 @@
     <row r="79" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A79" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B79" s="5" t="n"/>
@@ -3284,7 +3206,7 @@
     <row r="80" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A80" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B80" s="5" t="n"/>
@@ -3308,7 +3230,7 @@
     <row r="81" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A81" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B81" s="5" t="n"/>
@@ -3329,17 +3251,58 @@
       <c r="I81" s="33" t="n"/>
       <c r="J81" s="33" t="n"/>
     </row>
-    <row r="82" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="83" ht="26" customHeight="1">
-      <c r="A83" s="40">
-        <f>IF('Getting Started'!B32&lt;&gt;"","  "&amp;UPPER('Getting Started'!B32)&amp;"   ·   "&amp;'Getting Started'!F32,"  STUDENT 4")</f>
-        <v/>
-      </c>
+    <row r="82" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A82" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="n"/>
+      <c r="C82" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D82" s="32" t="n"/>
+      <c r="E82" s="32" t="n"/>
+      <c r="F82" s="26" t="n"/>
+      <c r="G82" s="5" t="n"/>
+      <c r="H82" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I82" s="32" t="n"/>
+      <c r="J82" s="32" t="n"/>
+    </row>
+    <row r="83" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A83" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="n"/>
+      <c r="C83" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D83" s="33" t="n"/>
+      <c r="E83" s="33" t="n"/>
+      <c r="F83" s="26" t="n"/>
+      <c r="G83" s="5" t="n"/>
+      <c r="H83" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I83" s="33" t="n"/>
+      <c r="J83" s="33" t="n"/>
     </row>
     <row r="84" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A84" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A84" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B84" s="5" t="n"/>
@@ -3361,9 +3324,9 @@
       <c r="J84" s="32" t="n"/>
     </row>
     <row r="85" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A85" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A85" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B85" s="5" t="n"/>
@@ -3384,58 +3347,17 @@
       <c r="I85" s="33" t="n"/>
       <c r="J85" s="33" t="n"/>
     </row>
-    <row r="86" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A86" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B86" s="5" t="n"/>
-      <c r="C86" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D86" s="32" t="n"/>
-      <c r="E86" s="32" t="n"/>
-      <c r="F86" s="26" t="n"/>
-      <c r="G86" s="5" t="n"/>
-      <c r="H86" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I86" s="32" t="n"/>
-      <c r="J86" s="32" t="n"/>
-    </row>
-    <row r="87" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A87" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="n"/>
-      <c r="C87" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D87" s="33" t="n"/>
-      <c r="E87" s="33" t="n"/>
-      <c r="F87" s="26" t="n"/>
-      <c r="G87" s="5" t="n"/>
-      <c r="H87" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I87" s="33" t="n"/>
-      <c r="J87" s="33" t="n"/>
+    <row r="86" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="38">
+        <f>IF('Getting Started'!B32&lt;&gt;"","  "&amp;UPPER('Getting Started'!B32)&amp;"   ·   "&amp;'Getting Started'!F32,"  STUDENT 4")</f>
+        <v/>
+      </c>
     </row>
     <row r="88" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A88" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B88" s="5" t="n"/>
@@ -3459,7 +3381,7 @@
     <row r="89" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A89" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B89" s="5" t="n"/>
@@ -3483,7 +3405,7 @@
     <row r="90" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A90" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B90" s="5" t="n"/>
@@ -3507,7 +3429,7 @@
     <row r="91" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A91" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B91" s="5" t="n"/>
@@ -3531,7 +3453,7 @@
     <row r="92" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A92" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B92" s="5" t="n"/>
@@ -3555,7 +3477,7 @@
     <row r="93" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A93" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B93" s="5" t="n"/>
@@ -3577,9 +3499,9 @@
       <c r="J93" s="33" t="n"/>
     </row>
     <row r="94" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A94" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A94" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B94" s="5" t="n"/>
@@ -3601,9 +3523,9 @@
       <c r="J94" s="32" t="n"/>
     </row>
     <row r="95" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A95" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A95" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B95" s="5" t="n"/>
@@ -3625,9 +3547,9 @@
       <c r="J95" s="33" t="n"/>
     </row>
     <row r="96" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A96" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A96" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B96" s="5" t="n"/>
@@ -3649,9 +3571,9 @@
       <c r="J96" s="32" t="n"/>
     </row>
     <row r="97" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A97" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A97" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B97" s="5" t="n"/>
@@ -3675,7 +3597,7 @@
     <row r="98" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A98" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B98" s="5" t="n"/>
@@ -3699,7 +3621,7 @@
     <row r="99" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A99" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B99" s="5" t="n"/>
@@ -3723,7 +3645,7 @@
     <row r="100" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A100" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B100" s="5" t="n"/>
@@ -3747,7 +3669,7 @@
     <row r="101" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A101" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B101" s="5" t="n"/>
@@ -3768,17 +3690,58 @@
       <c r="I101" s="33" t="n"/>
       <c r="J101" s="33" t="n"/>
     </row>
-    <row r="102" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="103" ht="26" customHeight="1">
-      <c r="A103" s="41">
-        <f>IF('Getting Started'!B33&lt;&gt;"","  "&amp;UPPER('Getting Started'!B33)&amp;"   ·   "&amp;'Getting Started'!F33,"  STUDENT 5")</f>
-        <v/>
-      </c>
+    <row r="102" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A102" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B102" s="5" t="n"/>
+      <c r="C102" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D102" s="32" t="n"/>
+      <c r="E102" s="32" t="n"/>
+      <c r="F102" s="26" t="n"/>
+      <c r="G102" s="5" t="n"/>
+      <c r="H102" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I102" s="32" t="n"/>
+      <c r="J102" s="32" t="n"/>
+    </row>
+    <row r="103" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A103" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="n"/>
+      <c r="C103" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D103" s="33" t="n"/>
+      <c r="E103" s="33" t="n"/>
+      <c r="F103" s="26" t="n"/>
+      <c r="G103" s="5" t="n"/>
+      <c r="H103" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I103" s="33" t="n"/>
+      <c r="J103" s="33" t="n"/>
     </row>
     <row r="104" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A104" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A104" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B104" s="5" t="n"/>
@@ -3800,9 +3763,9 @@
       <c r="J104" s="32" t="n"/>
     </row>
     <row r="105" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A105" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A105" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B105" s="5" t="n"/>
@@ -3823,58 +3786,17 @@
       <c r="I105" s="33" t="n"/>
       <c r="J105" s="33" t="n"/>
     </row>
-    <row r="106" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A106" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B106" s="5" t="n"/>
-      <c r="C106" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D106" s="32" t="n"/>
-      <c r="E106" s="32" t="n"/>
-      <c r="F106" s="26" t="n"/>
-      <c r="G106" s="5" t="n"/>
-      <c r="H106" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I106" s="32" t="n"/>
-      <c r="J106" s="32" t="n"/>
-    </row>
-    <row r="107" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A107" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B107" s="5" t="n"/>
-      <c r="C107" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D107" s="33" t="n"/>
-      <c r="E107" s="33" t="n"/>
-      <c r="F107" s="26" t="n"/>
-      <c r="G107" s="5" t="n"/>
-      <c r="H107" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I107" s="33" t="n"/>
-      <c r="J107" s="33" t="n"/>
+    <row r="106" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="107" ht="26" customHeight="1">
+      <c r="A107" s="39">
+        <f>IF('Getting Started'!B33&lt;&gt;"","  "&amp;UPPER('Getting Started'!B33)&amp;"   ·   "&amp;'Getting Started'!F33,"  STUDENT 5")</f>
+        <v/>
+      </c>
     </row>
     <row r="108" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A108" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B108" s="5" t="n"/>
@@ -3898,7 +3820,7 @@
     <row r="109" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A109" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B109" s="5" t="n"/>
@@ -3922,7 +3844,7 @@
     <row r="110" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A110" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B110" s="5" t="n"/>
@@ -3946,7 +3868,7 @@
     <row r="111" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A111" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B111" s="5" t="n"/>
@@ -3970,7 +3892,7 @@
     <row r="112" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A112" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B112" s="5" t="n"/>
@@ -3994,7 +3916,7 @@
     <row r="113" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A113" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B113" s="5" t="n"/>
@@ -4016,9 +3938,9 @@
       <c r="J113" s="33" t="n"/>
     </row>
     <row r="114" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A114" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A114" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B114" s="5" t="n"/>
@@ -4040,9 +3962,9 @@
       <c r="J114" s="32" t="n"/>
     </row>
     <row r="115" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A115" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A115" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B115" s="5" t="n"/>
@@ -4064,9 +3986,9 @@
       <c r="J115" s="33" t="n"/>
     </row>
     <row r="116" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A116" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A116" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B116" s="5" t="n"/>
@@ -4088,9 +4010,9 @@
       <c r="J116" s="32" t="n"/>
     </row>
     <row r="117" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A117" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A117" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B117" s="5" t="n"/>
@@ -4114,7 +4036,7 @@
     <row r="118" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A118" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B118" s="5" t="n"/>
@@ -4138,7 +4060,7 @@
     <row r="119" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A119" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B119" s="5" t="n"/>
@@ -4162,7 +4084,7 @@
     <row r="120" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A120" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B120" s="5" t="n"/>
@@ -4186,7 +4108,7 @@
     <row r="121" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A121" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B121" s="5" t="n"/>
@@ -4207,17 +4129,58 @@
       <c r="I121" s="33" t="n"/>
       <c r="J121" s="33" t="n"/>
     </row>
-    <row r="122" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="123" ht="26" customHeight="1">
-      <c r="A123" s="42">
-        <f>IF('Getting Started'!B34&lt;&gt;"","  "&amp;UPPER('Getting Started'!B34)&amp;"   ·   "&amp;'Getting Started'!F34,"  STUDENT 6")</f>
-        <v/>
-      </c>
+    <row r="122" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A122" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B122" s="5" t="n"/>
+      <c r="C122" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D122" s="32" t="n"/>
+      <c r="E122" s="32" t="n"/>
+      <c r="F122" s="26" t="n"/>
+      <c r="G122" s="5" t="n"/>
+      <c r="H122" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I122" s="32" t="n"/>
+      <c r="J122" s="32" t="n"/>
+    </row>
+    <row r="123" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A123" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="n"/>
+      <c r="C123" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D123" s="33" t="n"/>
+      <c r="E123" s="33" t="n"/>
+      <c r="F123" s="26" t="n"/>
+      <c r="G123" s="5" t="n"/>
+      <c r="H123" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I123" s="33" t="n"/>
+      <c r="J123" s="33" t="n"/>
     </row>
     <row r="124" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A124" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A124" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B124" s="5" t="n"/>
@@ -4239,9 +4202,9 @@
       <c r="J124" s="32" t="n"/>
     </row>
     <row r="125" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A125" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A125" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B125" s="5" t="n"/>
@@ -4262,58 +4225,17 @@
       <c r="I125" s="33" t="n"/>
       <c r="J125" s="33" t="n"/>
     </row>
-    <row r="126" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A126" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B126" s="5" t="n"/>
-      <c r="C126" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D126" s="32" t="n"/>
-      <c r="E126" s="32" t="n"/>
-      <c r="F126" s="26" t="n"/>
-      <c r="G126" s="5" t="n"/>
-      <c r="H126" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I126" s="32" t="n"/>
-      <c r="J126" s="32" t="n"/>
-    </row>
-    <row r="127" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A127" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B127" s="5" t="n"/>
-      <c r="C127" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D127" s="33" t="n"/>
-      <c r="E127" s="33" t="n"/>
-      <c r="F127" s="26" t="n"/>
-      <c r="G127" s="5" t="n"/>
-      <c r="H127" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I127" s="33" t="n"/>
-      <c r="J127" s="33" t="n"/>
+    <row r="126" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="127" ht="26" customHeight="1">
+      <c r="A127" s="40">
+        <f>IF('Getting Started'!B34&lt;&gt;"","  "&amp;UPPER('Getting Started'!B34)&amp;"   ·   "&amp;'Getting Started'!F34,"  STUDENT 6")</f>
+        <v/>
+      </c>
     </row>
     <row r="128" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A128" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B128" s="5" t="n"/>
@@ -4337,7 +4259,7 @@
     <row r="129" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A129" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B129" s="5" t="n"/>
@@ -4361,7 +4283,7 @@
     <row r="130" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A130" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B130" s="5" t="n"/>
@@ -4385,7 +4307,7 @@
     <row r="131" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A131" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B131" s="5" t="n"/>
@@ -4409,7 +4331,7 @@
     <row r="132" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A132" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B132" s="5" t="n"/>
@@ -4433,7 +4355,7 @@
     <row r="133" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A133" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B133" s="5" t="n"/>
@@ -4455,9 +4377,9 @@
       <c r="J133" s="33" t="n"/>
     </row>
     <row r="134" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A134" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A134" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B134" s="5" t="n"/>
@@ -4479,9 +4401,9 @@
       <c r="J134" s="32" t="n"/>
     </row>
     <row r="135" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A135" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A135" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B135" s="5" t="n"/>
@@ -4503,9 +4425,9 @@
       <c r="J135" s="33" t="n"/>
     </row>
     <row r="136" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A136" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A136" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B136" s="5" t="n"/>
@@ -4527,9 +4449,9 @@
       <c r="J136" s="32" t="n"/>
     </row>
     <row r="137" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A137" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A137" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B137" s="5" t="n"/>
@@ -4553,7 +4475,7 @@
     <row r="138" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A138" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B138" s="5" t="n"/>
@@ -4577,7 +4499,7 @@
     <row r="139" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A139" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B139" s="5" t="n"/>
@@ -4601,7 +4523,7 @@
     <row r="140" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A140" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B140" s="5" t="n"/>
@@ -4625,7 +4547,7 @@
     <row r="141" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A141" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B141" s="5" t="n"/>
@@ -4646,17 +4568,58 @@
       <c r="I141" s="33" t="n"/>
       <c r="J141" s="33" t="n"/>
     </row>
-    <row r="142" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="143" ht="26" customHeight="1">
-      <c r="A143" s="43">
-        <f>IF('Getting Started'!B35&lt;&gt;"","  "&amp;UPPER('Getting Started'!B35)&amp;"   ·   "&amp;'Getting Started'!F35,"  STUDENT 7")</f>
-        <v/>
-      </c>
+    <row r="142" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A142" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="n"/>
+      <c r="C142" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D142" s="32" t="n"/>
+      <c r="E142" s="32" t="n"/>
+      <c r="F142" s="26" t="n"/>
+      <c r="G142" s="5" t="n"/>
+      <c r="H142" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I142" s="32" t="n"/>
+      <c r="J142" s="32" t="n"/>
+    </row>
+    <row r="143" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A143" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="n"/>
+      <c r="C143" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D143" s="33" t="n"/>
+      <c r="E143" s="33" t="n"/>
+      <c r="F143" s="26" t="n"/>
+      <c r="G143" s="5" t="n"/>
+      <c r="H143" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I143" s="33" t="n"/>
+      <c r="J143" s="33" t="n"/>
     </row>
     <row r="144" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A144" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A144" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B144" s="5" t="n"/>
@@ -4678,9 +4641,9 @@
       <c r="J144" s="32" t="n"/>
     </row>
     <row r="145" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A145" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A145" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B145" s="5" t="n"/>
@@ -4701,58 +4664,17 @@
       <c r="I145" s="33" t="n"/>
       <c r="J145" s="33" t="n"/>
     </row>
-    <row r="146" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A146" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B146" s="5" t="n"/>
-      <c r="C146" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D146" s="32" t="n"/>
-      <c r="E146" s="32" t="n"/>
-      <c r="F146" s="26" t="n"/>
-      <c r="G146" s="5" t="n"/>
-      <c r="H146" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I146" s="32" t="n"/>
-      <c r="J146" s="32" t="n"/>
-    </row>
-    <row r="147" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A147" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B147" s="5" t="n"/>
-      <c r="C147" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D147" s="33" t="n"/>
-      <c r="E147" s="33" t="n"/>
-      <c r="F147" s="26" t="n"/>
-      <c r="G147" s="5" t="n"/>
-      <c r="H147" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I147" s="33" t="n"/>
-      <c r="J147" s="33" t="n"/>
+    <row r="146" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="147" ht="26" customHeight="1">
+      <c r="A147" s="41">
+        <f>IF('Getting Started'!B35&lt;&gt;"","  "&amp;UPPER('Getting Started'!B35)&amp;"   ·   "&amp;'Getting Started'!F35,"  STUDENT 7")</f>
+        <v/>
+      </c>
     </row>
     <row r="148" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A148" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B148" s="5" t="n"/>
@@ -4776,7 +4698,7 @@
     <row r="149" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A149" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B149" s="5" t="n"/>
@@ -4800,7 +4722,7 @@
     <row r="150" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A150" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B150" s="5" t="n"/>
@@ -4824,7 +4746,7 @@
     <row r="151" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A151" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B151" s="5" t="n"/>
@@ -4848,7 +4770,7 @@
     <row r="152" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A152" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B152" s="5" t="n"/>
@@ -4872,7 +4794,7 @@
     <row r="153" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A153" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B153" s="5" t="n"/>
@@ -4894,9 +4816,9 @@
       <c r="J153" s="33" t="n"/>
     </row>
     <row r="154" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A154" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A154" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B154" s="5" t="n"/>
@@ -4918,9 +4840,9 @@
       <c r="J154" s="32" t="n"/>
     </row>
     <row r="155" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A155" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A155" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B155" s="5" t="n"/>
@@ -4942,9 +4864,9 @@
       <c r="J155" s="33" t="n"/>
     </row>
     <row r="156" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A156" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A156" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B156" s="5" t="n"/>
@@ -4966,9 +4888,9 @@
       <c r="J156" s="32" t="n"/>
     </row>
     <row r="157" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A157" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A157" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B157" s="5" t="n"/>
@@ -4992,7 +4914,7 @@
     <row r="158" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A158" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B158" s="5" t="n"/>
@@ -5016,7 +4938,7 @@
     <row r="159" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A159" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B159" s="5" t="n"/>
@@ -5040,7 +4962,7 @@
     <row r="160" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A160" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B160" s="5" t="n"/>
@@ -5064,7 +4986,7 @@
     <row r="161" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A161" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B161" s="5" t="n"/>
@@ -5085,17 +5007,58 @@
       <c r="I161" s="33" t="n"/>
       <c r="J161" s="33" t="n"/>
     </row>
-    <row r="162" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="163" ht="26" customHeight="1">
-      <c r="A163" s="44">
-        <f>IF('Getting Started'!B36&lt;&gt;"","  "&amp;UPPER('Getting Started'!B36)&amp;"   ·   "&amp;'Getting Started'!F36,"  STUDENT 8")</f>
-        <v/>
-      </c>
+    <row r="162" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A162" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="n"/>
+      <c r="C162" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D162" s="32" t="n"/>
+      <c r="E162" s="32" t="n"/>
+      <c r="F162" s="26" t="n"/>
+      <c r="G162" s="5" t="n"/>
+      <c r="H162" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I162" s="32" t="n"/>
+      <c r="J162" s="32" t="n"/>
+    </row>
+    <row r="163" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A163" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="n"/>
+      <c r="C163" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D163" s="33" t="n"/>
+      <c r="E163" s="33" t="n"/>
+      <c r="F163" s="26" t="n"/>
+      <c r="G163" s="5" t="n"/>
+      <c r="H163" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I163" s="33" t="n"/>
+      <c r="J163" s="33" t="n"/>
     </row>
     <row r="164" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A164" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A164" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B164" s="5" t="n"/>
@@ -5117,9 +5080,9 @@
       <c r="J164" s="32" t="n"/>
     </row>
     <row r="165" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A165" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A165" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B165" s="5" t="n"/>
@@ -5140,58 +5103,17 @@
       <c r="I165" s="33" t="n"/>
       <c r="J165" s="33" t="n"/>
     </row>
-    <row r="166" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A166" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B166" s="5" t="n"/>
-      <c r="C166" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D166" s="32" t="n"/>
-      <c r="E166" s="32" t="n"/>
-      <c r="F166" s="26" t="n"/>
-      <c r="G166" s="5" t="n"/>
-      <c r="H166" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I166" s="32" t="n"/>
-      <c r="J166" s="32" t="n"/>
-    </row>
-    <row r="167" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A167" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B167" s="5" t="n"/>
-      <c r="C167" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D167" s="33" t="n"/>
-      <c r="E167" s="33" t="n"/>
-      <c r="F167" s="26" t="n"/>
-      <c r="G167" s="5" t="n"/>
-      <c r="H167" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I167" s="33" t="n"/>
-      <c r="J167" s="33" t="n"/>
+    <row r="166" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="167" ht="26" customHeight="1">
+      <c r="A167" s="42">
+        <f>IF('Getting Started'!B36&lt;&gt;"","  "&amp;UPPER('Getting Started'!B36)&amp;"   ·   "&amp;'Getting Started'!F36,"  STUDENT 8")</f>
+        <v/>
+      </c>
     </row>
     <row r="168" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A168" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B168" s="5" t="n"/>
@@ -5215,7 +5137,7 @@
     <row r="169" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A169" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B169" s="5" t="n"/>
@@ -5239,7 +5161,7 @@
     <row r="170" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A170" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B170" s="5" t="n"/>
@@ -5263,7 +5185,7 @@
     <row r="171" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A171" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B171" s="5" t="n"/>
@@ -5287,7 +5209,7 @@
     <row r="172" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A172" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B172" s="5" t="n"/>
@@ -5311,7 +5233,7 @@
     <row r="173" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A173" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B173" s="5" t="n"/>
@@ -5333,9 +5255,9 @@
       <c r="J173" s="33" t="n"/>
     </row>
     <row r="174" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A174" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A174" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B174" s="5" t="n"/>
@@ -5357,9 +5279,9 @@
       <c r="J174" s="32" t="n"/>
     </row>
     <row r="175" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A175" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A175" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B175" s="5" t="n"/>
@@ -5381,9 +5303,9 @@
       <c r="J175" s="33" t="n"/>
     </row>
     <row r="176" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A176" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A176" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B176" s="5" t="n"/>
@@ -5405,9 +5327,9 @@
       <c r="J176" s="32" t="n"/>
     </row>
     <row r="177" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A177" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A177" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B177" s="5" t="n"/>
@@ -5431,7 +5353,7 @@
     <row r="178" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A178" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B178" s="5" t="n"/>
@@ -5455,7 +5377,7 @@
     <row r="179" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A179" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B179" s="5" t="n"/>
@@ -5479,7 +5401,7 @@
     <row r="180" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A180" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B180" s="5" t="n"/>
@@ -5503,7 +5425,7 @@
     <row r="181" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A181" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B181" s="5" t="n"/>
@@ -5524,17 +5446,58 @@
       <c r="I181" s="33" t="n"/>
       <c r="J181" s="33" t="n"/>
     </row>
-    <row r="182" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="183" ht="26" customHeight="1">
-      <c r="A183" s="45">
-        <f>IF('Getting Started'!B37&lt;&gt;"","  "&amp;UPPER('Getting Started'!B37)&amp;"   ·   "&amp;'Getting Started'!F37,"  STUDENT 9")</f>
-        <v/>
-      </c>
+    <row r="182" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A182" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="n"/>
+      <c r="C182" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D182" s="32" t="n"/>
+      <c r="E182" s="32" t="n"/>
+      <c r="F182" s="26" t="n"/>
+      <c r="G182" s="5" t="n"/>
+      <c r="H182" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I182" s="32" t="n"/>
+      <c r="J182" s="32" t="n"/>
+    </row>
+    <row r="183" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A183" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="n"/>
+      <c r="C183" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D183" s="33" t="n"/>
+      <c r="E183" s="33" t="n"/>
+      <c r="F183" s="26" t="n"/>
+      <c r="G183" s="5" t="n"/>
+      <c r="H183" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I183" s="33" t="n"/>
+      <c r="J183" s="33" t="n"/>
     </row>
     <row r="184" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A184" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A184" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B184" s="5" t="n"/>
@@ -5556,9 +5519,9 @@
       <c r="J184" s="32" t="n"/>
     </row>
     <row r="185" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A185" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A185" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B185" s="5" t="n"/>
@@ -5579,58 +5542,17 @@
       <c r="I185" s="33" t="n"/>
       <c r="J185" s="33" t="n"/>
     </row>
-    <row r="186" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A186" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B186" s="5" t="n"/>
-      <c r="C186" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D186" s="32" t="n"/>
-      <c r="E186" s="32" t="n"/>
-      <c r="F186" s="26" t="n"/>
-      <c r="G186" s="5" t="n"/>
-      <c r="H186" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I186" s="32" t="n"/>
-      <c r="J186" s="32" t="n"/>
-    </row>
-    <row r="187" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A187" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B187" s="5" t="n"/>
-      <c r="C187" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D187" s="33" t="n"/>
-      <c r="E187" s="33" t="n"/>
-      <c r="F187" s="26" t="n"/>
-      <c r="G187" s="5" t="n"/>
-      <c r="H187" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I187" s="33" t="n"/>
-      <c r="J187" s="33" t="n"/>
+    <row r="186" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="187" ht="26" customHeight="1">
+      <c r="A187" s="43">
+        <f>IF('Getting Started'!B37&lt;&gt;"","  "&amp;UPPER('Getting Started'!B37)&amp;"   ·   "&amp;'Getting Started'!F37,"  STUDENT 9")</f>
+        <v/>
+      </c>
     </row>
     <row r="188" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A188" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B188" s="5" t="n"/>
@@ -5654,7 +5576,7 @@
     <row r="189" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A189" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B189" s="5" t="n"/>
@@ -5678,7 +5600,7 @@
     <row r="190" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A190" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B190" s="5" t="n"/>
@@ -5702,7 +5624,7 @@
     <row r="191" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A191" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B191" s="5" t="n"/>
@@ -5726,7 +5648,7 @@
     <row r="192" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A192" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B192" s="5" t="n"/>
@@ -5750,7 +5672,7 @@
     <row r="193" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A193" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B193" s="5" t="n"/>
@@ -5772,9 +5694,9 @@
       <c r="J193" s="33" t="n"/>
     </row>
     <row r="194" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A194" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A194" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B194" s="5" t="n"/>
@@ -5796,9 +5718,9 @@
       <c r="J194" s="32" t="n"/>
     </row>
     <row r="195" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A195" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A195" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B195" s="5" t="n"/>
@@ -5820,9 +5742,9 @@
       <c r="J195" s="33" t="n"/>
     </row>
     <row r="196" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A196" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A196" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B196" s="5" t="n"/>
@@ -5844,9 +5766,9 @@
       <c r="J196" s="32" t="n"/>
     </row>
     <row r="197" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A197" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A197" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B197" s="5" t="n"/>
@@ -5870,7 +5792,7 @@
     <row r="198" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A198" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B198" s="5" t="n"/>
@@ -5894,7 +5816,7 @@
     <row r="199" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A199" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B199" s="5" t="n"/>
@@ -5918,7 +5840,7 @@
     <row r="200" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A200" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B200" s="5" t="n"/>
@@ -5942,7 +5864,7 @@
     <row r="201" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A201" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B201" s="5" t="n"/>
@@ -5963,17 +5885,58 @@
       <c r="I201" s="33" t="n"/>
       <c r="J201" s="33" t="n"/>
     </row>
-    <row r="202" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
-    <row r="203" ht="26" customHeight="1">
-      <c r="A203" s="46">
-        <f>IF('Getting Started'!B38&lt;&gt;"","  "&amp;UPPER('Getting Started'!B38)&amp;"   ·   "&amp;'Getting Started'!F38,"  STUDENT 10")</f>
-        <v/>
-      </c>
+    <row r="202" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A202" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B202" s="5" t="n"/>
+      <c r="C202" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D202" s="32" t="n"/>
+      <c r="E202" s="32" t="n"/>
+      <c r="F202" s="26" t="n"/>
+      <c r="G202" s="5" t="n"/>
+      <c r="H202" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I202" s="32" t="n"/>
+      <c r="J202" s="32" t="n"/>
+    </row>
+    <row r="203" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A203" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="n"/>
+      <c r="C203" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D203" s="33" t="n"/>
+      <c r="E203" s="33" t="n"/>
+      <c r="F203" s="26" t="n"/>
+      <c r="G203" s="5" t="n"/>
+      <c r="H203" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I203" s="33" t="n"/>
+      <c r="J203" s="33" t="n"/>
     </row>
     <row r="204" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A204" s="31" t="inlineStr">
-        <is>
-          <t>Bible</t>
+      <c r="A204" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
         </is>
       </c>
       <c r="B204" s="5" t="n"/>
@@ -5995,9 +5958,9 @@
       <c r="J204" s="32" t="n"/>
     </row>
     <row r="205" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A205" s="31" t="inlineStr">
-        <is>
-          <t>Math</t>
+      <c r="A205" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
         </is>
       </c>
       <c r="B205" s="5" t="n"/>
@@ -6018,58 +5981,17 @@
       <c r="I205" s="33" t="n"/>
       <c r="J205" s="33" t="n"/>
     </row>
-    <row r="206" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A206" s="31" t="inlineStr">
-        <is>
-          <t>English / Language Arts</t>
-        </is>
-      </c>
-      <c r="B206" s="5" t="n"/>
-      <c r="C206" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D206" s="32" t="n"/>
-      <c r="E206" s="32" t="n"/>
-      <c r="F206" s="26" t="n"/>
-      <c r="G206" s="5" t="n"/>
-      <c r="H206" s="32" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I206" s="32" t="n"/>
-      <c r="J206" s="32" t="n"/>
-    </row>
-    <row r="207" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A207" s="31" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B207" s="5" t="n"/>
-      <c r="C207" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="D207" s="33" t="n"/>
-      <c r="E207" s="33" t="n"/>
-      <c r="F207" s="26" t="n"/>
-      <c r="G207" s="5" t="n"/>
-      <c r="H207" s="33" t="inlineStr">
-        <is>
-          <t>pages</t>
-        </is>
-      </c>
-      <c r="I207" s="33" t="n"/>
-      <c r="J207" s="33" t="n"/>
+    <row r="206" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="207" ht="26" customHeight="1">
+      <c r="A207" s="44">
+        <f>IF('Getting Started'!B38&lt;&gt;"","  "&amp;UPPER('Getting Started'!B38)&amp;"   ·   "&amp;'Getting Started'!F38,"  STUDENT 10")</f>
+        <v/>
+      </c>
     </row>
     <row r="208" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A208" s="31" t="inlineStr">
         <is>
-          <t>Writing / Composition</t>
+          <t>Bible</t>
         </is>
       </c>
       <c r="B208" s="5" t="n"/>
@@ -6093,7 +6015,7 @@
     <row r="209" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A209" s="31" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Math</t>
         </is>
       </c>
       <c r="B209" s="5" t="n"/>
@@ -6117,7 +6039,7 @@
     <row r="210" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A210" s="31" t="inlineStr">
         <is>
-          <t>Social Studies / History</t>
+          <t>English / Language Arts</t>
         </is>
       </c>
       <c r="B210" s="5" t="n"/>
@@ -6141,7 +6063,7 @@
     <row r="211" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A211" s="31" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Reading</t>
         </is>
       </c>
       <c r="B211" s="5" t="n"/>
@@ -6165,7 +6087,7 @@
     <row r="212" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A212" s="31" t="inlineStr">
         <is>
-          <t>Physical Education</t>
+          <t>Writing / Composition</t>
         </is>
       </c>
       <c r="B212" s="5" t="n"/>
@@ -6189,7 +6111,7 @@
     <row r="213" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A213" s="31" t="inlineStr">
         <is>
-          <t>Art / Music</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="B213" s="5" t="n"/>
@@ -6211,9 +6133,9 @@
       <c r="J213" s="33" t="n"/>
     </row>
     <row r="214" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A214" s="34" t="inlineStr">
-        <is>
-          <t>Other 1</t>
+      <c r="A214" s="31" t="inlineStr">
+        <is>
+          <t>Social Studies / History</t>
         </is>
       </c>
       <c r="B214" s="5" t="n"/>
@@ -6235,9 +6157,9 @@
       <c r="J214" s="32" t="n"/>
     </row>
     <row r="215" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A215" s="34" t="inlineStr">
-        <is>
-          <t>Other 2</t>
+      <c r="A215" s="31" t="inlineStr">
+        <is>
+          <t>Health</t>
         </is>
       </c>
       <c r="B215" s="5" t="n"/>
@@ -6259,9 +6181,9 @@
       <c r="J215" s="33" t="n"/>
     </row>
     <row r="216" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A216" s="34" t="inlineStr">
-        <is>
-          <t>Other 3</t>
+      <c r="A216" s="31" t="inlineStr">
+        <is>
+          <t>Physical Education</t>
         </is>
       </c>
       <c r="B216" s="5" t="n"/>
@@ -6283,9 +6205,9 @@
       <c r="J216" s="32" t="n"/>
     </row>
     <row r="217" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A217" s="34" t="inlineStr">
-        <is>
-          <t>Other 4</t>
+      <c r="A217" s="31" t="inlineStr">
+        <is>
+          <t>Art / Music</t>
         </is>
       </c>
       <c r="B217" s="5" t="n"/>
@@ -6309,7 +6231,7 @@
     <row r="218" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A218" s="34" t="inlineStr">
         <is>
-          <t>Other 5</t>
+          <t>Other 1</t>
         </is>
       </c>
       <c r="B218" s="5" t="n"/>
@@ -6333,7 +6255,7 @@
     <row r="219" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A219" s="34" t="inlineStr">
         <is>
-          <t>Other 6</t>
+          <t>Other 2</t>
         </is>
       </c>
       <c r="B219" s="5" t="n"/>
@@ -6357,7 +6279,7 @@
     <row r="220" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A220" s="34" t="inlineStr">
         <is>
-          <t>Other 7</t>
+          <t>Other 3</t>
         </is>
       </c>
       <c r="B220" s="5" t="n"/>
@@ -6381,7 +6303,7 @@
     <row r="221" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A221" s="34" t="inlineStr">
         <is>
-          <t>Other 8</t>
+          <t>Other 4</t>
         </is>
       </c>
       <c r="B221" s="5" t="n"/>
@@ -6402,29 +6324,125 @@
       <c r="I221" s="33" t="n"/>
       <c r="J221" s="33" t="n"/>
     </row>
-    <row r="222" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
+    <row r="222" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A222" s="34" t="inlineStr">
+        <is>
+          <t>Other 5</t>
+        </is>
+      </c>
+      <c r="B222" s="5" t="n"/>
+      <c r="C222" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D222" s="32" t="n"/>
+      <c r="E222" s="32" t="n"/>
+      <c r="F222" s="26" t="n"/>
+      <c r="G222" s="5" t="n"/>
+      <c r="H222" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I222" s="32" t="n"/>
+      <c r="J222" s="32" t="n"/>
+    </row>
+    <row r="223" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A223" s="34" t="inlineStr">
+        <is>
+          <t>Other 6</t>
+        </is>
+      </c>
+      <c r="B223" s="5" t="n"/>
+      <c r="C223" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D223" s="33" t="n"/>
+      <c r="E223" s="33" t="n"/>
+      <c r="F223" s="26" t="n"/>
+      <c r="G223" s="5" t="n"/>
+      <c r="H223" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I223" s="33" t="n"/>
+      <c r="J223" s="33" t="n"/>
+    </row>
+    <row r="224" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A224" s="34" t="inlineStr">
+        <is>
+          <t>Other 7</t>
+        </is>
+      </c>
+      <c r="B224" s="5" t="n"/>
+      <c r="C224" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D224" s="32" t="n"/>
+      <c r="E224" s="32" t="n"/>
+      <c r="F224" s="26" t="n"/>
+      <c r="G224" s="5" t="n"/>
+      <c r="H224" s="32" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I224" s="32" t="n"/>
+      <c r="J224" s="32" t="n"/>
+    </row>
+    <row r="225" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A225" s="34" t="inlineStr">
+        <is>
+          <t>Other 8</t>
+        </is>
+      </c>
+      <c r="B225" s="5" t="n"/>
+      <c r="C225" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="D225" s="33" t="n"/>
+      <c r="E225" s="33" t="n"/>
+      <c r="F225" s="26" t="n"/>
+      <c r="G225" s="5" t="n"/>
+      <c r="H225" s="33" t="inlineStr">
+        <is>
+          <t>pages</t>
+        </is>
+      </c>
+      <c r="I225" s="33" t="n"/>
+      <c r="J225" s="33" t="n"/>
+    </row>
+    <row r="226" hidden="1" outlineLevel="1" ht="6" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A203:J203"/>
+    <mergeCell ref="A47:J47"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A23:J23"/>
-    <mergeCell ref="A103:J103"/>
-    <mergeCell ref="A123:J123"/>
-    <mergeCell ref="A143:J143"/>
-    <mergeCell ref="A83:J83"/>
+    <mergeCell ref="A107:J107"/>
+    <mergeCell ref="A127:J127"/>
+    <mergeCell ref="A167:J167"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A67:J67"/>
+    <mergeCell ref="A187:J187"/>
+    <mergeCell ref="A87:J87"/>
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A43:J43"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A163:J163"/>
-    <mergeCell ref="A183:J183"/>
+    <mergeCell ref="A147:J147"/>
     <mergeCell ref="G5:J5"/>
-    <mergeCell ref="A63:J63"/>
+    <mergeCell ref="A207:J207"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C58 C59 C60 C61 C64 C65 C66 C67 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C84 C85 C86 C87 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C104 C105 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C118 C119 C120 C121 C124 C125 C126 C127 C128 C129 C130 C131 C132 C133 C134 C135 C136 C137 C138 C139 C140 C141 C144 C145 C146 C147 C148 C149 C150 C151 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C164 C165 C166 C167 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 C184 C185 C186 C187 C188 C189 C190 C191 C192 C193 C194 C195 C196 C197 C198 C199 C200 C201 C204 C205 C206 C207 C208 C209 C210 C211 C212 C213 C214 C215 C216 C217 C218 C219 C220 C221 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H144 H145 H146 H147 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H164 H165 H166 H167 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H184 H185 H186 H187 H188 H189 H190 H191 H192 H193 H194 H195 H196 H197 H198 H199 H200 H201 H204 H205 H206 H207 H208 H209 H210 H211 H212 H213 H214 H215 H216 H217 H218 H219 H220 H221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 C21 C22 C23 C24 C25 C28 C29 C30 C31 C32 C33 C34 C35 C36 C37 C38 C39 C40 C41 C42 C43 C44 C45 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C58 C59 C60 C61 C62 C63 C64 C65 C68 C69 C70 C71 C72 C73 C74 C75 C76 C77 C78 C79 C80 C81 C82 C83 C84 C85 C88 C89 C90 C91 C92 C93 C94 C95 C96 C97 C98 C99 C100 C101 C102 C103 C104 C105 C108 C109 C110 C111 C112 C113 C114 C115 C116 C117 C118 C119 C120 C121 C122 C123 C124 C125 C128 C129 C130 C131 C132 C133 C134 C135 C136 C137 C138 C139 C140 C141 C142 C143 C144 C145 C148 C149 C150 C151 C152 C153 C154 C155 C156 C157 C158 C159 C160 C161 C162 C163 C164 C165 C168 C169 C170 C171 C172 C173 C174 C175 C176 C177 C178 C179 C180 C181 C182 C183 C184 C185 C188 C189 C190 C191 C192 C193 C194 C195 C196 C197 C198 C199 C200 C201 C202 C203 C204 C205 C208 C209 C210 C211 C212 C213 C214 C215 C216 C217 C218 C219 C220 C221 C222 C223 C224 C225 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 H103 H104 H105 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H122 H123 H124 H125 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H182 H183 H184 H185 H188 H189 H190 H191 H192 H193 H194 H195 H196 H197 H198 H199 H200 H201 H202 H203 H204 H205 H208 H209 H210 H211 H212 H213 H214 H215 H216 H217 H218 H219 H220 H221 H222 H223 H224 H225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"pages,lessons,chapters,units,assignments,projects"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6463,40 +6481,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
-      <c r="A1" s="47">
+      <c r="A1" s="45">
         <f>IF('Getting Started'!B29="","Student 1",'Getting Started'!B29)</f>
         <v/>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="48">
+      <c r="A2" s="46">
         <f>IFERROR("Grade: "&amp;'Getting Started'!F29&amp;"   ·   School Year: "&amp;'Getting Started'!C6,"")</f>
         <v/>
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="49">
+      <c r="A4" s="47">
         <f>IFERROR("SEM 1   "&amp;TEXT('Getting Started'!C10,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C11,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C15&amp;" school wks)","SEMESTER 1")</f>
         <v/>
       </c>
       <c r="J4" s="26" t="n"/>
-      <c r="K4" s="50">
+      <c r="K4" s="48">
         <f>IFERROR("SEM 2   "&amp;TEXT('Getting Started'!C18,"MMM D")&amp;" – "&amp;TEXT('Getting Started'!C19,"MMM D, YYYY")&amp;"   ("&amp;'Getting Started'!C23&amp;" school wks)","SEMESTER 2")</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1"/>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="51" t="inlineStr">
+      <c r="A6" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  SCHOOL DAYS  ·  Mark each day this student attends</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="52" t="inlineStr"/>
-      <c r="B7" s="53" t="inlineStr">
+      <c r="A7" s="50" t="inlineStr"/>
+      <c r="B7" s="51" t="inlineStr">
         <is>
           <t>Typical school week  →</t>
         </is>
@@ -6537,25 +6555,25 @@
         </is>
       </c>
       <c r="J7" s="26" t="n"/>
-      <c r="K7" s="54" t="n"/>
-      <c r="L7" s="54" t="n"/>
-      <c r="M7" s="54" t="n"/>
-      <c r="N7" s="54" t="n"/>
-      <c r="O7" s="54" t="n"/>
-      <c r="P7" s="54" t="n"/>
-      <c r="Q7" s="54" t="n"/>
-      <c r="R7" s="54" t="n"/>
+      <c r="K7" s="52" t="n"/>
+      <c r="L7" s="52" t="n"/>
+      <c r="M7" s="52" t="n"/>
+      <c r="N7" s="52" t="n"/>
+      <c r="O7" s="52" t="n"/>
+      <c r="P7" s="52" t="n"/>
+      <c r="Q7" s="52" t="n"/>
+      <c r="R7" s="52" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="26" t="n"/>
       <c r="B8" s="26" t="n"/>
-      <c r="C8" s="55" t="n"/>
-      <c r="D8" s="55" t="n"/>
-      <c r="E8" s="55" t="n"/>
-      <c r="F8" s="55" t="n"/>
-      <c r="G8" s="55" t="n"/>
-      <c r="H8" s="55" t="n"/>
-      <c r="I8" s="56">
+      <c r="C8" s="53" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="53" t="n"/>
+      <c r="F8" s="53" t="n"/>
+      <c r="G8" s="53" t="n"/>
+      <c r="H8" s="53" t="n"/>
+      <c r="I8" s="54">
         <f>MAX(1,COUNTA(C8:H8))</f>
         <v/>
       </c>
@@ -6571,91 +6589,91 @@
     </row>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="57" t="inlineStr">
+      <c r="A10" s="55" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="B10" s="57" t="inlineStr">
+      <c r="B10" s="55" t="inlineStr">
         <is>
           <t>Curriculum / Book</t>
         </is>
       </c>
-      <c r="C10" s="57" t="inlineStr">
+      <c r="C10" s="55" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="D10" s="57" t="inlineStr">
+      <c r="D10" s="55" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="E10" s="57" t="inlineStr">
+      <c r="E10" s="55" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="F10" s="57" t="inlineStr">
+      <c r="F10" s="55" t="inlineStr">
         <is>
           <t>Th</t>
         </is>
       </c>
-      <c r="G10" s="57" t="inlineStr">
+      <c r="G10" s="55" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="H10" s="57" t="inlineStr">
+      <c r="H10" s="55" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="I10" s="57" t="inlineStr">
+      <c r="I10" s="55" t="inlineStr">
         <is>
           <t>Days
 /Wk</t>
         </is>
       </c>
       <c r="J10" s="26" t="n"/>
-      <c r="K10" s="58" t="inlineStr">
+      <c r="K10" s="56" t="inlineStr">
         <is>
           <t>S1
 Total</t>
         </is>
       </c>
-      <c r="L10" s="58" t="inlineStr">
+      <c r="L10" s="56" t="inlineStr">
         <is>
           <t>S1
 /Wk</t>
         </is>
       </c>
-      <c r="M10" s="58" t="inlineStr">
+      <c r="M10" s="56" t="inlineStr">
         <is>
           <t>S1
 /Day</t>
         </is>
       </c>
       <c r="N10" s="26" t="n"/>
-      <c r="O10" s="59" t="inlineStr">
+      <c r="O10" s="57" t="inlineStr">
         <is>
           <t>S2
 Total</t>
         </is>
       </c>
-      <c r="P10" s="59" t="inlineStr">
+      <c r="P10" s="57" t="inlineStr">
         <is>
           <t>S2
 /Wk</t>
         </is>
       </c>
-      <c r="Q10" s="59" t="inlineStr">
+      <c r="Q10" s="57" t="inlineStr">
         <is>
           <t>S2
 /Day</t>
         </is>
       </c>
-      <c r="R10" s="57" t="inlineStr">
+      <c r="R10" s="55" t="inlineStr">
         <is>
           <t>Unit
 Type</t>
@@ -6669,47 +6687,47 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>IFERROR(IF('Course Content'!B24&lt;&gt;"",'Course Content'!B24,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,IF('Course Content'!G24&lt;&gt;"",'Course Content'!G24,IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C11" s="60" t="n"/>
-      <c r="D11" s="60" t="n"/>
-      <c r="E11" s="60" t="n"/>
-      <c r="F11" s="60" t="n"/>
-      <c r="G11" s="60" t="n"/>
-      <c r="H11" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C11" s="58" t="n"/>
+      <c r="D11" s="58" t="n"/>
+      <c r="E11" s="58" t="n"/>
+      <c r="F11" s="58" t="n"/>
+      <c r="G11" s="58" t="n"/>
+      <c r="H11" s="58" t="n"/>
       <c r="I11" s="17">
         <f>IF(COUNTA(C11:H11)=0,$I$8,COUNTA(C11:H11))</f>
         <v/>
       </c>
       <c r="J11" s="26" t="n"/>
-      <c r="K11" s="61">
-        <f>IFERROR(IF(('Course Content'!D8="")*('Course Content'!I8="")*('Course Content'!D24="")*('Course Content'!I24=""),"—",IFERROR('Course Content'!D8*1,0)+IFERROR('Course Content'!I8*1,0)+IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="61">
+      <c r="K11" s="59">
+        <f>IFERROR(IF(('Course Content'!D8="")*('Course Content'!I8="")*('Course Content'!D28="")*('Course Content'!I28=""),"—",IFERROR('Course Content'!D8*1,0)+IFERROR('Course Content'!I8*1,0)+IFERROR('Course Content'!D28*1,0)+IFERROR('Course Content'!I28*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="59">
         <f>IFERROR(IF(K11="","",IF(K11="—","",FLOOR(K11/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M11" s="62">
+      <c r="M11" s="60">
         <f>IFERROR(IF(L11="","",IF(L11="—","",FLOOR(L11/I11,1))),"")</f>
         <v/>
       </c>
       <c r="N11" s="26" t="n"/>
-      <c r="O11" s="63">
-        <f>IFERROR(IF(('Course Content'!E8="")*('Course Content'!J8="")*('Course Content'!E24="")*('Course Content'!J24=""),"—",IFERROR('Course Content'!E8*1,0)+IFERROR('Course Content'!J8*1,0)+IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P11" s="63">
+      <c r="O11" s="61">
+        <f>IFERROR(IF(('Course Content'!E8="")*('Course Content'!J8="")*('Course Content'!E28="")*('Course Content'!J28=""),"—",IFERROR('Course Content'!E8*1,0)+IFERROR('Course Content'!J8*1,0)+IFERROR('Course Content'!E28*1,0)+IFERROR('Course Content'!J28*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="61">
         <f>IFERROR(IF(O11="","",IF(O11="—","",FLOOR(O11/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q11" s="64">
+      <c r="Q11" s="62">
         <f>IFERROR(IF(P11="","",IF(P11="—","",FLOOR(P11/I11,1))),"")</f>
         <v/>
       </c>
-      <c r="R11" s="65">
-        <f>IFERROR(IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,IF('Course Content'!H24&lt;&gt;"",'Course Content'!H24,IF('Course Content'!C8&lt;&gt;"",'Course Content'!C8,'Course Content'!H8))),"")</f>
+      <c r="R11" s="63">
+        <f>IFERROR(IF('Course Content'!C28&lt;&gt;"",'Course Content'!C28,IF('Course Content'!H28&lt;&gt;"",'Course Content'!H28,IF('Course Content'!C8&lt;&gt;"",'Course Content'!C8,'Course Content'!H8))),"")</f>
         <v/>
       </c>
     </row>
@@ -6720,47 +6738,47 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>IFERROR(IF('Course Content'!B25&lt;&gt;"",'Course Content'!B25,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,IF('Course Content'!G25&lt;&gt;"",'Course Content'!G25,IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C12" s="60" t="n"/>
-      <c r="D12" s="60" t="n"/>
-      <c r="E12" s="60" t="n"/>
-      <c r="F12" s="60" t="n"/>
-      <c r="G12" s="60" t="n"/>
-      <c r="H12" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C12" s="58" t="n"/>
+      <c r="D12" s="58" t="n"/>
+      <c r="E12" s="58" t="n"/>
+      <c r="F12" s="58" t="n"/>
+      <c r="G12" s="58" t="n"/>
+      <c r="H12" s="58" t="n"/>
       <c r="I12" s="17">
         <f>IF(COUNTA(C12:H12)=0,$I$8,COUNTA(C12:H12))</f>
         <v/>
       </c>
       <c r="J12" s="26" t="n"/>
-      <c r="K12" s="61">
-        <f>IFERROR(IF(('Course Content'!D9="")*('Course Content'!I9="")*('Course Content'!D25="")*('Course Content'!I25=""),"—",IFERROR('Course Content'!D9*1,0)+IFERROR('Course Content'!I9*1,0)+IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="61">
+      <c r="K12" s="59">
+        <f>IFERROR(IF(('Course Content'!D9="")*('Course Content'!I9="")*('Course Content'!D29="")*('Course Content'!I29=""),"—",IFERROR('Course Content'!D9*1,0)+IFERROR('Course Content'!I9*1,0)+IFERROR('Course Content'!D29*1,0)+IFERROR('Course Content'!I29*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="59">
         <f>IFERROR(IF(K12="","",IF(K12="—","",FLOOR(K12/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M12" s="62">
+      <c r="M12" s="60">
         <f>IFERROR(IF(L12="","",IF(L12="—","",FLOOR(L12/I12,1))),"")</f>
         <v/>
       </c>
       <c r="N12" s="26" t="n"/>
-      <c r="O12" s="63">
-        <f>IFERROR(IF(('Course Content'!E9="")*('Course Content'!J9="")*('Course Content'!E25="")*('Course Content'!J25=""),"—",IFERROR('Course Content'!E9*1,0)+IFERROR('Course Content'!J9*1,0)+IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P12" s="63">
+      <c r="O12" s="61">
+        <f>IFERROR(IF(('Course Content'!E9="")*('Course Content'!J9="")*('Course Content'!E29="")*('Course Content'!J29=""),"—",IFERROR('Course Content'!E9*1,0)+IFERROR('Course Content'!J9*1,0)+IFERROR('Course Content'!E29*1,0)+IFERROR('Course Content'!J29*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="61">
         <f>IFERROR(IF(O12="","",IF(O12="—","",FLOOR(O12/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q12" s="64">
+      <c r="Q12" s="62">
         <f>IFERROR(IF(P12="","",IF(P12="—","",FLOOR(P12/I12,1))),"")</f>
         <v/>
       </c>
-      <c r="R12" s="66">
-        <f>IFERROR(IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,IF('Course Content'!H25&lt;&gt;"",'Course Content'!H25,IF('Course Content'!C9&lt;&gt;"",'Course Content'!C9,'Course Content'!H9))),"")</f>
+      <c r="R12" s="64">
+        <f>IFERROR(IF('Course Content'!C29&lt;&gt;"",'Course Content'!C29,IF('Course Content'!H29&lt;&gt;"",'Course Content'!H29,IF('Course Content'!C9&lt;&gt;"",'Course Content'!C9,'Course Content'!H9))),"")</f>
         <v/>
       </c>
     </row>
@@ -6771,47 +6789,47 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>IFERROR(IF('Course Content'!B26&lt;&gt;"",'Course Content'!B26,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,IF('Course Content'!G26&lt;&gt;"",'Course Content'!G26,IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C13" s="60" t="n"/>
-      <c r="D13" s="60" t="n"/>
-      <c r="E13" s="60" t="n"/>
-      <c r="F13" s="60" t="n"/>
-      <c r="G13" s="60" t="n"/>
-      <c r="H13" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C13" s="58" t="n"/>
+      <c r="D13" s="58" t="n"/>
+      <c r="E13" s="58" t="n"/>
+      <c r="F13" s="58" t="n"/>
+      <c r="G13" s="58" t="n"/>
+      <c r="H13" s="58" t="n"/>
       <c r="I13" s="17">
         <f>IF(COUNTA(C13:H13)=0,$I$8,COUNTA(C13:H13))</f>
         <v/>
       </c>
       <c r="J13" s="26" t="n"/>
-      <c r="K13" s="61">
-        <f>IFERROR(IF(('Course Content'!D10="")*('Course Content'!I10="")*('Course Content'!D26="")*('Course Content'!I26=""),"—",IFERROR('Course Content'!D10*1,0)+IFERROR('Course Content'!I10*1,0)+IFERROR('Course Content'!D26*1,0)+IFERROR('Course Content'!I26*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="61">
+      <c r="K13" s="59">
+        <f>IFERROR(IF(('Course Content'!D10="")*('Course Content'!I10="")*('Course Content'!D30="")*('Course Content'!I30=""),"—",IFERROR('Course Content'!D10*1,0)+IFERROR('Course Content'!I10*1,0)+IFERROR('Course Content'!D30*1,0)+IFERROR('Course Content'!I30*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="59">
         <f>IFERROR(IF(K13="","",IF(K13="—","",FLOOR(K13/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M13" s="62">
+      <c r="M13" s="60">
         <f>IFERROR(IF(L13="","",IF(L13="—","",FLOOR(L13/I13,1))),"")</f>
         <v/>
       </c>
       <c r="N13" s="26" t="n"/>
-      <c r="O13" s="63">
-        <f>IFERROR(IF(('Course Content'!E10="")*('Course Content'!J10="")*('Course Content'!E26="")*('Course Content'!J26=""),"—",IFERROR('Course Content'!E10*1,0)+IFERROR('Course Content'!J10*1,0)+IFERROR('Course Content'!E26*1,0)+IFERROR('Course Content'!J26*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P13" s="63">
+      <c r="O13" s="61">
+        <f>IFERROR(IF(('Course Content'!E10="")*('Course Content'!J10="")*('Course Content'!E30="")*('Course Content'!J30=""),"—",IFERROR('Course Content'!E10*1,0)+IFERROR('Course Content'!J10*1,0)+IFERROR('Course Content'!E30*1,0)+IFERROR('Course Content'!J30*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="61">
         <f>IFERROR(IF(O13="","",IF(O13="—","",FLOOR(O13/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q13" s="64">
+      <c r="Q13" s="62">
         <f>IFERROR(IF(P13="","",IF(P13="—","",FLOOR(P13/I13,1))),"")</f>
         <v/>
       </c>
-      <c r="R13" s="65">
-        <f>IFERROR(IF('Course Content'!C26&lt;&gt;"",'Course Content'!C26,IF('Course Content'!H26&lt;&gt;"",'Course Content'!H26,IF('Course Content'!C10&lt;&gt;"",'Course Content'!C10,'Course Content'!H10))),"")</f>
+      <c r="R13" s="63">
+        <f>IFERROR(IF('Course Content'!C30&lt;&gt;"",'Course Content'!C30,IF('Course Content'!H30&lt;&gt;"",'Course Content'!H30,IF('Course Content'!C10&lt;&gt;"",'Course Content'!C10,'Course Content'!H10))),"")</f>
         <v/>
       </c>
     </row>
@@ -6822,47 +6840,47 @@
         </is>
       </c>
       <c r="B14" s="18">
-        <f>IFERROR(IF('Course Content'!B27&lt;&gt;"",'Course Content'!B27,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,IF('Course Content'!G27&lt;&gt;"",'Course Content'!G27,IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C14" s="60" t="n"/>
-      <c r="D14" s="60" t="n"/>
-      <c r="E14" s="60" t="n"/>
-      <c r="F14" s="60" t="n"/>
-      <c r="G14" s="60" t="n"/>
-      <c r="H14" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C14" s="58" t="n"/>
+      <c r="D14" s="58" t="n"/>
+      <c r="E14" s="58" t="n"/>
+      <c r="F14" s="58" t="n"/>
+      <c r="G14" s="58" t="n"/>
+      <c r="H14" s="58" t="n"/>
       <c r="I14" s="17">
         <f>IF(COUNTA(C14:H14)=0,$I$8,COUNTA(C14:H14))</f>
         <v/>
       </c>
       <c r="J14" s="26" t="n"/>
-      <c r="K14" s="61">
-        <f>IFERROR(IF(('Course Content'!D11="")*('Course Content'!I11="")*('Course Content'!D27="")*('Course Content'!I27=""),"—",IFERROR('Course Content'!D11*1,0)+IFERROR('Course Content'!I11*1,0)+IFERROR('Course Content'!D27*1,0)+IFERROR('Course Content'!I27*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="61">
+      <c r="K14" s="59">
+        <f>IFERROR(IF(('Course Content'!D11="")*('Course Content'!I11="")*('Course Content'!D31="")*('Course Content'!I31=""),"—",IFERROR('Course Content'!D11*1,0)+IFERROR('Course Content'!I11*1,0)+IFERROR('Course Content'!D31*1,0)+IFERROR('Course Content'!I31*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="59">
         <f>IFERROR(IF(K14="","",IF(K14="—","",FLOOR(K14/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M14" s="62">
+      <c r="M14" s="60">
         <f>IFERROR(IF(L14="","",IF(L14="—","",FLOOR(L14/I14,1))),"")</f>
         <v/>
       </c>
       <c r="N14" s="26" t="n"/>
-      <c r="O14" s="63">
-        <f>IFERROR(IF(('Course Content'!E11="")*('Course Content'!J11="")*('Course Content'!E27="")*('Course Content'!J27=""),"—",IFERROR('Course Content'!E11*1,0)+IFERROR('Course Content'!J11*1,0)+IFERROR('Course Content'!E27*1,0)+IFERROR('Course Content'!J27*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P14" s="63">
+      <c r="O14" s="61">
+        <f>IFERROR(IF(('Course Content'!E11="")*('Course Content'!J11="")*('Course Content'!E31="")*('Course Content'!J31=""),"—",IFERROR('Course Content'!E11*1,0)+IFERROR('Course Content'!J11*1,0)+IFERROR('Course Content'!E31*1,0)+IFERROR('Course Content'!J31*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="61">
         <f>IFERROR(IF(O14="","",IF(O14="—","",FLOOR(O14/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q14" s="64">
+      <c r="Q14" s="62">
         <f>IFERROR(IF(P14="","",IF(P14="—","",FLOOR(P14/I14,1))),"")</f>
         <v/>
       </c>
-      <c r="R14" s="66">
-        <f>IFERROR(IF('Course Content'!C27&lt;&gt;"",'Course Content'!C27,IF('Course Content'!H27&lt;&gt;"",'Course Content'!H27,IF('Course Content'!C11&lt;&gt;"",'Course Content'!C11,'Course Content'!H11))),"")</f>
+      <c r="R14" s="64">
+        <f>IFERROR(IF('Course Content'!C31&lt;&gt;"",'Course Content'!C31,IF('Course Content'!H31&lt;&gt;"",'Course Content'!H31,IF('Course Content'!C11&lt;&gt;"",'Course Content'!C11,'Course Content'!H11))),"")</f>
         <v/>
       </c>
     </row>
@@ -6873,47 +6891,47 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>IFERROR(IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C15" s="60" t="n"/>
-      <c r="D15" s="60" t="n"/>
-      <c r="E15" s="60" t="n"/>
-      <c r="F15" s="60" t="n"/>
-      <c r="G15" s="60" t="n"/>
-      <c r="H15" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C15" s="58" t="n"/>
+      <c r="D15" s="58" t="n"/>
+      <c r="E15" s="58" t="n"/>
+      <c r="F15" s="58" t="n"/>
+      <c r="G15" s="58" t="n"/>
+      <c r="H15" s="58" t="n"/>
       <c r="I15" s="17">
         <f>IF(COUNTA(C15:H15)=0,$I$8,COUNTA(C15:H15))</f>
         <v/>
       </c>
       <c r="J15" s="26" t="n"/>
-      <c r="K15" s="61">
-        <f>IFERROR(IF(('Course Content'!D12="")*('Course Content'!I12="")*('Course Content'!D28="")*('Course Content'!I28=""),"—",IFERROR('Course Content'!D12*1,0)+IFERROR('Course Content'!I12*1,0)+IFERROR('Course Content'!D28*1,0)+IFERROR('Course Content'!I28*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L15" s="61">
+      <c r="K15" s="59">
+        <f>IFERROR(IF(('Course Content'!D12="")*('Course Content'!I12="")*('Course Content'!D32="")*('Course Content'!I32=""),"—",IFERROR('Course Content'!D12*1,0)+IFERROR('Course Content'!I12*1,0)+IFERROR('Course Content'!D32*1,0)+IFERROR('Course Content'!I32*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="59">
         <f>IFERROR(IF(K15="","",IF(K15="—","",FLOOR(K15/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M15" s="62">
+      <c r="M15" s="60">
         <f>IFERROR(IF(L15="","",IF(L15="—","",FLOOR(L15/I15,1))),"")</f>
         <v/>
       </c>
       <c r="N15" s="26" t="n"/>
-      <c r="O15" s="63">
-        <f>IFERROR(IF(('Course Content'!E12="")*('Course Content'!J12="")*('Course Content'!E28="")*('Course Content'!J28=""),"—",IFERROR('Course Content'!E12*1,0)+IFERROR('Course Content'!J12*1,0)+IFERROR('Course Content'!E28*1,0)+IFERROR('Course Content'!J28*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P15" s="63">
+      <c r="O15" s="61">
+        <f>IFERROR(IF(('Course Content'!E12="")*('Course Content'!J12="")*('Course Content'!E32="")*('Course Content'!J32=""),"—",IFERROR('Course Content'!E12*1,0)+IFERROR('Course Content'!J12*1,0)+IFERROR('Course Content'!E32*1,0)+IFERROR('Course Content'!J32*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="61">
         <f>IFERROR(IF(O15="","",IF(O15="—","",FLOOR(O15/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q15" s="64">
+      <c r="Q15" s="62">
         <f>IFERROR(IF(P15="","",IF(P15="—","",FLOOR(P15/I15,1))),"")</f>
         <v/>
       </c>
-      <c r="R15" s="65">
-        <f>IFERROR(IF('Course Content'!C28&lt;&gt;"",'Course Content'!C28,IF('Course Content'!H28&lt;&gt;"",'Course Content'!H28,IF('Course Content'!C12&lt;&gt;"",'Course Content'!C12,'Course Content'!H12))),"")</f>
+      <c r="R15" s="63">
+        <f>IFERROR(IF('Course Content'!C32&lt;&gt;"",'Course Content'!C32,IF('Course Content'!H32&lt;&gt;"",'Course Content'!H32,IF('Course Content'!C12&lt;&gt;"",'Course Content'!C12,'Course Content'!H12))),"")</f>
         <v/>
       </c>
     </row>
@@ -6924,47 +6942,47 @@
         </is>
       </c>
       <c r="B16" s="18">
-        <f>IFERROR(IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C16" s="60" t="n"/>
-      <c r="D16" s="60" t="n"/>
-      <c r="E16" s="60" t="n"/>
-      <c r="F16" s="60" t="n"/>
-      <c r="G16" s="60" t="n"/>
-      <c r="H16" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C16" s="58" t="n"/>
+      <c r="D16" s="58" t="n"/>
+      <c r="E16" s="58" t="n"/>
+      <c r="F16" s="58" t="n"/>
+      <c r="G16" s="58" t="n"/>
+      <c r="H16" s="58" t="n"/>
       <c r="I16" s="17">
         <f>IF(COUNTA(C16:H16)=0,$I$8,COUNTA(C16:H16))</f>
         <v/>
       </c>
       <c r="J16" s="26" t="n"/>
-      <c r="K16" s="61">
-        <f>IFERROR(IF(('Course Content'!D13="")*('Course Content'!I13="")*('Course Content'!D29="")*('Course Content'!I29=""),"—",IFERROR('Course Content'!D13*1,0)+IFERROR('Course Content'!I13*1,0)+IFERROR('Course Content'!D29*1,0)+IFERROR('Course Content'!I29*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L16" s="61">
+      <c r="K16" s="59">
+        <f>IFERROR(IF(('Course Content'!D13="")*('Course Content'!I13="")*('Course Content'!D33="")*('Course Content'!I33=""),"—",IFERROR('Course Content'!D13*1,0)+IFERROR('Course Content'!I13*1,0)+IFERROR('Course Content'!D33*1,0)+IFERROR('Course Content'!I33*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="59">
         <f>IFERROR(IF(K16="","",IF(K16="—","",FLOOR(K16/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M16" s="62">
+      <c r="M16" s="60">
         <f>IFERROR(IF(L16="","",IF(L16="—","",FLOOR(L16/I16,1))),"")</f>
         <v/>
       </c>
       <c r="N16" s="26" t="n"/>
-      <c r="O16" s="63">
-        <f>IFERROR(IF(('Course Content'!E13="")*('Course Content'!J13="")*('Course Content'!E29="")*('Course Content'!J29=""),"—",IFERROR('Course Content'!E13*1,0)+IFERROR('Course Content'!J13*1,0)+IFERROR('Course Content'!E29*1,0)+IFERROR('Course Content'!J29*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P16" s="63">
+      <c r="O16" s="61">
+        <f>IFERROR(IF(('Course Content'!E13="")*('Course Content'!J13="")*('Course Content'!E33="")*('Course Content'!J33=""),"—",IFERROR('Course Content'!E13*1,0)+IFERROR('Course Content'!J13*1,0)+IFERROR('Course Content'!E33*1,0)+IFERROR('Course Content'!J33*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="61">
         <f>IFERROR(IF(O16="","",IF(O16="—","",FLOOR(O16/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q16" s="64">
+      <c r="Q16" s="62">
         <f>IFERROR(IF(P16="","",IF(P16="—","",FLOOR(P16/I16,1))),"")</f>
         <v/>
       </c>
-      <c r="R16" s="66">
-        <f>IFERROR(IF('Course Content'!C29&lt;&gt;"",'Course Content'!C29,IF('Course Content'!H29&lt;&gt;"",'Course Content'!H29,IF('Course Content'!C13&lt;&gt;"",'Course Content'!C13,'Course Content'!H13))),"")</f>
+      <c r="R16" s="64">
+        <f>IFERROR(IF('Course Content'!C33&lt;&gt;"",'Course Content'!C33,IF('Course Content'!H33&lt;&gt;"",'Course Content'!H33,IF('Course Content'!C13&lt;&gt;"",'Course Content'!C13,'Course Content'!H13))),"")</f>
         <v/>
       </c>
     </row>
@@ -6975,47 +6993,47 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>IFERROR(IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C17" s="60" t="n"/>
-      <c r="D17" s="60" t="n"/>
-      <c r="E17" s="60" t="n"/>
-      <c r="F17" s="60" t="n"/>
-      <c r="G17" s="60" t="n"/>
-      <c r="H17" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C17" s="58" t="n"/>
+      <c r="D17" s="58" t="n"/>
+      <c r="E17" s="58" t="n"/>
+      <c r="F17" s="58" t="n"/>
+      <c r="G17" s="58" t="n"/>
+      <c r="H17" s="58" t="n"/>
       <c r="I17" s="17">
         <f>IF(COUNTA(C17:H17)=0,$I$8,COUNTA(C17:H17))</f>
         <v/>
       </c>
       <c r="J17" s="26" t="n"/>
-      <c r="K17" s="61">
-        <f>IFERROR(IF(('Course Content'!D14="")*('Course Content'!I14="")*('Course Content'!D30="")*('Course Content'!I30=""),"—",IFERROR('Course Content'!D14*1,0)+IFERROR('Course Content'!I14*1,0)+IFERROR('Course Content'!D30*1,0)+IFERROR('Course Content'!I30*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="61">
+      <c r="K17" s="59">
+        <f>IFERROR(IF(('Course Content'!D14="")*('Course Content'!I14="")*('Course Content'!D34="")*('Course Content'!I34=""),"—",IFERROR('Course Content'!D14*1,0)+IFERROR('Course Content'!I14*1,0)+IFERROR('Course Content'!D34*1,0)+IFERROR('Course Content'!I34*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="59">
         <f>IFERROR(IF(K17="","",IF(K17="—","",FLOOR(K17/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M17" s="62">
+      <c r="M17" s="60">
         <f>IFERROR(IF(L17="","",IF(L17="—","",FLOOR(L17/I17,1))),"")</f>
         <v/>
       </c>
       <c r="N17" s="26" t="n"/>
-      <c r="O17" s="63">
-        <f>IFERROR(IF(('Course Content'!E14="")*('Course Content'!J14="")*('Course Content'!E30="")*('Course Content'!J30=""),"—",IFERROR('Course Content'!E14*1,0)+IFERROR('Course Content'!J14*1,0)+IFERROR('Course Content'!E30*1,0)+IFERROR('Course Content'!J30*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P17" s="63">
+      <c r="O17" s="61">
+        <f>IFERROR(IF(('Course Content'!E14="")*('Course Content'!J14="")*('Course Content'!E34="")*('Course Content'!J34=""),"—",IFERROR('Course Content'!E14*1,0)+IFERROR('Course Content'!J14*1,0)+IFERROR('Course Content'!E34*1,0)+IFERROR('Course Content'!J34*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="61">
         <f>IFERROR(IF(O17="","",IF(O17="—","",FLOOR(O17/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q17" s="64">
+      <c r="Q17" s="62">
         <f>IFERROR(IF(P17="","",IF(P17="—","",FLOOR(P17/I17,1))),"")</f>
         <v/>
       </c>
-      <c r="R17" s="65">
-        <f>IFERROR(IF('Course Content'!C30&lt;&gt;"",'Course Content'!C30,IF('Course Content'!H30&lt;&gt;"",'Course Content'!H30,IF('Course Content'!C14&lt;&gt;"",'Course Content'!C14,'Course Content'!H14))),"")</f>
+      <c r="R17" s="63">
+        <f>IFERROR(IF('Course Content'!C34&lt;&gt;"",'Course Content'!C34,IF('Course Content'!H34&lt;&gt;"",'Course Content'!H34,IF('Course Content'!C14&lt;&gt;"",'Course Content'!C14,'Course Content'!H14))),"")</f>
         <v/>
       </c>
     </row>
@@ -7026,47 +7044,47 @@
         </is>
       </c>
       <c r="B18" s="18">
-        <f>IFERROR(IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C18" s="60" t="n"/>
-      <c r="D18" s="60" t="n"/>
-      <c r="E18" s="60" t="n"/>
-      <c r="F18" s="60" t="n"/>
-      <c r="G18" s="60" t="n"/>
-      <c r="H18" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C18" s="58" t="n"/>
+      <c r="D18" s="58" t="n"/>
+      <c r="E18" s="58" t="n"/>
+      <c r="F18" s="58" t="n"/>
+      <c r="G18" s="58" t="n"/>
+      <c r="H18" s="58" t="n"/>
       <c r="I18" s="17">
         <f>IF(COUNTA(C18:H18)=0,$I$8,COUNTA(C18:H18))</f>
         <v/>
       </c>
       <c r="J18" s="26" t="n"/>
-      <c r="K18" s="61">
-        <f>IFERROR(IF(('Course Content'!D15="")*('Course Content'!I15="")*('Course Content'!D31="")*('Course Content'!I31=""),"—",IFERROR('Course Content'!D15*1,0)+IFERROR('Course Content'!I15*1,0)+IFERROR('Course Content'!D31*1,0)+IFERROR('Course Content'!I31*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="61">
+      <c r="K18" s="59">
+        <f>IFERROR(IF(('Course Content'!D15="")*('Course Content'!I15="")*('Course Content'!D35="")*('Course Content'!I35=""),"—",IFERROR('Course Content'!D15*1,0)+IFERROR('Course Content'!I15*1,0)+IFERROR('Course Content'!D35*1,0)+IFERROR('Course Content'!I35*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="59">
         <f>IFERROR(IF(K18="","",IF(K18="—","",FLOOR(K18/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M18" s="62">
+      <c r="M18" s="60">
         <f>IFERROR(IF(L18="","",IF(L18="—","",FLOOR(L18/I18,1))),"")</f>
         <v/>
       </c>
       <c r="N18" s="26" t="n"/>
-      <c r="O18" s="63">
-        <f>IFERROR(IF(('Course Content'!E15="")*('Course Content'!J15="")*('Course Content'!E31="")*('Course Content'!J31=""),"—",IFERROR('Course Content'!E15*1,0)+IFERROR('Course Content'!J15*1,0)+IFERROR('Course Content'!E31*1,0)+IFERROR('Course Content'!J31*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P18" s="63">
+      <c r="O18" s="61">
+        <f>IFERROR(IF(('Course Content'!E15="")*('Course Content'!J15="")*('Course Content'!E35="")*('Course Content'!J35=""),"—",IFERROR('Course Content'!E15*1,0)+IFERROR('Course Content'!J15*1,0)+IFERROR('Course Content'!E35*1,0)+IFERROR('Course Content'!J35*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="61">
         <f>IFERROR(IF(O18="","",IF(O18="—","",FLOOR(O18/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q18" s="64">
+      <c r="Q18" s="62">
         <f>IFERROR(IF(P18="","",IF(P18="—","",FLOOR(P18/I18,1))),"")</f>
         <v/>
       </c>
-      <c r="R18" s="66">
-        <f>IFERROR(IF('Course Content'!C31&lt;&gt;"",'Course Content'!C31,IF('Course Content'!H31&lt;&gt;"",'Course Content'!H31,IF('Course Content'!C15&lt;&gt;"",'Course Content'!C15,'Course Content'!H15))),"")</f>
+      <c r="R18" s="64">
+        <f>IFERROR(IF('Course Content'!C35&lt;&gt;"",'Course Content'!C35,IF('Course Content'!H35&lt;&gt;"",'Course Content'!H35,IF('Course Content'!C15&lt;&gt;"",'Course Content'!C15,'Course Content'!H15))),"")</f>
         <v/>
       </c>
     </row>
@@ -7077,47 +7095,47 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>IFERROR(IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C19" s="60" t="n"/>
-      <c r="D19" s="60" t="n"/>
-      <c r="E19" s="60" t="n"/>
-      <c r="F19" s="60" t="n"/>
-      <c r="G19" s="60" t="n"/>
-      <c r="H19" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C19" s="58" t="n"/>
+      <c r="D19" s="58" t="n"/>
+      <c r="E19" s="58" t="n"/>
+      <c r="F19" s="58" t="n"/>
+      <c r="G19" s="58" t="n"/>
+      <c r="H19" s="58" t="n"/>
       <c r="I19" s="17">
         <f>IF(COUNTA(C19:H19)=0,$I$8,COUNTA(C19:H19))</f>
         <v/>
       </c>
       <c r="J19" s="26" t="n"/>
-      <c r="K19" s="61">
-        <f>IFERROR(IF(('Course Content'!D16="")*('Course Content'!I16="")*('Course Content'!D32="")*('Course Content'!I32=""),"—",IFERROR('Course Content'!D16*1,0)+IFERROR('Course Content'!I16*1,0)+IFERROR('Course Content'!D32*1,0)+IFERROR('Course Content'!I32*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="61">
+      <c r="K19" s="59">
+        <f>IFERROR(IF(('Course Content'!D16="")*('Course Content'!I16="")*('Course Content'!D36="")*('Course Content'!I36=""),"—",IFERROR('Course Content'!D16*1,0)+IFERROR('Course Content'!I16*1,0)+IFERROR('Course Content'!D36*1,0)+IFERROR('Course Content'!I36*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="59">
         <f>IFERROR(IF(K19="","",IF(K19="—","",FLOOR(K19/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M19" s="62">
+      <c r="M19" s="60">
         <f>IFERROR(IF(L19="","",IF(L19="—","",FLOOR(L19/I19,1))),"")</f>
         <v/>
       </c>
       <c r="N19" s="26" t="n"/>
-      <c r="O19" s="63">
-        <f>IFERROR(IF(('Course Content'!E16="")*('Course Content'!J16="")*('Course Content'!E32="")*('Course Content'!J32=""),"—",IFERROR('Course Content'!E16*1,0)+IFERROR('Course Content'!J16*1,0)+IFERROR('Course Content'!E32*1,0)+IFERROR('Course Content'!J32*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P19" s="63">
+      <c r="O19" s="61">
+        <f>IFERROR(IF(('Course Content'!E16="")*('Course Content'!J16="")*('Course Content'!E36="")*('Course Content'!J36=""),"—",IFERROR('Course Content'!E16*1,0)+IFERROR('Course Content'!J16*1,0)+IFERROR('Course Content'!E36*1,0)+IFERROR('Course Content'!J36*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="61">
         <f>IFERROR(IF(O19="","",IF(O19="—","",FLOOR(O19/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q19" s="64">
+      <c r="Q19" s="62">
         <f>IFERROR(IF(P19="","",IF(P19="—","",FLOOR(P19/I19,1))),"")</f>
         <v/>
       </c>
-      <c r="R19" s="65">
-        <f>IFERROR(IF('Course Content'!C32&lt;&gt;"",'Course Content'!C32,IF('Course Content'!H32&lt;&gt;"",'Course Content'!H32,IF('Course Content'!C16&lt;&gt;"",'Course Content'!C16,'Course Content'!H16))),"")</f>
+      <c r="R19" s="63">
+        <f>IFERROR(IF('Course Content'!C36&lt;&gt;"",'Course Content'!C36,IF('Course Content'!H36&lt;&gt;"",'Course Content'!H36,IF('Course Content'!C16&lt;&gt;"",'Course Content'!C16,'Course Content'!H16))),"")</f>
         <v/>
       </c>
     </row>
@@ -7128,447 +7146,447 @@
         </is>
       </c>
       <c r="B20" s="18">
-        <f>IFERROR(IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C20" s="60" t="n"/>
-      <c r="D20" s="60" t="n"/>
-      <c r="E20" s="60" t="n"/>
-      <c r="F20" s="60" t="n"/>
-      <c r="G20" s="60" t="n"/>
-      <c r="H20" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C20" s="58" t="n"/>
+      <c r="D20" s="58" t="n"/>
+      <c r="E20" s="58" t="n"/>
+      <c r="F20" s="58" t="n"/>
+      <c r="G20" s="58" t="n"/>
+      <c r="H20" s="58" t="n"/>
       <c r="I20" s="17">
         <f>IF(COUNTA(C20:H20)=0,$I$8,COUNTA(C20:H20))</f>
         <v/>
       </c>
       <c r="J20" s="26" t="n"/>
-      <c r="K20" s="61">
-        <f>IFERROR(IF(('Course Content'!D17="")*('Course Content'!I17="")*('Course Content'!D33="")*('Course Content'!I33=""),"—",IFERROR('Course Content'!D17*1,0)+IFERROR('Course Content'!I17*1,0)+IFERROR('Course Content'!D33*1,0)+IFERROR('Course Content'!I33*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="61">
+      <c r="K20" s="59">
+        <f>IFERROR(IF(('Course Content'!D17="")*('Course Content'!I17="")*('Course Content'!D37="")*('Course Content'!I37=""),"—",IFERROR('Course Content'!D17*1,0)+IFERROR('Course Content'!I17*1,0)+IFERROR('Course Content'!D37*1,0)+IFERROR('Course Content'!I37*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="59">
         <f>IFERROR(IF(K20="","",IF(K20="—","",FLOOR(K20/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M20" s="62">
+      <c r="M20" s="60">
         <f>IFERROR(IF(L20="","",IF(L20="—","",FLOOR(L20/I20,1))),"")</f>
         <v/>
       </c>
       <c r="N20" s="26" t="n"/>
-      <c r="O20" s="63">
-        <f>IFERROR(IF(('Course Content'!E17="")*('Course Content'!J17="")*('Course Content'!E33="")*('Course Content'!J33=""),"—",IFERROR('Course Content'!E17*1,0)+IFERROR('Course Content'!J17*1,0)+IFERROR('Course Content'!E33*1,0)+IFERROR('Course Content'!J33*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P20" s="63">
+      <c r="O20" s="61">
+        <f>IFERROR(IF(('Course Content'!E17="")*('Course Content'!J17="")*('Course Content'!E37="")*('Course Content'!J37=""),"—",IFERROR('Course Content'!E17*1,0)+IFERROR('Course Content'!J17*1,0)+IFERROR('Course Content'!E37*1,0)+IFERROR('Course Content'!J37*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P20" s="61">
         <f>IFERROR(IF(O20="","",IF(O20="—","",FLOOR(O20/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q20" s="64">
+      <c r="Q20" s="62">
         <f>IFERROR(IF(P20="","",IF(P20="—","",FLOOR(P20/I20,1))),"")</f>
         <v/>
       </c>
-      <c r="R20" s="66">
-        <f>IFERROR(IF('Course Content'!C33&lt;&gt;"",'Course Content'!C33,IF('Course Content'!H33&lt;&gt;"",'Course Content'!H33,IF('Course Content'!C17&lt;&gt;"",'Course Content'!C17,'Course Content'!H17))),"")</f>
+      <c r="R20" s="64">
+        <f>IFERROR(IF('Course Content'!C37&lt;&gt;"",'Course Content'!C37,IF('Course Content'!H37&lt;&gt;"",'Course Content'!H37,IF('Course Content'!C17&lt;&gt;"",'Course Content'!C17,'Course Content'!H17))),"")</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="31">
-        <f>IF('Course Content'!A34="Other 1","Other 1",'Course Content'!A34)</f>
+        <f>IF('Course Content'!A38="Other 1","Other 1",'Course Content'!A38)</f>
         <v/>
       </c>
       <c r="B21" s="5">
-        <f>IFERROR(IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C21" s="60" t="n"/>
-      <c r="D21" s="60" t="n"/>
-      <c r="E21" s="60" t="n"/>
-      <c r="F21" s="60" t="n"/>
-      <c r="G21" s="60" t="n"/>
-      <c r="H21" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B38&lt;&gt;"",'Course Content'!B38,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,IF('Course Content'!G38&lt;&gt;"",'Course Content'!G38,IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C21" s="58" t="n"/>
+      <c r="D21" s="58" t="n"/>
+      <c r="E21" s="58" t="n"/>
+      <c r="F21" s="58" t="n"/>
+      <c r="G21" s="58" t="n"/>
+      <c r="H21" s="58" t="n"/>
       <c r="I21" s="17">
         <f>IF(COUNTA(C21:H21)=0,$I$8,COUNTA(C21:H21))</f>
         <v/>
       </c>
       <c r="J21" s="26" t="n"/>
-      <c r="K21" s="61">
-        <f>IFERROR(IF(('Course Content'!D18="")*('Course Content'!I18="")*('Course Content'!D34="")*('Course Content'!I34=""),"—",IFERROR('Course Content'!D18*1,0)+IFERROR('Course Content'!I18*1,0)+IFERROR('Course Content'!D34*1,0)+IFERROR('Course Content'!I34*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L21" s="61">
+      <c r="K21" s="59">
+        <f>IFERROR(IF(('Course Content'!D18="")*('Course Content'!I18="")*('Course Content'!D38="")*('Course Content'!I38=""),"—",IFERROR('Course Content'!D18*1,0)+IFERROR('Course Content'!I18*1,0)+IFERROR('Course Content'!D38*1,0)+IFERROR('Course Content'!I38*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L21" s="59">
         <f>IFERROR(IF(K21="","",IF(K21="—","",FLOOR(K21/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M21" s="62">
+      <c r="M21" s="60">
         <f>IFERROR(IF(L21="","",IF(L21="—","",FLOOR(L21/I21,1))),"")</f>
         <v/>
       </c>
       <c r="N21" s="26" t="n"/>
-      <c r="O21" s="63">
-        <f>IFERROR(IF(('Course Content'!E18="")*('Course Content'!J18="")*('Course Content'!E34="")*('Course Content'!J34=""),"—",IFERROR('Course Content'!E18*1,0)+IFERROR('Course Content'!J18*1,0)+IFERROR('Course Content'!E34*1,0)+IFERROR('Course Content'!J34*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P21" s="63">
+      <c r="O21" s="61">
+        <f>IFERROR(IF(('Course Content'!E18="")*('Course Content'!J18="")*('Course Content'!E38="")*('Course Content'!J38=""),"—",IFERROR('Course Content'!E18*1,0)+IFERROR('Course Content'!J18*1,0)+IFERROR('Course Content'!E38*1,0)+IFERROR('Course Content'!J38*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P21" s="61">
         <f>IFERROR(IF(O21="","",IF(O21="—","",FLOOR(O21/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q21" s="64">
+      <c r="Q21" s="62">
         <f>IFERROR(IF(P21="","",IF(P21="—","",FLOOR(P21/I21,1))),"")</f>
         <v/>
       </c>
-      <c r="R21" s="65">
-        <f>IFERROR(IF('Course Content'!C34&lt;&gt;"",'Course Content'!C34,IF('Course Content'!H34&lt;&gt;"",'Course Content'!H34,IF('Course Content'!C18&lt;&gt;"",'Course Content'!C18,'Course Content'!H18))),"")</f>
+      <c r="R21" s="63">
+        <f>IFERROR(IF('Course Content'!C38&lt;&gt;"",'Course Content'!C38,IF('Course Content'!H38&lt;&gt;"",'Course Content'!H38,IF('Course Content'!C18&lt;&gt;"",'Course Content'!C18,'Course Content'!H18))),"")</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="31">
-        <f>IF('Course Content'!A35="Other 2","Other 2",'Course Content'!A35)</f>
+        <f>IF('Course Content'!A39="Other 2","Other 2",'Course Content'!A39)</f>
         <v/>
       </c>
       <c r="B22" s="18">
-        <f>IFERROR(IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C22" s="60" t="n"/>
-      <c r="D22" s="60" t="n"/>
-      <c r="E22" s="60" t="n"/>
-      <c r="F22" s="60" t="n"/>
-      <c r="G22" s="60" t="n"/>
-      <c r="H22" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B39&lt;&gt;"",'Course Content'!B39,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,IF('Course Content'!G39&lt;&gt;"",'Course Content'!G39,IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C22" s="58" t="n"/>
+      <c r="D22" s="58" t="n"/>
+      <c r="E22" s="58" t="n"/>
+      <c r="F22" s="58" t="n"/>
+      <c r="G22" s="58" t="n"/>
+      <c r="H22" s="58" t="n"/>
       <c r="I22" s="17">
         <f>IF(COUNTA(C22:H22)=0,$I$8,COUNTA(C22:H22))</f>
         <v/>
       </c>
       <c r="J22" s="26" t="n"/>
-      <c r="K22" s="61">
-        <f>IFERROR(IF(('Course Content'!D19="")*('Course Content'!I19="")*('Course Content'!D35="")*('Course Content'!I35=""),"—",IFERROR('Course Content'!D19*1,0)+IFERROR('Course Content'!I19*1,0)+IFERROR('Course Content'!D35*1,0)+IFERROR('Course Content'!I35*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L22" s="61">
+      <c r="K22" s="59">
+        <f>IFERROR(IF(('Course Content'!D19="")*('Course Content'!I19="")*('Course Content'!D39="")*('Course Content'!I39=""),"—",IFERROR('Course Content'!D19*1,0)+IFERROR('Course Content'!I19*1,0)+IFERROR('Course Content'!D39*1,0)+IFERROR('Course Content'!I39*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L22" s="59">
         <f>IFERROR(IF(K22="","",IF(K22="—","",FLOOR(K22/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M22" s="62">
+      <c r="M22" s="60">
         <f>IFERROR(IF(L22="","",IF(L22="—","",FLOOR(L22/I22,1))),"")</f>
         <v/>
       </c>
       <c r="N22" s="26" t="n"/>
-      <c r="O22" s="63">
-        <f>IFERROR(IF(('Course Content'!E19="")*('Course Content'!J19="")*('Course Content'!E35="")*('Course Content'!J35=""),"—",IFERROR('Course Content'!E19*1,0)+IFERROR('Course Content'!J19*1,0)+IFERROR('Course Content'!E35*1,0)+IFERROR('Course Content'!J35*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P22" s="63">
+      <c r="O22" s="61">
+        <f>IFERROR(IF(('Course Content'!E19="")*('Course Content'!J19="")*('Course Content'!E39="")*('Course Content'!J39=""),"—",IFERROR('Course Content'!E19*1,0)+IFERROR('Course Content'!J19*1,0)+IFERROR('Course Content'!E39*1,0)+IFERROR('Course Content'!J39*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P22" s="61">
         <f>IFERROR(IF(O22="","",IF(O22="—","",FLOOR(O22/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q22" s="64">
+      <c r="Q22" s="62">
         <f>IFERROR(IF(P22="","",IF(P22="—","",FLOOR(P22/I22,1))),"")</f>
         <v/>
       </c>
-      <c r="R22" s="66">
-        <f>IFERROR(IF('Course Content'!C35&lt;&gt;"",'Course Content'!C35,IF('Course Content'!H35&lt;&gt;"",'Course Content'!H35,IF('Course Content'!C19&lt;&gt;"",'Course Content'!C19,'Course Content'!H19))),"")</f>
+      <c r="R22" s="64">
+        <f>IFERROR(IF('Course Content'!C39&lt;&gt;"",'Course Content'!C39,IF('Course Content'!H39&lt;&gt;"",'Course Content'!H39,IF('Course Content'!C19&lt;&gt;"",'Course Content'!C19,'Course Content'!H19))),"")</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="31">
-        <f>IF('Course Content'!A36="Other 3","Other 3",'Course Content'!A36)</f>
+        <f>IF('Course Content'!A40="Other 3","Other 3",'Course Content'!A40)</f>
         <v/>
       </c>
       <c r="B23" s="5">
-        <f>IFERROR(IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C23" s="60" t="n"/>
-      <c r="D23" s="60" t="n"/>
-      <c r="E23" s="60" t="n"/>
-      <c r="F23" s="60" t="n"/>
-      <c r="G23" s="60" t="n"/>
-      <c r="H23" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B40&lt;&gt;"",'Course Content'!B40,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,IF('Course Content'!G40&lt;&gt;"",'Course Content'!G40,IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C23" s="58" t="n"/>
+      <c r="D23" s="58" t="n"/>
+      <c r="E23" s="58" t="n"/>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="58" t="n"/>
+      <c r="H23" s="58" t="n"/>
       <c r="I23" s="17">
         <f>IF(COUNTA(C23:H23)=0,$I$8,COUNTA(C23:H23))</f>
         <v/>
       </c>
       <c r="J23" s="26" t="n"/>
-      <c r="K23" s="61">
-        <f>IFERROR(IF(('Course Content'!D20="")*('Course Content'!I20="")*('Course Content'!D36="")*('Course Content'!I36=""),"—",IFERROR('Course Content'!D20*1,0)+IFERROR('Course Content'!I20*1,0)+IFERROR('Course Content'!D36*1,0)+IFERROR('Course Content'!I36*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L23" s="61">
+      <c r="K23" s="59">
+        <f>IFERROR(IF(('Course Content'!D20="")*('Course Content'!I20="")*('Course Content'!D40="")*('Course Content'!I40=""),"—",IFERROR('Course Content'!D20*1,0)+IFERROR('Course Content'!I20*1,0)+IFERROR('Course Content'!D40*1,0)+IFERROR('Course Content'!I40*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="59">
         <f>IFERROR(IF(K23="","",IF(K23="—","",FLOOR(K23/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M23" s="62">
+      <c r="M23" s="60">
         <f>IFERROR(IF(L23="","",IF(L23="—","",FLOOR(L23/I23,1))),"")</f>
         <v/>
       </c>
       <c r="N23" s="26" t="n"/>
-      <c r="O23" s="63">
-        <f>IFERROR(IF(('Course Content'!E20="")*('Course Content'!J20="")*('Course Content'!E36="")*('Course Content'!J36=""),"—",IFERROR('Course Content'!E20*1,0)+IFERROR('Course Content'!J20*1,0)+IFERROR('Course Content'!E36*1,0)+IFERROR('Course Content'!J36*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P23" s="63">
+      <c r="O23" s="61">
+        <f>IFERROR(IF(('Course Content'!E20="")*('Course Content'!J20="")*('Course Content'!E40="")*('Course Content'!J40=""),"—",IFERROR('Course Content'!E20*1,0)+IFERROR('Course Content'!J20*1,0)+IFERROR('Course Content'!E40*1,0)+IFERROR('Course Content'!J40*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P23" s="61">
         <f>IFERROR(IF(O23="","",IF(O23="—","",FLOOR(O23/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q23" s="64">
+      <c r="Q23" s="62">
         <f>IFERROR(IF(P23="","",IF(P23="—","",FLOOR(P23/I23,1))),"")</f>
         <v/>
       </c>
-      <c r="R23" s="65">
-        <f>IFERROR(IF('Course Content'!C36&lt;&gt;"",'Course Content'!C36,IF('Course Content'!H36&lt;&gt;"",'Course Content'!H36,IF('Course Content'!C20&lt;&gt;"",'Course Content'!C20,'Course Content'!H20))),"")</f>
+      <c r="R23" s="63">
+        <f>IFERROR(IF('Course Content'!C40&lt;&gt;"",'Course Content'!C40,IF('Course Content'!H40&lt;&gt;"",'Course Content'!H40,IF('Course Content'!C20&lt;&gt;"",'Course Content'!C20,'Course Content'!H20))),"")</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="31">
-        <f>IF('Course Content'!A37="Other 4","Other 4",'Course Content'!A37)</f>
+        <f>IF('Course Content'!A41="Other 4","Other 4",'Course Content'!A41)</f>
         <v/>
       </c>
       <c r="B24" s="18">
-        <f>IFERROR(IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C24" s="60" t="n"/>
-      <c r="D24" s="60" t="n"/>
-      <c r="E24" s="60" t="n"/>
-      <c r="F24" s="60" t="n"/>
-      <c r="G24" s="60" t="n"/>
-      <c r="H24" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B41&lt;&gt;"",'Course Content'!B41,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,IF('Course Content'!G41&lt;&gt;"",'Course Content'!G41,IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C24" s="58" t="n"/>
+      <c r="D24" s="58" t="n"/>
+      <c r="E24" s="58" t="n"/>
+      <c r="F24" s="58" t="n"/>
+      <c r="G24" s="58" t="n"/>
+      <c r="H24" s="58" t="n"/>
       <c r="I24" s="17">
         <f>IF(COUNTA(C24:H24)=0,$I$8,COUNTA(C24:H24))</f>
         <v/>
       </c>
       <c r="J24" s="26" t="n"/>
-      <c r="K24" s="61">
-        <f>IFERROR(IF(('Course Content'!D21="")*('Course Content'!I21="")*('Course Content'!D37="")*('Course Content'!I37=""),"—",IFERROR('Course Content'!D21*1,0)+IFERROR('Course Content'!I21*1,0)+IFERROR('Course Content'!D37*1,0)+IFERROR('Course Content'!I37*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L24" s="61">
+      <c r="K24" s="59">
+        <f>IFERROR(IF(('Course Content'!D21="")*('Course Content'!I21="")*('Course Content'!D41="")*('Course Content'!I41=""),"—",IFERROR('Course Content'!D21*1,0)+IFERROR('Course Content'!I21*1,0)+IFERROR('Course Content'!D41*1,0)+IFERROR('Course Content'!I41*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="59">
         <f>IFERROR(IF(K24="","",IF(K24="—","",FLOOR(K24/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M24" s="62">
+      <c r="M24" s="60">
         <f>IFERROR(IF(L24="","",IF(L24="—","",FLOOR(L24/I24,1))),"")</f>
         <v/>
       </c>
       <c r="N24" s="26" t="n"/>
-      <c r="O24" s="63">
-        <f>IFERROR(IF(('Course Content'!E21="")*('Course Content'!J21="")*('Course Content'!E37="")*('Course Content'!J37=""),"—",IFERROR('Course Content'!E21*1,0)+IFERROR('Course Content'!J21*1,0)+IFERROR('Course Content'!E37*1,0)+IFERROR('Course Content'!J37*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P24" s="63">
+      <c r="O24" s="61">
+        <f>IFERROR(IF(('Course Content'!E21="")*('Course Content'!J21="")*('Course Content'!E41="")*('Course Content'!J41=""),"—",IFERROR('Course Content'!E21*1,0)+IFERROR('Course Content'!J21*1,0)+IFERROR('Course Content'!E41*1,0)+IFERROR('Course Content'!J41*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P24" s="61">
         <f>IFERROR(IF(O24="","",IF(O24="—","",FLOOR(O24/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q24" s="64">
+      <c r="Q24" s="62">
         <f>IFERROR(IF(P24="","",IF(P24="—","",FLOOR(P24/I24,1))),"")</f>
         <v/>
       </c>
-      <c r="R24" s="66">
-        <f>IFERROR(IF('Course Content'!C37&lt;&gt;"",'Course Content'!C37,IF('Course Content'!H37&lt;&gt;"",'Course Content'!H37,IF('Course Content'!C21&lt;&gt;"",'Course Content'!C21,'Course Content'!H21))),"")</f>
+      <c r="R24" s="64">
+        <f>IFERROR(IF('Course Content'!C41&lt;&gt;"",'Course Content'!C41,IF('Course Content'!H41&lt;&gt;"",'Course Content'!H41,IF('Course Content'!C21&lt;&gt;"",'Course Content'!C21,'Course Content'!H21))),"")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="31">
-        <f>IF('Course Content'!A38="Other 5","Other 5",'Course Content'!A38)</f>
+        <f>IF('Course Content'!A42="Other 5","Other 5",'Course Content'!A42)</f>
         <v/>
       </c>
       <c r="B25" s="5">
-        <f>IFERROR(IF('Course Content'!B38&lt;&gt;"",'Course Content'!B38,IF('Course Content'!B22&lt;&gt;"","[Grp] "&amp;'Course Content'!B22,IF('Course Content'!G38&lt;&gt;"",'Course Content'!G38,IF('Course Content'!G22&lt;&gt;"","[Grp] "&amp;'Course Content'!G22,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C25" s="60" t="n"/>
-      <c r="D25" s="60" t="n"/>
-      <c r="E25" s="60" t="n"/>
-      <c r="F25" s="60" t="n"/>
-      <c r="G25" s="60" t="n"/>
-      <c r="H25" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B42&lt;&gt;"",'Course Content'!B42,IF('Course Content'!B22&lt;&gt;"","[Grp] "&amp;'Course Content'!B22,IF('Course Content'!G42&lt;&gt;"",'Course Content'!G42,IF('Course Content'!G22&lt;&gt;"","[Grp] "&amp;'Course Content'!G22,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C25" s="58" t="n"/>
+      <c r="D25" s="58" t="n"/>
+      <c r="E25" s="58" t="n"/>
+      <c r="F25" s="58" t="n"/>
+      <c r="G25" s="58" t="n"/>
+      <c r="H25" s="58" t="n"/>
       <c r="I25" s="17">
         <f>IF(COUNTA(C25:H25)=0,$I$8,COUNTA(C25:H25))</f>
         <v/>
       </c>
       <c r="J25" s="26" t="n"/>
-      <c r="K25" s="61">
-        <f>IFERROR(IF(('Course Content'!D22="")*('Course Content'!I22="")*('Course Content'!D38="")*('Course Content'!I38=""),"—",IFERROR('Course Content'!D22*1,0)+IFERROR('Course Content'!I22*1,0)+IFERROR('Course Content'!D38*1,0)+IFERROR('Course Content'!I38*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L25" s="61">
+      <c r="K25" s="59">
+        <f>IFERROR(IF(('Course Content'!D22="")*('Course Content'!I22="")*('Course Content'!D42="")*('Course Content'!I42=""),"—",IFERROR('Course Content'!D22*1,0)+IFERROR('Course Content'!I22*1,0)+IFERROR('Course Content'!D42*1,0)+IFERROR('Course Content'!I42*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="59">
         <f>IFERROR(IF(K25="","",IF(K25="—","",FLOOR(K25/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M25" s="62">
+      <c r="M25" s="60">
         <f>IFERROR(IF(L25="","",IF(L25="—","",FLOOR(L25/I25,1))),"")</f>
         <v/>
       </c>
       <c r="N25" s="26" t="n"/>
-      <c r="O25" s="63">
-        <f>IFERROR(IF(('Course Content'!E22="")*('Course Content'!J22="")*('Course Content'!E38="")*('Course Content'!J38=""),"—",IFERROR('Course Content'!E22*1,0)+IFERROR('Course Content'!J22*1,0)+IFERROR('Course Content'!E38*1,0)+IFERROR('Course Content'!J38*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P25" s="63">
+      <c r="O25" s="61">
+        <f>IFERROR(IF(('Course Content'!E22="")*('Course Content'!J22="")*('Course Content'!E42="")*('Course Content'!J42=""),"—",IFERROR('Course Content'!E22*1,0)+IFERROR('Course Content'!J22*1,0)+IFERROR('Course Content'!E42*1,0)+IFERROR('Course Content'!J42*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P25" s="61">
         <f>IFERROR(IF(O25="","",IF(O25="—","",FLOOR(O25/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q25" s="64">
+      <c r="Q25" s="62">
         <f>IFERROR(IF(P25="","",IF(P25="—","",FLOOR(P25/I25,1))),"")</f>
         <v/>
       </c>
-      <c r="R25" s="65">
-        <f>IFERROR(IF('Course Content'!C38&lt;&gt;"",'Course Content'!C38,IF('Course Content'!H38&lt;&gt;"",'Course Content'!H38,IF('Course Content'!C22&lt;&gt;"",'Course Content'!C22,'Course Content'!H22))),"")</f>
+      <c r="R25" s="63">
+        <f>IFERROR(IF('Course Content'!C42&lt;&gt;"",'Course Content'!C42,IF('Course Content'!H42&lt;&gt;"",'Course Content'!H42,IF('Course Content'!C22&lt;&gt;"",'Course Content'!C22,'Course Content'!H22))),"")</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="31">
-        <f>IF('Course Content'!A39="Other 6","Other 6",'Course Content'!A39)</f>
+        <f>IF('Course Content'!A43="Other 6","Other 6",'Course Content'!A43)</f>
         <v/>
       </c>
       <c r="B26" s="18">
-        <f>IFERROR(IF('Course Content'!B39&lt;&gt;"",'Course Content'!B39,IF('Course Content'!B23&lt;&gt;"","[Grp] "&amp;'Course Content'!B23,IF('Course Content'!G39&lt;&gt;"",'Course Content'!G39,IF('Course Content'!G23&lt;&gt;"","[Grp] "&amp;'Course Content'!G23,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C26" s="60" t="n"/>
-      <c r="D26" s="60" t="n"/>
-      <c r="E26" s="60" t="n"/>
-      <c r="F26" s="60" t="n"/>
-      <c r="G26" s="60" t="n"/>
-      <c r="H26" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B43&lt;&gt;"",'Course Content'!B43,IF('Course Content'!B23&lt;&gt;"","[Grp] "&amp;'Course Content'!B23,IF('Course Content'!G43&lt;&gt;"",'Course Content'!G43,IF('Course Content'!G23&lt;&gt;"","[Grp] "&amp;'Course Content'!G23,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C26" s="58" t="n"/>
+      <c r="D26" s="58" t="n"/>
+      <c r="E26" s="58" t="n"/>
+      <c r="F26" s="58" t="n"/>
+      <c r="G26" s="58" t="n"/>
+      <c r="H26" s="58" t="n"/>
       <c r="I26" s="17">
         <f>IF(COUNTA(C26:H26)=0,$I$8,COUNTA(C26:H26))</f>
         <v/>
       </c>
       <c r="J26" s="26" t="n"/>
-      <c r="K26" s="61">
-        <f>IFERROR(IF(('Course Content'!D23="")*('Course Content'!I23="")*('Course Content'!D39="")*('Course Content'!I39=""),"—",IFERROR('Course Content'!D23*1,0)+IFERROR('Course Content'!I23*1,0)+IFERROR('Course Content'!D39*1,0)+IFERROR('Course Content'!I39*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L26" s="61">
+      <c r="K26" s="59">
+        <f>IFERROR(IF(('Course Content'!D23="")*('Course Content'!I23="")*('Course Content'!D43="")*('Course Content'!I43=""),"—",IFERROR('Course Content'!D23*1,0)+IFERROR('Course Content'!I23*1,0)+IFERROR('Course Content'!D43*1,0)+IFERROR('Course Content'!I43*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="59">
         <f>IFERROR(IF(K26="","",IF(K26="—","",FLOOR(K26/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M26" s="62">
+      <c r="M26" s="60">
         <f>IFERROR(IF(L26="","",IF(L26="—","",FLOOR(L26/I26,1))),"")</f>
         <v/>
       </c>
       <c r="N26" s="26" t="n"/>
-      <c r="O26" s="63">
-        <f>IFERROR(IF(('Course Content'!E23="")*('Course Content'!J23="")*('Course Content'!E39="")*('Course Content'!J39=""),"—",IFERROR('Course Content'!E23*1,0)+IFERROR('Course Content'!J23*1,0)+IFERROR('Course Content'!E39*1,0)+IFERROR('Course Content'!J39*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P26" s="63">
+      <c r="O26" s="61">
+        <f>IFERROR(IF(('Course Content'!E23="")*('Course Content'!J23="")*('Course Content'!E43="")*('Course Content'!J43=""),"—",IFERROR('Course Content'!E23*1,0)+IFERROR('Course Content'!J23*1,0)+IFERROR('Course Content'!E43*1,0)+IFERROR('Course Content'!J43*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P26" s="61">
         <f>IFERROR(IF(O26="","",IF(O26="—","",FLOOR(O26/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q26" s="64">
+      <c r="Q26" s="62">
         <f>IFERROR(IF(P26="","",IF(P26="—","",FLOOR(P26/I26,1))),"")</f>
         <v/>
       </c>
-      <c r="R26" s="66">
-        <f>IFERROR(IF('Course Content'!C39&lt;&gt;"",'Course Content'!C39,IF('Course Content'!H39&lt;&gt;"",'Course Content'!H39,IF('Course Content'!C23&lt;&gt;"",'Course Content'!C23,'Course Content'!H23))),"")</f>
+      <c r="R26" s="64">
+        <f>IFERROR(IF('Course Content'!C43&lt;&gt;"",'Course Content'!C43,IF('Course Content'!H43&lt;&gt;"",'Course Content'!H43,IF('Course Content'!C23&lt;&gt;"",'Course Content'!C23,'Course Content'!H23))),"")</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="31">
-        <f>IF('Course Content'!A40="Other 7","Other 7",'Course Content'!A40)</f>
+        <f>IF('Course Content'!A44="Other 7","Other 7",'Course Content'!A44)</f>
         <v/>
       </c>
       <c r="B27" s="5">
-        <f>IFERROR(IF('Course Content'!B40&lt;&gt;"",'Course Content'!B40,IF('Course Content'!B24&lt;&gt;"","[Grp] "&amp;'Course Content'!B24,IF('Course Content'!G40&lt;&gt;"",'Course Content'!G40,IF('Course Content'!G24&lt;&gt;"","[Grp] "&amp;'Course Content'!G24,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C27" s="60" t="n"/>
-      <c r="D27" s="60" t="n"/>
-      <c r="E27" s="60" t="n"/>
-      <c r="F27" s="60" t="n"/>
-      <c r="G27" s="60" t="n"/>
-      <c r="H27" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B44&lt;&gt;"",'Course Content'!B44,IF('Course Content'!B24&lt;&gt;"","[Grp] "&amp;'Course Content'!B24,IF('Course Content'!G44&lt;&gt;"",'Course Content'!G44,IF('Course Content'!G24&lt;&gt;"","[Grp] "&amp;'Course Content'!G24,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C27" s="58" t="n"/>
+      <c r="D27" s="58" t="n"/>
+      <c r="E27" s="58" t="n"/>
+      <c r="F27" s="58" t="n"/>
+      <c r="G27" s="58" t="n"/>
+      <c r="H27" s="58" t="n"/>
       <c r="I27" s="17">
         <f>IF(COUNTA(C27:H27)=0,$I$8,COUNTA(C27:H27))</f>
         <v/>
       </c>
       <c r="J27" s="26" t="n"/>
-      <c r="K27" s="61">
-        <f>IFERROR(IF(('Course Content'!D24="")*('Course Content'!I24="")*('Course Content'!D40="")*('Course Content'!I40=""),"—",IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)+IFERROR('Course Content'!D40*1,0)+IFERROR('Course Content'!I40*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L27" s="61">
+      <c r="K27" s="59">
+        <f>IFERROR(IF(('Course Content'!D24="")*('Course Content'!I24="")*('Course Content'!D44="")*('Course Content'!I44=""),"—",IFERROR('Course Content'!D24*1,0)+IFERROR('Course Content'!I24*1,0)+IFERROR('Course Content'!D44*1,0)+IFERROR('Course Content'!I44*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="59">
         <f>IFERROR(IF(K27="","",IF(K27="—","",FLOOR(K27/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M27" s="62">
+      <c r="M27" s="60">
         <f>IFERROR(IF(L27="","",IF(L27="—","",FLOOR(L27/I27,1))),"")</f>
         <v/>
       </c>
       <c r="N27" s="26" t="n"/>
-      <c r="O27" s="63">
-        <f>IFERROR(IF(('Course Content'!E24="")*('Course Content'!J24="")*('Course Content'!E40="")*('Course Content'!J40=""),"—",IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)+IFERROR('Course Content'!E40*1,0)+IFERROR('Course Content'!J40*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P27" s="63">
+      <c r="O27" s="61">
+        <f>IFERROR(IF(('Course Content'!E24="")*('Course Content'!J24="")*('Course Content'!E44="")*('Course Content'!J44=""),"—",IFERROR('Course Content'!E24*1,0)+IFERROR('Course Content'!J24*1,0)+IFERROR('Course Content'!E44*1,0)+IFERROR('Course Content'!J44*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P27" s="61">
         <f>IFERROR(IF(O27="","",IF(O27="—","",FLOOR(O27/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q27" s="64">
+      <c r="Q27" s="62">
         <f>IFERROR(IF(P27="","",IF(P27="—","",FLOOR(P27/I27,1))),"")</f>
         <v/>
       </c>
-      <c r="R27" s="65">
-        <f>IFERROR(IF('Course Content'!C40&lt;&gt;"",'Course Content'!C40,IF('Course Content'!H40&lt;&gt;"",'Course Content'!H40,IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,'Course Content'!H24))),"")</f>
+      <c r="R27" s="63">
+        <f>IFERROR(IF('Course Content'!C44&lt;&gt;"",'Course Content'!C44,IF('Course Content'!H44&lt;&gt;"",'Course Content'!H44,IF('Course Content'!C24&lt;&gt;"",'Course Content'!C24,'Course Content'!H24))),"")</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="31">
-        <f>IF('Course Content'!A41="Other 8","Other 8",'Course Content'!A41)</f>
+        <f>IF('Course Content'!A45="Other 8","Other 8",'Course Content'!A45)</f>
         <v/>
       </c>
       <c r="B28" s="18">
-        <f>IFERROR(IF('Course Content'!B41&lt;&gt;"",'Course Content'!B41,IF('Course Content'!B25&lt;&gt;"","[Grp] "&amp;'Course Content'!B25,IF('Course Content'!G41&lt;&gt;"",'Course Content'!G41,IF('Course Content'!G25&lt;&gt;"","[Grp] "&amp;'Course Content'!G25,"—")))),"—")</f>
-        <v/>
-      </c>
-      <c r="C28" s="60" t="n"/>
-      <c r="D28" s="60" t="n"/>
-      <c r="E28" s="60" t="n"/>
-      <c r="F28" s="60" t="n"/>
-      <c r="G28" s="60" t="n"/>
-      <c r="H28" s="60" t="n"/>
+        <f>IFERROR(IF('Course Content'!B45&lt;&gt;"",'Course Content'!B45,IF('Course Content'!B25&lt;&gt;"","[Grp] "&amp;'Course Content'!B25,IF('Course Content'!G45&lt;&gt;"",'Course Content'!G45,IF('Course Content'!G25&lt;&gt;"","[Grp] "&amp;'Course Content'!G25,"—")))),"—")</f>
+        <v/>
+      </c>
+      <c r="C28" s="58" t="n"/>
+      <c r="D28" s="58" t="n"/>
+      <c r="E28" s="58" t="n"/>
+      <c r="F28" s="58" t="n"/>
+      <c r="G28" s="58" t="n"/>
+      <c r="H28" s="58" t="n"/>
       <c r="I28" s="17">
         <f>IF(COUNTA(C28:H28)=0,$I$8,COUNTA(C28:H28))</f>
         <v/>
       </c>
       <c r="J28" s="26" t="n"/>
-      <c r="K28" s="61">
-        <f>IFERROR(IF(('Course Content'!D25="")*('Course Content'!I25="")*('Course Content'!D41="")*('Course Content'!I41=""),"—",IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)+IFERROR('Course Content'!D41*1,0)+IFERROR('Course Content'!I41*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="L28" s="61">
+      <c r="K28" s="59">
+        <f>IFERROR(IF(('Course Content'!D25="")*('Course Content'!I25="")*('Course Content'!D45="")*('Course Content'!I45=""),"—",IFERROR('Course Content'!D25*1,0)+IFERROR('Course Content'!I25*1,0)+IFERROR('Course Content'!D45*1,0)+IFERROR('Course Content'!I45*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="59">
         <f>IFERROR(IF(K28="","",IF(K28="—","",FLOOR(K28/'Getting Started'!C15,1))),"")</f>
         <v/>
       </c>
-      <c r="M28" s="62">
+      <c r="M28" s="60">
         <f>IFERROR(IF(L28="","",IF(L28="—","",FLOOR(L28/I28,1))),"")</f>
         <v/>
       </c>
       <c r="N28" s="26" t="n"/>
-      <c r="O28" s="63">
-        <f>IFERROR(IF(('Course Content'!E25="")*('Course Content'!J25="")*('Course Content'!E41="")*('Course Content'!J41=""),"—",IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)+IFERROR('Course Content'!E41*1,0)+IFERROR('Course Content'!J41*1,0)),"")</f>
-        <v/>
-      </c>
-      <c r="P28" s="63">
+      <c r="O28" s="61">
+        <f>IFERROR(IF(('Course Content'!E25="")*('Course Content'!J25="")*('Course Content'!E45="")*('Course Content'!J45=""),"—",IFERROR('Course Content'!E25*1,0)+IFERROR('Course Content'!J25*1,0)+IFERROR('Course Content'!E45*1,0)+IFERROR('Course Content'!J45*1,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P28" s="61">
         <f>IFERROR(IF(O28="","",IF(O28="—","",FLOOR(O28/'Getting Started'!C23,1))),"")</f>
         <v/>
       </c>
-      <c r="Q28" s="64">
+      <c r="Q28" s="62">
         <f>IFERROR(IF(P28="","",IF(P28="—","",FLOOR(P28/I28,1))),"")</f>
         <v/>
       </c>
-      <c r="R28" s="66">
-        <f>IFERROR(IF('Course Content'!C41&lt;&gt;"",'Course Content'!C41,IF('Course Content'!H41&lt;&gt;"",'Course Content'!H41,IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,'Course Content'!H25))),"")</f>
+      <c r="R28" s="64">
+        <f>IFERROR(IF('Course Content'!C45&lt;&gt;"",'Course Content'!C45,IF('Course Content'!H45&lt;&gt;"",'Course Content'!H45,IF('Course Content'!C25&lt;&gt;"",'Course Content'!C25,'Course Content'!H25))),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Show all curriculum slots in student schedule curriculum column
Changed col B from first-non-blank to TEXTJOIN of all non-blank titles
(Group Slot 1 & 2 prefixed [Grp], Individual Slot 1 & 2 plain).
wrap_text stays off so row height is never affected by long strings.
Totals were already correct — this fixes the visibility issue only.

https://claude.ai/code/session_01LsZPQzKg22cdQ6reZhSm9C
</commit_message>
<xml_diff>
--- a/Homeschool_Curriculum_Planner.xlsx
+++ b/Homeschool_Curriculum_Planner.xlsx
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>IFERROR(IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B8&lt;&gt;"","[Grp] "&amp;'Course Content'!B8,""),IF('Course Content'!G8&lt;&gt;"","[Grp] "&amp;'Course Content'!G8,""),IF('Course Content'!B28&lt;&gt;"",'Course Content'!B28,""),IF('Course Content'!G28&lt;&gt;"",'Course Content'!G28,"")),"—")</f>
         <v/>
       </c>
       <c r="C11" s="58" t="n"/>
@@ -6738,7 +6738,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>IFERROR(IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B9&lt;&gt;"","[Grp] "&amp;'Course Content'!B9,""),IF('Course Content'!G9&lt;&gt;"","[Grp] "&amp;'Course Content'!G9,""),IF('Course Content'!B29&lt;&gt;"",'Course Content'!B29,""),IF('Course Content'!G29&lt;&gt;"",'Course Content'!G29,"")),"—")</f>
         <v/>
       </c>
       <c r="C12" s="58" t="n"/>
@@ -6789,7 +6789,7 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>IFERROR(IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B10&lt;&gt;"","[Grp] "&amp;'Course Content'!B10,""),IF('Course Content'!G10&lt;&gt;"","[Grp] "&amp;'Course Content'!G10,""),IF('Course Content'!B30&lt;&gt;"",'Course Content'!B30,""),IF('Course Content'!G30&lt;&gt;"",'Course Content'!G30,"")),"—")</f>
         <v/>
       </c>
       <c r="C13" s="58" t="n"/>
@@ -6840,7 +6840,7 @@
         </is>
       </c>
       <c r="B14" s="18">
-        <f>IFERROR(IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B11&lt;&gt;"","[Grp] "&amp;'Course Content'!B11,""),IF('Course Content'!G11&lt;&gt;"","[Grp] "&amp;'Course Content'!G11,""),IF('Course Content'!B31&lt;&gt;"",'Course Content'!B31,""),IF('Course Content'!G31&lt;&gt;"",'Course Content'!G31,"")),"—")</f>
         <v/>
       </c>
       <c r="C14" s="58" t="n"/>
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>IFERROR(IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B12&lt;&gt;"","[Grp] "&amp;'Course Content'!B12,""),IF('Course Content'!G12&lt;&gt;"","[Grp] "&amp;'Course Content'!G12,""),IF('Course Content'!B32&lt;&gt;"",'Course Content'!B32,""),IF('Course Content'!G32&lt;&gt;"",'Course Content'!G32,"")),"—")</f>
         <v/>
       </c>
       <c r="C15" s="58" t="n"/>
@@ -6942,7 +6942,7 @@
         </is>
       </c>
       <c r="B16" s="18">
-        <f>IFERROR(IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B13&lt;&gt;"","[Grp] "&amp;'Course Content'!B13,""),IF('Course Content'!G13&lt;&gt;"","[Grp] "&amp;'Course Content'!G13,""),IF('Course Content'!B33&lt;&gt;"",'Course Content'!B33,""),IF('Course Content'!G33&lt;&gt;"",'Course Content'!G33,"")),"—")</f>
         <v/>
       </c>
       <c r="C16" s="58" t="n"/>
@@ -6993,7 +6993,7 @@
         </is>
       </c>
       <c r="B17" s="5">
-        <f>IFERROR(IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B14&lt;&gt;"","[Grp] "&amp;'Course Content'!B14,""),IF('Course Content'!G14&lt;&gt;"","[Grp] "&amp;'Course Content'!G14,""),IF('Course Content'!B34&lt;&gt;"",'Course Content'!B34,""),IF('Course Content'!G34&lt;&gt;"",'Course Content'!G34,"")),"—")</f>
         <v/>
       </c>
       <c r="C17" s="58" t="n"/>
@@ -7044,7 +7044,7 @@
         </is>
       </c>
       <c r="B18" s="18">
-        <f>IFERROR(IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B15&lt;&gt;"","[Grp] "&amp;'Course Content'!B15,""),IF('Course Content'!G15&lt;&gt;"","[Grp] "&amp;'Course Content'!G15,""),IF('Course Content'!B35&lt;&gt;"",'Course Content'!B35,""),IF('Course Content'!G35&lt;&gt;"",'Course Content'!G35,"")),"—")</f>
         <v/>
       </c>
       <c r="C18" s="58" t="n"/>
@@ -7095,7 +7095,7 @@
         </is>
       </c>
       <c r="B19" s="5">
-        <f>IFERROR(IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B16&lt;&gt;"","[Grp] "&amp;'Course Content'!B16,""),IF('Course Content'!G16&lt;&gt;"","[Grp] "&amp;'Course Content'!G16,""),IF('Course Content'!B36&lt;&gt;"",'Course Content'!B36,""),IF('Course Content'!G36&lt;&gt;"",'Course Content'!G36,"")),"—")</f>
         <v/>
       </c>
       <c r="C19" s="58" t="n"/>
@@ -7146,7 +7146,7 @@
         </is>
       </c>
       <c r="B20" s="18">
-        <f>IFERROR(IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B17&lt;&gt;"","[Grp] "&amp;'Course Content'!B17,""),IF('Course Content'!G17&lt;&gt;"","[Grp] "&amp;'Course Content'!G17,""),IF('Course Content'!B37&lt;&gt;"",'Course Content'!B37,""),IF('Course Content'!G37&lt;&gt;"",'Course Content'!G37,"")),"—")</f>
         <v/>
       </c>
       <c r="C20" s="58" t="n"/>
@@ -7196,7 +7196,7 @@
         <v/>
       </c>
       <c r="B21" s="5">
-        <f>IFERROR(IF('Course Content'!B38&lt;&gt;"",'Course Content'!B38,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,IF('Course Content'!G38&lt;&gt;"",'Course Content'!G38,IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B18&lt;&gt;"","[Grp] "&amp;'Course Content'!B18,""),IF('Course Content'!G18&lt;&gt;"","[Grp] "&amp;'Course Content'!G18,""),IF('Course Content'!B38&lt;&gt;"",'Course Content'!B38,""),IF('Course Content'!G38&lt;&gt;"",'Course Content'!G38,"")),"—")</f>
         <v/>
       </c>
       <c r="C21" s="58" t="n"/>
@@ -7246,7 +7246,7 @@
         <v/>
       </c>
       <c r="B22" s="18">
-        <f>IFERROR(IF('Course Content'!B39&lt;&gt;"",'Course Content'!B39,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,IF('Course Content'!G39&lt;&gt;"",'Course Content'!G39,IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B19&lt;&gt;"","[Grp] "&amp;'Course Content'!B19,""),IF('Course Content'!G19&lt;&gt;"","[Grp] "&amp;'Course Content'!G19,""),IF('Course Content'!B39&lt;&gt;"",'Course Content'!B39,""),IF('Course Content'!G39&lt;&gt;"",'Course Content'!G39,"")),"—")</f>
         <v/>
       </c>
       <c r="C22" s="58" t="n"/>
@@ -7296,7 +7296,7 @@
         <v/>
       </c>
       <c r="B23" s="5">
-        <f>IFERROR(IF('Course Content'!B40&lt;&gt;"",'Course Content'!B40,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,IF('Course Content'!G40&lt;&gt;"",'Course Content'!G40,IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B20&lt;&gt;"","[Grp] "&amp;'Course Content'!B20,""),IF('Course Content'!G20&lt;&gt;"","[Grp] "&amp;'Course Content'!G20,""),IF('Course Content'!B40&lt;&gt;"",'Course Content'!B40,""),IF('Course Content'!G40&lt;&gt;"",'Course Content'!G40,"")),"—")</f>
         <v/>
       </c>
       <c r="C23" s="58" t="n"/>
@@ -7346,7 +7346,7 @@
         <v/>
       </c>
       <c r="B24" s="18">
-        <f>IFERROR(IF('Course Content'!B41&lt;&gt;"",'Course Content'!B41,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,IF('Course Content'!G41&lt;&gt;"",'Course Content'!G41,IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B21&lt;&gt;"","[Grp] "&amp;'Course Content'!B21,""),IF('Course Content'!G21&lt;&gt;"","[Grp] "&amp;'Course Content'!G21,""),IF('Course Content'!B41&lt;&gt;"",'Course Content'!B41,""),IF('Course Content'!G41&lt;&gt;"",'Course Content'!G41,"")),"—")</f>
         <v/>
       </c>
       <c r="C24" s="58" t="n"/>
@@ -7396,7 +7396,7 @@
         <v/>
       </c>
       <c r="B25" s="5">
-        <f>IFERROR(IF('Course Content'!B42&lt;&gt;"",'Course Content'!B42,IF('Course Content'!B22&lt;&gt;"","[Grp] "&amp;'Course Content'!B22,IF('Course Content'!G42&lt;&gt;"",'Course Content'!G42,IF('Course Content'!G22&lt;&gt;"","[Grp] "&amp;'Course Content'!G22,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B22&lt;&gt;"","[Grp] "&amp;'Course Content'!B22,""),IF('Course Content'!G22&lt;&gt;"","[Grp] "&amp;'Course Content'!G22,""),IF('Course Content'!B42&lt;&gt;"",'Course Content'!B42,""),IF('Course Content'!G42&lt;&gt;"",'Course Content'!G42,"")),"—")</f>
         <v/>
       </c>
       <c r="C25" s="58" t="n"/>
@@ -7446,7 +7446,7 @@
         <v/>
       </c>
       <c r="B26" s="18">
-        <f>IFERROR(IF('Course Content'!B43&lt;&gt;"",'Course Content'!B43,IF('Course Content'!B23&lt;&gt;"","[Grp] "&amp;'Course Content'!B23,IF('Course Content'!G43&lt;&gt;"",'Course Content'!G43,IF('Course Content'!G23&lt;&gt;"","[Grp] "&amp;'Course Content'!G23,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B23&lt;&gt;"","[Grp] "&amp;'Course Content'!B23,""),IF('Course Content'!G23&lt;&gt;"","[Grp] "&amp;'Course Content'!G23,""),IF('Course Content'!B43&lt;&gt;"",'Course Content'!B43,""),IF('Course Content'!G43&lt;&gt;"",'Course Content'!G43,"")),"—")</f>
         <v/>
       </c>
       <c r="C26" s="58" t="n"/>
@@ -7496,7 +7496,7 @@
         <v/>
       </c>
       <c r="B27" s="5">
-        <f>IFERROR(IF('Course Content'!B44&lt;&gt;"",'Course Content'!B44,IF('Course Content'!B24&lt;&gt;"","[Grp] "&amp;'Course Content'!B24,IF('Course Content'!G44&lt;&gt;"",'Course Content'!G44,IF('Course Content'!G24&lt;&gt;"","[Grp] "&amp;'Course Content'!G24,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B24&lt;&gt;"","[Grp] "&amp;'Course Content'!B24,""),IF('Course Content'!G24&lt;&gt;"","[Grp] "&amp;'Course Content'!G24,""),IF('Course Content'!B44&lt;&gt;"",'Course Content'!B44,""),IF('Course Content'!G44&lt;&gt;"",'Course Content'!G44,"")),"—")</f>
         <v/>
       </c>
       <c r="C27" s="58" t="n"/>
@@ -7546,7 +7546,7 @@
         <v/>
       </c>
       <c r="B28" s="18">
-        <f>IFERROR(IF('Course Content'!B45&lt;&gt;"",'Course Content'!B45,IF('Course Content'!B25&lt;&gt;"","[Grp] "&amp;'Course Content'!B25,IF('Course Content'!G45&lt;&gt;"",'Course Content'!G45,IF('Course Content'!G25&lt;&gt;"","[Grp] "&amp;'Course Content'!G25,"—")))),"—")</f>
+        <f>IFERROR(TEXTJOIN(" · ",TRUE,IF('Course Content'!B25&lt;&gt;"","[Grp] "&amp;'Course Content'!B25,""),IF('Course Content'!G25&lt;&gt;"","[Grp] "&amp;'Course Content'!G25,""),IF('Course Content'!B45&lt;&gt;"",'Course Content'!B45,""),IF('Course Content'!G45&lt;&gt;"",'Course Content'!G45,"")),"—")</f>
         <v/>
       </c>
       <c r="C28" s="58" t="n"/>

</xml_diff>